<commit_message>
Actualiza precios Facilito 2026-09-13 06:16 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BR$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BS$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BR165"/>
+  <dimension ref="A1:BS165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -513,6 +513,7 @@
     <col width="16" customWidth="1" min="68" max="68"/>
     <col width="16" customWidth="1" min="69" max="69"/>
     <col width="16" customWidth="1" min="70" max="70"/>
+    <col width="16" customWidth="1" min="71" max="71"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -866,6 +867,11 @@
           <t>2026-09-12 22:09</t>
         </is>
       </c>
+      <c r="BS1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-13 01:16</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1084,6 +1090,9 @@
       <c r="BR2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="BS2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1302,6 +1311,9 @@
       <c r="BR3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="BS3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1520,6 +1532,9 @@
       <c r="BR4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="BS4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1738,6 +1753,9 @@
       <c r="BR5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BS5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1956,6 +1974,9 @@
       <c r="BR6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BS6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2174,6 +2195,9 @@
       <c r="BR7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="BS7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2392,6 +2416,9 @@
       <c r="BR8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="BS8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2610,6 +2637,9 @@
       <c r="BR9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="BS9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2828,6 +2858,9 @@
       <c r="BR10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BS10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3046,6 +3079,9 @@
       <c r="BR11" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS11" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3264,6 +3300,9 @@
       <c r="BR12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3482,6 +3521,9 @@
       <c r="BR13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="BS13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3700,6 +3742,9 @@
       <c r="BR14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3918,6 +3963,9 @@
       <c r="BR15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="BS15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4136,6 +4184,9 @@
       <c r="BR16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BS16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4354,6 +4405,9 @@
       <c r="BR17" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BS17" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -4572,6 +4626,9 @@
       <c r="BR18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BS18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -4790,6 +4847,9 @@
       <c r="BR19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="BS19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5008,6 +5068,9 @@
       <c r="BR20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="BS20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -5226,6 +5289,9 @@
       <c r="BR21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="BS21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -5444,6 +5510,9 @@
       <c r="BR22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BS22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -5662,6 +5731,9 @@
       <c r="BR23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BS23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -5880,6 +5952,9 @@
       <c r="BR24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BS24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -6098,6 +6173,9 @@
       <c r="BR25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -6316,6 +6394,9 @@
       <c r="BR26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="BS26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -6534,6 +6615,9 @@
       <c r="BR27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BS27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -6752,6 +6836,9 @@
       <c r="BR28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BS28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -6970,6 +7057,9 @@
       <c r="BR29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BS29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -7188,6 +7278,9 @@
       <c r="BR30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -7406,6 +7499,9 @@
       <c r="BR31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -7624,6 +7720,9 @@
       <c r="BR32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -7842,6 +7941,9 @@
       <c r="BR33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BS33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -8060,6 +8162,9 @@
       <c r="BR34" s="3" t="n">
         <v>21.22</v>
       </c>
+      <c r="BS34" s="3" t="n">
+        <v>21.22</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -8278,6 +8383,9 @@
       <c r="BR35" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BS35" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -8496,6 +8604,9 @@
       <c r="BR36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BS36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -8714,6 +8825,9 @@
       <c r="BR37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BS37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -8932,6 +9046,9 @@
       <c r="BR38" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS38" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -9150,6 +9267,9 @@
       <c r="BR39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="BS39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -9368,6 +9488,9 @@
       <c r="BR40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -9586,6 +9709,9 @@
       <c r="BR41" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS41" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -9804,6 +9930,9 @@
       <c r="BR42" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS42" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -10022,6 +10151,9 @@
       <c r="BR43" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BS43" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -10240,6 +10372,9 @@
       <c r="BR44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BS44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -10458,6 +10593,9 @@
       <c r="BR45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BS45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -10676,6 +10814,9 @@
       <c r="BR46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="BS46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -10894,6 +11035,9 @@
       <c r="BR47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BS47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -11112,6 +11256,9 @@
       <c r="BR48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BS48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -11330,6 +11477,9 @@
       <c r="BR49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BS49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -11548,6 +11698,9 @@
       <c r="BR50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BS50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -11766,6 +11919,9 @@
       <c r="BR51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="BS51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -11984,6 +12140,9 @@
       <c r="BR52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BS52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -12202,6 +12361,9 @@
       <c r="BR53" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BS53" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -12420,6 +12582,9 @@
       <c r="BR54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BS54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -12638,6 +12803,9 @@
       <c r="BR55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="BS55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -12856,6 +13024,9 @@
       <c r="BR56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BS56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -13074,6 +13245,9 @@
       <c r="BR57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -13292,6 +13466,9 @@
       <c r="BR58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="BS58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -13510,6 +13687,9 @@
       <c r="BR59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="BS59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -13728,6 +13908,9 @@
       <c r="BR60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="BS60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -13946,6 +14129,9 @@
       <c r="BR61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="BS61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -14164,6 +14350,9 @@
       <c r="BR62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="BS62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -14382,6 +14571,9 @@
       <c r="BR63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="BS63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -14600,6 +14792,9 @@
       <c r="BR64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BS64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -14818,6 +15013,9 @@
       <c r="BR65" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BS65" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -15036,6 +15234,9 @@
       <c r="BR66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -15254,6 +15455,9 @@
       <c r="BR67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BS67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -15472,6 +15676,9 @@
       <c r="BR68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -15690,6 +15897,9 @@
       <c r="BR69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BS69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -15908,6 +16118,9 @@
       <c r="BR70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BS70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -16126,6 +16339,9 @@
       <c r="BR71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -16344,6 +16560,9 @@
       <c r="BR72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -16562,6 +16781,9 @@
       <c r="BR73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BS73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -16780,6 +17002,9 @@
       <c r="BR74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BS74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -16998,6 +17223,9 @@
       <c r="BR75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -17216,6 +17444,9 @@
       <c r="BR76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -17434,6 +17665,9 @@
       <c r="BR77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -17652,6 +17886,9 @@
       <c r="BR78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BS78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -17870,6 +18107,9 @@
       <c r="BR79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -18088,6 +18328,9 @@
       <c r="BR80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BS80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -18306,6 +18549,9 @@
       <c r="BR81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -18524,6 +18770,9 @@
       <c r="BR82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -18742,6 +18991,9 @@
       <c r="BR83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -18960,6 +19212,9 @@
       <c r="BR84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BS84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -19178,6 +19433,9 @@
       <c r="BR85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BS85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -19396,6 +19654,9 @@
       <c r="BR86" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BS86" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -19614,6 +19875,9 @@
       <c r="BR87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -19832,6 +20096,9 @@
       <c r="BR88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -20050,6 +20317,9 @@
       <c r="BR89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -20268,6 +20538,9 @@
       <c r="BR90" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BS90" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -20486,6 +20759,9 @@
       <c r="BR91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -20704,6 +20980,9 @@
       <c r="BR92" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="BS92" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -20922,6 +21201,9 @@
       <c r="BR93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="BS93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -21140,6 +21422,9 @@
       <c r="BR94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BS94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -21358,6 +21643,9 @@
       <c r="BR95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BS95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -21576,6 +21864,9 @@
       <c r="BR96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BS96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -21794,6 +22085,9 @@
       <c r="BR97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BS97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -22012,6 +22306,9 @@
       <c r="BR98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BS98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -22230,6 +22527,9 @@
       <c r="BR99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BS99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -22448,6 +22748,9 @@
       <c r="BR100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BS100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -22666,6 +22969,9 @@
       <c r="BR101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BS101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -22884,6 +23190,9 @@
       <c r="BR102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BS102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -23102,6 +23411,9 @@
       <c r="BR103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BS103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -23320,6 +23632,9 @@
       <c r="BR104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BS104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -23538,6 +23853,9 @@
       <c r="BR105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BS105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -23756,6 +24074,9 @@
       <c r="BR106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BS106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -23974,6 +24295,9 @@
       <c r="BR107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BS107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -24192,6 +24516,9 @@
       <c r="BR108" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BS108" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -24410,6 +24737,9 @@
       <c r="BR109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BS109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -24628,6 +24958,9 @@
       <c r="BR110" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BS110" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -24846,6 +25179,9 @@
       <c r="BR111" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BS111" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -25064,6 +25400,9 @@
       <c r="BR112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BS112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -25282,6 +25621,9 @@
       <c r="BR113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BS113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -25500,6 +25842,9 @@
       <c r="BR114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BS114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -25718,6 +26063,9 @@
       <c r="BR115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BS115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -25936,6 +26284,9 @@
       <c r="BR116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BS116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -26154,6 +26505,9 @@
       <c r="BR117" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BS117" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -26372,6 +26726,9 @@
       <c r="BR118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BS118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -26590,6 +26947,9 @@
       <c r="BR119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BS119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -26808,6 +27168,9 @@
       <c r="BR120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BS120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -27026,6 +27389,9 @@
       <c r="BR121" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BS121" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -27244,6 +27610,9 @@
       <c r="BR122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BS122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -27462,6 +27831,9 @@
       <c r="BR123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="BS123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -27680,6 +28052,9 @@
       <c r="BR124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BS124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -27898,6 +28273,9 @@
       <c r="BR125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BS125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -28116,6 +28494,9 @@
       <c r="BR126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BS126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -28334,6 +28715,9 @@
       <c r="BR127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BS127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -28552,6 +28936,9 @@
       <c r="BR128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BS128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -28770,6 +29157,9 @@
       <c r="BR129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BS129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -28988,6 +29378,9 @@
       <c r="BR130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BS130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -29206,6 +29599,9 @@
       <c r="BR131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BS131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -29424,6 +29820,9 @@
       <c r="BR132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="BS132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -29642,6 +30041,9 @@
       <c r="BR133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BS133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -29860,6 +30262,9 @@
       <c r="BR134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="BS134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -30078,6 +30483,9 @@
       <c r="BR135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BS135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -30296,6 +30704,9 @@
       <c r="BR136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BS136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -30514,6 +30925,9 @@
       <c r="BR137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BS137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -30732,6 +31146,9 @@
       <c r="BR138" s="3" t="n">
         <v>23.29</v>
       </c>
+      <c r="BS138" s="3" t="n">
+        <v>23.29</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -30950,6 +31367,9 @@
       <c r="BR139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BS139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -31168,6 +31588,9 @@
       <c r="BR140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BS140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -31386,6 +31809,9 @@
       <c r="BR141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BS141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -31604,6 +32030,9 @@
       <c r="BR142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BS142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -31822,6 +32251,9 @@
       <c r="BR143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BS143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -32040,6 +32472,9 @@
       <c r="BR144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BS144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -32258,6 +32693,9 @@
       <c r="BR145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="BS145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -32476,6 +32914,9 @@
       <c r="BR146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BS146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -32694,6 +33135,9 @@
       <c r="BR147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BS147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -32912,6 +33356,9 @@
       <c r="BR148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BS148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -33130,6 +33577,9 @@
       <c r="BR149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="BS149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -33348,6 +33798,9 @@
       <c r="BR150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BS150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -33566,6 +34019,9 @@
       <c r="BR151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BS151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -33784,6 +34240,9 @@
       <c r="BR152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BS152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -34002,6 +34461,9 @@
       <c r="BR153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BS153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -34220,6 +34682,9 @@
       <c r="BR154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="BS154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -34438,6 +34903,9 @@
       <c r="BR155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BS155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -34656,6 +35124,9 @@
       <c r="BR156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BS156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -34874,6 +35345,9 @@
       <c r="BR157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BS157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -35092,6 +35566,9 @@
       <c r="BR158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BS158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -35310,6 +35787,9 @@
       <c r="BR159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="BS159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -35528,6 +36008,9 @@
       <c r="BR160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BS160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -35746,6 +36229,9 @@
       <c r="BR161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BS161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -35964,6 +36450,9 @@
       <c r="BR162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="BS162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -36182,6 +36671,9 @@
       <c r="BR163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="BS163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -36400,6 +36892,9 @@
       <c r="BR164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="BS164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -36519,9 +37014,12 @@
       <c r="BR165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="BS165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BR165"/>
+  <autoFilter ref="A1:BS165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-13 09:33 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BS$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BT$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BS165"/>
+  <dimension ref="A1:BT165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -514,6 +514,7 @@
     <col width="16" customWidth="1" min="69" max="69"/>
     <col width="16" customWidth="1" min="70" max="70"/>
     <col width="16" customWidth="1" min="71" max="71"/>
+    <col width="16" customWidth="1" min="72" max="72"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -872,6 +873,11 @@
           <t>2026-09-13 01:16</t>
         </is>
       </c>
+      <c r="BT1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-13 04:33</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1093,6 +1099,9 @@
       <c r="BS2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="BT2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1314,6 +1323,9 @@
       <c r="BS3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="BT3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1535,6 +1547,9 @@
       <c r="BS4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="BT4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1756,6 +1771,9 @@
       <c r="BS5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BT5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1977,6 +1995,9 @@
       <c r="BS6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BT6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2198,6 +2219,9 @@
       <c r="BS7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="BT7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2419,6 +2443,9 @@
       <c r="BS8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="BT8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2640,6 +2667,9 @@
       <c r="BS9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="BT9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2861,6 +2891,9 @@
       <c r="BS10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BT10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3082,6 +3115,9 @@
       <c r="BS11" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT11" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3303,6 +3339,9 @@
       <c r="BS12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3524,6 +3563,9 @@
       <c r="BS13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="BT13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3745,6 +3787,9 @@
       <c r="BS14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3966,6 +4011,9 @@
       <c r="BS15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="BT15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4187,6 +4235,9 @@
       <c r="BS16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BT16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4408,6 +4459,9 @@
       <c r="BS17" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BT17" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -4629,6 +4683,9 @@
       <c r="BS18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BT18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -4850,6 +4907,9 @@
       <c r="BS19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="BT19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5071,6 +5131,9 @@
       <c r="BS20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="BT20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -5292,6 +5355,9 @@
       <c r="BS21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="BT21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -5513,6 +5579,9 @@
       <c r="BS22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BT22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -5734,6 +5803,9 @@
       <c r="BS23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BT23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -5955,6 +6027,9 @@
       <c r="BS24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BT24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -6176,6 +6251,9 @@
       <c r="BS25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -6397,6 +6475,9 @@
       <c r="BS26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="BT26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -6618,6 +6699,9 @@
       <c r="BS27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BT27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -6839,6 +6923,9 @@
       <c r="BS28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BT28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -7060,6 +7147,9 @@
       <c r="BS29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BT29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -7281,6 +7371,9 @@
       <c r="BS30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -7502,6 +7595,9 @@
       <c r="BS31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -7723,6 +7819,9 @@
       <c r="BS32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -7944,6 +8043,9 @@
       <c r="BS33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BT33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -8165,6 +8267,9 @@
       <c r="BS34" s="3" t="n">
         <v>21.22</v>
       </c>
+      <c r="BT34" s="3" t="n">
+        <v>21.22</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -8386,6 +8491,9 @@
       <c r="BS35" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BT35" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -8607,6 +8715,9 @@
       <c r="BS36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BT36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -8828,6 +8939,9 @@
       <c r="BS37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BT37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -9049,6 +9163,9 @@
       <c r="BS38" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT38" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -9270,6 +9387,9 @@
       <c r="BS39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="BT39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -9491,6 +9611,9 @@
       <c r="BS40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -9712,6 +9835,9 @@
       <c r="BS41" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT41" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -9933,6 +10059,9 @@
       <c r="BS42" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT42" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -10154,6 +10283,9 @@
       <c r="BS43" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BT43" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -10375,6 +10507,9 @@
       <c r="BS44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BT44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -10596,6 +10731,9 @@
       <c r="BS45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BT45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -10817,6 +10955,9 @@
       <c r="BS46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="BT46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -11038,6 +11179,9 @@
       <c r="BS47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BT47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -11259,6 +11403,9 @@
       <c r="BS48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BT48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -11480,6 +11627,9 @@
       <c r="BS49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BT49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -11701,6 +11851,9 @@
       <c r="BS50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BT50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -11922,6 +12075,9 @@
       <c r="BS51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="BT51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -12143,6 +12299,9 @@
       <c r="BS52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BT52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -12364,6 +12523,9 @@
       <c r="BS53" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BT53" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -12585,6 +12747,9 @@
       <c r="BS54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BT54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -12806,6 +12971,9 @@
       <c r="BS55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="BT55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -13027,6 +13195,9 @@
       <c r="BS56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BT56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -13248,6 +13419,9 @@
       <c r="BS57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -13469,6 +13643,9 @@
       <c r="BS58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="BT58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -13690,6 +13867,9 @@
       <c r="BS59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="BT59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -13911,6 +14091,9 @@
       <c r="BS60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="BT60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -14132,6 +14315,9 @@
       <c r="BS61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="BT61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -14353,6 +14539,9 @@
       <c r="BS62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="BT62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -14574,6 +14763,9 @@
       <c r="BS63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="BT63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -14795,6 +14987,9 @@
       <c r="BS64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BT64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -15016,6 +15211,9 @@
       <c r="BS65" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BT65" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -15237,6 +15435,9 @@
       <c r="BS66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -15458,6 +15659,9 @@
       <c r="BS67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BT67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -15679,6 +15883,9 @@
       <c r="BS68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -15900,6 +16107,9 @@
       <c r="BS69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BT69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -16121,6 +16331,9 @@
       <c r="BS70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BT70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -16342,6 +16555,9 @@
       <c r="BS71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -16563,6 +16779,9 @@
       <c r="BS72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -16784,6 +17003,9 @@
       <c r="BS73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BT73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -17005,6 +17227,9 @@
       <c r="BS74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BT74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -17226,6 +17451,9 @@
       <c r="BS75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -17447,6 +17675,9 @@
       <c r="BS76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -17668,6 +17899,9 @@
       <c r="BS77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -17889,6 +18123,9 @@
       <c r="BS78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BT78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -18110,6 +18347,9 @@
       <c r="BS79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -18331,6 +18571,9 @@
       <c r="BS80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BT80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -18552,6 +18795,9 @@
       <c r="BS81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -18773,6 +19019,9 @@
       <c r="BS82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -18994,6 +19243,9 @@
       <c r="BS83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -19215,6 +19467,9 @@
       <c r="BS84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BT84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -19436,6 +19691,9 @@
       <c r="BS85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BT85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -19657,6 +19915,9 @@
       <c r="BS86" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BT86" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -19878,6 +20139,9 @@
       <c r="BS87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -20099,6 +20363,9 @@
       <c r="BS88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -20320,6 +20587,9 @@
       <c r="BS89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -20541,6 +20811,9 @@
       <c r="BS90" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BT90" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -20762,6 +21035,9 @@
       <c r="BS91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -20983,6 +21259,9 @@
       <c r="BS92" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="BT92" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -21204,6 +21483,9 @@
       <c r="BS93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="BT93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -21425,6 +21707,9 @@
       <c r="BS94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BT94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -21646,6 +21931,9 @@
       <c r="BS95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BT95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -21867,6 +22155,9 @@
       <c r="BS96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BT96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -22088,6 +22379,9 @@
       <c r="BS97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BT97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -22309,6 +22603,9 @@
       <c r="BS98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BT98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -22530,6 +22827,9 @@
       <c r="BS99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BT99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -22751,6 +23051,9 @@
       <c r="BS100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BT100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -22972,6 +23275,9 @@
       <c r="BS101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BT101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -23193,6 +23499,9 @@
       <c r="BS102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BT102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -23414,6 +23723,9 @@
       <c r="BS103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BT103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -23635,6 +23947,9 @@
       <c r="BS104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BT104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -23856,6 +24171,9 @@
       <c r="BS105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BT105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -24077,6 +24395,9 @@
       <c r="BS106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BT106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -24298,6 +24619,9 @@
       <c r="BS107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BT107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -24519,6 +24843,9 @@
       <c r="BS108" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BT108" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -24740,6 +25067,9 @@
       <c r="BS109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BT109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -24961,6 +25291,9 @@
       <c r="BS110" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BT110" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -25182,6 +25515,9 @@
       <c r="BS111" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BT111" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -25403,6 +25739,9 @@
       <c r="BS112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BT112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -25624,6 +25963,9 @@
       <c r="BS113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BT113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -25845,6 +26187,9 @@
       <c r="BS114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BT114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -26066,6 +26411,9 @@
       <c r="BS115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BT115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -26287,6 +26635,9 @@
       <c r="BS116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BT116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -26508,6 +26859,9 @@
       <c r="BS117" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BT117" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -26729,6 +27083,9 @@
       <c r="BS118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BT118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -26950,6 +27307,9 @@
       <c r="BS119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BT119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -27171,6 +27531,9 @@
       <c r="BS120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BT120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -27392,6 +27755,9 @@
       <c r="BS121" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BT121" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -27613,6 +27979,9 @@
       <c r="BS122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BT122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -27834,6 +28203,9 @@
       <c r="BS123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="BT123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -28055,6 +28427,9 @@
       <c r="BS124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BT124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -28276,6 +28651,9 @@
       <c r="BS125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BT125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -28497,6 +28875,9 @@
       <c r="BS126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BT126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -28718,6 +29099,9 @@
       <c r="BS127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BT127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -28939,6 +29323,9 @@
       <c r="BS128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BT128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -29160,6 +29547,9 @@
       <c r="BS129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BT129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -29381,6 +29771,9 @@
       <c r="BS130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BT130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -29602,6 +29995,9 @@
       <c r="BS131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BT131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -29823,6 +30219,9 @@
       <c r="BS132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="BT132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -30044,6 +30443,9 @@
       <c r="BS133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BT133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -30265,6 +30667,9 @@
       <c r="BS134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="BT134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -30486,6 +30891,9 @@
       <c r="BS135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BT135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -30707,6 +31115,9 @@
       <c r="BS136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BT136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -30928,6 +31339,9 @@
       <c r="BS137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BT137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -31149,6 +31563,9 @@
       <c r="BS138" s="3" t="n">
         <v>23.29</v>
       </c>
+      <c r="BT138" s="3" t="n">
+        <v>23.29</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -31370,6 +31787,9 @@
       <c r="BS139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BT139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -31591,6 +32011,9 @@
       <c r="BS140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BT140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -31812,6 +32235,9 @@
       <c r="BS141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BT141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -32033,6 +32459,9 @@
       <c r="BS142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BT142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -32254,6 +32683,9 @@
       <c r="BS143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BT143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -32475,6 +32907,9 @@
       <c r="BS144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BT144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -32696,6 +33131,9 @@
       <c r="BS145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="BT145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -32917,6 +33355,9 @@
       <c r="BS146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BT146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -33138,6 +33579,9 @@
       <c r="BS147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BT147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -33359,6 +33803,9 @@
       <c r="BS148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BT148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -33580,6 +34027,9 @@
       <c r="BS149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="BT149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -33801,6 +34251,9 @@
       <c r="BS150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BT150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -34022,6 +34475,9 @@
       <c r="BS151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BT151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -34243,6 +34699,9 @@
       <c r="BS152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BT152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -34464,6 +34923,9 @@
       <c r="BS153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BT153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -34685,6 +35147,9 @@
       <c r="BS154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="BT154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -34906,6 +35371,9 @@
       <c r="BS155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BT155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -35127,6 +35595,9 @@
       <c r="BS156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BT156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -35348,6 +35819,9 @@
       <c r="BS157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BT157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -35569,6 +36043,9 @@
       <c r="BS158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BT158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -35790,6 +36267,9 @@
       <c r="BS159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="BT159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -36011,6 +36491,9 @@
       <c r="BS160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BT160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -36232,6 +36715,9 @@
       <c r="BS161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BT161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -36453,6 +36939,9 @@
       <c r="BS162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="BT162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -36674,6 +37163,9 @@
       <c r="BS163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="BT163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -36895,6 +37387,9 @@
       <c r="BS164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="BT164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -37017,9 +37512,12 @@
       <c r="BS165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="BT165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BS165"/>
+  <autoFilter ref="A1:BT165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-13 12:11 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BT$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BU$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BT165"/>
+  <dimension ref="A1:BU165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -515,6 +515,7 @@
     <col width="16" customWidth="1" min="70" max="70"/>
     <col width="16" customWidth="1" min="71" max="71"/>
     <col width="16" customWidth="1" min="72" max="72"/>
+    <col width="16" customWidth="1" min="73" max="73"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -878,6 +879,11 @@
           <t>2026-09-13 04:33</t>
         </is>
       </c>
+      <c r="BU1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-13 07:11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1102,6 +1108,9 @@
       <c r="BT2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="BU2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1326,6 +1335,9 @@
       <c r="BT3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="BU3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1550,6 +1562,9 @@
       <c r="BT4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="BU4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1774,6 +1789,9 @@
       <c r="BT5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BU5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1998,6 +2016,9 @@
       <c r="BT6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BU6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2222,6 +2243,9 @@
       <c r="BT7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="BU7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2446,6 +2470,9 @@
       <c r="BT8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="BU8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2670,6 +2697,9 @@
       <c r="BT9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="BU9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2894,6 +2924,9 @@
       <c r="BT10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BU10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3118,6 +3151,9 @@
       <c r="BT11" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU11" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3342,6 +3378,9 @@
       <c r="BT12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3566,6 +3605,9 @@
       <c r="BT13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="BU13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3790,6 +3832,9 @@
       <c r="BT14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4014,6 +4059,9 @@
       <c r="BT15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="BU15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4238,6 +4286,9 @@
       <c r="BT16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BU16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4462,6 +4513,9 @@
       <c r="BT17" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BU17" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -4686,6 +4740,9 @@
       <c r="BT18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BU18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -4910,6 +4967,9 @@
       <c r="BT19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="BU19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5134,6 +5194,9 @@
       <c r="BT20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="BU20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -5358,6 +5421,9 @@
       <c r="BT21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="BU21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -5582,6 +5648,9 @@
       <c r="BT22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BU22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -5806,6 +5875,9 @@
       <c r="BT23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BU23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -6030,6 +6102,9 @@
       <c r="BT24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BU24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -6254,6 +6329,9 @@
       <c r="BT25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -6478,6 +6556,9 @@
       <c r="BT26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="BU26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -6702,6 +6783,9 @@
       <c r="BT27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BU27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -6926,6 +7010,9 @@
       <c r="BT28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BU28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -7150,6 +7237,9 @@
       <c r="BT29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BU29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -7374,6 +7464,9 @@
       <c r="BT30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -7598,6 +7691,9 @@
       <c r="BT31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -7822,6 +7918,9 @@
       <c r="BT32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -8046,6 +8145,9 @@
       <c r="BT33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BU33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -8270,6 +8372,9 @@
       <c r="BT34" s="3" t="n">
         <v>21.22</v>
       </c>
+      <c r="BU34" s="3" t="n">
+        <v>21.22</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -8494,6 +8599,9 @@
       <c r="BT35" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BU35" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -8718,6 +8826,9 @@
       <c r="BT36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BU36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -8942,6 +9053,9 @@
       <c r="BT37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BU37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -9166,6 +9280,9 @@
       <c r="BT38" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU38" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -9390,6 +9507,9 @@
       <c r="BT39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="BU39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -9614,6 +9734,9 @@
       <c r="BT40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -9838,6 +9961,9 @@
       <c r="BT41" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU41" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -10062,6 +10188,9 @@
       <c r="BT42" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU42" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -10286,6 +10415,9 @@
       <c r="BT43" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BU43" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -10510,6 +10642,9 @@
       <c r="BT44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BU44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -10734,6 +10869,9 @@
       <c r="BT45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BU45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -10958,6 +11096,9 @@
       <c r="BT46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="BU46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -11182,6 +11323,9 @@
       <c r="BT47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BU47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -11406,6 +11550,9 @@
       <c r="BT48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BU48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -11630,6 +11777,9 @@
       <c r="BT49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BU49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -11854,6 +12004,9 @@
       <c r="BT50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BU50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -12078,6 +12231,9 @@
       <c r="BT51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="BU51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -12302,6 +12458,9 @@
       <c r="BT52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BU52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -12526,6 +12685,9 @@
       <c r="BT53" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BU53" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -12750,6 +12912,9 @@
       <c r="BT54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BU54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -12974,6 +13139,9 @@
       <c r="BT55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="BU55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -13198,6 +13366,9 @@
       <c r="BT56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BU56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -13422,6 +13593,9 @@
       <c r="BT57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -13646,6 +13820,9 @@
       <c r="BT58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="BU58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -13870,6 +14047,9 @@
       <c r="BT59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="BU59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -14094,6 +14274,9 @@
       <c r="BT60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="BU60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -14318,6 +14501,9 @@
       <c r="BT61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="BU61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -14542,6 +14728,9 @@
       <c r="BT62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="BU62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -14766,6 +14955,9 @@
       <c r="BT63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="BU63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -14990,6 +15182,9 @@
       <c r="BT64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BU64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -15214,6 +15409,9 @@
       <c r="BT65" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BU65" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -15438,6 +15636,9 @@
       <c r="BT66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -15662,6 +15863,9 @@
       <c r="BT67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BU67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -15886,6 +16090,9 @@
       <c r="BT68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -16110,6 +16317,9 @@
       <c r="BT69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BU69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -16334,6 +16544,9 @@
       <c r="BT70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BU70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -16558,6 +16771,9 @@
       <c r="BT71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -16782,6 +16998,9 @@
       <c r="BT72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -17006,6 +17225,9 @@
       <c r="BT73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BU73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -17230,6 +17452,9 @@
       <c r="BT74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BU74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -17454,6 +17679,9 @@
       <c r="BT75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -17678,6 +17906,9 @@
       <c r="BT76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -17902,6 +18133,9 @@
       <c r="BT77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -18126,6 +18360,9 @@
       <c r="BT78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BU78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -18350,6 +18587,9 @@
       <c r="BT79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -18574,6 +18814,9 @@
       <c r="BT80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BU80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -18798,6 +19041,9 @@
       <c r="BT81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -19022,6 +19268,9 @@
       <c r="BT82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -19246,6 +19495,9 @@
       <c r="BT83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -19470,6 +19722,9 @@
       <c r="BT84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BU84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -19694,6 +19949,9 @@
       <c r="BT85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BU85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -19918,6 +20176,9 @@
       <c r="BT86" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BU86" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -20142,6 +20403,9 @@
       <c r="BT87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -20366,6 +20630,9 @@
       <c r="BT88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -20590,6 +20857,9 @@
       <c r="BT89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -20814,6 +21084,9 @@
       <c r="BT90" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BU90" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -21038,6 +21311,9 @@
       <c r="BT91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -21262,6 +21538,9 @@
       <c r="BT92" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="BU92" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -21486,6 +21765,9 @@
       <c r="BT93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="BU93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -21710,6 +21992,9 @@
       <c r="BT94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BU94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -21934,6 +22219,9 @@
       <c r="BT95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BU95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -22158,6 +22446,9 @@
       <c r="BT96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BU96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -22382,6 +22673,9 @@
       <c r="BT97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BU97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -22606,6 +22900,9 @@
       <c r="BT98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BU98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -22830,6 +23127,9 @@
       <c r="BT99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BU99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -23054,6 +23354,9 @@
       <c r="BT100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BU100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -23278,6 +23581,9 @@
       <c r="BT101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BU101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -23502,6 +23808,9 @@
       <c r="BT102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BU102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -23726,6 +24035,9 @@
       <c r="BT103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BU103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -23950,6 +24262,9 @@
       <c r="BT104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BU104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -24174,6 +24489,9 @@
       <c r="BT105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BU105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -24398,6 +24716,9 @@
       <c r="BT106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BU106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -24622,6 +24943,9 @@
       <c r="BT107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BU107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -24846,6 +25170,9 @@
       <c r="BT108" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BU108" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -25070,6 +25397,9 @@
       <c r="BT109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BU109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -25294,6 +25624,9 @@
       <c r="BT110" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BU110" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -25518,6 +25851,9 @@
       <c r="BT111" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BU111" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -25742,6 +26078,9 @@
       <c r="BT112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BU112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -25966,6 +26305,9 @@
       <c r="BT113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BU113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -26190,6 +26532,9 @@
       <c r="BT114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BU114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -26414,6 +26759,9 @@
       <c r="BT115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BU115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -26638,6 +26986,9 @@
       <c r="BT116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BU116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -26862,6 +27213,9 @@
       <c r="BT117" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BU117" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -27086,6 +27440,9 @@
       <c r="BT118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BU118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -27310,6 +27667,9 @@
       <c r="BT119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BU119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -27534,6 +27894,9 @@
       <c r="BT120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BU120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -27758,6 +28121,9 @@
       <c r="BT121" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BU121" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -27982,6 +28348,9 @@
       <c r="BT122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BU122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -28206,6 +28575,9 @@
       <c r="BT123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="BU123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -28430,6 +28802,9 @@
       <c r="BT124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BU124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -28654,6 +29029,9 @@
       <c r="BT125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BU125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -28878,6 +29256,9 @@
       <c r="BT126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BU126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -29102,6 +29483,9 @@
       <c r="BT127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BU127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -29326,6 +29710,9 @@
       <c r="BT128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BU128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -29550,6 +29937,9 @@
       <c r="BT129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BU129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -29774,6 +30164,9 @@
       <c r="BT130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BU130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -29998,6 +30391,9 @@
       <c r="BT131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BU131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -30222,6 +30618,9 @@
       <c r="BT132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="BU132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -30446,6 +30845,9 @@
       <c r="BT133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BU133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -30670,6 +31072,9 @@
       <c r="BT134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="BU134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -30894,6 +31299,9 @@
       <c r="BT135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BU135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -31118,6 +31526,9 @@
       <c r="BT136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BU136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -31342,6 +31753,9 @@
       <c r="BT137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BU137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -31566,6 +31980,9 @@
       <c r="BT138" s="3" t="n">
         <v>23.29</v>
       </c>
+      <c r="BU138" s="3" t="n">
+        <v>23.29</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -31790,6 +32207,9 @@
       <c r="BT139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BU139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -32014,6 +32434,9 @@
       <c r="BT140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BU140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -32238,6 +32661,9 @@
       <c r="BT141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BU141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -32462,6 +32888,9 @@
       <c r="BT142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BU142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -32686,6 +33115,9 @@
       <c r="BT143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BU143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -32910,6 +33342,9 @@
       <c r="BT144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BU144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -33134,6 +33569,9 @@
       <c r="BT145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="BU145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -33358,6 +33796,9 @@
       <c r="BT146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BU146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -33582,6 +34023,9 @@
       <c r="BT147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BU147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -33806,6 +34250,9 @@
       <c r="BT148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BU148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -34030,6 +34477,9 @@
       <c r="BT149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="BU149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -34254,6 +34704,9 @@
       <c r="BT150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BU150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -34478,6 +34931,9 @@
       <c r="BT151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BU151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -34702,6 +35158,9 @@
       <c r="BT152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BU152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -34926,6 +35385,9 @@
       <c r="BT153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BU153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -35150,6 +35612,9 @@
       <c r="BT154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="BU154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -35374,6 +35839,9 @@
       <c r="BT155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BU155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -35598,6 +36066,9 @@
       <c r="BT156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BU156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -35822,6 +36293,9 @@
       <c r="BT157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BU157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -36046,6 +36520,9 @@
       <c r="BT158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BU158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -36270,6 +36747,9 @@
       <c r="BT159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="BU159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -36494,6 +36974,9 @@
       <c r="BT160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BU160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -36718,6 +37201,9 @@
       <c r="BT161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BU161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -36942,6 +37428,9 @@
       <c r="BT162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="BU162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -37166,6 +37655,9 @@
       <c r="BT163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="BU163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -37390,6 +37882,9 @@
       <c r="BT164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="BU164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -37515,9 +38010,12 @@
       <c r="BT165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="BU165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BT165"/>
+  <autoFilter ref="A1:BU165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-13 15:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BU$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BV$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BU165"/>
+  <dimension ref="A1:BV165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -516,6 +516,7 @@
     <col width="16" customWidth="1" min="71" max="71"/>
     <col width="16" customWidth="1" min="72" max="72"/>
     <col width="16" customWidth="1" min="73" max="73"/>
+    <col width="16" customWidth="1" min="74" max="74"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -884,6 +885,11 @@
           <t>2026-09-13 07:11</t>
         </is>
       </c>
+      <c r="BV1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-13 10:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1111,6 +1117,9 @@
       <c r="BU2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="BV2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1338,6 +1347,9 @@
       <c r="BU3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="BV3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1565,6 +1577,9 @@
       <c r="BU4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="BV4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1792,6 +1807,9 @@
       <c r="BU5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BV5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2019,6 +2037,9 @@
       <c r="BU6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BV6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2246,6 +2267,9 @@
       <c r="BU7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="BV7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2473,6 +2497,9 @@
       <c r="BU8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="BV8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2700,6 +2727,9 @@
       <c r="BU9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="BV9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2927,6 +2957,9 @@
       <c r="BU10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BV10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3154,6 +3187,9 @@
       <c r="BU11" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV11" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3381,6 +3417,9 @@
       <c r="BU12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3608,6 +3647,9 @@
       <c r="BU13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="BV13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3835,6 +3877,9 @@
       <c r="BU14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4062,6 +4107,9 @@
       <c r="BU15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="BV15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4289,6 +4337,9 @@
       <c r="BU16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BV16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4516,6 +4567,9 @@
       <c r="BU17" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BV17" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -4743,6 +4797,9 @@
       <c r="BU18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BV18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -4970,6 +5027,9 @@
       <c r="BU19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="BV19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5197,6 +5257,9 @@
       <c r="BU20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="BV20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -5424,6 +5487,9 @@
       <c r="BU21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="BV21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -5651,6 +5717,9 @@
       <c r="BU22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BV22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -5878,6 +5947,9 @@
       <c r="BU23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BV23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -6105,6 +6177,9 @@
       <c r="BU24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BV24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -6332,6 +6407,9 @@
       <c r="BU25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -6559,6 +6637,9 @@
       <c r="BU26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="BV26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -6786,6 +6867,9 @@
       <c r="BU27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BV27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -7013,6 +7097,9 @@
       <c r="BU28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BV28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -7240,6 +7327,9 @@
       <c r="BU29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BV29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -7467,6 +7557,9 @@
       <c r="BU30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -7694,6 +7787,9 @@
       <c r="BU31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -7921,6 +8017,9 @@
       <c r="BU32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -8148,6 +8247,9 @@
       <c r="BU33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BV33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -8375,6 +8477,9 @@
       <c r="BU34" s="3" t="n">
         <v>21.22</v>
       </c>
+      <c r="BV34" s="3" t="n">
+        <v>21.22</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -8602,6 +8707,9 @@
       <c r="BU35" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BV35" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -8829,6 +8937,9 @@
       <c r="BU36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BV36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -9056,6 +9167,9 @@
       <c r="BU37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BV37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -9283,6 +9397,9 @@
       <c r="BU38" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV38" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -9510,6 +9627,9 @@
       <c r="BU39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="BV39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -9737,6 +9857,9 @@
       <c r="BU40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -9964,6 +10087,9 @@
       <c r="BU41" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV41" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -10191,6 +10317,9 @@
       <c r="BU42" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV42" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -10418,6 +10547,9 @@
       <c r="BU43" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BV43" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -10645,6 +10777,9 @@
       <c r="BU44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BV44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -10872,6 +11007,9 @@
       <c r="BU45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BV45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -11099,6 +11237,9 @@
       <c r="BU46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="BV46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -11326,6 +11467,9 @@
       <c r="BU47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BV47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -11553,6 +11697,9 @@
       <c r="BU48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BV48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -11780,6 +11927,9 @@
       <c r="BU49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BV49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -12007,6 +12157,9 @@
       <c r="BU50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BV50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -12234,6 +12387,9 @@
       <c r="BU51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="BV51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -12461,6 +12617,9 @@
       <c r="BU52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BV52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -12688,6 +12847,9 @@
       <c r="BU53" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BV53" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -12915,6 +13077,9 @@
       <c r="BU54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BV54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -13142,6 +13307,9 @@
       <c r="BU55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="BV55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -13369,6 +13537,9 @@
       <c r="BU56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BV56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -13596,6 +13767,9 @@
       <c r="BU57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -13823,6 +13997,9 @@
       <c r="BU58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="BV58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -14050,6 +14227,9 @@
       <c r="BU59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="BV59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -14277,6 +14457,9 @@
       <c r="BU60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="BV60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -14504,6 +14687,9 @@
       <c r="BU61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="BV61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -14731,6 +14917,9 @@
       <c r="BU62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="BV62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -14958,6 +15147,9 @@
       <c r="BU63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="BV63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -15185,6 +15377,9 @@
       <c r="BU64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BV64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -15412,6 +15607,9 @@
       <c r="BU65" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BV65" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -15639,6 +15837,9 @@
       <c r="BU66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -15866,6 +16067,9 @@
       <c r="BU67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BV67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -16093,6 +16297,9 @@
       <c r="BU68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -16320,6 +16527,9 @@
       <c r="BU69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BV69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -16547,6 +16757,9 @@
       <c r="BU70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BV70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -16774,6 +16987,9 @@
       <c r="BU71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -17001,6 +17217,9 @@
       <c r="BU72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -17228,6 +17447,9 @@
       <c r="BU73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BV73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -17455,6 +17677,9 @@
       <c r="BU74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BV74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -17682,6 +17907,9 @@
       <c r="BU75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -17909,6 +18137,9 @@
       <c r="BU76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -18136,6 +18367,9 @@
       <c r="BU77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -18363,6 +18597,9 @@
       <c r="BU78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BV78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -18590,6 +18827,9 @@
       <c r="BU79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -18817,6 +19057,9 @@
       <c r="BU80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BV80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -19044,6 +19287,9 @@
       <c r="BU81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -19271,6 +19517,9 @@
       <c r="BU82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -19498,6 +19747,9 @@
       <c r="BU83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -19725,6 +19977,9 @@
       <c r="BU84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BV84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -19952,6 +20207,9 @@
       <c r="BU85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BV85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -20179,6 +20437,9 @@
       <c r="BU86" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BV86" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -20406,6 +20667,9 @@
       <c r="BU87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -20633,6 +20897,9 @@
       <c r="BU88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -20860,6 +21127,9 @@
       <c r="BU89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -21087,6 +21357,9 @@
       <c r="BU90" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BV90" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -21314,6 +21587,9 @@
       <c r="BU91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -21541,6 +21817,9 @@
       <c r="BU92" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="BV92" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -21768,6 +22047,9 @@
       <c r="BU93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="BV93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -21995,6 +22277,9 @@
       <c r="BU94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BV94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -22222,6 +22507,9 @@
       <c r="BU95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BV95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -22449,6 +22737,9 @@
       <c r="BU96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BV96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -22676,6 +22967,9 @@
       <c r="BU97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BV97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -22903,6 +23197,9 @@
       <c r="BU98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BV98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -23130,6 +23427,9 @@
       <c r="BU99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BV99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -23357,6 +23657,9 @@
       <c r="BU100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BV100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -23584,6 +23887,9 @@
       <c r="BU101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BV101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -23811,6 +24117,9 @@
       <c r="BU102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BV102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -24038,6 +24347,9 @@
       <c r="BU103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BV103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -24265,6 +24577,9 @@
       <c r="BU104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BV104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -24492,6 +24807,9 @@
       <c r="BU105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BV105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -24719,6 +25037,9 @@
       <c r="BU106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BV106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -24946,6 +25267,9 @@
       <c r="BU107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BV107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -25173,6 +25497,9 @@
       <c r="BU108" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BV108" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -25400,6 +25727,9 @@
       <c r="BU109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BV109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -25627,6 +25957,9 @@
       <c r="BU110" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BV110" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -25854,6 +26187,9 @@
       <c r="BU111" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BV111" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -26081,6 +26417,9 @@
       <c r="BU112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BV112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -26308,6 +26647,9 @@
       <c r="BU113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BV113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -26535,6 +26877,9 @@
       <c r="BU114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BV114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -26762,6 +27107,9 @@
       <c r="BU115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BV115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -26989,6 +27337,9 @@
       <c r="BU116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BV116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -27216,6 +27567,9 @@
       <c r="BU117" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BV117" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -27443,6 +27797,9 @@
       <c r="BU118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BV118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -27670,6 +28027,9 @@
       <c r="BU119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BV119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -27897,6 +28257,9 @@
       <c r="BU120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BV120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -28124,6 +28487,9 @@
       <c r="BU121" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BV121" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -28351,6 +28717,9 @@
       <c r="BU122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BV122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -28578,6 +28947,9 @@
       <c r="BU123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="BV123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -28805,6 +29177,9 @@
       <c r="BU124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BV124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -29032,6 +29407,9 @@
       <c r="BU125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BV125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -29259,6 +29637,9 @@
       <c r="BU126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BV126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -29486,6 +29867,9 @@
       <c r="BU127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BV127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -29713,6 +30097,9 @@
       <c r="BU128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BV128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -29940,6 +30327,9 @@
       <c r="BU129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BV129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -30167,6 +30557,9 @@
       <c r="BU130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BV130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -30394,6 +30787,9 @@
       <c r="BU131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BV131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -30621,6 +31017,9 @@
       <c r="BU132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="BV132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -30848,6 +31247,9 @@
       <c r="BU133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BV133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -31075,6 +31477,9 @@
       <c r="BU134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="BV134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -31302,6 +31707,9 @@
       <c r="BU135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BV135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -31529,6 +31937,9 @@
       <c r="BU136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BV136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -31756,6 +32167,9 @@
       <c r="BU137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BV137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -31983,6 +32397,9 @@
       <c r="BU138" s="3" t="n">
         <v>23.29</v>
       </c>
+      <c r="BV138" s="3" t="n">
+        <v>23.29</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -32210,6 +32627,9 @@
       <c r="BU139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BV139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -32437,6 +32857,9 @@
       <c r="BU140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BV140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -32664,6 +33087,9 @@
       <c r="BU141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BV141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -32891,6 +33317,9 @@
       <c r="BU142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BV142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -33118,6 +33547,9 @@
       <c r="BU143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BV143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -33345,6 +33777,9 @@
       <c r="BU144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BV144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -33572,6 +34007,9 @@
       <c r="BU145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="BV145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -33799,6 +34237,9 @@
       <c r="BU146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BV146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -34026,6 +34467,9 @@
       <c r="BU147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BV147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -34253,6 +34697,9 @@
       <c r="BU148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BV148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -34480,6 +34927,9 @@
       <c r="BU149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="BV149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -34707,6 +35157,9 @@
       <c r="BU150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BV150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -34934,6 +35387,9 @@
       <c r="BU151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BV151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -35161,6 +35617,9 @@
       <c r="BU152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BV152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -35388,6 +35847,9 @@
       <c r="BU153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BV153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -35615,6 +36077,9 @@
       <c r="BU154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="BV154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -35842,6 +36307,9 @@
       <c r="BU155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BV155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -36069,6 +36537,9 @@
       <c r="BU156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BV156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -36296,6 +36767,9 @@
       <c r="BU157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BV157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -36523,6 +36997,9 @@
       <c r="BU158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BV158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -36750,6 +37227,9 @@
       <c r="BU159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="BV159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -36977,6 +37457,9 @@
       <c r="BU160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BV160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -37204,6 +37687,9 @@
       <c r="BU161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BV161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -37431,6 +37917,9 @@
       <c r="BU162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="BV162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -37658,6 +38147,9 @@
       <c r="BU163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="BV163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -37885,6 +38377,9 @@
       <c r="BU164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="BV164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -38013,9 +38508,12 @@
       <c r="BU165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="BV165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BU165"/>
+  <autoFilter ref="A1:BV165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-13 18:10 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BV$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BW$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BV165"/>
+  <dimension ref="A1:BW165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -517,6 +517,7 @@
     <col width="16" customWidth="1" min="72" max="72"/>
     <col width="16" customWidth="1" min="73" max="73"/>
     <col width="16" customWidth="1" min="74" max="74"/>
+    <col width="16" customWidth="1" min="75" max="75"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -890,6 +891,11 @@
           <t>2026-09-13 10:09</t>
         </is>
       </c>
+      <c r="BW1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-13 13:10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1120,6 +1126,9 @@
       <c r="BV2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="BW2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1350,6 +1359,9 @@
       <c r="BV3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="BW3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1580,6 +1592,9 @@
       <c r="BV4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="BW4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1810,6 +1825,9 @@
       <c r="BV5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BW5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2040,6 +2058,9 @@
       <c r="BV6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BW6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2270,6 +2291,9 @@
       <c r="BV7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="BW7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2500,6 +2524,9 @@
       <c r="BV8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="BW8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2730,6 +2757,9 @@
       <c r="BV9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="BW9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2960,6 +2990,9 @@
       <c r="BV10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BW10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3190,6 +3223,9 @@
       <c r="BV11" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW11" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3420,6 +3456,9 @@
       <c r="BV12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3650,6 +3689,9 @@
       <c r="BV13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="BW13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3880,6 +3922,9 @@
       <c r="BV14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4110,6 +4155,9 @@
       <c r="BV15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="BW15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4340,6 +4388,9 @@
       <c r="BV16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BW16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4570,6 +4621,9 @@
       <c r="BV17" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BW17" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -4800,6 +4854,9 @@
       <c r="BV18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BW18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5030,6 +5087,9 @@
       <c r="BV19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="BW19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5260,6 +5320,9 @@
       <c r="BV20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="BW20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -5490,6 +5553,9 @@
       <c r="BV21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="BW21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -5720,6 +5786,9 @@
       <c r="BV22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BW22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -5950,6 +6019,9 @@
       <c r="BV23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BW23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -6180,6 +6252,9 @@
       <c r="BV24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BW24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -6410,6 +6485,9 @@
       <c r="BV25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -6640,6 +6718,9 @@
       <c r="BV26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="BW26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -6870,6 +6951,9 @@
       <c r="BV27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BW27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -7100,6 +7184,9 @@
       <c r="BV28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BW28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -7330,6 +7417,9 @@
       <c r="BV29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BW29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -7560,6 +7650,9 @@
       <c r="BV30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -7790,6 +7883,9 @@
       <c r="BV31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -8020,6 +8116,9 @@
       <c r="BV32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -8250,6 +8349,9 @@
       <c r="BV33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BW33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -8480,6 +8582,9 @@
       <c r="BV34" s="3" t="n">
         <v>21.22</v>
       </c>
+      <c r="BW34" s="3" t="n">
+        <v>21.22</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -8710,6 +8815,9 @@
       <c r="BV35" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BW35" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -8940,6 +9048,9 @@
       <c r="BV36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BW36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -9170,6 +9281,9 @@
       <c r="BV37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BW37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -9400,6 +9514,9 @@
       <c r="BV38" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW38" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -9630,6 +9747,9 @@
       <c r="BV39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="BW39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -9860,6 +9980,9 @@
       <c r="BV40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -10090,6 +10213,9 @@
       <c r="BV41" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW41" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -10320,6 +10446,9 @@
       <c r="BV42" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW42" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -10550,6 +10679,9 @@
       <c r="BV43" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BW43" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -10780,6 +10912,9 @@
       <c r="BV44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BW44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -11010,6 +11145,9 @@
       <c r="BV45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BW45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -11240,6 +11378,9 @@
       <c r="BV46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="BW46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -11470,6 +11611,9 @@
       <c r="BV47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BW47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -11700,6 +11844,9 @@
       <c r="BV48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BW48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -11930,6 +12077,9 @@
       <c r="BV49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BW49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -12160,6 +12310,9 @@
       <c r="BV50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BW50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -12390,6 +12543,9 @@
       <c r="BV51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="BW51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -12620,6 +12776,9 @@
       <c r="BV52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BW52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -12850,6 +13009,9 @@
       <c r="BV53" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BW53" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -13080,6 +13242,9 @@
       <c r="BV54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BW54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -13310,6 +13475,9 @@
       <c r="BV55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="BW55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -13540,6 +13708,9 @@
       <c r="BV56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BW56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -13770,6 +13941,9 @@
       <c r="BV57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -14000,6 +14174,9 @@
       <c r="BV58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="BW58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -14230,6 +14407,9 @@
       <c r="BV59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="BW59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -14460,6 +14640,9 @@
       <c r="BV60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="BW60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -14690,6 +14873,9 @@
       <c r="BV61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="BW61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -14920,6 +15106,9 @@
       <c r="BV62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="BW62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -15150,6 +15339,9 @@
       <c r="BV63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="BW63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -15380,6 +15572,9 @@
       <c r="BV64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BW64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -15610,6 +15805,9 @@
       <c r="BV65" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BW65" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -15840,6 +16038,9 @@
       <c r="BV66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -16070,6 +16271,9 @@
       <c r="BV67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BW67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -16300,6 +16504,9 @@
       <c r="BV68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -16530,6 +16737,9 @@
       <c r="BV69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BW69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -16760,6 +16970,9 @@
       <c r="BV70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BW70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -16990,6 +17203,9 @@
       <c r="BV71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -17220,6 +17436,9 @@
       <c r="BV72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -17450,6 +17669,9 @@
       <c r="BV73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BW73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -17680,6 +17902,9 @@
       <c r="BV74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BW74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -17910,6 +18135,9 @@
       <c r="BV75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -18140,6 +18368,9 @@
       <c r="BV76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -18370,6 +18601,9 @@
       <c r="BV77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -18600,6 +18834,9 @@
       <c r="BV78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BW78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -18830,6 +19067,9 @@
       <c r="BV79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -19060,6 +19300,9 @@
       <c r="BV80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BW80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -19290,6 +19533,9 @@
       <c r="BV81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -19520,6 +19766,9 @@
       <c r="BV82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -19750,6 +19999,9 @@
       <c r="BV83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -19980,6 +20232,9 @@
       <c r="BV84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BW84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -20210,6 +20465,9 @@
       <c r="BV85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BW85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -20440,6 +20698,9 @@
       <c r="BV86" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BW86" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -20670,6 +20931,9 @@
       <c r="BV87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -20900,6 +21164,9 @@
       <c r="BV88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -21130,6 +21397,9 @@
       <c r="BV89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -21360,6 +21630,9 @@
       <c r="BV90" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BW90" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -21590,6 +21863,9 @@
       <c r="BV91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -21820,6 +22096,9 @@
       <c r="BV92" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="BW92" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -22050,6 +22329,9 @@
       <c r="BV93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="BW93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -22280,6 +22562,9 @@
       <c r="BV94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BW94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -22510,6 +22795,9 @@
       <c r="BV95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BW95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -22740,6 +23028,9 @@
       <c r="BV96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BW96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -22970,6 +23261,9 @@
       <c r="BV97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BW97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -23200,6 +23494,9 @@
       <c r="BV98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BW98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -23430,6 +23727,9 @@
       <c r="BV99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BW99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -23660,6 +23960,9 @@
       <c r="BV100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BW100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -23890,6 +24193,9 @@
       <c r="BV101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BW101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -24120,6 +24426,9 @@
       <c r="BV102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BW102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -24350,6 +24659,9 @@
       <c r="BV103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BW103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -24580,6 +24892,9 @@
       <c r="BV104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BW104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -24810,6 +25125,9 @@
       <c r="BV105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BW105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -25040,6 +25358,9 @@
       <c r="BV106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BW106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -25270,6 +25591,9 @@
       <c r="BV107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BW107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -25500,6 +25824,9 @@
       <c r="BV108" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BW108" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -25730,6 +26057,9 @@
       <c r="BV109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BW109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -25960,6 +26290,9 @@
       <c r="BV110" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BW110" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -26190,6 +26523,9 @@
       <c r="BV111" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BW111" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -26420,6 +26756,9 @@
       <c r="BV112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BW112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -26650,6 +26989,9 @@
       <c r="BV113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BW113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -26880,6 +27222,9 @@
       <c r="BV114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BW114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -27110,6 +27455,9 @@
       <c r="BV115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BW115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -27340,6 +27688,9 @@
       <c r="BV116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BW116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -27570,6 +27921,9 @@
       <c r="BV117" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BW117" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -27800,6 +28154,9 @@
       <c r="BV118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BW118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -28030,6 +28387,9 @@
       <c r="BV119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BW119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -28260,6 +28620,9 @@
       <c r="BV120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BW120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -28490,6 +28853,9 @@
       <c r="BV121" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BW121" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -28720,6 +29086,9 @@
       <c r="BV122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BW122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -28950,6 +29319,9 @@
       <c r="BV123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="BW123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -29180,6 +29552,9 @@
       <c r="BV124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BW124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -29410,6 +29785,9 @@
       <c r="BV125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BW125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -29640,6 +30018,9 @@
       <c r="BV126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BW126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -29870,6 +30251,9 @@
       <c r="BV127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BW127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -30100,6 +30484,9 @@
       <c r="BV128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BW128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -30330,6 +30717,9 @@
       <c r="BV129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BW129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -30560,6 +30950,9 @@
       <c r="BV130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BW130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -30790,6 +31183,9 @@
       <c r="BV131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BW131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -31020,6 +31416,9 @@
       <c r="BV132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="BW132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -31250,6 +31649,9 @@
       <c r="BV133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BW133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -31480,6 +31882,9 @@
       <c r="BV134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="BW134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -31710,6 +32115,9 @@
       <c r="BV135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BW135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -31940,6 +32348,9 @@
       <c r="BV136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BW136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -32170,6 +32581,9 @@
       <c r="BV137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BW137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -32400,6 +32814,9 @@
       <c r="BV138" s="3" t="n">
         <v>23.29</v>
       </c>
+      <c r="BW138" s="3" t="n">
+        <v>23.29</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -32630,6 +33047,9 @@
       <c r="BV139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BW139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -32860,6 +33280,9 @@
       <c r="BV140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BW140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -33090,6 +33513,9 @@
       <c r="BV141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BW141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -33320,6 +33746,9 @@
       <c r="BV142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BW142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -33550,6 +33979,9 @@
       <c r="BV143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BW143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -33780,6 +34212,9 @@
       <c r="BV144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BW144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -34010,6 +34445,9 @@
       <c r="BV145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="BW145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -34240,6 +34678,9 @@
       <c r="BV146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BW146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -34470,6 +34911,9 @@
       <c r="BV147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BW147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -34700,6 +35144,9 @@
       <c r="BV148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BW148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -34930,6 +35377,9 @@
       <c r="BV149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="BW149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -35160,6 +35610,9 @@
       <c r="BV150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BW150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -35390,6 +35843,9 @@
       <c r="BV151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BW151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -35620,6 +36076,9 @@
       <c r="BV152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BW152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -35850,6 +36309,9 @@
       <c r="BV153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BW153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -36080,6 +36542,9 @@
       <c r="BV154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="BW154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -36310,6 +36775,9 @@
       <c r="BV155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BW155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -36540,6 +37008,9 @@
       <c r="BV156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BW156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -36770,6 +37241,9 @@
       <c r="BV157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BW157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -37000,6 +37474,9 @@
       <c r="BV158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BW158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -37230,6 +37707,9 @@
       <c r="BV159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="BW159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -37460,6 +37940,9 @@
       <c r="BV160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BW160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -37690,6 +38173,9 @@
       <c r="BV161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BW161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -37920,6 +38406,9 @@
       <c r="BV162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="BW162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -38150,6 +38639,9 @@
       <c r="BV163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="BW163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -38380,6 +38872,9 @@
       <c r="BV164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="BW164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -38511,9 +39006,12 @@
       <c r="BV165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="BW165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BV165"/>
+  <autoFilter ref="A1:BW165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-13 21:08 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BW$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BX$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BW165"/>
+  <dimension ref="A1:BX165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -518,6 +518,7 @@
     <col width="16" customWidth="1" min="73" max="73"/>
     <col width="16" customWidth="1" min="74" max="74"/>
     <col width="16" customWidth="1" min="75" max="75"/>
+    <col width="16" customWidth="1" min="76" max="76"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -896,6 +897,11 @@
           <t>2026-09-13 13:10</t>
         </is>
       </c>
+      <c r="BX1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-13 16:08</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1129,6 +1135,9 @@
       <c r="BW2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="BX2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1362,6 +1371,9 @@
       <c r="BW3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="BX3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1595,6 +1607,9 @@
       <c r="BW4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="BX4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1828,6 +1843,9 @@
       <c r="BW5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BX5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2061,6 +2079,9 @@
       <c r="BW6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BX6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2294,6 +2315,9 @@
       <c r="BW7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="BX7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2527,6 +2551,9 @@
       <c r="BW8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="BX8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2760,6 +2787,9 @@
       <c r="BW9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="BX9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2993,6 +3023,9 @@
       <c r="BW10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BX10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3226,6 +3259,9 @@
       <c r="BW11" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX11" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3459,6 +3495,9 @@
       <c r="BW12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3692,6 +3731,9 @@
       <c r="BW13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="BX13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3925,6 +3967,9 @@
       <c r="BW14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4158,6 +4203,9 @@
       <c r="BW15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="BX15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4391,6 +4439,9 @@
       <c r="BW16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BX16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4624,6 +4675,9 @@
       <c r="BW17" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BX17" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -4857,6 +4911,9 @@
       <c r="BW18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BX18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5090,6 +5147,9 @@
       <c r="BW19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="BX19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5323,6 +5383,9 @@
       <c r="BW20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="BX20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -5556,6 +5619,9 @@
       <c r="BW21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="BX21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -5789,6 +5855,9 @@
       <c r="BW22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BX22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -6022,6 +6091,9 @@
       <c r="BW23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BX23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -6255,6 +6327,9 @@
       <c r="BW24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BX24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -6488,6 +6563,9 @@
       <c r="BW25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -6721,6 +6799,9 @@
       <c r="BW26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="BX26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -6954,6 +7035,9 @@
       <c r="BW27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BX27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -7187,6 +7271,9 @@
       <c r="BW28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BX28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -7420,6 +7507,9 @@
       <c r="BW29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BX29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -7653,6 +7743,9 @@
       <c r="BW30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -7886,6 +7979,9 @@
       <c r="BW31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -8119,6 +8215,9 @@
       <c r="BW32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -8352,6 +8451,9 @@
       <c r="BW33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BX33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -8585,6 +8687,9 @@
       <c r="BW34" s="3" t="n">
         <v>21.22</v>
       </c>
+      <c r="BX34" s="3" t="n">
+        <v>21.22</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -8818,6 +8923,9 @@
       <c r="BW35" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BX35" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -9051,6 +9159,9 @@
       <c r="BW36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BX36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -9284,6 +9395,9 @@
       <c r="BW37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BX37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -9517,6 +9631,9 @@
       <c r="BW38" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX38" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -9750,6 +9867,9 @@
       <c r="BW39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="BX39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -9983,6 +10103,9 @@
       <c r="BW40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -10216,6 +10339,9 @@
       <c r="BW41" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX41" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -10449,6 +10575,9 @@
       <c r="BW42" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX42" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -10682,6 +10811,9 @@
       <c r="BW43" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BX43" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -10915,6 +11047,9 @@
       <c r="BW44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BX44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -11148,6 +11283,9 @@
       <c r="BW45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BX45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -11381,6 +11519,9 @@
       <c r="BW46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="BX46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -11614,6 +11755,9 @@
       <c r="BW47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BX47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -11847,6 +11991,9 @@
       <c r="BW48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BX48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -12080,6 +12227,9 @@
       <c r="BW49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BX49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -12313,6 +12463,9 @@
       <c r="BW50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BX50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -12546,6 +12699,9 @@
       <c r="BW51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="BX51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -12779,6 +12935,9 @@
       <c r="BW52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BX52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -13012,6 +13171,9 @@
       <c r="BW53" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BX53" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -13245,6 +13407,9 @@
       <c r="BW54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BX54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -13478,6 +13643,9 @@
       <c r="BW55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="BX55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -13711,6 +13879,9 @@
       <c r="BW56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BX56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -13944,6 +14115,9 @@
       <c r="BW57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -14177,6 +14351,9 @@
       <c r="BW58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="BX58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -14410,6 +14587,9 @@
       <c r="BW59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="BX59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -14643,6 +14823,9 @@
       <c r="BW60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="BX60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -14876,6 +15059,9 @@
       <c r="BW61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="BX61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -15109,6 +15295,9 @@
       <c r="BW62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="BX62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -15342,6 +15531,9 @@
       <c r="BW63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="BX63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -15575,6 +15767,9 @@
       <c r="BW64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BX64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -15808,6 +16003,9 @@
       <c r="BW65" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BX65" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -16041,6 +16239,9 @@
       <c r="BW66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -16274,6 +16475,9 @@
       <c r="BW67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BX67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -16507,6 +16711,9 @@
       <c r="BW68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -16740,6 +16947,9 @@
       <c r="BW69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BX69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -16973,6 +17183,9 @@
       <c r="BW70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BX70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -17206,6 +17419,9 @@
       <c r="BW71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -17439,6 +17655,9 @@
       <c r="BW72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -17672,6 +17891,9 @@
       <c r="BW73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BX73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -17905,6 +18127,9 @@
       <c r="BW74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BX74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -18138,6 +18363,9 @@
       <c r="BW75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -18371,6 +18599,9 @@
       <c r="BW76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -18604,6 +18835,9 @@
       <c r="BW77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -18837,6 +19071,9 @@
       <c r="BW78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BX78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -19070,6 +19307,9 @@
       <c r="BW79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -19303,6 +19543,9 @@
       <c r="BW80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BX80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -19536,6 +19779,9 @@
       <c r="BW81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -19769,6 +20015,9 @@
       <c r="BW82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -20002,6 +20251,9 @@
       <c r="BW83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -20235,6 +20487,9 @@
       <c r="BW84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BX84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -20468,6 +20723,9 @@
       <c r="BW85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BX85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -20701,6 +20959,9 @@
       <c r="BW86" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BX86" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -20934,6 +21195,9 @@
       <c r="BW87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -21167,6 +21431,9 @@
       <c r="BW88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -21400,6 +21667,9 @@
       <c r="BW89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -21633,6 +21903,9 @@
       <c r="BW90" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BX90" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -21866,6 +22139,9 @@
       <c r="BW91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -22099,6 +22375,9 @@
       <c r="BW92" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="BX92" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -22332,6 +22611,9 @@
       <c r="BW93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="BX93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -22565,6 +22847,9 @@
       <c r="BW94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BX94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -22798,6 +23083,9 @@
       <c r="BW95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BX95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -23031,6 +23319,9 @@
       <c r="BW96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BX96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -23264,6 +23555,9 @@
       <c r="BW97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BX97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -23497,6 +23791,9 @@
       <c r="BW98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BX98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -23730,6 +24027,9 @@
       <c r="BW99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BX99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -23963,6 +24263,9 @@
       <c r="BW100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BX100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -24196,6 +24499,9 @@
       <c r="BW101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BX101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -24429,6 +24735,9 @@
       <c r="BW102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BX102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -24662,6 +24971,9 @@
       <c r="BW103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BX103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -24895,6 +25207,9 @@
       <c r="BW104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BX104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -25128,6 +25443,9 @@
       <c r="BW105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BX105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -25361,6 +25679,9 @@
       <c r="BW106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BX106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -25594,6 +25915,9 @@
       <c r="BW107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BX107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -25827,6 +26151,9 @@
       <c r="BW108" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BX108" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -26060,6 +26387,9 @@
       <c r="BW109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BX109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -26293,6 +26623,9 @@
       <c r="BW110" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BX110" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -26526,6 +26859,9 @@
       <c r="BW111" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BX111" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -26759,6 +27095,9 @@
       <c r="BW112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BX112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -26992,6 +27331,9 @@
       <c r="BW113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BX113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -27225,6 +27567,9 @@
       <c r="BW114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BX114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -27458,6 +27803,9 @@
       <c r="BW115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BX115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -27691,6 +28039,9 @@
       <c r="BW116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BX116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -27924,6 +28275,9 @@
       <c r="BW117" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BX117" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -28157,6 +28511,9 @@
       <c r="BW118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BX118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -28390,6 +28747,9 @@
       <c r="BW119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BX119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -28623,6 +28983,9 @@
       <c r="BW120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BX120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -28856,6 +29219,9 @@
       <c r="BW121" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BX121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -29089,6 +29455,9 @@
       <c r="BW122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BX122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -29322,6 +29691,9 @@
       <c r="BW123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="BX123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -29555,6 +29927,9 @@
       <c r="BW124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BX124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -29788,6 +30163,9 @@
       <c r="BW125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BX125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -30021,6 +30399,9 @@
       <c r="BW126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BX126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -30254,6 +30635,9 @@
       <c r="BW127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BX127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -30487,6 +30871,9 @@
       <c r="BW128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BX128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -30720,6 +31107,9 @@
       <c r="BW129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BX129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -30953,6 +31343,9 @@
       <c r="BW130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BX130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -31186,6 +31579,9 @@
       <c r="BW131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BX131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -31419,6 +31815,9 @@
       <c r="BW132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="BX132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -31652,6 +32051,9 @@
       <c r="BW133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BX133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -31885,6 +32287,9 @@
       <c r="BW134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="BX134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -32118,6 +32523,9 @@
       <c r="BW135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BX135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -32351,6 +32759,9 @@
       <c r="BW136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BX136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -32584,6 +32995,9 @@
       <c r="BW137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BX137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -32817,6 +33231,9 @@
       <c r="BW138" s="3" t="n">
         <v>23.29</v>
       </c>
+      <c r="BX138" s="3" t="n">
+        <v>23.29</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -33050,6 +33467,9 @@
       <c r="BW139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BX139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -33283,6 +33703,9 @@
       <c r="BW140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BX140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -33516,6 +33939,9 @@
       <c r="BW141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BX141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -33749,6 +34175,9 @@
       <c r="BW142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BX142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -33982,6 +34411,9 @@
       <c r="BW143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BX143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -34215,6 +34647,9 @@
       <c r="BW144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BX144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -34448,6 +34883,9 @@
       <c r="BW145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="BX145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -34681,6 +35119,9 @@
       <c r="BW146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BX146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -34914,6 +35355,9 @@
       <c r="BW147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BX147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -35147,6 +35591,9 @@
       <c r="BW148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BX148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -35380,6 +35827,9 @@
       <c r="BW149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="BX149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -35613,6 +36063,9 @@
       <c r="BW150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BX150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -35846,6 +36299,9 @@
       <c r="BW151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BX151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -36079,6 +36535,9 @@
       <c r="BW152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BX152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -36312,6 +36771,9 @@
       <c r="BW153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BX153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -36545,6 +37007,9 @@
       <c r="BW154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="BX154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -36778,6 +37243,9 @@
       <c r="BW155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BX155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -37011,6 +37479,9 @@
       <c r="BW156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BX156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -37244,6 +37715,9 @@
       <c r="BW157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BX157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -37477,6 +37951,9 @@
       <c r="BW158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BX158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -37710,6 +38187,9 @@
       <c r="BW159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="BX159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -37943,6 +38423,9 @@
       <c r="BW160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BX160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -38176,6 +38659,9 @@
       <c r="BW161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BX161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -38409,6 +38895,9 @@
       <c r="BW162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="BX162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -38642,6 +39131,9 @@
       <c r="BW163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="BX163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -38875,6 +39367,9 @@
       <c r="BW164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="BX164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -39009,9 +39504,12 @@
       <c r="BW165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="BX165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BW165"/>
+  <autoFilter ref="A1:BX165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-14 00:14 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BX$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BY$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BX165"/>
+  <dimension ref="A1:BY165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -519,6 +519,7 @@
     <col width="16" customWidth="1" min="74" max="74"/>
     <col width="16" customWidth="1" min="75" max="75"/>
     <col width="16" customWidth="1" min="76" max="76"/>
+    <col width="16" customWidth="1" min="77" max="77"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -902,6 +903,11 @@
           <t>2026-09-13 16:08</t>
         </is>
       </c>
+      <c r="BY1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-13 19:14</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1138,6 +1144,9 @@
       <c r="BX2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="BY2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1374,6 +1383,9 @@
       <c r="BX3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="BY3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1610,6 +1622,9 @@
       <c r="BX4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="BY4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1846,6 +1861,9 @@
       <c r="BX5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BY5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2082,6 +2100,9 @@
       <c r="BX6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BY6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2318,6 +2339,9 @@
       <c r="BX7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="BY7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2554,6 +2578,9 @@
       <c r="BX8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="BY8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2790,6 +2817,9 @@
       <c r="BX9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="BY9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3026,6 +3056,9 @@
       <c r="BX10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BY10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3262,6 +3295,9 @@
       <c r="BX11" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY11" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3498,6 +3534,9 @@
       <c r="BX12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3734,6 +3773,9 @@
       <c r="BX13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="BY13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -3970,6 +4012,9 @@
       <c r="BX14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4206,6 +4251,9 @@
       <c r="BX15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="BY15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4442,6 +4490,9 @@
       <c r="BX16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BY16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4678,6 +4729,9 @@
       <c r="BX17" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BY17" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -4914,6 +4968,9 @@
       <c r="BX18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BY18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5150,6 +5207,9 @@
       <c r="BX19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="BY19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5386,6 +5446,9 @@
       <c r="BX20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="BY20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -5622,6 +5685,9 @@
       <c r="BX21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="BY21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -5858,6 +5924,9 @@
       <c r="BX22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BY22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -6094,6 +6163,9 @@
       <c r="BX23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BY23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -6330,6 +6402,9 @@
       <c r="BX24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BY24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -6566,6 +6641,9 @@
       <c r="BX25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -6802,6 +6880,9 @@
       <c r="BX26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="BY26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -7038,6 +7119,9 @@
       <c r="BX27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BY27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -7274,6 +7358,9 @@
       <c r="BX28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BY28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -7510,6 +7597,9 @@
       <c r="BX29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BY29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -7746,6 +7836,9 @@
       <c r="BX30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -7982,6 +8075,9 @@
       <c r="BX31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -8218,6 +8314,9 @@
       <c r="BX32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -8454,6 +8553,9 @@
       <c r="BX33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BY33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -8690,6 +8792,9 @@
       <c r="BX34" s="3" t="n">
         <v>21.22</v>
       </c>
+      <c r="BY34" s="3" t="n">
+        <v>21.22</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -8926,6 +9031,9 @@
       <c r="BX35" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BY35" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -9162,6 +9270,9 @@
       <c r="BX36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BY36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -9398,6 +9509,9 @@
       <c r="BX37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BY37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -9634,6 +9748,9 @@
       <c r="BX38" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY38" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -9870,6 +9987,9 @@
       <c r="BX39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="BY39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -10106,6 +10226,9 @@
       <c r="BX40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -10342,6 +10465,9 @@
       <c r="BX41" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY41" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -10578,6 +10704,9 @@
       <c r="BX42" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY42" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -10814,6 +10943,9 @@
       <c r="BX43" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BY43" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -11050,6 +11182,9 @@
       <c r="BX44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BY44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -11286,6 +11421,9 @@
       <c r="BX45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BY45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -11522,6 +11660,9 @@
       <c r="BX46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="BY46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -11758,6 +11899,9 @@
       <c r="BX47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BY47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -11994,6 +12138,9 @@
       <c r="BX48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BY48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -12230,6 +12377,9 @@
       <c r="BX49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BY49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -12466,6 +12616,9 @@
       <c r="BX50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BY50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -12702,6 +12855,9 @@
       <c r="BX51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="BY51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -12938,6 +13094,9 @@
       <c r="BX52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BY52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -13174,6 +13333,9 @@
       <c r="BX53" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BY53" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -13410,6 +13572,9 @@
       <c r="BX54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BY54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -13646,6 +13811,9 @@
       <c r="BX55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="BY55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -13882,6 +14050,9 @@
       <c r="BX56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BY56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -14118,6 +14289,9 @@
       <c r="BX57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -14354,6 +14528,9 @@
       <c r="BX58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="BY58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -14590,6 +14767,9 @@
       <c r="BX59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="BY59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -14826,6 +15006,9 @@
       <c r="BX60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="BY60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -15062,6 +15245,9 @@
       <c r="BX61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="BY61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -15298,6 +15484,9 @@
       <c r="BX62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="BY62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -15534,6 +15723,9 @@
       <c r="BX63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="BY63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -15770,6 +15962,9 @@
       <c r="BX64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BY64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -16006,6 +16201,9 @@
       <c r="BX65" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BY65" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -16242,6 +16440,9 @@
       <c r="BX66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -16478,6 +16679,9 @@
       <c r="BX67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BY67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -16714,6 +16918,9 @@
       <c r="BX68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -16950,6 +17157,9 @@
       <c r="BX69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BY69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -17186,6 +17396,9 @@
       <c r="BX70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BY70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -17422,6 +17635,9 @@
       <c r="BX71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -17658,6 +17874,9 @@
       <c r="BX72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -17894,6 +18113,9 @@
       <c r="BX73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BY73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -18130,6 +18352,9 @@
       <c r="BX74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BY74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -18366,6 +18591,9 @@
       <c r="BX75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -18602,6 +18830,9 @@
       <c r="BX76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -18838,6 +19069,9 @@
       <c r="BX77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -19074,6 +19308,9 @@
       <c r="BX78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BY78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -19310,6 +19547,9 @@
       <c r="BX79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -19546,6 +19786,9 @@
       <c r="BX80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BY80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -19782,6 +20025,9 @@
       <c r="BX81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -20018,6 +20264,9 @@
       <c r="BX82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -20254,6 +20503,9 @@
       <c r="BX83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -20490,6 +20742,9 @@
       <c r="BX84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BY84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -20726,6 +20981,9 @@
       <c r="BX85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BY85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -20962,6 +21220,9 @@
       <c r="BX86" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BY86" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -21198,6 +21459,9 @@
       <c r="BX87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -21434,6 +21698,9 @@
       <c r="BX88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -21670,6 +21937,9 @@
       <c r="BX89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -21906,6 +22176,9 @@
       <c r="BX90" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BY90" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -22142,6 +22415,9 @@
       <c r="BX91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -22378,6 +22654,9 @@
       <c r="BX92" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="BY92" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -22614,6 +22893,9 @@
       <c r="BX93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="BY93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -22850,6 +23132,9 @@
       <c r="BX94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BY94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -23086,6 +23371,9 @@
       <c r="BX95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BY95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -23322,6 +23610,9 @@
       <c r="BX96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BY96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -23558,6 +23849,9 @@
       <c r="BX97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BY97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -23794,6 +24088,9 @@
       <c r="BX98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BY98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -24030,6 +24327,9 @@
       <c r="BX99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BY99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -24266,6 +24566,9 @@
       <c r="BX100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BY100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -24502,6 +24805,9 @@
       <c r="BX101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BY101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -24738,6 +25044,9 @@
       <c r="BX102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BY102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -24974,6 +25283,9 @@
       <c r="BX103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BY103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -25210,6 +25522,9 @@
       <c r="BX104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BY104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -25446,6 +25761,9 @@
       <c r="BX105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BY105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -25682,6 +26000,9 @@
       <c r="BX106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BY106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -25918,6 +26239,9 @@
       <c r="BX107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BY107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -26154,6 +26478,9 @@
       <c r="BX108" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BY108" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -26390,6 +26717,9 @@
       <c r="BX109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BY109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -26626,6 +26956,9 @@
       <c r="BX110" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BY110" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -26862,6 +27195,9 @@
       <c r="BX111" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BY111" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -27098,6 +27434,9 @@
       <c r="BX112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BY112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -27334,6 +27673,9 @@
       <c r="BX113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BY113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -27570,6 +27912,9 @@
       <c r="BX114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BY114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -27806,6 +28151,9 @@
       <c r="BX115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BY115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -28042,6 +28390,9 @@
       <c r="BX116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BY116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -28278,6 +28629,9 @@
       <c r="BX117" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BY117" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -28514,6 +28868,9 @@
       <c r="BX118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BY118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -28750,6 +29107,9 @@
       <c r="BX119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BY119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -28986,6 +29346,9 @@
       <c r="BX120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BY120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -29222,6 +29585,9 @@
       <c r="BX121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="BY121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -29458,6 +29824,9 @@
       <c r="BX122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BY122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -29694,6 +30063,9 @@
       <c r="BX123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="BY123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -29930,6 +30302,9 @@
       <c r="BX124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BY124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -30166,6 +30541,9 @@
       <c r="BX125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BY125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -30402,6 +30780,9 @@
       <c r="BX126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BY126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -30638,6 +31019,9 @@
       <c r="BX127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BY127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -30874,6 +31258,9 @@
       <c r="BX128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BY128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -31110,6 +31497,9 @@
       <c r="BX129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BY129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -31346,6 +31736,9 @@
       <c r="BX130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BY130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -31582,6 +31975,9 @@
       <c r="BX131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BY131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -31818,6 +32214,9 @@
       <c r="BX132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="BY132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -32054,6 +32453,9 @@
       <c r="BX133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BY133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -32290,6 +32692,9 @@
       <c r="BX134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="BY134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -32526,6 +32931,9 @@
       <c r="BX135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BY135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -32762,6 +33170,9 @@
       <c r="BX136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BY136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -32998,6 +33409,9 @@
       <c r="BX137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BY137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -33234,6 +33648,9 @@
       <c r="BX138" s="3" t="n">
         <v>23.29</v>
       </c>
+      <c r="BY138" s="3" t="n">
+        <v>23.29</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -33470,6 +33887,9 @@
       <c r="BX139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BY139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -33706,6 +34126,9 @@
       <c r="BX140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BY140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -33942,6 +34365,9 @@
       <c r="BX141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BY141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -34178,6 +34604,9 @@
       <c r="BX142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BY142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -34414,6 +34843,9 @@
       <c r="BX143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BY143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -34650,6 +35082,9 @@
       <c r="BX144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BY144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -34886,6 +35321,9 @@
       <c r="BX145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="BY145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -35122,6 +35560,9 @@
       <c r="BX146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BY146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -35358,6 +35799,9 @@
       <c r="BX147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BY147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -35594,6 +36038,9 @@
       <c r="BX148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BY148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -35830,6 +36277,9 @@
       <c r="BX149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="BY149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -36066,6 +36516,9 @@
       <c r="BX150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BY150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -36302,6 +36755,9 @@
       <c r="BX151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BY151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -36538,6 +36994,9 @@
       <c r="BX152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BY152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -36774,6 +37233,9 @@
       <c r="BX153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BY153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -37010,6 +37472,9 @@
       <c r="BX154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="BY154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -37246,6 +37711,9 @@
       <c r="BX155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BY155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -37482,6 +37950,9 @@
       <c r="BX156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BY156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -37718,6 +38189,9 @@
       <c r="BX157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BY157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -37954,6 +38428,9 @@
       <c r="BX158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BY158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -38190,6 +38667,9 @@
       <c r="BX159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="BY159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -38426,6 +38906,9 @@
       <c r="BX160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BY160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -38662,6 +39145,9 @@
       <c r="BX161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BY161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -38898,6 +39384,9 @@
       <c r="BX162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="BY162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -39134,6 +39623,9 @@
       <c r="BX163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="BY163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -39370,6 +39862,9 @@
       <c r="BX164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="BY164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -39507,9 +40002,12 @@
       <c r="BX165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="BY165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BX165"/>
+  <autoFilter ref="A1:BY165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-14 03:10 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BY$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BZ$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BY165"/>
+  <dimension ref="A1:BZ165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -520,6 +520,7 @@
     <col width="16" customWidth="1" min="75" max="75"/>
     <col width="16" customWidth="1" min="76" max="76"/>
     <col width="16" customWidth="1" min="77" max="77"/>
+    <col width="16" customWidth="1" min="78" max="78"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -908,6 +909,11 @@
           <t>2026-09-13 19:14</t>
         </is>
       </c>
+      <c r="BZ1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-13 22:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1147,6 +1153,9 @@
       <c r="BY2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="BZ2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1386,6 +1395,9 @@
       <c r="BY3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="BZ3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1625,6 +1637,9 @@
       <c r="BY4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="BZ4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1864,6 +1879,9 @@
       <c r="BY5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BZ5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2103,6 +2121,9 @@
       <c r="BY6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="BZ6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2342,6 +2363,9 @@
       <c r="BY7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="BZ7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2581,6 +2605,9 @@
       <c r="BY8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="BZ8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2820,6 +2847,9 @@
       <c r="BY9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="BZ9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3059,6 +3089,9 @@
       <c r="BY10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BZ10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3298,6 +3331,9 @@
       <c r="BY11" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ11" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3537,6 +3573,9 @@
       <c r="BY12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3776,6 +3815,9 @@
       <c r="BY13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="BZ13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4015,6 +4057,9 @@
       <c r="BY14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4254,6 +4299,9 @@
       <c r="BY15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="BZ15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4493,6 +4541,9 @@
       <c r="BY16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BZ16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4732,6 +4783,9 @@
       <c r="BY17" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BZ17" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -4971,6 +5025,9 @@
       <c r="BY18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BZ18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5210,6 +5267,9 @@
       <c r="BY19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="BZ19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5449,6 +5509,9 @@
       <c r="BY20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="BZ20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -5688,6 +5751,9 @@
       <c r="BY21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="BZ21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -5927,6 +5993,9 @@
       <c r="BY22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BZ22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -6166,6 +6235,9 @@
       <c r="BY23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BZ23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -6405,6 +6477,9 @@
       <c r="BY24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BZ24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -6644,6 +6719,9 @@
       <c r="BY25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -6883,6 +6961,9 @@
       <c r="BY26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="BZ26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -7122,6 +7203,9 @@
       <c r="BY27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BZ27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -7361,6 +7445,9 @@
       <c r="BY28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BZ28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -7600,6 +7687,9 @@
       <c r="BY29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BZ29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -7839,6 +7929,9 @@
       <c r="BY30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -8078,6 +8171,9 @@
       <c r="BY31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -8317,6 +8413,9 @@
       <c r="BY32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -8556,6 +8655,9 @@
       <c r="BY33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BZ33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -8795,6 +8897,9 @@
       <c r="BY34" s="3" t="n">
         <v>21.22</v>
       </c>
+      <c r="BZ34" s="3" t="n">
+        <v>21.22</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -9034,6 +9139,9 @@
       <c r="BY35" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BZ35" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -9273,6 +9381,9 @@
       <c r="BY36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BZ36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -9512,6 +9623,9 @@
       <c r="BY37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="BZ37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -9751,6 +9865,9 @@
       <c r="BY38" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ38" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -9990,6 +10107,9 @@
       <c r="BY39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="BZ39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -10229,6 +10349,9 @@
       <c r="BY40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -10468,6 +10591,9 @@
       <c r="BY41" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ41" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -10707,6 +10833,9 @@
       <c r="BY42" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ42" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -10946,6 +11075,9 @@
       <c r="BY43" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BZ43" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -11185,6 +11317,9 @@
       <c r="BY44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BZ44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -11424,6 +11559,9 @@
       <c r="BY45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="BZ45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -11663,6 +11801,9 @@
       <c r="BY46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="BZ46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -11902,6 +12043,9 @@
       <c r="BY47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BZ47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -12141,6 +12285,9 @@
       <c r="BY48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BZ48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -12380,6 +12527,9 @@
       <c r="BY49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BZ49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -12619,6 +12769,9 @@
       <c r="BY50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BZ50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -12858,6 +13011,9 @@
       <c r="BY51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="BZ51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -13097,6 +13253,9 @@
       <c r="BY52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BZ52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -13336,6 +13495,9 @@
       <c r="BY53" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BZ53" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -13575,6 +13737,9 @@
       <c r="BY54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BZ54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -13814,6 +13979,9 @@
       <c r="BY55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="BZ55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -14053,6 +14221,9 @@
       <c r="BY56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="BZ56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -14292,6 +14463,9 @@
       <c r="BY57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -14531,6 +14705,9 @@
       <c r="BY58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="BZ58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -14770,6 +14947,9 @@
       <c r="BY59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="BZ59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -15009,6 +15189,9 @@
       <c r="BY60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="BZ60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -15248,6 +15431,9 @@
       <c r="BY61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="BZ61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -15487,6 +15673,9 @@
       <c r="BY62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="BZ62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -15726,6 +15915,9 @@
       <c r="BY63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="BZ63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -15965,6 +16157,9 @@
       <c r="BY64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BZ64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -16204,6 +16399,9 @@
       <c r="BY65" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BZ65" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -16443,6 +16641,9 @@
       <c r="BY66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -16682,6 +16883,9 @@
       <c r="BY67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BZ67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -16921,6 +17125,9 @@
       <c r="BY68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -17160,6 +17367,9 @@
       <c r="BY69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BZ69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -17399,6 +17609,9 @@
       <c r="BY70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BZ70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -17638,6 +17851,9 @@
       <c r="BY71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -17877,6 +18093,9 @@
       <c r="BY72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -18116,6 +18335,9 @@
       <c r="BY73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BZ73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -18355,6 +18577,9 @@
       <c r="BY74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BZ74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -18594,6 +18819,9 @@
       <c r="BY75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -18833,6 +19061,9 @@
       <c r="BY76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -19072,6 +19303,9 @@
       <c r="BY77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -19311,6 +19545,9 @@
       <c r="BY78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BZ78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -19550,6 +19787,9 @@
       <c r="BY79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -19789,6 +20029,9 @@
       <c r="BY80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BZ80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -20028,6 +20271,9 @@
       <c r="BY81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -20267,6 +20513,9 @@
       <c r="BY82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -20506,6 +20755,9 @@
       <c r="BY83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -20745,6 +20997,9 @@
       <c r="BY84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BZ84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -20984,6 +21239,9 @@
       <c r="BY85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BZ85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -21223,6 +21481,9 @@
       <c r="BY86" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BZ86" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -21462,6 +21723,9 @@
       <c r="BY87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -21701,6 +21965,9 @@
       <c r="BY88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -21940,6 +22207,9 @@
       <c r="BY89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -22179,6 +22449,9 @@
       <c r="BY90" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BZ90" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -22418,6 +22691,9 @@
       <c r="BY91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -22657,6 +22933,9 @@
       <c r="BY92" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="BZ92" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -22896,6 +23175,9 @@
       <c r="BY93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="BZ93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -23135,6 +23417,9 @@
       <c r="BY94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BZ94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -23374,6 +23659,9 @@
       <c r="BY95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BZ95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -23613,6 +23901,9 @@
       <c r="BY96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="BZ96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -23852,6 +24143,9 @@
       <c r="BY97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BZ97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -24091,6 +24385,9 @@
       <c r="BY98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="BZ98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -24330,6 +24627,9 @@
       <c r="BY99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="BZ99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -24569,6 +24869,9 @@
       <c r="BY100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BZ100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -24808,6 +25111,9 @@
       <c r="BY101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BZ101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -25047,6 +25353,9 @@
       <c r="BY102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BZ102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -25286,6 +25595,9 @@
       <c r="BY103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="BZ103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -25525,6 +25837,9 @@
       <c r="BY104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BZ104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -25764,6 +26079,9 @@
       <c r="BY105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BZ105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -26003,6 +26321,9 @@
       <c r="BY106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="BZ106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -26242,6 +26563,9 @@
       <c r="BY107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="BZ107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -26481,6 +26805,9 @@
       <c r="BY108" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BZ108" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -26720,6 +27047,9 @@
       <c r="BY109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BZ109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -26959,6 +27289,9 @@
       <c r="BY110" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="BZ110" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -27198,6 +27531,9 @@
       <c r="BY111" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BZ111" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -27437,6 +27773,9 @@
       <c r="BY112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BZ112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -27676,6 +28015,9 @@
       <c r="BY113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BZ113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -27915,6 +28257,9 @@
       <c r="BY114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BZ114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -28154,6 +28499,9 @@
       <c r="BY115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="BZ115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -28393,6 +28741,9 @@
       <c r="BY116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BZ116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -28632,6 +28983,9 @@
       <c r="BY117" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="BZ117" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -28871,6 +29225,9 @@
       <c r="BY118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="BZ118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -29110,6 +29467,9 @@
       <c r="BY119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="BZ119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -29349,6 +29709,9 @@
       <c r="BY120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="BZ120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -29588,6 +29951,9 @@
       <c r="BY121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="BZ121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -29827,6 +30193,9 @@
       <c r="BY122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="BZ122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -30066,6 +30435,9 @@
       <c r="BY123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="BZ123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -30305,6 +30677,9 @@
       <c r="BY124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BZ124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -30544,6 +30919,9 @@
       <c r="BY125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BZ125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -30783,6 +31161,9 @@
       <c r="BY126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BZ126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -31022,6 +31403,9 @@
       <c r="BY127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="BZ127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -31261,6 +31645,9 @@
       <c r="BY128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BZ128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -31500,6 +31887,9 @@
       <c r="BY129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BZ129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -31739,6 +32129,9 @@
       <c r="BY130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BZ130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -31978,6 +32371,9 @@
       <c r="BY131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="BZ131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -32217,6 +32613,9 @@
       <c r="BY132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="BZ132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -32456,6 +32855,9 @@
       <c r="BY133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BZ133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -32695,6 +33097,9 @@
       <c r="BY134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="BZ134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -32934,6 +33339,9 @@
       <c r="BY135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BZ135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -33173,6 +33581,9 @@
       <c r="BY136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BZ136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -33412,6 +33823,9 @@
       <c r="BY137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="BZ137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -33651,6 +34065,9 @@
       <c r="BY138" s="3" t="n">
         <v>23.29</v>
       </c>
+      <c r="BZ138" s="3" t="n">
+        <v>23.29</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -33890,6 +34307,9 @@
       <c r="BY139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BZ139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -34129,6 +34549,9 @@
       <c r="BY140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BZ140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -34368,6 +34791,9 @@
       <c r="BY141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BZ141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -34607,6 +35033,9 @@
       <c r="BY142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BZ142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -34846,6 +35275,9 @@
       <c r="BY143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BZ143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -35085,6 +35517,9 @@
       <c r="BY144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="BZ144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -35324,6 +35759,9 @@
       <c r="BY145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="BZ145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -35563,6 +36001,9 @@
       <c r="BY146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BZ146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -35802,6 +36243,9 @@
       <c r="BY147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="BZ147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -36041,6 +36485,9 @@
       <c r="BY148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="BZ148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -36280,6 +36727,9 @@
       <c r="BY149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="BZ149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -36519,6 +36969,9 @@
       <c r="BY150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="BZ150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -36758,6 +37211,9 @@
       <c r="BY151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BZ151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -36997,6 +37453,9 @@
       <c r="BY152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BZ152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -37236,6 +37695,9 @@
       <c r="BY153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="BZ153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -37475,6 +37937,9 @@
       <c r="BY154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="BZ154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -37714,6 +38179,9 @@
       <c r="BY155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="BZ155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -37953,6 +38421,9 @@
       <c r="BY156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BZ156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -38192,6 +38663,9 @@
       <c r="BY157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="BZ157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -38431,6 +38905,9 @@
       <c r="BY158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BZ158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -38670,6 +39147,9 @@
       <c r="BY159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="BZ159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -38909,6 +39389,9 @@
       <c r="BY160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BZ160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -39148,6 +39631,9 @@
       <c r="BY161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="BZ161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -39387,6 +39873,9 @@
       <c r="BY162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="BZ162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -39626,6 +40115,9 @@
       <c r="BY163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="BZ163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -39865,6 +40357,9 @@
       <c r="BY164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="BZ164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -40005,9 +40500,12 @@
       <c r="BY165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="BZ165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BY165"/>
+  <autoFilter ref="A1:BZ165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-14 06:14 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$BZ$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CA$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BZ165"/>
+  <dimension ref="A1:CA165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -521,6 +521,7 @@
     <col width="16" customWidth="1" min="76" max="76"/>
     <col width="16" customWidth="1" min="77" max="77"/>
     <col width="16" customWidth="1" min="78" max="78"/>
+    <col width="16" customWidth="1" min="79" max="79"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -914,6 +915,11 @@
           <t>2026-09-13 22:09</t>
         </is>
       </c>
+      <c r="CA1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-14 01:13</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1156,6 +1162,9 @@
       <c r="BZ2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CA2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1398,6 +1407,9 @@
       <c r="BZ3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CA3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1640,6 +1652,9 @@
       <c r="BZ4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CA4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1882,6 +1897,9 @@
       <c r="BZ5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CA5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2124,6 +2142,9 @@
       <c r="BZ6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CA6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2366,6 +2387,9 @@
       <c r="BZ7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CA7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2608,6 +2632,9 @@
       <c r="BZ8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="CA8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2850,6 +2877,9 @@
       <c r="BZ9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CA9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3092,6 +3122,9 @@
       <c r="BZ10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CA10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3334,6 +3367,9 @@
       <c r="BZ11" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA11" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3576,6 +3612,9 @@
       <c r="BZ12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3818,6 +3857,9 @@
       <c r="BZ13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CA13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4060,6 +4102,9 @@
       <c r="BZ14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4302,6 +4347,9 @@
       <c r="BZ15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="CA15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4544,6 +4592,9 @@
       <c r="BZ16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CA16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4786,6 +4837,9 @@
       <c r="BZ17" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CA17" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5028,6 +5082,9 @@
       <c r="BZ18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CA18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5270,6 +5327,9 @@
       <c r="BZ19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="CA19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5512,6 +5572,9 @@
       <c r="BZ20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="CA20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -5754,6 +5817,9 @@
       <c r="BZ21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="CA21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -5996,6 +6062,9 @@
       <c r="BZ22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CA22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -6238,6 +6307,9 @@
       <c r="BZ23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CA23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -6480,6 +6552,9 @@
       <c r="BZ24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CA24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -6722,6 +6797,9 @@
       <c r="BZ25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -6964,6 +7042,9 @@
       <c r="BZ26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="CA26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -7206,6 +7287,9 @@
       <c r="BZ27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CA27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -7448,6 +7532,9 @@
       <c r="BZ28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CA28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -7690,6 +7777,9 @@
       <c r="BZ29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CA29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -7932,6 +8022,9 @@
       <c r="BZ30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -8174,6 +8267,9 @@
       <c r="BZ31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -8416,6 +8512,9 @@
       <c r="BZ32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -8658,6 +8757,9 @@
       <c r="BZ33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CA33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -8900,6 +9002,9 @@
       <c r="BZ34" s="3" t="n">
         <v>21.22</v>
       </c>
+      <c r="CA34" s="3" t="n">
+        <v>21.22</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -9142,6 +9247,9 @@
       <c r="BZ35" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CA35" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -9384,6 +9492,9 @@
       <c r="BZ36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CA36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -9626,6 +9737,9 @@
       <c r="BZ37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CA37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -9868,6 +9982,9 @@
       <c r="BZ38" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA38" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -10110,6 +10227,9 @@
       <c r="BZ39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CA39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -10352,6 +10472,9 @@
       <c r="BZ40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -10594,6 +10717,9 @@
       <c r="BZ41" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA41" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -10836,6 +10962,9 @@
       <c r="BZ42" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA42" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -11078,6 +11207,9 @@
       <c r="BZ43" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CA43" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -11320,6 +11452,9 @@
       <c r="BZ44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CA44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -11562,6 +11697,9 @@
       <c r="BZ45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="CA45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -11804,6 +11942,9 @@
       <c r="BZ46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="CA46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -12046,6 +12187,9 @@
       <c r="BZ47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CA47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -12288,6 +12432,9 @@
       <c r="BZ48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CA48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -12530,6 +12677,9 @@
       <c r="BZ49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CA49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -12772,6 +12922,9 @@
       <c r="BZ50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CA50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -13014,6 +13167,9 @@
       <c r="BZ51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CA51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -13256,6 +13412,9 @@
       <c r="BZ52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CA52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -13498,6 +13657,9 @@
       <c r="BZ53" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CA53" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -13740,6 +13902,9 @@
       <c r="BZ54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CA54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -13982,6 +14147,9 @@
       <c r="BZ55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="CA55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -14224,6 +14392,9 @@
       <c r="BZ56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CA56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -14466,6 +14637,9 @@
       <c r="BZ57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -14708,6 +14882,9 @@
       <c r="BZ58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CA58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -14950,6 +15127,9 @@
       <c r="BZ59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CA59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -15192,6 +15372,9 @@
       <c r="BZ60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CA60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -15434,6 +15617,9 @@
       <c r="BZ61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CA61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -15676,6 +15862,9 @@
       <c r="BZ62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CA62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -15918,6 +16107,9 @@
       <c r="BZ63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CA63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -16160,6 +16352,9 @@
       <c r="BZ64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CA64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -16402,6 +16597,9 @@
       <c r="BZ65" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CA65" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -16644,6 +16842,9 @@
       <c r="BZ66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -16886,6 +17087,9 @@
       <c r="BZ67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CA67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -17128,6 +17332,9 @@
       <c r="BZ68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -17370,6 +17577,9 @@
       <c r="BZ69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CA69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -17612,6 +17822,9 @@
       <c r="BZ70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CA70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -17854,6 +18067,9 @@
       <c r="BZ71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -18096,6 +18312,9 @@
       <c r="BZ72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -18338,6 +18557,9 @@
       <c r="BZ73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CA73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -18580,6 +18802,9 @@
       <c r="BZ74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CA74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -18822,6 +19047,9 @@
       <c r="BZ75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -19064,6 +19292,9 @@
       <c r="BZ76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -19306,6 +19537,9 @@
       <c r="BZ77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -19548,6 +19782,9 @@
       <c r="BZ78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CA78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -19790,6 +20027,9 @@
       <c r="BZ79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -20032,6 +20272,9 @@
       <c r="BZ80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CA80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -20274,6 +20517,9 @@
       <c r="BZ81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -20516,6 +20762,9 @@
       <c r="BZ82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -20758,6 +21007,9 @@
       <c r="BZ83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -21000,6 +21252,9 @@
       <c r="BZ84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CA84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -21242,6 +21497,9 @@
       <c r="BZ85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CA85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -21484,6 +21742,9 @@
       <c r="BZ86" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CA86" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -21726,6 +21987,9 @@
       <c r="BZ87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -21968,6 +22232,9 @@
       <c r="BZ88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -22210,6 +22477,9 @@
       <c r="BZ89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -22452,6 +22722,9 @@
       <c r="BZ90" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CA90" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -22694,6 +22967,9 @@
       <c r="BZ91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -22936,6 +23212,9 @@
       <c r="BZ92" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CA92" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -23178,6 +23457,9 @@
       <c r="BZ93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CA93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -23420,6 +23702,9 @@
       <c r="BZ94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CA94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -23662,6 +23947,9 @@
       <c r="BZ95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CA95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -23904,6 +24192,9 @@
       <c r="BZ96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CA96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -24146,6 +24437,9 @@
       <c r="BZ97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CA97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -24388,6 +24682,9 @@
       <c r="BZ98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="CA98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -24630,6 +24927,9 @@
       <c r="BZ99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CA99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -24872,6 +25172,9 @@
       <c r="BZ100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CA100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -25114,6 +25417,9 @@
       <c r="BZ101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CA101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -25356,6 +25662,9 @@
       <c r="BZ102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CA102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -25598,6 +25907,9 @@
       <c r="BZ103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CA103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -25840,6 +26152,9 @@
       <c r="BZ104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CA104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -26082,6 +26397,9 @@
       <c r="BZ105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CA105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -26324,6 +26642,9 @@
       <c r="BZ106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CA106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -26566,6 +26887,9 @@
       <c r="BZ107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CA107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -26808,6 +27132,9 @@
       <c r="BZ108" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CA108" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -27050,6 +27377,9 @@
       <c r="BZ109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CA109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -27292,6 +27622,9 @@
       <c r="BZ110" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CA110" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -27534,6 +27867,9 @@
       <c r="BZ111" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CA111" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -27776,6 +28112,9 @@
       <c r="BZ112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CA112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -28018,6 +28357,9 @@
       <c r="BZ113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CA113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -28260,6 +28602,9 @@
       <c r="BZ114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CA114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -28502,6 +28847,9 @@
       <c r="BZ115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CA115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -28744,6 +29092,9 @@
       <c r="BZ116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CA116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -28986,6 +29337,9 @@
       <c r="BZ117" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CA117" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -29228,6 +29582,9 @@
       <c r="BZ118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="CA118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -29470,6 +29827,9 @@
       <c r="BZ119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CA119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -29712,6 +30072,9 @@
       <c r="BZ120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CA120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -29954,6 +30317,9 @@
       <c r="BZ121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CA121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -30196,6 +30562,9 @@
       <c r="BZ122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CA122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -30438,6 +30807,9 @@
       <c r="BZ123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CA123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -30680,6 +31052,9 @@
       <c r="BZ124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CA124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -30922,6 +31297,9 @@
       <c r="BZ125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CA125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -31164,6 +31542,9 @@
       <c r="BZ126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CA126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -31406,6 +31787,9 @@
       <c r="BZ127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CA127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -31648,6 +32032,9 @@
       <c r="BZ128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CA128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -31890,6 +32277,9 @@
       <c r="BZ129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CA129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -32132,6 +32522,9 @@
       <c r="BZ130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CA130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -32374,6 +32767,9 @@
       <c r="BZ131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CA131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -32616,6 +33012,9 @@
       <c r="BZ132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="CA132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -32858,6 +33257,9 @@
       <c r="BZ133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CA133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -33100,6 +33502,9 @@
       <c r="BZ134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="CA134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -33342,6 +33747,9 @@
       <c r="BZ135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CA135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -33584,6 +33992,9 @@
       <c r="BZ136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CA136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -33826,6 +34237,9 @@
       <c r="BZ137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CA137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -34068,6 +34482,9 @@
       <c r="BZ138" s="3" t="n">
         <v>23.29</v>
       </c>
+      <c r="CA138" s="3" t="n">
+        <v>23.29</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -34310,6 +34727,9 @@
       <c r="BZ139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CA139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -34552,6 +34972,9 @@
       <c r="BZ140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CA140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -34794,6 +35217,9 @@
       <c r="BZ141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CA141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -35036,6 +35462,9 @@
       <c r="BZ142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CA142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -35278,6 +35707,9 @@
       <c r="BZ143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CA143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -35520,6 +35952,9 @@
       <c r="BZ144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CA144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -35762,6 +36197,9 @@
       <c r="BZ145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CA145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -36004,6 +36442,9 @@
       <c r="BZ146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CA146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -36246,6 +36687,9 @@
       <c r="BZ147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CA147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -36488,6 +36932,9 @@
       <c r="BZ148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CA148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -36730,6 +37177,9 @@
       <c r="BZ149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CA149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -36972,6 +37422,9 @@
       <c r="BZ150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CA150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -37214,6 +37667,9 @@
       <c r="BZ151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CA151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -37456,6 +37912,9 @@
       <c r="BZ152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CA152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -37698,6 +38157,9 @@
       <c r="BZ153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CA153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -37940,6 +38402,9 @@
       <c r="BZ154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CA154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -38182,6 +38647,9 @@
       <c r="BZ155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CA155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -38424,6 +38892,9 @@
       <c r="BZ156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CA156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -38666,6 +39137,9 @@
       <c r="BZ157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CA157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -38908,6 +39382,9 @@
       <c r="BZ158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CA158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -39150,6 +39627,9 @@
       <c r="BZ159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CA159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -39392,6 +39872,9 @@
       <c r="BZ160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CA160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -39634,6 +40117,9 @@
       <c r="BZ161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CA161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -39876,6 +40362,9 @@
       <c r="BZ162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CA162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -40118,6 +40607,9 @@
       <c r="BZ163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CA163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -40360,6 +40852,9 @@
       <c r="BZ164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CA164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -40503,9 +40998,12 @@
       <c r="BZ165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CA165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BZ165"/>
+  <autoFilter ref="A1:CA165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-14 09:11 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CA$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CB$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CA165"/>
+  <dimension ref="A1:CB165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -522,6 +522,7 @@
     <col width="16" customWidth="1" min="77" max="77"/>
     <col width="16" customWidth="1" min="78" max="78"/>
     <col width="16" customWidth="1" min="79" max="79"/>
+    <col width="16" customWidth="1" min="80" max="80"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -920,6 +921,11 @@
           <t>2026-09-14 01:13</t>
         </is>
       </c>
+      <c r="CB1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-14 04:11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1165,6 +1171,9 @@
       <c r="CA2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CB2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1410,6 +1419,9 @@
       <c r="CA3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CB3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1655,6 +1667,9 @@
       <c r="CA4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CB4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1900,6 +1915,9 @@
       <c r="CA5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CB5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2145,6 +2163,9 @@
       <c r="CA6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CB6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2390,6 +2411,9 @@
       <c r="CA7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CB7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2635,6 +2659,9 @@
       <c r="CA8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="CB8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2880,6 +2907,9 @@
       <c r="CA9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CB9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3125,6 +3155,9 @@
       <c r="CA10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CB10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3370,6 +3403,9 @@
       <c r="CA11" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB11" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3615,6 +3651,9 @@
       <c r="CA12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3860,6 +3899,9 @@
       <c r="CA13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CB13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4105,6 +4147,9 @@
       <c r="CA14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4350,6 +4395,9 @@
       <c r="CA15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="CB15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4595,6 +4643,9 @@
       <c r="CA16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CB16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4840,6 +4891,9 @@
       <c r="CA17" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CB17" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5085,6 +5139,9 @@
       <c r="CA18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CB18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5330,6 +5387,9 @@
       <c r="CA19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="CB19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5575,6 +5635,9 @@
       <c r="CA20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="CB20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -5820,6 +5883,9 @@
       <c r="CA21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="CB21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -6065,6 +6131,9 @@
       <c r="CA22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CB22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -6310,6 +6379,9 @@
       <c r="CA23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CB23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -6555,6 +6627,9 @@
       <c r="CA24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CB24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -6800,6 +6875,9 @@
       <c r="CA25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -7045,6 +7123,9 @@
       <c r="CA26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="CB26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -7290,6 +7371,9 @@
       <c r="CA27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CB27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -7535,6 +7619,9 @@
       <c r="CA28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CB28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -7780,6 +7867,9 @@
       <c r="CA29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CB29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -8025,6 +8115,9 @@
       <c r="CA30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -8270,6 +8363,9 @@
       <c r="CA31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -8515,6 +8611,9 @@
       <c r="CA32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -8760,6 +8859,9 @@
       <c r="CA33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CB33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -9005,6 +9107,9 @@
       <c r="CA34" s="3" t="n">
         <v>21.22</v>
       </c>
+      <c r="CB34" s="3" t="n">
+        <v>21.22</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -9250,6 +9355,9 @@
       <c r="CA35" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CB35" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -9495,6 +9603,9 @@
       <c r="CA36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CB36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -9740,6 +9851,9 @@
       <c r="CA37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CB37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -9985,6 +10099,9 @@
       <c r="CA38" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB38" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -10230,6 +10347,9 @@
       <c r="CA39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CB39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -10475,6 +10595,9 @@
       <c r="CA40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -10720,6 +10843,9 @@
       <c r="CA41" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB41" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -10965,6 +11091,9 @@
       <c r="CA42" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB42" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -11210,6 +11339,9 @@
       <c r="CA43" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CB43" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -11455,6 +11587,9 @@
       <c r="CA44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CB44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -11700,6 +11835,9 @@
       <c r="CA45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="CB45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -11945,6 +12083,9 @@
       <c r="CA46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="CB46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -12190,6 +12331,9 @@
       <c r="CA47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CB47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -12435,6 +12579,9 @@
       <c r="CA48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CB48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -12680,6 +12827,9 @@
       <c r="CA49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CB49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -12925,6 +13075,9 @@
       <c r="CA50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CB50" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -13170,6 +13323,9 @@
       <c r="CA51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CB51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -13415,6 +13571,9 @@
       <c r="CA52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CB52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -13660,6 +13819,9 @@
       <c r="CA53" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CB53" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -13905,6 +14067,9 @@
       <c r="CA54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CB54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -14150,6 +14315,9 @@
       <c r="CA55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="CB55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -14395,6 +14563,9 @@
       <c r="CA56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CB56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -14640,6 +14811,9 @@
       <c r="CA57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -14885,6 +15059,9 @@
       <c r="CA58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CB58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -15130,6 +15307,9 @@
       <c r="CA59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CB59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -15375,6 +15555,9 @@
       <c r="CA60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CB60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -15620,6 +15803,9 @@
       <c r="CA61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CB61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -15865,6 +16051,9 @@
       <c r="CA62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CB62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -16110,6 +16299,9 @@
       <c r="CA63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CB63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -16355,6 +16547,9 @@
       <c r="CA64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CB64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -16600,6 +16795,9 @@
       <c r="CA65" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CB65" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -16845,6 +17043,9 @@
       <c r="CA66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -17090,6 +17291,9 @@
       <c r="CA67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CB67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -17335,6 +17539,9 @@
       <c r="CA68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -17580,6 +17787,9 @@
       <c r="CA69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CB69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -17825,6 +18035,9 @@
       <c r="CA70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CB70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -18070,6 +18283,9 @@
       <c r="CA71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -18315,6 +18531,9 @@
       <c r="CA72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -18560,6 +18779,9 @@
       <c r="CA73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CB73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -18805,6 +19027,9 @@
       <c r="CA74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CB74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -19050,6 +19275,9 @@
       <c r="CA75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -19295,6 +19523,9 @@
       <c r="CA76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -19540,6 +19771,9 @@
       <c r="CA77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -19785,6 +20019,9 @@
       <c r="CA78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CB78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -20030,6 +20267,9 @@
       <c r="CA79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -20275,6 +20515,9 @@
       <c r="CA80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CB80" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -20520,6 +20763,9 @@
       <c r="CA81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -20765,6 +21011,9 @@
       <c r="CA82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -21010,6 +21259,9 @@
       <c r="CA83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -21255,6 +21507,9 @@
       <c r="CA84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CB84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -21500,6 +21755,9 @@
       <c r="CA85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CB85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -21745,6 +22003,9 @@
       <c r="CA86" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CB86" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -21990,6 +22251,9 @@
       <c r="CA87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -22235,6 +22499,9 @@
       <c r="CA88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -22480,6 +22747,9 @@
       <c r="CA89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -22725,6 +22995,9 @@
       <c r="CA90" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CB90" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -22970,6 +23243,9 @@
       <c r="CA91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -23215,6 +23491,9 @@
       <c r="CA92" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CB92" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -23460,6 +23739,9 @@
       <c r="CA93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CB93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -23705,6 +23987,9 @@
       <c r="CA94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CB94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -23950,6 +24235,9 @@
       <c r="CA95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CB95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -24195,6 +24483,9 @@
       <c r="CA96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CB96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -24440,6 +24731,9 @@
       <c r="CA97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CB97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -24685,6 +24979,9 @@
       <c r="CA98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="CB98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -24930,6 +25227,9 @@
       <c r="CA99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CB99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -25175,6 +25475,9 @@
       <c r="CA100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CB100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -25420,6 +25723,9 @@
       <c r="CA101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CB101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -25665,6 +25971,9 @@
       <c r="CA102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CB102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -25910,6 +26219,9 @@
       <c r="CA103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CB103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -26155,6 +26467,9 @@
       <c r="CA104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CB104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -26400,6 +26715,9 @@
       <c r="CA105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CB105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -26645,6 +26963,9 @@
       <c r="CA106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CB106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -26890,6 +27211,9 @@
       <c r="CA107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CB107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -27135,6 +27459,9 @@
       <c r="CA108" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CB108" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -27380,6 +27707,9 @@
       <c r="CA109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CB109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -27625,6 +27955,9 @@
       <c r="CA110" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CB110" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -27870,6 +28203,9 @@
       <c r="CA111" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CB111" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -28115,6 +28451,9 @@
       <c r="CA112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CB112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -28360,6 +28699,9 @@
       <c r="CA113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CB113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -28605,6 +28947,9 @@
       <c r="CA114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CB114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -28850,6 +29195,9 @@
       <c r="CA115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CB115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -29095,6 +29443,9 @@
       <c r="CA116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CB116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -29340,6 +29691,9 @@
       <c r="CA117" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CB117" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -29585,6 +29939,9 @@
       <c r="CA118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="CB118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -29830,6 +30187,9 @@
       <c r="CA119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CB119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -30075,6 +30435,9 @@
       <c r="CA120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CB120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -30320,6 +30683,9 @@
       <c r="CA121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CB121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -30565,6 +30931,9 @@
       <c r="CA122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CB122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -30810,6 +31179,9 @@
       <c r="CA123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CB123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -31055,6 +31427,9 @@
       <c r="CA124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CB124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -31300,6 +31675,9 @@
       <c r="CA125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CB125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -31545,6 +31923,9 @@
       <c r="CA126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CB126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -31790,6 +32171,9 @@
       <c r="CA127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CB127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -32035,6 +32419,9 @@
       <c r="CA128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CB128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -32280,6 +32667,9 @@
       <c r="CA129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CB129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -32525,6 +32915,9 @@
       <c r="CA130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CB130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -32770,6 +33163,9 @@
       <c r="CA131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CB131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -33015,6 +33411,9 @@
       <c r="CA132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="CB132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -33260,6 +33659,9 @@
       <c r="CA133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CB133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -33505,6 +33907,9 @@
       <c r="CA134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="CB134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -33750,6 +34155,9 @@
       <c r="CA135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CB135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -33995,6 +34403,9 @@
       <c r="CA136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CB136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -34240,6 +34651,9 @@
       <c r="CA137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CB137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -34485,6 +34899,9 @@
       <c r="CA138" s="3" t="n">
         <v>23.29</v>
       </c>
+      <c r="CB138" s="3" t="n">
+        <v>23.29</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -34730,6 +35147,9 @@
       <c r="CA139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CB139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -34975,6 +35395,9 @@
       <c r="CA140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CB140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -35220,6 +35643,9 @@
       <c r="CA141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CB141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -35465,6 +35891,9 @@
       <c r="CA142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CB142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -35710,6 +36139,9 @@
       <c r="CA143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CB143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -35955,6 +36387,9 @@
       <c r="CA144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CB144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -36200,6 +36635,9 @@
       <c r="CA145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CB145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -36445,6 +36883,9 @@
       <c r="CA146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CB146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -36690,6 +37131,9 @@
       <c r="CA147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CB147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -36935,6 +37379,9 @@
       <c r="CA148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CB148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -37180,6 +37627,9 @@
       <c r="CA149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CB149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -37425,6 +37875,9 @@
       <c r="CA150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CB150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -37670,6 +38123,9 @@
       <c r="CA151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CB151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -37915,6 +38371,9 @@
       <c r="CA152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CB152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -38160,6 +38619,9 @@
       <c r="CA153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CB153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -38405,6 +38867,9 @@
       <c r="CA154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CB154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -38650,6 +39115,9 @@
       <c r="CA155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CB155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -38895,6 +39363,9 @@
       <c r="CA156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CB156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -39140,6 +39611,9 @@
       <c r="CA157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CB157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -39385,6 +39859,9 @@
       <c r="CA158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CB158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -39630,6 +40107,9 @@
       <c r="CA159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CB159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -39875,6 +40355,9 @@
       <c r="CA160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CB160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -40120,6 +40603,9 @@
       <c r="CA161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CB161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -40365,6 +40851,9 @@
       <c r="CA162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CB162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -40610,6 +41099,9 @@
       <c r="CA163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CB163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -40855,6 +41347,9 @@
       <c r="CA164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CB164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -41001,9 +41496,12 @@
       <c r="CA165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CB165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CA165"/>
+  <autoFilter ref="A1:CB165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-14 12:12 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CB$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CC$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CB165"/>
+  <dimension ref="A1:CC165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -523,6 +523,7 @@
     <col width="16" customWidth="1" min="78" max="78"/>
     <col width="16" customWidth="1" min="79" max="79"/>
     <col width="16" customWidth="1" min="80" max="80"/>
+    <col width="16" customWidth="1" min="81" max="81"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -926,6 +927,11 @@
           <t>2026-09-14 04:11</t>
         </is>
       </c>
+      <c r="CC1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1174,6 +1180,9 @@
       <c r="CB2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CC2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1422,6 +1431,9 @@
       <c r="CB3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CC3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1670,6 +1682,9 @@
       <c r="CB4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CC4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1918,6 +1933,9 @@
       <c r="CB5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CC5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2166,6 +2184,9 @@
       <c r="CB6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CC6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2414,6 +2435,9 @@
       <c r="CB7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CC7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2662,6 +2686,9 @@
       <c r="CB8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="CC8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2910,6 +2937,9 @@
       <c r="CB9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CC9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3158,6 +3188,9 @@
       <c r="CB10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CC10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3406,6 +3439,9 @@
       <c r="CB11" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC11" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3654,6 +3690,9 @@
       <c r="CB12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3902,6 +3941,9 @@
       <c r="CB13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CC13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4150,6 +4192,9 @@
       <c r="CB14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4398,6 +4443,9 @@
       <c r="CB15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="CC15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4646,6 +4694,9 @@
       <c r="CB16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CC16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4894,6 +4945,9 @@
       <c r="CB17" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CC17" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5142,6 +5196,9 @@
       <c r="CB18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CC18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5390,6 +5447,9 @@
       <c r="CB19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="CC19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5638,6 +5698,9 @@
       <c r="CB20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="CC20" s="3" t="n">
+        <v>20.65</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -5886,6 +5949,9 @@
       <c r="CB21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="CC21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -6134,6 +6200,9 @@
       <c r="CB22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CC22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -6382,6 +6451,9 @@
       <c r="CB23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CC23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -6630,6 +6702,9 @@
       <c r="CB24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CC24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -6878,6 +6953,9 @@
       <c r="CB25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -7126,6 +7204,9 @@
       <c r="CB26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="CC26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -7374,6 +7455,9 @@
       <c r="CB27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CC27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -7622,6 +7706,9 @@
       <c r="CB28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CC28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -7870,6 +7957,9 @@
       <c r="CB29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CC29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -8118,6 +8208,9 @@
       <c r="CB30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -8366,6 +8459,9 @@
       <c r="CB31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -8614,6 +8710,9 @@
       <c r="CB32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -8862,6 +8961,9 @@
       <c r="CB33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CC33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -9110,6 +9212,9 @@
       <c r="CB34" s="3" t="n">
         <v>21.22</v>
       </c>
+      <c r="CC34" s="3" t="n">
+        <v>21.22</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -9358,6 +9463,9 @@
       <c r="CB35" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CC35" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -9606,6 +9714,9 @@
       <c r="CB36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CC36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -9854,6 +9965,9 @@
       <c r="CB37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CC37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -10102,6 +10216,9 @@
       <c r="CB38" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC38" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -10350,6 +10467,9 @@
       <c r="CB39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CC39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -10598,6 +10718,9 @@
       <c r="CB40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -10846,6 +10969,9 @@
       <c r="CB41" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC41" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -11094,6 +11220,9 @@
       <c r="CB42" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC42" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -11342,6 +11471,9 @@
       <c r="CB43" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CC43" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -11590,6 +11722,9 @@
       <c r="CB44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CC44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -11838,6 +11973,9 @@
       <c r="CB45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="CC45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -12086,6 +12224,9 @@
       <c r="CB46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="CC46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -12334,6 +12475,9 @@
       <c r="CB47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CC47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -12582,6 +12726,9 @@
       <c r="CB48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CC48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -12830,6 +12977,9 @@
       <c r="CB49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CC49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -13078,6 +13228,9 @@
       <c r="CB50" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CC50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -13326,6 +13479,9 @@
       <c r="CB51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CC51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -13574,6 +13730,9 @@
       <c r="CB52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CC52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -13822,6 +13981,9 @@
       <c r="CB53" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CC53" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -14070,6 +14232,9 @@
       <c r="CB54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CC54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -14318,6 +14483,9 @@
       <c r="CB55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="CC55" s="3" t="n">
+        <v>21.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -14566,6 +14734,9 @@
       <c r="CB56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CC56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -14814,6 +14985,9 @@
       <c r="CB57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -15062,6 +15236,9 @@
       <c r="CB58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CC58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -15310,6 +15487,9 @@
       <c r="CB59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CC59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -15558,6 +15738,9 @@
       <c r="CB60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CC60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -15806,6 +15989,9 @@
       <c r="CB61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CC61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -16054,6 +16240,9 @@
       <c r="CB62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CC62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -16302,6 +16491,9 @@
       <c r="CB63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CC63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -16550,6 +16742,9 @@
       <c r="CB64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CC64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -16798,6 +16993,9 @@
       <c r="CB65" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CC65" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -17046,6 +17244,9 @@
       <c r="CB66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -17294,6 +17495,9 @@
       <c r="CB67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CC67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -17542,6 +17746,9 @@
       <c r="CB68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -17790,6 +17997,9 @@
       <c r="CB69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CC69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -18038,6 +18248,9 @@
       <c r="CB70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CC70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -18286,6 +18499,9 @@
       <c r="CB71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -18534,6 +18750,9 @@
       <c r="CB72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -18782,6 +19001,9 @@
       <c r="CB73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CC73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -19030,6 +19252,9 @@
       <c r="CB74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CC74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -19278,6 +19503,9 @@
       <c r="CB75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -19526,6 +19754,9 @@
       <c r="CB76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC76" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -19774,6 +20005,9 @@
       <c r="CB77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -20022,6 +20256,9 @@
       <c r="CB78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CC78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -20270,6 +20507,9 @@
       <c r="CB79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -20518,6 +20758,9 @@
       <c r="CB80" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CC80" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -20766,6 +21009,9 @@
       <c r="CB81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -21014,6 +21260,9 @@
       <c r="CB82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -21262,6 +21511,9 @@
       <c r="CB83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -21510,6 +21762,9 @@
       <c r="CB84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CC84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -21758,6 +22013,9 @@
       <c r="CB85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CC85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -22006,6 +22264,9 @@
       <c r="CB86" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CC86" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -22254,6 +22515,9 @@
       <c r="CB87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -22502,6 +22766,9 @@
       <c r="CB88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -22750,6 +23017,9 @@
       <c r="CB89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -22998,6 +23268,9 @@
       <c r="CB90" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CC90" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -23246,6 +23519,9 @@
       <c r="CB91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -23494,6 +23770,9 @@
       <c r="CB92" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CC92" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -23742,6 +24021,9 @@
       <c r="CB93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CC93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -23990,6 +24272,9 @@
       <c r="CB94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CC94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -24238,6 +24523,9 @@
       <c r="CB95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CC95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -24486,6 +24774,9 @@
       <c r="CB96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CC96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -24734,6 +25025,9 @@
       <c r="CB97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CC97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -24982,6 +25276,9 @@
       <c r="CB98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="CC98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -25230,6 +25527,9 @@
       <c r="CB99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CC99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -25478,6 +25778,9 @@
       <c r="CB100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CC100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -25726,6 +26029,9 @@
       <c r="CB101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CC101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -25974,6 +26280,9 @@
       <c r="CB102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CC102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -26222,6 +26531,9 @@
       <c r="CB103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CC103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -26470,6 +26782,9 @@
       <c r="CB104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CC104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -26718,6 +27033,9 @@
       <c r="CB105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CC105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -26966,6 +27284,9 @@
       <c r="CB106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CC106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -27214,6 +27535,9 @@
       <c r="CB107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CC107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -27462,6 +27786,9 @@
       <c r="CB108" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CC108" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -27710,6 +28037,9 @@
       <c r="CB109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CC109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -27958,6 +28288,9 @@
       <c r="CB110" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CC110" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -28206,6 +28539,9 @@
       <c r="CB111" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CC111" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -28454,6 +28790,9 @@
       <c r="CB112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CC112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -28702,6 +29041,9 @@
       <c r="CB113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CC113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -28950,6 +29292,9 @@
       <c r="CB114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CC114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -29198,6 +29543,9 @@
       <c r="CB115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CC115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -29446,6 +29794,9 @@
       <c r="CB116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CC116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -29694,6 +30045,9 @@
       <c r="CB117" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CC117" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -29942,6 +30296,9 @@
       <c r="CB118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="CC118" s="3" t="n">
+        <v>21.75</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -30190,6 +30547,9 @@
       <c r="CB119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CC119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -30438,6 +30798,9 @@
       <c r="CB120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CC120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -30686,6 +31049,9 @@
       <c r="CB121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CC121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -30934,6 +31300,9 @@
       <c r="CB122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CC122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -31182,6 +31551,9 @@
       <c r="CB123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CC123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -31430,6 +31802,9 @@
       <c r="CB124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CC124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -31678,6 +32053,9 @@
       <c r="CB125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CC125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -31926,6 +32304,9 @@
       <c r="CB126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CC126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -32174,6 +32555,9 @@
       <c r="CB127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CC127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -32422,6 +32806,9 @@
       <c r="CB128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CC128" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -32670,6 +33057,9 @@
       <c r="CB129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CC129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -32918,6 +33308,9 @@
       <c r="CB130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CC130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -33166,6 +33559,9 @@
       <c r="CB131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CC131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -33414,6 +33810,9 @@
       <c r="CB132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="CC132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -33662,6 +34061,9 @@
       <c r="CB133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CC133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -33910,6 +34312,9 @@
       <c r="CB134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="CC134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -34158,6 +34563,9 @@
       <c r="CB135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CC135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -34406,6 +34814,9 @@
       <c r="CB136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CC136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -34654,6 +35065,9 @@
       <c r="CB137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CC137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -34902,6 +35316,9 @@
       <c r="CB138" s="3" t="n">
         <v>23.29</v>
       </c>
+      <c r="CC138" s="3" t="n">
+        <v>23.29</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -35150,6 +35567,9 @@
       <c r="CB139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CC139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -35398,6 +35818,9 @@
       <c r="CB140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CC140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -35646,6 +36069,9 @@
       <c r="CB141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CC141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -35894,6 +36320,9 @@
       <c r="CB142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CC142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -36142,6 +36571,9 @@
       <c r="CB143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CC143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -36390,6 +36822,9 @@
       <c r="CB144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CC144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -36638,6 +37073,9 @@
       <c r="CB145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CC145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -36886,6 +37324,9 @@
       <c r="CB146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CC146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -37134,6 +37575,9 @@
       <c r="CB147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CC147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -37382,6 +37826,9 @@
       <c r="CB148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CC148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -37630,6 +38077,9 @@
       <c r="CB149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CC149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -37878,6 +38328,9 @@
       <c r="CB150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CC150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -38126,6 +38579,9 @@
       <c r="CB151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CC151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -38374,6 +38830,9 @@
       <c r="CB152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CC152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -38622,6 +39081,9 @@
       <c r="CB153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CC153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -38870,6 +39332,9 @@
       <c r="CB154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CC154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -39118,6 +39583,9 @@
       <c r="CB155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CC155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -39366,6 +39834,9 @@
       <c r="CB156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CC156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -39614,6 +40085,9 @@
       <c r="CB157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CC157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -39862,6 +40336,9 @@
       <c r="CB158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CC158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -40110,6 +40587,9 @@
       <c r="CB159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CC159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -40358,6 +40838,9 @@
       <c r="CB160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CC160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -40606,6 +41089,9 @@
       <c r="CB161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CC161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -40854,6 +41340,9 @@
       <c r="CB162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CC162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -41102,6 +41591,9 @@
       <c r="CB163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CC163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -41350,6 +41842,9 @@
       <c r="CB164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CC164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -41499,9 +41994,12 @@
       <c r="CB165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CC165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CB165"/>
+  <autoFilter ref="A1:CC165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-14 15:11 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CC$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CD$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CC165"/>
+  <dimension ref="A1:CD165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -524,6 +524,7 @@
     <col width="16" customWidth="1" min="79" max="79"/>
     <col width="16" customWidth="1" min="80" max="80"/>
     <col width="16" customWidth="1" min="81" max="81"/>
+    <col width="16" customWidth="1" min="82" max="82"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -932,6 +933,11 @@
           <t>2026-09-14 07:12</t>
         </is>
       </c>
+      <c r="CD1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-14 10:11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1183,6 +1189,9 @@
       <c r="CC2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CD2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1434,6 +1443,9 @@
       <c r="CC3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CD3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1685,6 +1697,9 @@
       <c r="CC4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CD4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1936,6 +1951,9 @@
       <c r="CC5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CD5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2187,6 +2205,9 @@
       <c r="CC6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CD6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2438,6 +2459,9 @@
       <c r="CC7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CD7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2689,6 +2713,9 @@
       <c r="CC8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="CD8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2940,6 +2967,9 @@
       <c r="CC9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CD9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3191,6 +3221,9 @@
       <c r="CC10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CD10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3442,6 +3475,9 @@
       <c r="CC11" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD11" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3693,6 +3729,9 @@
       <c r="CC12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3944,6 +3983,9 @@
       <c r="CC13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CD13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4195,6 +4237,9 @@
       <c r="CC14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4446,6 +4491,9 @@
       <c r="CC15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="CD15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4697,6 +4745,9 @@
       <c r="CC16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CD16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4948,6 +4999,9 @@
       <c r="CC17" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CD17" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5199,6 +5253,9 @@
       <c r="CC18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CD18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5450,6 +5507,9 @@
       <c r="CC19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="CD19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5701,6 +5761,9 @@
       <c r="CC20" s="3" t="n">
         <v>20.65</v>
       </c>
+      <c r="CD20" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -5952,6 +6015,9 @@
       <c r="CC21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="CD21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -6203,6 +6269,9 @@
       <c r="CC22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CD22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -6454,6 +6523,9 @@
       <c r="CC23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CD23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -6705,6 +6777,9 @@
       <c r="CC24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CD24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -6956,6 +7031,9 @@
       <c r="CC25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -7207,6 +7285,9 @@
       <c r="CC26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="CD26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -7458,6 +7539,9 @@
       <c r="CC27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CD27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -7709,6 +7793,9 @@
       <c r="CC28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CD28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -7960,6 +8047,9 @@
       <c r="CC29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CD29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -8211,6 +8301,9 @@
       <c r="CC30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -8462,6 +8555,9 @@
       <c r="CC31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -8713,6 +8809,9 @@
       <c r="CC32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -8964,6 +9063,9 @@
       <c r="CC33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CD33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -9215,6 +9317,9 @@
       <c r="CC34" s="3" t="n">
         <v>21.22</v>
       </c>
+      <c r="CD34" s="3" t="n">
+        <v>21.22</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -9466,6 +9571,9 @@
       <c r="CC35" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CD35" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -9717,6 +9825,9 @@
       <c r="CC36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CD36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -9968,6 +10079,9 @@
       <c r="CC37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CD37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -10219,6 +10333,9 @@
       <c r="CC38" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD38" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -10470,6 +10587,9 @@
       <c r="CC39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CD39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -10721,6 +10841,9 @@
       <c r="CC40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -10972,6 +11095,9 @@
       <c r="CC41" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD41" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -11223,6 +11349,9 @@
       <c r="CC42" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD42" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -11474,6 +11603,9 @@
       <c r="CC43" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CD43" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -11725,6 +11857,9 @@
       <c r="CC44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CD44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -11976,6 +12111,9 @@
       <c r="CC45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="CD45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -12227,6 +12365,9 @@
       <c r="CC46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="CD46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -12478,6 +12619,9 @@
       <c r="CC47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CD47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -12729,6 +12873,9 @@
       <c r="CC48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CD48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -12980,6 +13127,9 @@
       <c r="CC49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CD49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -13231,6 +13381,9 @@
       <c r="CC50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CD50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -13482,6 +13635,9 @@
       <c r="CC51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CD51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -13733,6 +13889,9 @@
       <c r="CC52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CD52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -13984,6 +14143,9 @@
       <c r="CC53" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CD53" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -14235,6 +14397,9 @@
       <c r="CC54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CD54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -14486,6 +14651,9 @@
       <c r="CC55" s="3" t="n">
         <v>21.3</v>
       </c>
+      <c r="CD55" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -14737,6 +14905,9 @@
       <c r="CC56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CD56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -14988,6 +15159,9 @@
       <c r="CC57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -15239,6 +15413,9 @@
       <c r="CC58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CD58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -15490,6 +15667,9 @@
       <c r="CC59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CD59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -15741,6 +15921,9 @@
       <c r="CC60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CD60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -15992,6 +16175,9 @@
       <c r="CC61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CD61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -16243,6 +16429,9 @@
       <c r="CC62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CD62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -16494,6 +16683,9 @@
       <c r="CC63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CD63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -16745,6 +16937,9 @@
       <c r="CC64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CD64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -16996,6 +17191,9 @@
       <c r="CC65" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CD65" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -17247,6 +17445,9 @@
       <c r="CC66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -17498,6 +17699,9 @@
       <c r="CC67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CD67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -17749,6 +17953,9 @@
       <c r="CC68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -18000,6 +18207,9 @@
       <c r="CC69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CD69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -18251,6 +18461,9 @@
       <c r="CC70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CD70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -18502,6 +18715,9 @@
       <c r="CC71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -18753,6 +18969,9 @@
       <c r="CC72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -19004,6 +19223,9 @@
       <c r="CC73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CD73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -19255,6 +19477,9 @@
       <c r="CC74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CD74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -19506,6 +19731,9 @@
       <c r="CC75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -19757,6 +19985,9 @@
       <c r="CC76" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD76" s="3" t="n">
+        <v>21.67</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -20008,6 +20239,9 @@
       <c r="CC77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -20259,6 +20493,9 @@
       <c r="CC78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CD78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -20510,6 +20747,9 @@
       <c r="CC79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -20761,6 +21001,9 @@
       <c r="CC80" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CD80" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -21012,6 +21255,9 @@
       <c r="CC81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -21263,6 +21509,9 @@
       <c r="CC82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -21514,6 +21763,9 @@
       <c r="CC83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -21765,6 +22017,9 @@
       <c r="CC84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CD84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -22016,6 +22271,9 @@
       <c r="CC85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CD85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -22267,6 +22525,9 @@
       <c r="CC86" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CD86" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -22518,6 +22779,9 @@
       <c r="CC87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -22769,6 +23033,9 @@
       <c r="CC88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -23020,6 +23287,9 @@
       <c r="CC89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -23271,6 +23541,9 @@
       <c r="CC90" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CD90" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -23522,6 +23795,9 @@
       <c r="CC91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -23773,6 +24049,9 @@
       <c r="CC92" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CD92" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -24024,6 +24303,9 @@
       <c r="CC93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CD93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -24275,6 +24557,9 @@
       <c r="CC94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CD94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -24526,6 +24811,9 @@
       <c r="CC95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CD95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -24777,6 +25065,9 @@
       <c r="CC96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CD96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -25028,6 +25319,9 @@
       <c r="CC97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CD97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -25279,6 +25573,9 @@
       <c r="CC98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="CD98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -25530,6 +25827,9 @@
       <c r="CC99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CD99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -25781,6 +26081,9 @@
       <c r="CC100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CD100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -26032,6 +26335,9 @@
       <c r="CC101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CD101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -26283,6 +26589,9 @@
       <c r="CC102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CD102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -26534,6 +26843,9 @@
       <c r="CC103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CD103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -26785,6 +27097,9 @@
       <c r="CC104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CD104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -27036,6 +27351,9 @@
       <c r="CC105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CD105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -27287,6 +27605,9 @@
       <c r="CC106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CD106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -27538,6 +27859,9 @@
       <c r="CC107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CD107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -27789,6 +28113,9 @@
       <c r="CC108" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CD108" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -28040,6 +28367,9 @@
       <c r="CC109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CD109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -28291,6 +28621,9 @@
       <c r="CC110" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CD110" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -28542,6 +28875,9 @@
       <c r="CC111" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CD111" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -28793,6 +29129,9 @@
       <c r="CC112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CD112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -29044,6 +29383,9 @@
       <c r="CC113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CD113" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -29295,6 +29637,9 @@
       <c r="CC114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CD114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -29546,6 +29891,9 @@
       <c r="CC115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CD115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -29797,6 +30145,9 @@
       <c r="CC116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CD116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -30048,6 +30399,9 @@
       <c r="CC117" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CD117" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -30299,6 +30653,9 @@
       <c r="CC118" s="3" t="n">
         <v>21.75</v>
       </c>
+      <c r="CD118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -30550,6 +30907,9 @@
       <c r="CC119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CD119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -30801,6 +31161,9 @@
       <c r="CC120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CD120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -31052,6 +31415,9 @@
       <c r="CC121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CD121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -31303,6 +31669,9 @@
       <c r="CC122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CD122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -31554,6 +31923,9 @@
       <c r="CC123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CD123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -31805,6 +32177,9 @@
       <c r="CC124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CD124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -32056,6 +32431,9 @@
       <c r="CC125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CD125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -32307,6 +32685,9 @@
       <c r="CC126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CD126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -32558,6 +32939,9 @@
       <c r="CC127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CD127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -32809,6 +33193,9 @@
       <c r="CC128" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CD128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -33060,6 +33447,9 @@
       <c r="CC129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CD129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -33311,6 +33701,9 @@
       <c r="CC130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CD130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -33562,6 +33955,9 @@
       <c r="CC131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CD131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -33813,6 +34209,9 @@
       <c r="CC132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="CD132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -34064,6 +34463,9 @@
       <c r="CC133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CD133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -34315,6 +34717,9 @@
       <c r="CC134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="CD134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -34566,6 +34971,9 @@
       <c r="CC135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CD135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -34817,6 +35225,9 @@
       <c r="CC136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CD136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -35068,6 +35479,9 @@
       <c r="CC137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CD137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -35319,6 +35733,9 @@
       <c r="CC138" s="3" t="n">
         <v>23.29</v>
       </c>
+      <c r="CD138" s="3" t="n">
+        <v>23.29</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -35570,6 +35987,9 @@
       <c r="CC139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CD139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -35821,6 +36241,9 @@
       <c r="CC140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CD140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -36072,6 +36495,9 @@
       <c r="CC141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CD141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -36323,6 +36749,9 @@
       <c r="CC142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CD142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -36574,6 +37003,9 @@
       <c r="CC143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CD143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -36825,6 +37257,9 @@
       <c r="CC144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CD144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -37076,6 +37511,9 @@
       <c r="CC145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CD145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -37327,6 +37765,9 @@
       <c r="CC146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CD146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -37578,6 +38019,9 @@
       <c r="CC147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CD147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -37829,6 +38273,9 @@
       <c r="CC148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CD148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -38080,6 +38527,9 @@
       <c r="CC149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CD149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -38331,6 +38781,9 @@
       <c r="CC150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CD150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -38582,6 +39035,9 @@
       <c r="CC151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CD151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -38833,6 +39289,9 @@
       <c r="CC152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CD152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -39084,6 +39543,9 @@
       <c r="CC153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CD153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -39335,6 +39797,9 @@
       <c r="CC154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CD154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -39586,6 +40051,9 @@
       <c r="CC155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CD155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -39837,6 +40305,9 @@
       <c r="CC156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CD156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -40088,6 +40559,9 @@
       <c r="CC157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CD157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -40339,6 +40813,9 @@
       <c r="CC158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CD158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -40590,6 +41067,9 @@
       <c r="CC159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CD159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -40841,6 +41321,9 @@
       <c r="CC160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CD160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -41092,6 +41575,9 @@
       <c r="CC161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CD161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -41343,6 +41829,9 @@
       <c r="CC162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CD162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -41594,6 +42083,9 @@
       <c r="CC163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CD163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -41845,6 +42337,9 @@
       <c r="CC164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CD164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -41997,9 +42492,12 @@
       <c r="CC165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CD165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CC165"/>
+  <autoFilter ref="A1:CD165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-14 18:11 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CD$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CE$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CD165"/>
+  <dimension ref="A1:CE165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -525,6 +525,7 @@
     <col width="16" customWidth="1" min="80" max="80"/>
     <col width="16" customWidth="1" min="81" max="81"/>
     <col width="16" customWidth="1" min="82" max="82"/>
+    <col width="16" customWidth="1" min="83" max="83"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -938,6 +939,11 @@
           <t>2026-09-14 10:11</t>
         </is>
       </c>
+      <c r="CE1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-14 13:11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1192,6 +1198,9 @@
       <c r="CD2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CE2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1446,6 +1455,9 @@
       <c r="CD3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CE3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1700,6 +1712,9 @@
       <c r="CD4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CE4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1954,6 +1969,9 @@
       <c r="CD5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CE5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2208,6 +2226,9 @@
       <c r="CD6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CE6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2462,6 +2483,9 @@
       <c r="CD7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CE7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2716,6 +2740,9 @@
       <c r="CD8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="CE8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2970,6 +2997,9 @@
       <c r="CD9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CE9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3224,6 +3254,9 @@
       <c r="CD10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CE10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3478,6 +3511,9 @@
       <c r="CD11" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE11" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3732,6 +3768,9 @@
       <c r="CD12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3986,6 +4025,9 @@
       <c r="CD13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CE13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4240,6 +4282,9 @@
       <c r="CD14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4494,6 +4539,9 @@
       <c r="CD15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="CE15" s="3" t="n">
+        <v>20.34</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4748,6 +4796,9 @@
       <c r="CD16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CE16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5002,6 +5053,9 @@
       <c r="CD17" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CE17" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5256,6 +5310,9 @@
       <c r="CD18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CE18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5510,6 +5567,9 @@
       <c r="CD19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="CE19" s="3" t="n">
+        <v>20.77</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5764,6 +5824,9 @@
       <c r="CD20" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE20" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -6018,6 +6081,9 @@
       <c r="CD21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="CE21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -6272,6 +6338,9 @@
       <c r="CD22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CE22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -6526,6 +6595,9 @@
       <c r="CD23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CE23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -6780,6 +6852,9 @@
       <c r="CD24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CE24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -7034,6 +7109,9 @@
       <c r="CD25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -7288,6 +7366,9 @@
       <c r="CD26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="CE26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -7542,6 +7623,9 @@
       <c r="CD27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CE27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -7796,6 +7880,9 @@
       <c r="CD28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CE28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -8050,6 +8137,9 @@
       <c r="CD29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CE29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -8304,6 +8394,9 @@
       <c r="CD30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -8558,6 +8651,9 @@
       <c r="CD31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -8812,6 +8908,9 @@
       <c r="CD32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -9066,6 +9165,9 @@
       <c r="CD33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CE33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -9320,6 +9422,9 @@
       <c r="CD34" s="3" t="n">
         <v>21.22</v>
       </c>
+      <c r="CE34" s="3" t="n">
+        <v>21.22</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -9574,6 +9679,9 @@
       <c r="CD35" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CE35" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -9828,6 +9936,9 @@
       <c r="CD36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CE36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -10082,6 +10193,9 @@
       <c r="CD37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CE37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -10336,6 +10450,9 @@
       <c r="CD38" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE38" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -10590,6 +10707,9 @@
       <c r="CD39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CE39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -10844,6 +10964,9 @@
       <c r="CD40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -11098,6 +11221,9 @@
       <c r="CD41" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE41" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -11352,6 +11478,9 @@
       <c r="CD42" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE42" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -11606,6 +11735,9 @@
       <c r="CD43" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CE43" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -11860,6 +11992,9 @@
       <c r="CD44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CE44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -12114,6 +12249,9 @@
       <c r="CD45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="CE45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -12368,6 +12506,9 @@
       <c r="CD46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="CE46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -12622,6 +12763,9 @@
       <c r="CD47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CE47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -12876,6 +13020,9 @@
       <c r="CD48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CE48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -13130,6 +13277,9 @@
       <c r="CD49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CE49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -13384,6 +13534,9 @@
       <c r="CD50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CE50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -13638,6 +13791,9 @@
       <c r="CD51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CE51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -13892,6 +14048,9 @@
       <c r="CD52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CE52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -14146,6 +14305,9 @@
       <c r="CD53" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CE53" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -14400,6 +14562,9 @@
       <c r="CD54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CE54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -14654,6 +14819,9 @@
       <c r="CD55" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CE55" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -14908,6 +15076,9 @@
       <c r="CD56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CE56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -15162,6 +15333,9 @@
       <c r="CD57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -15416,6 +15590,9 @@
       <c r="CD58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CE58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -15670,6 +15847,9 @@
       <c r="CD59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CE59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -15924,6 +16104,9 @@
       <c r="CD60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CE60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -16178,6 +16361,9 @@
       <c r="CD61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CE61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -16432,6 +16618,9 @@
       <c r="CD62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CE62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -16686,6 +16875,9 @@
       <c r="CD63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CE63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -16940,6 +17132,9 @@
       <c r="CD64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CE64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -17194,6 +17389,9 @@
       <c r="CD65" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CE65" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -17448,6 +17646,9 @@
       <c r="CD66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -17702,6 +17903,9 @@
       <c r="CD67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CE67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -17956,6 +18160,9 @@
       <c r="CD68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -18210,6 +18417,9 @@
       <c r="CD69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CE69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -18464,6 +18674,9 @@
       <c r="CD70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CE70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -18718,6 +18931,9 @@
       <c r="CD71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -18972,6 +19188,9 @@
       <c r="CD72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -19226,6 +19445,9 @@
       <c r="CD73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CE73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -19480,6 +19702,9 @@
       <c r="CD74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CE74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -19734,6 +19959,9 @@
       <c r="CD75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -19988,6 +20216,9 @@
       <c r="CD76" s="3" t="n">
         <v>21.67</v>
       </c>
+      <c r="CE76" s="3" t="n">
+        <v>21.67</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -20242,6 +20473,9 @@
       <c r="CD77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -20496,6 +20730,9 @@
       <c r="CD78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CE78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -20750,6 +20987,9 @@
       <c r="CD79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -21004,6 +21244,9 @@
       <c r="CD80" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CE80" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -21258,6 +21501,9 @@
       <c r="CD81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -21512,6 +21758,9 @@
       <c r="CD82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -21766,6 +22015,9 @@
       <c r="CD83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -22020,6 +22272,9 @@
       <c r="CD84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CE84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -22274,6 +22529,9 @@
       <c r="CD85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CE85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -22528,6 +22786,9 @@
       <c r="CD86" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CE86" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -22782,6 +23043,9 @@
       <c r="CD87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -23036,6 +23300,9 @@
       <c r="CD88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -23290,6 +23557,9 @@
       <c r="CD89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -23544,6 +23814,9 @@
       <c r="CD90" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CE90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -23798,6 +24071,9 @@
       <c r="CD91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -24052,6 +24328,9 @@
       <c r="CD92" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CE92" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -24306,6 +24585,9 @@
       <c r="CD93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CE93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -24560,6 +24842,9 @@
       <c r="CD94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CE94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -24814,6 +25099,9 @@
       <c r="CD95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CE95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -25068,6 +25356,9 @@
       <c r="CD96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CE96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -25322,6 +25613,9 @@
       <c r="CD97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CE97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -25576,6 +25870,9 @@
       <c r="CD98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="CE98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -25830,6 +26127,9 @@
       <c r="CD99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CE99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -26084,6 +26384,9 @@
       <c r="CD100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CE100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -26338,6 +26641,9 @@
       <c r="CD101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CE101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -26592,6 +26898,9 @@
       <c r="CD102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CE102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -26846,6 +27155,9 @@
       <c r="CD103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CE103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -27100,6 +27412,9 @@
       <c r="CD104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CE104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -27354,6 +27669,9 @@
       <c r="CD105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CE105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -27608,6 +27926,9 @@
       <c r="CD106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CE106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -27862,6 +28183,9 @@
       <c r="CD107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CE107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -28116,6 +28440,9 @@
       <c r="CD108" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CE108" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -28370,6 +28697,9 @@
       <c r="CD109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CE109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -28624,6 +28954,9 @@
       <c r="CD110" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CE110" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -28878,6 +29211,9 @@
       <c r="CD111" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CE111" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -29132,6 +29468,9 @@
       <c r="CD112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CE112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -29386,6 +29725,9 @@
       <c r="CD113" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CE113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -29640,6 +29982,9 @@
       <c r="CD114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CE114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -29894,6 +30239,9 @@
       <c r="CD115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CE115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -30148,6 +30496,9 @@
       <c r="CD116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CE116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -30402,6 +30753,9 @@
       <c r="CD117" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CE117" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -30656,6 +31010,9 @@
       <c r="CD118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CE118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -30910,6 +31267,9 @@
       <c r="CD119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CE119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -31164,6 +31524,9 @@
       <c r="CD120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CE120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -31418,6 +31781,9 @@
       <c r="CD121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CE121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -31672,6 +32038,9 @@
       <c r="CD122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CE122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -31926,6 +32295,9 @@
       <c r="CD123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CE123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -32180,6 +32552,9 @@
       <c r="CD124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CE124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -32434,6 +32809,9 @@
       <c r="CD125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CE125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -32688,6 +33066,9 @@
       <c r="CD126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CE126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -32942,6 +33323,9 @@
       <c r="CD127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CE127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -33196,6 +33580,9 @@
       <c r="CD128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CE128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -33450,6 +33837,9 @@
       <c r="CD129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CE129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -33704,6 +34094,9 @@
       <c r="CD130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CE130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -33958,6 +34351,9 @@
       <c r="CD131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CE131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -34212,6 +34608,9 @@
       <c r="CD132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="CE132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -34466,6 +34865,9 @@
       <c r="CD133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CE133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -34720,6 +35122,9 @@
       <c r="CD134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="CE134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -34974,6 +35379,9 @@
       <c r="CD135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CE135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -35228,6 +35636,9 @@
       <c r="CD136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CE136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -35482,6 +35893,9 @@
       <c r="CD137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CE137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -35736,6 +36150,9 @@
       <c r="CD138" s="3" t="n">
         <v>23.29</v>
       </c>
+      <c r="CE138" s="3" t="n">
+        <v>23.29</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -35990,6 +36407,9 @@
       <c r="CD139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CE139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -36244,6 +36664,9 @@
       <c r="CD140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CE140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -36498,6 +36921,9 @@
       <c r="CD141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CE141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -36752,6 +37178,9 @@
       <c r="CD142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CE142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -37006,6 +37435,9 @@
       <c r="CD143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CE143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -37260,6 +37692,9 @@
       <c r="CD144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CE144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -37514,6 +37949,9 @@
       <c r="CD145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CE145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -37768,6 +38206,9 @@
       <c r="CD146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CE146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -38022,6 +38463,9 @@
       <c r="CD147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CE147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -38276,6 +38720,9 @@
       <c r="CD148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CE148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -38530,6 +38977,9 @@
       <c r="CD149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CE149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -38784,6 +39234,9 @@
       <c r="CD150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CE150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -39038,6 +39491,9 @@
       <c r="CD151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CE151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -39292,6 +39748,9 @@
       <c r="CD152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CE152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -39546,6 +40005,9 @@
       <c r="CD153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CE153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -39800,6 +40262,9 @@
       <c r="CD154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CE154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -40054,6 +40519,9 @@
       <c r="CD155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CE155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -40308,6 +40776,9 @@
       <c r="CD156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CE156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -40562,6 +41033,9 @@
       <c r="CD157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CE157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -40816,6 +41290,9 @@
       <c r="CD158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CE158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -41070,6 +41547,9 @@
       <c r="CD159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CE159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -41324,6 +41804,9 @@
       <c r="CD160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CE160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -41578,6 +42061,9 @@
       <c r="CD161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CE161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -41832,6 +42318,9 @@
       <c r="CD162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CE162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -42086,6 +42575,9 @@
       <c r="CD163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CE163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -42340,6 +42832,9 @@
       <c r="CD164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CE164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -42495,9 +42990,12 @@
       <c r="CD165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CE165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CD165"/>
+  <autoFilter ref="A1:CE165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-14 21:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CE$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CF$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CE165"/>
+  <dimension ref="A1:CF165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -526,6 +526,7 @@
     <col width="16" customWidth="1" min="81" max="81"/>
     <col width="16" customWidth="1" min="82" max="82"/>
     <col width="16" customWidth="1" min="83" max="83"/>
+    <col width="16" customWidth="1" min="84" max="84"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -944,6 +945,11 @@
           <t>2026-09-14 13:11</t>
         </is>
       </c>
+      <c r="CF1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-14 16:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1201,6 +1207,9 @@
       <c r="CE2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CF2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1458,6 +1467,9 @@
       <c r="CE3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CF3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1715,6 +1727,9 @@
       <c r="CE4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CF4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1972,6 +1987,9 @@
       <c r="CE5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CF5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2229,6 +2247,9 @@
       <c r="CE6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CF6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2486,6 +2507,9 @@
       <c r="CE7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CF7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2743,6 +2767,9 @@
       <c r="CE8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="CF8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3000,6 +3027,9 @@
       <c r="CE9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CF9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3257,6 +3287,9 @@
       <c r="CE10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CF10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3514,6 +3547,9 @@
       <c r="CE11" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF11" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3771,6 +3807,9 @@
       <c r="CE12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4028,6 +4067,9 @@
       <c r="CE13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CF13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4285,6 +4327,9 @@
       <c r="CE14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4542,6 +4587,9 @@
       <c r="CE15" s="3" t="n">
         <v>20.34</v>
       </c>
+      <c r="CF15" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4799,6 +4847,9 @@
       <c r="CE16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CF16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5056,6 +5107,9 @@
       <c r="CE17" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CF17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5313,6 +5367,9 @@
       <c r="CE18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CF18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5570,6 +5627,9 @@
       <c r="CE19" s="3" t="n">
         <v>20.77</v>
       </c>
+      <c r="CF19" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5827,6 +5887,9 @@
       <c r="CE20" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF20" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -6084,6 +6147,9 @@
       <c r="CE21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="CF21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -6341,6 +6407,9 @@
       <c r="CE22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CF22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -6598,6 +6667,9 @@
       <c r="CE23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CF23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -6855,6 +6927,9 @@
       <c r="CE24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CF24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -7112,6 +7187,9 @@
       <c r="CE25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -7369,6 +7447,9 @@
       <c r="CE26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="CF26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -7626,6 +7707,9 @@
       <c r="CE27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CF27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -7883,6 +7967,9 @@
       <c r="CE28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CF28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -8140,6 +8227,9 @@
       <c r="CE29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CF29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -8397,6 +8487,9 @@
       <c r="CE30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -8654,6 +8747,9 @@
       <c r="CE31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -8911,6 +9007,9 @@
       <c r="CE32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -9168,6 +9267,9 @@
       <c r="CE33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CF33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -9425,6 +9527,9 @@
       <c r="CE34" s="3" t="n">
         <v>21.22</v>
       </c>
+      <c r="CF34" s="3" t="n">
+        <v>21.22</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -9682,6 +9787,9 @@
       <c r="CE35" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CF35" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -9939,6 +10047,9 @@
       <c r="CE36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CF36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -10196,6 +10307,9 @@
       <c r="CE37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CF37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -10453,6 +10567,9 @@
       <c r="CE38" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF38" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -10710,6 +10827,9 @@
       <c r="CE39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CF39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -10967,6 +11087,9 @@
       <c r="CE40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -11224,6 +11347,9 @@
       <c r="CE41" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF41" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -11481,6 +11607,9 @@
       <c r="CE42" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF42" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -11738,6 +11867,9 @@
       <c r="CE43" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CF43" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -11995,6 +12127,9 @@
       <c r="CE44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CF44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -12252,6 +12387,9 @@
       <c r="CE45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="CF45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -12509,6 +12647,9 @@
       <c r="CE46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="CF46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -12766,6 +12907,9 @@
       <c r="CE47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CF47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -13023,6 +13167,9 @@
       <c r="CE48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CF48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -13280,6 +13427,9 @@
       <c r="CE49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CF49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -13537,6 +13687,9 @@
       <c r="CE50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CF50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -13794,6 +13947,9 @@
       <c r="CE51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CF51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -14051,6 +14207,9 @@
       <c r="CE52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CF52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -14308,6 +14467,9 @@
       <c r="CE53" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CF53" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -14565,6 +14727,9 @@
       <c r="CE54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CF54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -14822,6 +14987,9 @@
       <c r="CE55" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CF55" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -15079,6 +15247,9 @@
       <c r="CE56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CF56" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -15336,6 +15507,9 @@
       <c r="CE57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -15593,6 +15767,9 @@
       <c r="CE58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CF58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -15850,6 +16027,9 @@
       <c r="CE59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CF59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -16107,6 +16287,9 @@
       <c r="CE60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CF60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -16364,6 +16547,9 @@
       <c r="CE61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CF61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -16621,6 +16807,9 @@
       <c r="CE62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CF62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -16878,6 +17067,9 @@
       <c r="CE63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CF63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -17135,6 +17327,9 @@
       <c r="CE64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CF64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -17392,6 +17587,9 @@
       <c r="CE65" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CF65" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -17649,6 +17847,9 @@
       <c r="CE66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -17906,6 +18107,9 @@
       <c r="CE67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CF67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -18163,6 +18367,9 @@
       <c r="CE68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -18420,6 +18627,9 @@
       <c r="CE69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CF69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -18677,6 +18887,9 @@
       <c r="CE70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CF70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -18934,6 +19147,9 @@
       <c r="CE71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -19191,6 +19407,9 @@
       <c r="CE72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -19448,6 +19667,9 @@
       <c r="CE73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CF73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -19705,6 +19927,9 @@
       <c r="CE74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CF74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -19962,6 +20187,9 @@
       <c r="CE75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -20219,6 +20447,9 @@
       <c r="CE76" s="3" t="n">
         <v>21.67</v>
       </c>
+      <c r="CF76" s="3" t="n">
+        <v>21.67</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -20476,6 +20707,9 @@
       <c r="CE77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -20733,6 +20967,9 @@
       <c r="CE78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CF78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -20990,6 +21227,9 @@
       <c r="CE79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -21247,6 +21487,9 @@
       <c r="CE80" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CF80" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -21504,6 +21747,9 @@
       <c r="CE81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -21761,6 +22007,9 @@
       <c r="CE82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -22018,6 +22267,9 @@
       <c r="CE83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -22275,6 +22527,9 @@
       <c r="CE84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CF84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -22532,6 +22787,9 @@
       <c r="CE85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CF85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -22789,6 +23047,9 @@
       <c r="CE86" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CF86" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -23046,6 +23307,9 @@
       <c r="CE87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -23303,6 +23567,9 @@
       <c r="CE88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -23560,6 +23827,9 @@
       <c r="CE89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -23817,6 +24087,9 @@
       <c r="CE90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CF90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -24074,6 +24347,9 @@
       <c r="CE91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -24331,6 +24607,9 @@
       <c r="CE92" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CF92" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -24588,6 +24867,9 @@
       <c r="CE93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CF93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -24845,6 +25127,9 @@
       <c r="CE94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CF94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -25102,6 +25387,9 @@
       <c r="CE95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CF95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -25359,6 +25647,9 @@
       <c r="CE96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CF96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -25616,6 +25907,9 @@
       <c r="CE97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CF97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -25873,6 +26167,9 @@
       <c r="CE98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="CF98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -26130,6 +26427,9 @@
       <c r="CE99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CF99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -26387,6 +26687,9 @@
       <c r="CE100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CF100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -26644,6 +26947,9 @@
       <c r="CE101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CF101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -26901,6 +27207,9 @@
       <c r="CE102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CF102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -27158,6 +27467,9 @@
       <c r="CE103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CF103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -27415,6 +27727,9 @@
       <c r="CE104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CF104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -27672,6 +27987,9 @@
       <c r="CE105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CF105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -27929,6 +28247,9 @@
       <c r="CE106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CF106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -28186,6 +28507,9 @@
       <c r="CE107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CF107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -28443,6 +28767,9 @@
       <c r="CE108" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CF108" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -28700,6 +29027,9 @@
       <c r="CE109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CF109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -28957,6 +29287,9 @@
       <c r="CE110" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CF110" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -29214,6 +29547,9 @@
       <c r="CE111" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CF111" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -29471,6 +29807,9 @@
       <c r="CE112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CF112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -29728,6 +30067,9 @@
       <c r="CE113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CF113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -29985,6 +30327,9 @@
       <c r="CE114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CF114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -30242,6 +30587,9 @@
       <c r="CE115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CF115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -30499,6 +30847,9 @@
       <c r="CE116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CF116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -30756,6 +31107,9 @@
       <c r="CE117" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CF117" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -31013,6 +31367,9 @@
       <c r="CE118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CF118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -31270,6 +31627,9 @@
       <c r="CE119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CF119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -31527,6 +31887,9 @@
       <c r="CE120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CF120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -31784,6 +32147,9 @@
       <c r="CE121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CF121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -32041,6 +32407,9 @@
       <c r="CE122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CF122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -32298,6 +32667,9 @@
       <c r="CE123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CF123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -32555,6 +32927,9 @@
       <c r="CE124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CF124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -32812,6 +33187,9 @@
       <c r="CE125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CF125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -33069,6 +33447,9 @@
       <c r="CE126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CF126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -33326,6 +33707,9 @@
       <c r="CE127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CF127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -33583,6 +33967,9 @@
       <c r="CE128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CF128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -33840,6 +34227,9 @@
       <c r="CE129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CF129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -34097,6 +34487,9 @@
       <c r="CE130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CF130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -34354,6 +34747,9 @@
       <c r="CE131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CF131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -34611,6 +35007,9 @@
       <c r="CE132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="CF132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -34868,6 +35267,9 @@
       <c r="CE133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CF133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -35125,6 +35527,9 @@
       <c r="CE134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="CF134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -35382,6 +35787,9 @@
       <c r="CE135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CF135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -35639,6 +36047,9 @@
       <c r="CE136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CF136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -35896,6 +36307,9 @@
       <c r="CE137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CF137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -36153,6 +36567,9 @@
       <c r="CE138" s="3" t="n">
         <v>23.29</v>
       </c>
+      <c r="CF138" s="3" t="n">
+        <v>23.29</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -36410,6 +36827,9 @@
       <c r="CE139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CF139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -36667,6 +37087,9 @@
       <c r="CE140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CF140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -36924,6 +37347,9 @@
       <c r="CE141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CF141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -37181,6 +37607,9 @@
       <c r="CE142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CF142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -37438,6 +37867,9 @@
       <c r="CE143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CF143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -37695,6 +38127,9 @@
       <c r="CE144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CF144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -37952,6 +38387,9 @@
       <c r="CE145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CF145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -38209,6 +38647,9 @@
       <c r="CE146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CF146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -38466,6 +38907,9 @@
       <c r="CE147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CF147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -38723,6 +39167,9 @@
       <c r="CE148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CF148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -38980,6 +39427,9 @@
       <c r="CE149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CF149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -39237,6 +39687,9 @@
       <c r="CE150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CF150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -39494,6 +39947,9 @@
       <c r="CE151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CF151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -39751,6 +40207,9 @@
       <c r="CE152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CF152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -40008,6 +40467,9 @@
       <c r="CE153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CF153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -40265,6 +40727,9 @@
       <c r="CE154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CF154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -40522,6 +40987,9 @@
       <c r="CE155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CF155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -40779,6 +41247,9 @@
       <c r="CE156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CF156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -41036,6 +41507,9 @@
       <c r="CE157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CF157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -41293,6 +41767,9 @@
       <c r="CE158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CF158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -41550,6 +42027,9 @@
       <c r="CE159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CF159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -41807,6 +42287,9 @@
       <c r="CE160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CF160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -42064,6 +42547,9 @@
       <c r="CE161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CF161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -42321,6 +42807,9 @@
       <c r="CE162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CF162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -42578,6 +43067,9 @@
       <c r="CE163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CF163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -42835,6 +43327,9 @@
       <c r="CE164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CF164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -42993,9 +43488,12 @@
       <c r="CE165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CF165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CE165"/>
+  <autoFilter ref="A1:CF165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-15 00:14 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CF$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CG$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CF165"/>
+  <dimension ref="A1:CG165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -527,6 +527,7 @@
     <col width="16" customWidth="1" min="82" max="82"/>
     <col width="16" customWidth="1" min="83" max="83"/>
     <col width="16" customWidth="1" min="84" max="84"/>
+    <col width="16" customWidth="1" min="85" max="85"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -950,6 +951,11 @@
           <t>2026-09-14 16:09</t>
         </is>
       </c>
+      <c r="CG1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-14 19:14</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1210,6 +1216,9 @@
       <c r="CF2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CG2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1470,6 +1479,9 @@
       <c r="CF3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CG3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1730,6 +1742,9 @@
       <c r="CF4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CG4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1990,6 +2005,9 @@
       <c r="CF5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CG5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2250,6 +2268,9 @@
       <c r="CF6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CG6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2510,6 +2531,9 @@
       <c r="CF7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CG7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2770,6 +2794,9 @@
       <c r="CF8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="CG8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3030,6 +3057,9 @@
       <c r="CF9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CG9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3290,6 +3320,9 @@
       <c r="CF10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CG10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3550,6 +3583,9 @@
       <c r="CF11" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG11" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3810,6 +3846,9 @@
       <c r="CF12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4070,6 +4109,9 @@
       <c r="CF13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CG13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4330,6 +4372,9 @@
       <c r="CF14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4590,6 +4635,9 @@
       <c r="CF15" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="CG15" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4850,6 +4898,9 @@
       <c r="CF16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CG16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5110,6 +5161,9 @@
       <c r="CF17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5370,6 +5424,9 @@
       <c r="CF18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CG18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5630,6 +5687,9 @@
       <c r="CF19" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="CG19" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5890,6 +5950,9 @@
       <c r="CF20" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG20" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -6150,6 +6213,9 @@
       <c r="CF21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="CG21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -6410,6 +6476,9 @@
       <c r="CF22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CG22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -6670,6 +6739,9 @@
       <c r="CF23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CG23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -6930,6 +7002,9 @@
       <c r="CF24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CG24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -7190,6 +7265,9 @@
       <c r="CF25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -7450,6 +7528,9 @@
       <c r="CF26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="CG26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -7710,6 +7791,9 @@
       <c r="CF27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CG27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -7970,6 +8054,9 @@
       <c r="CF28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CG28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -8230,6 +8317,9 @@
       <c r="CF29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CG29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -8490,6 +8580,9 @@
       <c r="CF30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -8750,6 +8843,9 @@
       <c r="CF31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -9010,6 +9106,9 @@
       <c r="CF32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -9270,6 +9369,9 @@
       <c r="CF33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CG33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -9530,6 +9632,9 @@
       <c r="CF34" s="3" t="n">
         <v>21.22</v>
       </c>
+      <c r="CG34" s="3" t="n">
+        <v>21.22</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -9790,6 +9895,9 @@
       <c r="CF35" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CG35" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -10050,6 +10158,9 @@
       <c r="CF36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CG36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -10310,6 +10421,9 @@
       <c r="CF37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CG37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -10570,6 +10684,9 @@
       <c r="CF38" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG38" s="3" t="n">
+        <v>21.46</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -10830,6 +10947,9 @@
       <c r="CF39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CG39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -11090,6 +11210,9 @@
       <c r="CF40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -11350,6 +11473,9 @@
       <c r="CF41" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -11610,6 +11736,9 @@
       <c r="CF42" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -11870,6 +11999,9 @@
       <c r="CF43" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CG43" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -12130,6 +12262,9 @@
       <c r="CF44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CG44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -12390,6 +12525,9 @@
       <c r="CF45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="CG45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -12650,6 +12788,9 @@
       <c r="CF46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="CG46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -12910,6 +13051,9 @@
       <c r="CF47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CG47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -13170,6 +13314,9 @@
       <c r="CF48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CG48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -13430,6 +13577,9 @@
       <c r="CF49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CG49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -13690,6 +13840,9 @@
       <c r="CF50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CG50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -13950,6 +14103,9 @@
       <c r="CF51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CG51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -14210,6 +14366,9 @@
       <c r="CF52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CG52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -14470,6 +14629,9 @@
       <c r="CF53" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CG53" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -14730,6 +14892,9 @@
       <c r="CF54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CG54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -14990,6 +15155,9 @@
       <c r="CF55" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CG55" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -15250,6 +15418,9 @@
       <c r="CF56" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CG56" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -15510,6 +15681,9 @@
       <c r="CF57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -15770,6 +15944,9 @@
       <c r="CF58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CG58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -16030,6 +16207,9 @@
       <c r="CF59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CG59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -16290,6 +16470,9 @@
       <c r="CF60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CG60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -16550,6 +16733,9 @@
       <c r="CF61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CG61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -16810,6 +16996,9 @@
       <c r="CF62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CG62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -17070,6 +17259,9 @@
       <c r="CF63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CG63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -17330,6 +17522,9 @@
       <c r="CF64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CG64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -17590,6 +17785,9 @@
       <c r="CF65" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CG65" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -17850,6 +18048,9 @@
       <c r="CF66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -18110,6 +18311,9 @@
       <c r="CF67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CG67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -18370,6 +18574,9 @@
       <c r="CF68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -18630,6 +18837,9 @@
       <c r="CF69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CG69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -18890,6 +19100,9 @@
       <c r="CF70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CG70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -19150,6 +19363,9 @@
       <c r="CF71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -19410,6 +19626,9 @@
       <c r="CF72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -19670,6 +19889,9 @@
       <c r="CF73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CG73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -19930,6 +20152,9 @@
       <c r="CF74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CG74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -20190,6 +20415,9 @@
       <c r="CF75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -20450,6 +20678,9 @@
       <c r="CF76" s="3" t="n">
         <v>21.67</v>
       </c>
+      <c r="CG76" s="3" t="n">
+        <v>21.67</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -20710,6 +20941,9 @@
       <c r="CF77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -20970,6 +21204,9 @@
       <c r="CF78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CG78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -21230,6 +21467,9 @@
       <c r="CF79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -21490,6 +21730,9 @@
       <c r="CF80" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CG80" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -21750,6 +21993,9 @@
       <c r="CF81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -22010,6 +22256,9 @@
       <c r="CF82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -22270,6 +22519,9 @@
       <c r="CF83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -22530,6 +22782,9 @@
       <c r="CF84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CG84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -22790,6 +23045,9 @@
       <c r="CF85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CG85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -23050,6 +23308,9 @@
       <c r="CF86" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CG86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -23310,6 +23571,9 @@
       <c r="CF87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -23570,6 +23834,9 @@
       <c r="CF88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -23830,6 +24097,9 @@
       <c r="CF89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -24090,6 +24360,9 @@
       <c r="CF90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CG90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -24350,6 +24623,9 @@
       <c r="CF91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -24610,6 +24886,9 @@
       <c r="CF92" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CG92" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -24870,6 +25149,9 @@
       <c r="CF93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CG93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -25130,6 +25412,9 @@
       <c r="CF94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CG94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -25390,6 +25675,9 @@
       <c r="CF95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CG95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -25650,6 +25938,9 @@
       <c r="CF96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CG96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -25910,6 +26201,9 @@
       <c r="CF97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CG97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -26170,6 +26464,9 @@
       <c r="CF98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="CG98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -26430,6 +26727,9 @@
       <c r="CF99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CG99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -26690,6 +26990,9 @@
       <c r="CF100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CG100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -26950,6 +27253,9 @@
       <c r="CF101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CG101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -27210,6 +27516,9 @@
       <c r="CF102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CG102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -27470,6 +27779,9 @@
       <c r="CF103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CG103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -27730,6 +28042,9 @@
       <c r="CF104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CG104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -27990,6 +28305,9 @@
       <c r="CF105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CG105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -28250,6 +28568,9 @@
       <c r="CF106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CG106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -28510,6 +28831,9 @@
       <c r="CF107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CG107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -28770,6 +29094,9 @@
       <c r="CF108" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CG108" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -29030,6 +29357,9 @@
       <c r="CF109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CG109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -29290,6 +29620,9 @@
       <c r="CF110" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CG110" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -29550,6 +29883,9 @@
       <c r="CF111" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CG111" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -29810,6 +30146,9 @@
       <c r="CF112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CG112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -30070,6 +30409,9 @@
       <c r="CF113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CG113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -30330,6 +30672,9 @@
       <c r="CF114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CG114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -30590,6 +30935,9 @@
       <c r="CF115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CG115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -30850,6 +31198,9 @@
       <c r="CF116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CG116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -31110,6 +31461,9 @@
       <c r="CF117" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CG117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -31370,6 +31724,9 @@
       <c r="CF118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CG118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -31630,6 +31987,9 @@
       <c r="CF119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CG119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -31890,6 +32250,9 @@
       <c r="CF120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CG120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -32150,6 +32513,9 @@
       <c r="CF121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CG121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -32410,6 +32776,9 @@
       <c r="CF122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CG122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -32670,6 +33039,9 @@
       <c r="CF123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CG123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -32930,6 +33302,9 @@
       <c r="CF124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CG124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -33190,6 +33565,9 @@
       <c r="CF125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CG125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -33450,6 +33828,9 @@
       <c r="CF126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CG126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -33710,6 +34091,9 @@
       <c r="CF127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CG127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -33970,6 +34354,9 @@
       <c r="CF128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CG128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -34230,6 +34617,9 @@
       <c r="CF129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CG129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -34490,6 +34880,9 @@
       <c r="CF130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CG130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -34750,6 +35143,9 @@
       <c r="CF131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CG131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -35010,6 +35406,9 @@
       <c r="CF132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="CG132" s="3" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -35270,6 +35669,9 @@
       <c r="CF133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CG133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -35530,6 +35932,9 @@
       <c r="CF134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="CG134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -35790,6 +36195,9 @@
       <c r="CF135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CG135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -36050,6 +36458,9 @@
       <c r="CF136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CG136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -36310,6 +36721,9 @@
       <c r="CF137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CG137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -36570,6 +36984,9 @@
       <c r="CF138" s="3" t="n">
         <v>23.29</v>
       </c>
+      <c r="CG138" s="3" t="n">
+        <v>23.29</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -36830,6 +37247,9 @@
       <c r="CF139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CG139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -37090,6 +37510,9 @@
       <c r="CF140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CG140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -37350,6 +37773,9 @@
       <c r="CF141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CG141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -37610,6 +38036,9 @@
       <c r="CF142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CG142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -37870,6 +38299,9 @@
       <c r="CF143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CG143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -38130,6 +38562,9 @@
       <c r="CF144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CG144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -38390,6 +38825,9 @@
       <c r="CF145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CG145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -38650,6 +39088,9 @@
       <c r="CF146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CG146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -38910,6 +39351,9 @@
       <c r="CF147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CG147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -39170,6 +39614,9 @@
       <c r="CF148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CG148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -39430,6 +39877,9 @@
       <c r="CF149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CG149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -39690,6 +40140,9 @@
       <c r="CF150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CG150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -39950,6 +40403,9 @@
       <c r="CF151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CG151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -40210,6 +40666,9 @@
       <c r="CF152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CG152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -40470,6 +40929,9 @@
       <c r="CF153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CG153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -40730,6 +41192,9 @@
       <c r="CF154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CG154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -40990,6 +41455,9 @@
       <c r="CF155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CG155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -41250,6 +41718,9 @@
       <c r="CF156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CG156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -41510,6 +41981,9 @@
       <c r="CF157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CG157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -41770,6 +42244,9 @@
       <c r="CF158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CG158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -42030,6 +42507,9 @@
       <c r="CF159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CG159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -42290,6 +42770,9 @@
       <c r="CF160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CG160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -42550,6 +43033,9 @@
       <c r="CF161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CG161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -42810,6 +43296,9 @@
       <c r="CF162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CG162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -43070,6 +43559,9 @@
       <c r="CF163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CG163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -43330,6 +43822,9 @@
       <c r="CF164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CG164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -43491,9 +43986,12 @@
       <c r="CF165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CG165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CF165"/>
+  <autoFilter ref="A1:CG165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-15 03:10 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CG$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CH$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CG165"/>
+  <dimension ref="A1:CH165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -528,6 +528,7 @@
     <col width="16" customWidth="1" min="83" max="83"/>
     <col width="16" customWidth="1" min="84" max="84"/>
     <col width="16" customWidth="1" min="85" max="85"/>
+    <col width="16" customWidth="1" min="86" max="86"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -956,6 +957,11 @@
           <t>2026-09-14 19:14</t>
         </is>
       </c>
+      <c r="CH1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-14 22:10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1219,6 +1225,9 @@
       <c r="CG2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CH2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1482,6 +1491,9 @@
       <c r="CG3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CH3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1745,6 +1757,9 @@
       <c r="CG4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CH4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2008,6 +2023,9 @@
       <c r="CG5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CH5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2271,6 +2289,9 @@
       <c r="CG6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CH6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2534,6 +2555,9 @@
       <c r="CG7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CH7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2797,6 +2821,9 @@
       <c r="CG8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="CH8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3060,6 +3087,9 @@
       <c r="CG9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CH9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3323,6 +3353,9 @@
       <c r="CG10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CH10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3586,6 +3619,9 @@
       <c r="CG11" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH11" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3849,6 +3885,9 @@
       <c r="CG12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4112,6 +4151,9 @@
       <c r="CG13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CH13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4375,6 +4417,9 @@
       <c r="CG14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4638,6 +4683,9 @@
       <c r="CG15" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="CH15" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4901,6 +4949,9 @@
       <c r="CG16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CH16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5164,6 +5215,9 @@
       <c r="CG17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5427,6 +5481,9 @@
       <c r="CG18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CH18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5690,6 +5747,9 @@
       <c r="CG19" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="CH19" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -5953,6 +6013,9 @@
       <c r="CG20" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH20" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -6216,6 +6279,9 @@
       <c r="CG21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="CH21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -6479,6 +6545,9 @@
       <c r="CG22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CH22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -6742,6 +6811,9 @@
       <c r="CG23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CH23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -7005,6 +7077,9 @@
       <c r="CG24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CH24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -7268,6 +7343,9 @@
       <c r="CG25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -7531,6 +7609,9 @@
       <c r="CG26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="CH26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -7794,6 +7875,9 @@
       <c r="CG27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CH27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -8057,6 +8141,9 @@
       <c r="CG28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CH28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -8320,6 +8407,9 @@
       <c r="CG29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CH29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -8583,6 +8673,9 @@
       <c r="CG30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -8846,6 +8939,9 @@
       <c r="CG31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -9109,6 +9205,9 @@
       <c r="CG32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -9372,6 +9471,9 @@
       <c r="CG33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CH33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -9635,6 +9737,9 @@
       <c r="CG34" s="3" t="n">
         <v>21.22</v>
       </c>
+      <c r="CH34" s="3" t="n">
+        <v>21.33</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -9898,6 +10003,9 @@
       <c r="CG35" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CH35" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -10161,6 +10269,9 @@
       <c r="CG36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CH36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -10424,6 +10535,9 @@
       <c r="CG37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CH37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -10687,6 +10801,9 @@
       <c r="CG38" s="3" t="n">
         <v>21.46</v>
       </c>
+      <c r="CH38" s="3" t="n">
+        <v>21.46</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -10950,6 +11067,9 @@
       <c r="CG39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CH39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -11213,6 +11333,9 @@
       <c r="CG40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -11476,6 +11599,9 @@
       <c r="CG41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CH41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -11739,6 +11865,9 @@
       <c r="CG42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CH42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -12002,6 +12131,9 @@
       <c r="CG43" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CH43" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -12265,6 +12397,9 @@
       <c r="CG44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CH44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -12528,6 +12663,9 @@
       <c r="CG45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="CH45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -12791,6 +12929,9 @@
       <c r="CG46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="CH46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -13054,6 +13195,9 @@
       <c r="CG47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CH47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -13317,6 +13461,9 @@
       <c r="CG48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CH48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -13580,6 +13727,9 @@
       <c r="CG49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CH49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -13843,6 +13993,9 @@
       <c r="CG50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CH50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -14106,6 +14259,9 @@
       <c r="CG51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CH51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -14369,6 +14525,9 @@
       <c r="CG52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CH52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -14632,6 +14791,9 @@
       <c r="CG53" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CH53" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -14895,6 +15057,9 @@
       <c r="CG54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CH54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -15158,6 +15323,9 @@
       <c r="CG55" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CH55" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -15421,6 +15589,9 @@
       <c r="CG56" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CH56" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -15684,6 +15855,9 @@
       <c r="CG57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -15947,6 +16121,9 @@
       <c r="CG58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CH58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -16210,6 +16387,9 @@
       <c r="CG59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CH59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -16473,6 +16653,9 @@
       <c r="CG60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CH60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -16736,6 +16919,9 @@
       <c r="CG61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CH61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -16999,6 +17185,9 @@
       <c r="CG62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CH62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -17262,6 +17451,9 @@
       <c r="CG63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CH63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -17525,6 +17717,9 @@
       <c r="CG64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CH64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -17788,6 +17983,9 @@
       <c r="CG65" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CH65" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -18051,6 +18249,9 @@
       <c r="CG66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -18314,6 +18515,9 @@
       <c r="CG67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CH67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -18577,6 +18781,9 @@
       <c r="CG68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -18840,6 +19047,9 @@
       <c r="CG69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CH69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -19103,6 +19313,9 @@
       <c r="CG70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CH70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -19366,6 +19579,9 @@
       <c r="CG71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -19629,6 +19845,9 @@
       <c r="CG72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -19892,6 +20111,9 @@
       <c r="CG73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CH73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -20155,6 +20377,9 @@
       <c r="CG74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CH74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -20418,6 +20643,9 @@
       <c r="CG75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -20681,6 +20909,9 @@
       <c r="CG76" s="3" t="n">
         <v>21.67</v>
       </c>
+      <c r="CH76" s="3" t="n">
+        <v>21.67</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -20944,6 +21175,9 @@
       <c r="CG77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -21207,6 +21441,9 @@
       <c r="CG78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CH78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -21470,6 +21707,9 @@
       <c r="CG79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -21733,6 +21973,9 @@
       <c r="CG80" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CH80" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -21996,6 +22239,9 @@
       <c r="CG81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -22259,6 +22505,9 @@
       <c r="CG82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -22522,6 +22771,9 @@
       <c r="CG83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -22785,6 +23037,9 @@
       <c r="CG84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CH84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -23048,6 +23303,9 @@
       <c r="CG85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CH85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -23311,6 +23569,9 @@
       <c r="CG86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="CH86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -23574,6 +23835,9 @@
       <c r="CG87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -23837,6 +24101,9 @@
       <c r="CG88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -24100,6 +24367,9 @@
       <c r="CG89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -24363,6 +24633,9 @@
       <c r="CG90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CH90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -24626,6 +24899,9 @@
       <c r="CG91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -24889,6 +25165,9 @@
       <c r="CG92" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CH92" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -25152,6 +25431,9 @@
       <c r="CG93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CH93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -25415,6 +25697,9 @@
       <c r="CG94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CH94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -25678,6 +25963,9 @@
       <c r="CG95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CH95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -25941,6 +26229,9 @@
       <c r="CG96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CH96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -26204,6 +26495,9 @@
       <c r="CG97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CH97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -26467,6 +26761,9 @@
       <c r="CG98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="CH98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -26730,6 +27027,9 @@
       <c r="CG99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CH99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -26993,6 +27293,9 @@
       <c r="CG100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CH100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -27256,6 +27559,9 @@
       <c r="CG101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CH101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -27519,6 +27825,9 @@
       <c r="CG102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CH102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -27782,6 +28091,9 @@
       <c r="CG103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CH103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -28045,6 +28357,9 @@
       <c r="CG104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CH104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -28308,6 +28623,9 @@
       <c r="CG105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CH105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -28571,6 +28889,9 @@
       <c r="CG106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CH106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -28834,6 +29155,9 @@
       <c r="CG107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CH107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -29097,6 +29421,9 @@
       <c r="CG108" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CH108" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -29360,6 +29687,9 @@
       <c r="CG109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CH109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -29623,6 +29953,9 @@
       <c r="CG110" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CH110" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -29886,6 +30219,9 @@
       <c r="CG111" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CH111" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -30149,6 +30485,9 @@
       <c r="CG112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CH112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -30412,6 +30751,9 @@
       <c r="CG113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CH113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -30675,6 +31017,9 @@
       <c r="CG114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CH114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -30938,6 +31283,9 @@
       <c r="CG115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CH115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -31201,6 +31549,9 @@
       <c r="CG116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CH116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -31464,6 +31815,9 @@
       <c r="CG117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CH117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -31727,6 +32081,9 @@
       <c r="CG118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CH118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -31990,6 +32347,9 @@
       <c r="CG119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CH119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -32253,6 +32613,9 @@
       <c r="CG120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CH120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -32516,6 +32879,9 @@
       <c r="CG121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CH121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -32779,6 +33145,9 @@
       <c r="CG122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CH122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -33042,6 +33411,9 @@
       <c r="CG123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CH123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -33305,6 +33677,9 @@
       <c r="CG124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CH124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -33568,6 +33943,9 @@
       <c r="CG125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CH125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -33831,6 +34209,9 @@
       <c r="CG126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CH126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -34094,6 +34475,9 @@
       <c r="CG127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CH127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -34357,6 +34741,9 @@
       <c r="CG128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CH128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -34620,6 +35007,9 @@
       <c r="CG129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CH129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -34883,6 +35273,9 @@
       <c r="CG130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CH130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -35146,6 +35539,9 @@
       <c r="CG131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CH131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -35409,6 +35805,9 @@
       <c r="CG132" s="3" t="n">
         <v>21.6</v>
       </c>
+      <c r="CH132" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -35672,6 +36071,9 @@
       <c r="CG133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CH133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -35935,6 +36337,9 @@
       <c r="CG134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="CH134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -36198,6 +36603,9 @@
       <c r="CG135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CH135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -36461,6 +36869,9 @@
       <c r="CG136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CH136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -36724,6 +37135,9 @@
       <c r="CG137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CH137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -36987,6 +37401,9 @@
       <c r="CG138" s="3" t="n">
         <v>23.29</v>
       </c>
+      <c r="CH138" s="3" t="n">
+        <v>23.29</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -37250,6 +37667,9 @@
       <c r="CG139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CH139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -37513,6 +37933,9 @@
       <c r="CG140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CH140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -37776,6 +38199,9 @@
       <c r="CG141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CH141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -38039,6 +38465,9 @@
       <c r="CG142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CH142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -38302,6 +38731,9 @@
       <c r="CG143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CH143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -38565,6 +38997,9 @@
       <c r="CG144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CH144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -38828,6 +39263,9 @@
       <c r="CG145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CH145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -39091,6 +39529,9 @@
       <c r="CG146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CH146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -39354,6 +39795,9 @@
       <c r="CG147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CH147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -39617,6 +40061,9 @@
       <c r="CG148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CH148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -39880,6 +40327,9 @@
       <c r="CG149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CH149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -40143,6 +40593,9 @@
       <c r="CG150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CH150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -40406,6 +40859,9 @@
       <c r="CG151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CH151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -40669,6 +41125,9 @@
       <c r="CG152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CH152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -40932,6 +41391,9 @@
       <c r="CG153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CH153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -41195,6 +41657,9 @@
       <c r="CG154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CH154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -41458,6 +41923,9 @@
       <c r="CG155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CH155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -41721,6 +42189,9 @@
       <c r="CG156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CH156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -41984,6 +42455,9 @@
       <c r="CG157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CH157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -42247,6 +42721,9 @@
       <c r="CG158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CH158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -42510,6 +42987,9 @@
       <c r="CG159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CH159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -42773,6 +43253,9 @@
       <c r="CG160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CH160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -43036,6 +43519,9 @@
       <c r="CG161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CH161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -43299,6 +43785,9 @@
       <c r="CG162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CH162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -43562,6 +44051,9 @@
       <c r="CG163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CH163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -43825,6 +44317,9 @@
       <c r="CG164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CH164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -43989,9 +44484,12 @@
       <c r="CG165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CH165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CG165"/>
+  <autoFilter ref="A1:CH165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-15 06:12 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CH$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CI$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CH165"/>
+  <dimension ref="A1:CI165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -529,6 +529,7 @@
     <col width="16" customWidth="1" min="84" max="84"/>
     <col width="16" customWidth="1" min="85" max="85"/>
     <col width="16" customWidth="1" min="86" max="86"/>
+    <col width="16" customWidth="1" min="87" max="87"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -962,6 +963,11 @@
           <t>2026-09-14 22:10</t>
         </is>
       </c>
+      <c r="CI1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-15 01:12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1228,6 +1234,9 @@
       <c r="CH2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CI2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1494,6 +1503,9 @@
       <c r="CH3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CI3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1760,6 +1772,9 @@
       <c r="CH4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CI4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2026,6 +2041,9 @@
       <c r="CH5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CI5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2292,6 +2310,9 @@
       <c r="CH6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CI6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2558,6 +2579,9 @@
       <c r="CH7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CI7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2824,6 +2848,9 @@
       <c r="CH8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="CI8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3090,6 +3117,9 @@
       <c r="CH9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CI9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3356,6 +3386,9 @@
       <c r="CH10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CI10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3622,6 +3655,9 @@
       <c r="CH11" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI11" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3888,6 +3924,9 @@
       <c r="CH12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4154,6 +4193,9 @@
       <c r="CH13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CI13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4420,6 +4462,9 @@
       <c r="CH14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4686,6 +4731,9 @@
       <c r="CH15" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="CI15" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -4952,6 +5000,9 @@
       <c r="CH16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CI16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5218,6 +5269,9 @@
       <c r="CH17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5484,6 +5538,9 @@
       <c r="CH18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CI18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5750,6 +5807,9 @@
       <c r="CH19" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="CI19" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -6016,6 +6076,9 @@
       <c r="CH20" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI20" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -6282,6 +6345,9 @@
       <c r="CH21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="CI21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -6548,6 +6614,9 @@
       <c r="CH22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CI22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -6814,6 +6883,9 @@
       <c r="CH23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CI23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -7080,6 +7152,9 @@
       <c r="CH24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CI24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -7346,6 +7421,9 @@
       <c r="CH25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -7612,6 +7690,9 @@
       <c r="CH26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="CI26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -7878,6 +7959,9 @@
       <c r="CH27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CI27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -8144,6 +8228,9 @@
       <c r="CH28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CI28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -8410,6 +8497,9 @@
       <c r="CH29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CI29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -8676,6 +8766,9 @@
       <c r="CH30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -8942,6 +9035,9 @@
       <c r="CH31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -9208,6 +9304,9 @@
       <c r="CH32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -9474,6 +9573,9 @@
       <c r="CH33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CI33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -9740,6 +9842,9 @@
       <c r="CH34" s="3" t="n">
         <v>21.33</v>
       </c>
+      <c r="CI34" s="3" t="n">
+        <v>21.33</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -10006,6 +10111,9 @@
       <c r="CH35" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CI35" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -10272,6 +10380,9 @@
       <c r="CH36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CI36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -10538,6 +10649,9 @@
       <c r="CH37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CI37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -10804,6 +10918,9 @@
       <c r="CH38" s="3" t="n">
         <v>21.46</v>
       </c>
+      <c r="CI38" s="3" t="n">
+        <v>21.46</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -11070,6 +11187,9 @@
       <c r="CH39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CI39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -11336,6 +11456,9 @@
       <c r="CH40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -11602,6 +11725,9 @@
       <c r="CH41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CI41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -11868,6 +11994,9 @@
       <c r="CH42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CI42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -12134,6 +12263,9 @@
       <c r="CH43" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CI43" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -12400,6 +12532,9 @@
       <c r="CH44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CI44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -12666,6 +12801,9 @@
       <c r="CH45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="CI45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -12932,6 +13070,9 @@
       <c r="CH46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="CI46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -13198,6 +13339,9 @@
       <c r="CH47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CI47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -13464,6 +13608,9 @@
       <c r="CH48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CI48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -13730,6 +13877,9 @@
       <c r="CH49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CI49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -13996,6 +14146,9 @@
       <c r="CH50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CI50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -14262,6 +14415,9 @@
       <c r="CH51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CI51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -14528,6 +14684,9 @@
       <c r="CH52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CI52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -14794,6 +14953,9 @@
       <c r="CH53" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CI53" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -15060,6 +15222,9 @@
       <c r="CH54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CI54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -15326,6 +15491,9 @@
       <c r="CH55" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CI55" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -15592,6 +15760,9 @@
       <c r="CH56" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CI56" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -15858,6 +16029,9 @@
       <c r="CH57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -16124,6 +16298,9 @@
       <c r="CH58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CI58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -16390,6 +16567,9 @@
       <c r="CH59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CI59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -16656,6 +16836,9 @@
       <c r="CH60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CI60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -16922,6 +17105,9 @@
       <c r="CH61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CI61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -17188,6 +17374,9 @@
       <c r="CH62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CI62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -17454,6 +17643,9 @@
       <c r="CH63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CI63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -17720,6 +17912,9 @@
       <c r="CH64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CI64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -17986,6 +18181,9 @@
       <c r="CH65" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CI65" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -18252,6 +18450,9 @@
       <c r="CH66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -18518,6 +18719,9 @@
       <c r="CH67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CI67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -18784,6 +18988,9 @@
       <c r="CH68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -19050,6 +19257,9 @@
       <c r="CH69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CI69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -19316,6 +19526,9 @@
       <c r="CH70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CI70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -19582,6 +19795,9 @@
       <c r="CH71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -19848,6 +20064,9 @@
       <c r="CH72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -20114,6 +20333,9 @@
       <c r="CH73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CI73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -20380,6 +20602,9 @@
       <c r="CH74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CI74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -20646,6 +20871,9 @@
       <c r="CH75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -20912,6 +21140,9 @@
       <c r="CH76" s="3" t="n">
         <v>21.67</v>
       </c>
+      <c r="CI76" s="3" t="n">
+        <v>21.67</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -21178,6 +21409,9 @@
       <c r="CH77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -21444,6 +21678,9 @@
       <c r="CH78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CI78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -21710,6 +21947,9 @@
       <c r="CH79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -21976,6 +22216,9 @@
       <c r="CH80" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CI80" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -22242,6 +22485,9 @@
       <c r="CH81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -22508,6 +22754,9 @@
       <c r="CH82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -22774,6 +23023,9 @@
       <c r="CH83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -23040,6 +23292,9 @@
       <c r="CH84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CI84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -23306,6 +23561,9 @@
       <c r="CH85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CI85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -23572,6 +23830,9 @@
       <c r="CH86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="CI86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -23838,6 +24099,9 @@
       <c r="CH87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -24104,6 +24368,9 @@
       <c r="CH88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -24370,6 +24637,9 @@
       <c r="CH89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -24636,6 +24906,9 @@
       <c r="CH90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CI90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -24902,6 +25175,9 @@
       <c r="CH91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -25168,6 +25444,9 @@
       <c r="CH92" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CI92" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -25434,6 +25713,9 @@
       <c r="CH93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CI93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -25700,6 +25982,9 @@
       <c r="CH94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CI94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -25966,6 +26251,9 @@
       <c r="CH95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CI95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -26232,6 +26520,9 @@
       <c r="CH96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CI96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -26498,6 +26789,9 @@
       <c r="CH97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CI97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -26764,6 +27058,9 @@
       <c r="CH98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="CI98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -27030,6 +27327,9 @@
       <c r="CH99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CI99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -27296,6 +27596,9 @@
       <c r="CH100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CI100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -27562,6 +27865,9 @@
       <c r="CH101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CI101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -27828,6 +28134,9 @@
       <c r="CH102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CI102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -28094,6 +28403,9 @@
       <c r="CH103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CI103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -28360,6 +28672,9 @@
       <c r="CH104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CI104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -28626,6 +28941,9 @@
       <c r="CH105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CI105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -28892,6 +29210,9 @@
       <c r="CH106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CI106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -29158,6 +29479,9 @@
       <c r="CH107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CI107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -29424,6 +29748,9 @@
       <c r="CH108" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CI108" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -29690,6 +30017,9 @@
       <c r="CH109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CI109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -29956,6 +30286,9 @@
       <c r="CH110" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CI110" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -30222,6 +30555,9 @@
       <c r="CH111" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CI111" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -30488,6 +30824,9 @@
       <c r="CH112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CI112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -30754,6 +31093,9 @@
       <c r="CH113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CI113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -31020,6 +31362,9 @@
       <c r="CH114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CI114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -31286,6 +31631,9 @@
       <c r="CH115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CI115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -31552,6 +31900,9 @@
       <c r="CH116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CI116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -31818,6 +32169,9 @@
       <c r="CH117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CI117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -32084,6 +32438,9 @@
       <c r="CH118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CI118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -32350,6 +32707,9 @@
       <c r="CH119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CI119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -32616,6 +32976,9 @@
       <c r="CH120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CI120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -32882,6 +33245,9 @@
       <c r="CH121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CI121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -33148,6 +33514,9 @@
       <c r="CH122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CI122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -33414,6 +33783,9 @@
       <c r="CH123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CI123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -33680,6 +34052,9 @@
       <c r="CH124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CI124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -33946,6 +34321,9 @@
       <c r="CH125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CI125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -34212,6 +34590,9 @@
       <c r="CH126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CI126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -34478,6 +34859,9 @@
       <c r="CH127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CI127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -34744,6 +35128,9 @@
       <c r="CH128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CI128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -35010,6 +35397,9 @@
       <c r="CH129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CI129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -35276,6 +35666,9 @@
       <c r="CH130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CI130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -35542,6 +35935,9 @@
       <c r="CH131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CI131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -35808,6 +36204,9 @@
       <c r="CH132" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CI132" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -36074,6 +36473,9 @@
       <c r="CH133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CI133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -36340,6 +36742,9 @@
       <c r="CH134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="CI134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -36606,6 +37011,9 @@
       <c r="CH135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CI135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -36872,6 +37280,9 @@
       <c r="CH136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CI136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -37138,6 +37549,9 @@
       <c r="CH137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CI137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -37404,6 +37818,9 @@
       <c r="CH138" s="3" t="n">
         <v>23.29</v>
       </c>
+      <c r="CI138" s="3" t="n">
+        <v>23.29</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -37670,6 +38087,9 @@
       <c r="CH139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CI139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -37936,6 +38356,9 @@
       <c r="CH140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CI140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -38202,6 +38625,9 @@
       <c r="CH141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CI141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -38468,6 +38894,9 @@
       <c r="CH142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CI142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -38734,6 +39163,9 @@
       <c r="CH143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CI143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -39000,6 +39432,9 @@
       <c r="CH144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CI144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -39266,6 +39701,9 @@
       <c r="CH145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CI145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -39532,6 +39970,9 @@
       <c r="CH146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CI146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -39798,6 +40239,9 @@
       <c r="CH147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CI147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -40064,6 +40508,9 @@
       <c r="CH148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CI148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -40330,6 +40777,9 @@
       <c r="CH149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CI149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -40596,6 +41046,9 @@
       <c r="CH150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CI150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -40862,6 +41315,9 @@
       <c r="CH151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CI151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -41128,6 +41584,9 @@
       <c r="CH152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CI152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -41394,6 +41853,9 @@
       <c r="CH153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CI153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -41660,6 +42122,9 @@
       <c r="CH154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CI154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -41926,6 +42391,9 @@
       <c r="CH155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CI155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -42192,6 +42660,9 @@
       <c r="CH156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CI156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -42458,6 +42929,9 @@
       <c r="CH157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CI157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -42724,6 +43198,9 @@
       <c r="CH158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CI158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -42990,6 +43467,9 @@
       <c r="CH159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CI159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -43256,6 +43736,9 @@
       <c r="CH160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CI160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -43522,6 +44005,9 @@
       <c r="CH161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CI161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -43788,6 +44274,9 @@
       <c r="CH162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CI162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -44054,6 +44543,9 @@
       <c r="CH163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CI163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -44320,6 +44812,9 @@
       <c r="CH164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CI164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -44487,9 +44982,12 @@
       <c r="CH165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CI165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CH165"/>
+  <autoFilter ref="A1:CI165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-15 09:11 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CI$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CJ$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CI165"/>
+  <dimension ref="A1:CJ165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -530,6 +530,7 @@
     <col width="16" customWidth="1" min="85" max="85"/>
     <col width="16" customWidth="1" min="86" max="86"/>
     <col width="16" customWidth="1" min="87" max="87"/>
+    <col width="16" customWidth="1" min="88" max="88"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -968,6 +969,11 @@
           <t>2026-09-15 01:12</t>
         </is>
       </c>
+      <c r="CJ1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-15 04:11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1237,6 +1243,9 @@
       <c r="CI2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CJ2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1506,6 +1515,9 @@
       <c r="CI3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CJ3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1775,6 +1787,9 @@
       <c r="CI4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CJ4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2044,6 +2059,9 @@
       <c r="CI5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CJ5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2313,6 +2331,9 @@
       <c r="CI6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CJ6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2582,6 +2603,9 @@
       <c r="CI7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CJ7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2851,6 +2875,9 @@
       <c r="CI8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="CJ8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3120,6 +3147,9 @@
       <c r="CI9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CJ9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3389,6 +3419,9 @@
       <c r="CI10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CJ10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3658,6 +3691,9 @@
       <c r="CI11" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ11" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3927,6 +3963,9 @@
       <c r="CI12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4196,6 +4235,9 @@
       <c r="CI13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CJ13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4465,6 +4507,9 @@
       <c r="CI14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4734,6 +4779,9 @@
       <c r="CI15" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="CJ15" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5003,6 +5051,9 @@
       <c r="CI16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CJ16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5272,6 +5323,9 @@
       <c r="CI17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5541,6 +5595,9 @@
       <c r="CI18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CJ18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5810,6 +5867,9 @@
       <c r="CI19" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="CJ19" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -6079,6 +6139,9 @@
       <c r="CI20" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ20" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -6348,6 +6411,9 @@
       <c r="CI21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="CJ21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -6617,6 +6683,9 @@
       <c r="CI22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CJ22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -6886,6 +6955,9 @@
       <c r="CI23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CJ23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -7155,6 +7227,9 @@
       <c r="CI24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CJ24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -7424,6 +7499,9 @@
       <c r="CI25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -7693,6 +7771,9 @@
       <c r="CI26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="CJ26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -7962,6 +8043,9 @@
       <c r="CI27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CJ27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -8231,6 +8315,9 @@
       <c r="CI28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CJ28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -8500,6 +8587,9 @@
       <c r="CI29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CJ29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -8769,6 +8859,9 @@
       <c r="CI30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -9038,6 +9131,9 @@
       <c r="CI31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -9307,6 +9403,9 @@
       <c r="CI32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -9576,6 +9675,9 @@
       <c r="CI33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CJ33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -9845,6 +9947,9 @@
       <c r="CI34" s="3" t="n">
         <v>21.33</v>
       </c>
+      <c r="CJ34" s="3" t="n">
+        <v>21.33</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -10114,6 +10219,9 @@
       <c r="CI35" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CJ35" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -10383,6 +10491,9 @@
       <c r="CI36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CJ36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -10652,6 +10763,9 @@
       <c r="CI37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CJ37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -10921,6 +11035,9 @@
       <c r="CI38" s="3" t="n">
         <v>21.46</v>
       </c>
+      <c r="CJ38" s="3" t="n">
+        <v>21.46</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -11190,6 +11307,9 @@
       <c r="CI39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CJ39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -11459,6 +11579,9 @@
       <c r="CI40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -11728,6 +11851,9 @@
       <c r="CI41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CJ41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -11997,6 +12123,9 @@
       <c r="CI42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CJ42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -12266,6 +12395,9 @@
       <c r="CI43" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CJ43" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -12535,6 +12667,9 @@
       <c r="CI44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CJ44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -12804,6 +12939,9 @@
       <c r="CI45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="CJ45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -13073,6 +13211,9 @@
       <c r="CI46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="CJ46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -13342,6 +13483,9 @@
       <c r="CI47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CJ47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -13611,6 +13755,9 @@
       <c r="CI48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CJ48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -13880,6 +14027,9 @@
       <c r="CI49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CJ49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -14149,6 +14299,9 @@
       <c r="CI50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CJ50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -14418,6 +14571,9 @@
       <c r="CI51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CJ51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -14687,6 +14843,9 @@
       <c r="CI52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CJ52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -14956,6 +15115,9 @@
       <c r="CI53" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CJ53" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -15225,6 +15387,9 @@
       <c r="CI54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CJ54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -15494,6 +15659,9 @@
       <c r="CI55" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CJ55" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -15763,6 +15931,9 @@
       <c r="CI56" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CJ56" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -16032,6 +16203,9 @@
       <c r="CI57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -16301,6 +16475,9 @@
       <c r="CI58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CJ58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -16570,6 +16747,9 @@
       <c r="CI59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CJ59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -16839,6 +17019,9 @@
       <c r="CI60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CJ60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -17108,6 +17291,9 @@
       <c r="CI61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CJ61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -17377,6 +17563,9 @@
       <c r="CI62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CJ62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -17646,6 +17835,9 @@
       <c r="CI63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CJ63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -17915,6 +18107,9 @@
       <c r="CI64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CJ64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -18184,6 +18379,9 @@
       <c r="CI65" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CJ65" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -18453,6 +18651,9 @@
       <c r="CI66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -18722,6 +18923,9 @@
       <c r="CI67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CJ67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -18991,6 +19195,9 @@
       <c r="CI68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -19260,6 +19467,9 @@
       <c r="CI69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CJ69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -19529,6 +19739,9 @@
       <c r="CI70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CJ70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -19798,6 +20011,9 @@
       <c r="CI71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -20067,6 +20283,9 @@
       <c r="CI72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -20336,6 +20555,9 @@
       <c r="CI73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CJ73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -20605,6 +20827,9 @@
       <c r="CI74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CJ74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -20874,6 +21099,9 @@
       <c r="CI75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -21143,6 +21371,9 @@
       <c r="CI76" s="3" t="n">
         <v>21.67</v>
       </c>
+      <c r="CJ76" s="3" t="n">
+        <v>21.67</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -21412,6 +21643,9 @@
       <c r="CI77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -21681,6 +21915,9 @@
       <c r="CI78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CJ78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -21950,6 +22187,9 @@
       <c r="CI79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -22219,6 +22459,9 @@
       <c r="CI80" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CJ80" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -22488,6 +22731,9 @@
       <c r="CI81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -22757,6 +23003,9 @@
       <c r="CI82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -23026,6 +23275,9 @@
       <c r="CI83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -23295,6 +23547,9 @@
       <c r="CI84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CJ84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -23564,6 +23819,9 @@
       <c r="CI85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CJ85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -23833,6 +24091,9 @@
       <c r="CI86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="CJ86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -24102,6 +24363,9 @@
       <c r="CI87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -24371,6 +24635,9 @@
       <c r="CI88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -24640,6 +24907,9 @@
       <c r="CI89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -24909,6 +25179,9 @@
       <c r="CI90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CJ90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -25178,6 +25451,9 @@
       <c r="CI91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -25447,6 +25723,9 @@
       <c r="CI92" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CJ92" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -25716,6 +25995,9 @@
       <c r="CI93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CJ93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -25985,6 +26267,9 @@
       <c r="CI94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CJ94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -26254,6 +26539,9 @@
       <c r="CI95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CJ95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -26523,6 +26811,9 @@
       <c r="CI96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CJ96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -26792,6 +27083,9 @@
       <c r="CI97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CJ97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -27061,6 +27355,9 @@
       <c r="CI98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="CJ98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -27330,6 +27627,9 @@
       <c r="CI99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CJ99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -27599,6 +27899,9 @@
       <c r="CI100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CJ100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -27868,6 +28171,9 @@
       <c r="CI101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CJ101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -28137,6 +28443,9 @@
       <c r="CI102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CJ102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -28406,6 +28715,9 @@
       <c r="CI103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CJ103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -28675,6 +28987,9 @@
       <c r="CI104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CJ104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -28944,6 +29259,9 @@
       <c r="CI105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CJ105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -29213,6 +29531,9 @@
       <c r="CI106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CJ106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -29482,6 +29803,9 @@
       <c r="CI107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CJ107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -29751,6 +30075,9 @@
       <c r="CI108" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CJ108" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -30020,6 +30347,9 @@
       <c r="CI109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CJ109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -30289,6 +30619,9 @@
       <c r="CI110" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CJ110" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -30558,6 +30891,9 @@
       <c r="CI111" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CJ111" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -30827,6 +31163,9 @@
       <c r="CI112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CJ112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -31096,6 +31435,9 @@
       <c r="CI113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CJ113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -31365,6 +31707,9 @@
       <c r="CI114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CJ114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -31634,6 +31979,9 @@
       <c r="CI115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CJ115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -31903,6 +32251,9 @@
       <c r="CI116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CJ116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -32172,6 +32523,9 @@
       <c r="CI117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CJ117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -32441,6 +32795,9 @@
       <c r="CI118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CJ118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -32710,6 +33067,9 @@
       <c r="CI119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CJ119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -32979,6 +33339,9 @@
       <c r="CI120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CJ120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -33248,6 +33611,9 @@
       <c r="CI121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CJ121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -33517,6 +33883,9 @@
       <c r="CI122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CJ122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -33786,6 +34155,9 @@
       <c r="CI123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CJ123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -34055,6 +34427,9 @@
       <c r="CI124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CJ124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -34324,6 +34699,9 @@
       <c r="CI125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CJ125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -34593,6 +34971,9 @@
       <c r="CI126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CJ126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -34862,6 +35243,9 @@
       <c r="CI127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CJ127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -35131,6 +35515,9 @@
       <c r="CI128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CJ128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -35400,6 +35787,9 @@
       <c r="CI129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CJ129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -35669,6 +36059,9 @@
       <c r="CI130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CJ130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -35938,6 +36331,9 @@
       <c r="CI131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CJ131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -36207,6 +36603,9 @@
       <c r="CI132" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CJ132" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -36476,6 +36875,9 @@
       <c r="CI133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CJ133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -36745,6 +37147,9 @@
       <c r="CI134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="CJ134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -37014,6 +37419,9 @@
       <c r="CI135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CJ135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -37283,6 +37691,9 @@
       <c r="CI136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CJ136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -37552,6 +37963,9 @@
       <c r="CI137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CJ137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -37821,6 +38235,9 @@
       <c r="CI138" s="3" t="n">
         <v>23.29</v>
       </c>
+      <c r="CJ138" s="3" t="n">
+        <v>23.29</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -38090,6 +38507,9 @@
       <c r="CI139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CJ139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -38359,6 +38779,9 @@
       <c r="CI140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CJ140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -38628,6 +39051,9 @@
       <c r="CI141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CJ141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -38897,6 +39323,9 @@
       <c r="CI142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CJ142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -39166,6 +39595,9 @@
       <c r="CI143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CJ143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -39435,6 +39867,9 @@
       <c r="CI144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CJ144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -39704,6 +40139,9 @@
       <c r="CI145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CJ145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -39973,6 +40411,9 @@
       <c r="CI146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CJ146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -40242,6 +40683,9 @@
       <c r="CI147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CJ147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -40511,6 +40955,9 @@
       <c r="CI148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CJ148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -40780,6 +41227,9 @@
       <c r="CI149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CJ149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -41049,6 +41499,9 @@
       <c r="CI150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CJ150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -41318,6 +41771,9 @@
       <c r="CI151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CJ151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -41587,6 +42043,9 @@
       <c r="CI152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CJ152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -41856,6 +42315,9 @@
       <c r="CI153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CJ153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -42125,6 +42587,9 @@
       <c r="CI154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CJ154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -42394,6 +42859,9 @@
       <c r="CI155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CJ155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -42663,6 +43131,9 @@
       <c r="CI156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CJ156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -42932,6 +43403,9 @@
       <c r="CI157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CJ157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -43201,6 +43675,9 @@
       <c r="CI158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CJ158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -43470,6 +43947,9 @@
       <c r="CI159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CJ159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -43739,6 +44219,9 @@
       <c r="CI160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CJ160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -44008,6 +44491,9 @@
       <c r="CI161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CJ161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -44277,6 +44763,9 @@
       <c r="CI162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CJ162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -44546,6 +45035,9 @@
       <c r="CI163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CJ163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -44815,6 +45307,9 @@
       <c r="CI164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CJ164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -44985,9 +45480,12 @@
       <c r="CI165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CJ165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CI165"/>
+  <autoFilter ref="A1:CJ165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-15 12:12 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CJ$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CK$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CJ165"/>
+  <dimension ref="A1:CK165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -531,6 +531,7 @@
     <col width="16" customWidth="1" min="86" max="86"/>
     <col width="16" customWidth="1" min="87" max="87"/>
     <col width="16" customWidth="1" min="88" max="88"/>
+    <col width="16" customWidth="1" min="89" max="89"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -974,6 +975,11 @@
           <t>2026-09-15 04:11</t>
         </is>
       </c>
+      <c r="CK1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1246,6 +1252,9 @@
       <c r="CJ2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CK2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1518,6 +1527,9 @@
       <c r="CJ3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CK3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1790,6 +1802,9 @@
       <c r="CJ4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CK4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2062,6 +2077,9 @@
       <c r="CJ5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CK5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2334,6 +2352,9 @@
       <c r="CJ6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CK6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2606,6 +2627,9 @@
       <c r="CJ7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CK7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2878,6 +2902,9 @@
       <c r="CJ8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="CK8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3150,6 +3177,9 @@
       <c r="CJ9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CK9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3422,6 +3452,9 @@
       <c r="CJ10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CK10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3694,6 +3727,9 @@
       <c r="CJ11" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK11" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3966,6 +4002,9 @@
       <c r="CJ12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4238,6 +4277,9 @@
       <c r="CJ13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CK13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4510,6 +4552,9 @@
       <c r="CJ14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4782,6 +4827,9 @@
       <c r="CJ15" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="CK15" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5054,6 +5102,9 @@
       <c r="CJ16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CK16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5326,6 +5377,9 @@
       <c r="CJ17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5598,6 +5652,9 @@
       <c r="CJ18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CK18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5870,6 +5927,9 @@
       <c r="CJ19" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="CK19" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -6142,6 +6202,9 @@
       <c r="CJ20" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK20" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -6414,6 +6477,9 @@
       <c r="CJ21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="CK21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -6686,6 +6752,9 @@
       <c r="CJ22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CK22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -6958,6 +7027,9 @@
       <c r="CJ23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CK23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -7230,6 +7302,9 @@
       <c r="CJ24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CK24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -7502,6 +7577,9 @@
       <c r="CJ25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -7774,6 +7852,9 @@
       <c r="CJ26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="CK26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -8046,6 +8127,9 @@
       <c r="CJ27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CK27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -8318,6 +8402,9 @@
       <c r="CJ28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CK28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -8590,6 +8677,9 @@
       <c r="CJ29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CK29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -8862,6 +8952,9 @@
       <c r="CJ30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -9134,6 +9227,9 @@
       <c r="CJ31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -9406,6 +9502,9 @@
       <c r="CJ32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -9678,6 +9777,9 @@
       <c r="CJ33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CK33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -9950,6 +10052,9 @@
       <c r="CJ34" s="3" t="n">
         <v>21.33</v>
       </c>
+      <c r="CK34" s="3" t="n">
+        <v>21.33</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -10222,6 +10327,9 @@
       <c r="CJ35" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CK35" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -10494,6 +10602,9 @@
       <c r="CJ36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CK36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -10766,6 +10877,9 @@
       <c r="CJ37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CK37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -11038,6 +11152,9 @@
       <c r="CJ38" s="3" t="n">
         <v>21.46</v>
       </c>
+      <c r="CK38" s="3" t="n">
+        <v>21.46</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -11310,6 +11427,9 @@
       <c r="CJ39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CK39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -11582,6 +11702,9 @@
       <c r="CJ40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK40" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -11854,6 +11977,9 @@
       <c r="CJ41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CK41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -12126,6 +12252,9 @@
       <c r="CJ42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CK42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -12398,6 +12527,9 @@
       <c r="CJ43" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CK43" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -12670,6 +12802,9 @@
       <c r="CJ44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CK44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -12942,6 +13077,9 @@
       <c r="CJ45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="CK45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -13214,6 +13352,9 @@
       <c r="CJ46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="CK46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -13486,6 +13627,9 @@
       <c r="CJ47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CK47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -13758,6 +13902,9 @@
       <c r="CJ48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CK48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -14030,6 +14177,9 @@
       <c r="CJ49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CK49" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -14302,6 +14452,9 @@
       <c r="CJ50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CK50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -14574,6 +14727,9 @@
       <c r="CJ51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CK51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -14846,6 +15002,9 @@
       <c r="CJ52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CK52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -15118,6 +15277,9 @@
       <c r="CJ53" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CK53" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -15390,6 +15552,9 @@
       <c r="CJ54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CK54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -15662,6 +15827,9 @@
       <c r="CJ55" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CK55" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -15934,6 +16102,9 @@
       <c r="CJ56" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CK56" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -16206,6 +16377,9 @@
       <c r="CJ57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -16478,6 +16652,9 @@
       <c r="CJ58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CK58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -16750,6 +16927,9 @@
       <c r="CJ59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CK59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -17022,6 +17202,9 @@
       <c r="CJ60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CK60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -17294,6 +17477,9 @@
       <c r="CJ61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CK61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -17566,6 +17752,9 @@
       <c r="CJ62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CK62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -17838,6 +18027,9 @@
       <c r="CJ63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CK63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -18110,6 +18302,9 @@
       <c r="CJ64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CK64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -18382,6 +18577,9 @@
       <c r="CJ65" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CK65" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -18654,6 +18852,9 @@
       <c r="CJ66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -18926,6 +19127,9 @@
       <c r="CJ67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CK67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -19198,6 +19402,9 @@
       <c r="CJ68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -19470,6 +19677,9 @@
       <c r="CJ69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CK69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -19742,6 +19952,9 @@
       <c r="CJ70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CK70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -20014,6 +20227,9 @@
       <c r="CJ71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -20286,6 +20502,9 @@
       <c r="CJ72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -20558,6 +20777,9 @@
       <c r="CJ73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CK73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -20830,6 +21052,9 @@
       <c r="CJ74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CK74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -21102,6 +21327,9 @@
       <c r="CJ75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -21374,6 +21602,9 @@
       <c r="CJ76" s="3" t="n">
         <v>21.67</v>
       </c>
+      <c r="CK76" s="3" t="n">
+        <v>21.67</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -21646,6 +21877,9 @@
       <c r="CJ77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -21918,6 +22152,9 @@
       <c r="CJ78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CK78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -22190,6 +22427,9 @@
       <c r="CJ79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -22462,6 +22702,9 @@
       <c r="CJ80" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CK80" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -22734,6 +22977,9 @@
       <c r="CJ81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -23006,6 +23252,9 @@
       <c r="CJ82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK82" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -23278,6 +23527,9 @@
       <c r="CJ83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -23550,6 +23802,9 @@
       <c r="CJ84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CK84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -23822,6 +24077,9 @@
       <c r="CJ85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CK85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -24094,6 +24352,9 @@
       <c r="CJ86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="CK86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -24366,6 +24627,9 @@
       <c r="CJ87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK87" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -24638,6 +24902,9 @@
       <c r="CJ88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -24910,6 +25177,9 @@
       <c r="CJ89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -25182,6 +25452,9 @@
       <c r="CJ90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CK90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -25454,6 +25727,9 @@
       <c r="CJ91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -25726,6 +26002,9 @@
       <c r="CJ92" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CK92" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -25998,6 +26277,9 @@
       <c r="CJ93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CK93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -26270,6 +26552,9 @@
       <c r="CJ94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CK94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -26542,6 +26827,9 @@
       <c r="CJ95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CK95" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -26814,6 +27102,9 @@
       <c r="CJ96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CK96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -27086,6 +27377,9 @@
       <c r="CJ97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CK97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -27358,6 +27652,9 @@
       <c r="CJ98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="CK98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -27630,6 +27927,9 @@
       <c r="CJ99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CK99" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -27902,6 +28202,9 @@
       <c r="CJ100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CK100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -28174,6 +28477,9 @@
       <c r="CJ101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CK101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -28446,6 +28752,9 @@
       <c r="CJ102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CK102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -28718,6 +29027,9 @@
       <c r="CJ103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CK103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -28990,6 +29302,9 @@
       <c r="CJ104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CK104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -29262,6 +29577,9 @@
       <c r="CJ105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CK105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -29534,6 +29852,9 @@
       <c r="CJ106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CK106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -29806,6 +30127,9 @@
       <c r="CJ107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CK107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -30078,6 +30402,9 @@
       <c r="CJ108" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CK108" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -30350,6 +30677,9 @@
       <c r="CJ109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CK109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -30622,6 +30952,9 @@
       <c r="CJ110" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CK110" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -30894,6 +31227,9 @@
       <c r="CJ111" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CK111" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -31166,6 +31502,9 @@
       <c r="CJ112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CK112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -31438,6 +31777,9 @@
       <c r="CJ113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CK113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -31710,6 +32052,9 @@
       <c r="CJ114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CK114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -31982,6 +32327,9 @@
       <c r="CJ115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CK115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -32254,6 +32602,9 @@
       <c r="CJ116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CK116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -32526,6 +32877,9 @@
       <c r="CJ117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CK117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -32798,6 +33152,9 @@
       <c r="CJ118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CK118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -33070,6 +33427,9 @@
       <c r="CJ119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CK119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -33342,6 +33702,9 @@
       <c r="CJ120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CK120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -33614,6 +33977,9 @@
       <c r="CJ121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CK121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -33886,6 +34252,9 @@
       <c r="CJ122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CK122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -34158,6 +34527,9 @@
       <c r="CJ123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CK123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -34430,6 +34802,9 @@
       <c r="CJ124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CK124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -34702,6 +35077,9 @@
       <c r="CJ125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CK125" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -34974,6 +35352,9 @@
       <c r="CJ126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CK126" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -35246,6 +35627,9 @@
       <c r="CJ127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CK127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -35518,6 +35902,9 @@
       <c r="CJ128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CK128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -35790,6 +36177,9 @@
       <c r="CJ129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CK129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -36062,6 +36452,9 @@
       <c r="CJ130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CK130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -36334,6 +36727,9 @@
       <c r="CJ131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CK131" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -36606,6 +37002,9 @@
       <c r="CJ132" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CK132" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -36878,6 +37277,9 @@
       <c r="CJ133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CK133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -37150,6 +37552,9 @@
       <c r="CJ134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="CK134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -37422,6 +37827,9 @@
       <c r="CJ135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CK135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -37694,6 +38102,9 @@
       <c r="CJ136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CK136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -37966,6 +38377,9 @@
       <c r="CJ137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CK137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -38238,6 +38652,9 @@
       <c r="CJ138" s="3" t="n">
         <v>23.29</v>
       </c>
+      <c r="CK138" s="3" t="n">
+        <v>23.29</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -38510,6 +38927,9 @@
       <c r="CJ139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CK139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -38782,6 +39202,9 @@
       <c r="CJ140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CK140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -39054,6 +39477,9 @@
       <c r="CJ141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CK141" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -39326,6 +39752,9 @@
       <c r="CJ142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CK142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -39598,6 +40027,9 @@
       <c r="CJ143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CK143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -39870,6 +40302,9 @@
       <c r="CJ144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CK144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -40142,6 +40577,9 @@
       <c r="CJ145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CK145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -40414,6 +40852,9 @@
       <c r="CJ146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CK146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -40686,6 +41127,9 @@
       <c r="CJ147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CK147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -40958,6 +41402,9 @@
       <c r="CJ148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CK148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -41230,6 +41677,9 @@
       <c r="CJ149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CK149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -41502,6 +41952,9 @@
       <c r="CJ150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CK150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -41774,6 +42227,9 @@
       <c r="CJ151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CK151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -42046,6 +42502,9 @@
       <c r="CJ152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CK152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -42318,6 +42777,9 @@
       <c r="CJ153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CK153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -42590,6 +43052,9 @@
       <c r="CJ154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CK154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -42862,6 +43327,9 @@
       <c r="CJ155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CK155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -43134,6 +43602,9 @@
       <c r="CJ156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CK156" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -43406,6 +43877,9 @@
       <c r="CJ157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CK157" s="3" t="n">
+        <v>22.8</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -43678,6 +44152,9 @@
       <c r="CJ158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CK158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -43950,6 +44427,9 @@
       <c r="CJ159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CK159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -44222,6 +44702,9 @@
       <c r="CJ160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CK160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -44494,6 +44977,9 @@
       <c r="CJ161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CK161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -44766,6 +45252,9 @@
       <c r="CJ162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CK162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -45038,6 +45527,9 @@
       <c r="CJ163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CK163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -45310,6 +45802,9 @@
       <c r="CJ164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CK164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -45483,9 +45978,12 @@
       <c r="CJ165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CK165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CJ165"/>
+  <autoFilter ref="A1:CK165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-15 15:10 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CK$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CL$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CK165"/>
+  <dimension ref="A1:CL165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -532,6 +532,7 @@
     <col width="16" customWidth="1" min="87" max="87"/>
     <col width="16" customWidth="1" min="88" max="88"/>
     <col width="16" customWidth="1" min="89" max="89"/>
+    <col width="16" customWidth="1" min="90" max="90"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -980,6 +981,11 @@
           <t>2026-09-15 07:12</t>
         </is>
       </c>
+      <c r="CL1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-15 10:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1255,6 +1261,9 @@
       <c r="CK2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CL2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1530,6 +1539,9 @@
       <c r="CK3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CL3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1805,6 +1817,9 @@
       <c r="CK4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CL4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2080,6 +2095,9 @@
       <c r="CK5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CL5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2355,6 +2373,9 @@
       <c r="CK6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CL6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2630,6 +2651,9 @@
       <c r="CK7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CL7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2905,6 +2929,9 @@
       <c r="CK8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="CL8" s="3" t="n">
+        <v>20.49</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3180,6 +3207,9 @@
       <c r="CK9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CL9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3455,6 +3485,9 @@
       <c r="CK10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CL10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3730,6 +3763,9 @@
       <c r="CK11" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL11" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4005,6 +4041,9 @@
       <c r="CK12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4280,6 +4319,9 @@
       <c r="CK13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CL13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4555,6 +4597,9 @@
       <c r="CK14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4830,6 +4875,9 @@
       <c r="CK15" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="CL15" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5105,6 +5153,9 @@
       <c r="CK16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CL16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5380,6 +5431,9 @@
       <c r="CK17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5655,6 +5709,9 @@
       <c r="CK18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CL18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5930,6 +5987,9 @@
       <c r="CK19" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="CL19" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -6205,6 +6265,9 @@
       <c r="CK20" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -6480,6 +6543,9 @@
       <c r="CK21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="CL21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -6755,6 +6821,9 @@
       <c r="CK22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CL22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -7030,6 +7099,9 @@
       <c r="CK23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CL23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -7305,6 +7377,9 @@
       <c r="CK24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CL24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -7580,6 +7655,9 @@
       <c r="CK25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -7855,6 +7933,9 @@
       <c r="CK26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="CL26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -8130,6 +8211,9 @@
       <c r="CK27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CL27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -8405,6 +8489,9 @@
       <c r="CK28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CL28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -8680,6 +8767,9 @@
       <c r="CK29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CL29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -8955,6 +9045,9 @@
       <c r="CK30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -9230,6 +9323,9 @@
       <c r="CK31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -9505,6 +9601,9 @@
       <c r="CK32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -9780,6 +9879,9 @@
       <c r="CK33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CL33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -10055,6 +10157,9 @@
       <c r="CK34" s="3" t="n">
         <v>21.33</v>
       </c>
+      <c r="CL34" s="3" t="n">
+        <v>21.33</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -10330,6 +10435,9 @@
       <c r="CK35" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CL35" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -10605,6 +10713,9 @@
       <c r="CK36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CL36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -10880,6 +10991,9 @@
       <c r="CK37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CL37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -11155,6 +11269,9 @@
       <c r="CK38" s="3" t="n">
         <v>21.46</v>
       </c>
+      <c r="CL38" s="3" t="n">
+        <v>21.46</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -11430,6 +11547,9 @@
       <c r="CK39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CL39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -11705,6 +11825,9 @@
       <c r="CK40" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -11980,6 +12103,9 @@
       <c r="CK41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CL41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -12255,6 +12381,9 @@
       <c r="CK42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CL42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -12530,6 +12659,9 @@
       <c r="CK43" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CL43" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -12805,6 +12937,9 @@
       <c r="CK44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CL44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -13080,6 +13215,9 @@
       <c r="CK45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="CL45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -13355,6 +13493,9 @@
       <c r="CK46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="CL46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -13630,6 +13771,9 @@
       <c r="CK47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CL47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -13905,6 +14049,9 @@
       <c r="CK48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CL48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -14180,6 +14327,9 @@
       <c r="CK49" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CL49" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -14455,6 +14605,9 @@
       <c r="CK50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CL50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -14730,6 +14883,9 @@
       <c r="CK51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CL51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -15005,6 +15161,9 @@
       <c r="CK52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CL52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -15280,6 +15439,9 @@
       <c r="CK53" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CL53" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -15555,6 +15717,9 @@
       <c r="CK54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CL54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -15830,6 +15995,9 @@
       <c r="CK55" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CL55" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -16105,6 +16273,9 @@
       <c r="CK56" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CL56" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -16380,6 +16551,9 @@
       <c r="CK57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -16655,6 +16829,9 @@
       <c r="CK58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CL58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -16930,6 +17107,9 @@
       <c r="CK59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CL59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -17205,6 +17385,9 @@
       <c r="CK60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CL60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -17480,6 +17663,9 @@
       <c r="CK61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CL61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -17755,6 +17941,9 @@
       <c r="CK62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CL62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -18030,6 +18219,9 @@
       <c r="CK63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CL63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -18305,6 +18497,9 @@
       <c r="CK64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CL64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -18580,6 +18775,9 @@
       <c r="CK65" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CL65" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -18855,6 +19053,9 @@
       <c r="CK66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL66" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -19130,6 +19331,9 @@
       <c r="CK67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CL67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -19405,6 +19609,9 @@
       <c r="CK68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -19680,6 +19887,9 @@
       <c r="CK69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CL69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -19955,6 +20165,9 @@
       <c r="CK70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CL70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -20230,6 +20443,9 @@
       <c r="CK71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL71" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -20505,6 +20721,9 @@
       <c r="CK72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -20780,6 +20999,9 @@
       <c r="CK73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CL73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -21055,6 +21277,9 @@
       <c r="CK74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CL74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -21330,6 +21555,9 @@
       <c r="CK75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL75" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -21605,6 +21833,9 @@
       <c r="CK76" s="3" t="n">
         <v>21.67</v>
       </c>
+      <c r="CL76" s="3" t="n">
+        <v>21.67</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -21880,6 +22111,9 @@
       <c r="CK77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -22155,6 +22389,9 @@
       <c r="CK78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CL78" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -22430,6 +22667,9 @@
       <c r="CK79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL79" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -22705,6 +22945,9 @@
       <c r="CK80" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CL80" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -22980,6 +23223,9 @@
       <c r="CK81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -23255,6 +23501,9 @@
       <c r="CK82" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -23530,6 +23779,9 @@
       <c r="CK83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -23805,6 +24057,9 @@
       <c r="CK84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CL84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -24080,6 +24335,9 @@
       <c r="CK85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CL85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -24355,6 +24613,9 @@
       <c r="CK86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="CL86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -24630,6 +24891,9 @@
       <c r="CK87" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -24905,6 +25169,9 @@
       <c r="CK88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -25180,6 +25447,9 @@
       <c r="CK89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -25455,6 +25725,9 @@
       <c r="CK90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CL90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -25730,6 +26003,9 @@
       <c r="CK91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL91" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -26005,6 +26281,9 @@
       <c r="CK92" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CL92" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -26280,6 +26559,9 @@
       <c r="CK93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CL93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -26555,6 +26837,9 @@
       <c r="CK94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CL94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -26830,6 +27115,9 @@
       <c r="CK95" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CL95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -27105,6 +27393,9 @@
       <c r="CK96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CL96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -27380,6 +27671,9 @@
       <c r="CK97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CL97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -27655,6 +27949,9 @@
       <c r="CK98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="CL98" s="3" t="n">
+        <v>20.95</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -27930,6 +28227,9 @@
       <c r="CK99" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CL99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -28205,6 +28505,9 @@
       <c r="CK100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CL100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -28480,6 +28783,9 @@
       <c r="CK101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CL101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -28755,6 +29061,9 @@
       <c r="CK102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CL102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -29030,6 +29339,9 @@
       <c r="CK103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CL103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -29305,6 +29617,9 @@
       <c r="CK104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CL104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -29580,6 +29895,9 @@
       <c r="CK105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CL105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -29855,6 +30173,9 @@
       <c r="CK106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CL106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -30130,6 +30451,9 @@
       <c r="CK107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CL107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -30405,6 +30729,9 @@
       <c r="CK108" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CL108" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -30680,6 +31007,9 @@
       <c r="CK109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CL109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -30955,6 +31285,9 @@
       <c r="CK110" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CL110" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -31230,6 +31563,9 @@
       <c r="CK111" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CL111" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -31505,6 +31841,9 @@
       <c r="CK112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CL112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -31780,6 +32119,9 @@
       <c r="CK113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CL113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -32055,6 +32397,9 @@
       <c r="CK114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CL114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -32330,6 +32675,9 @@
       <c r="CK115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CL115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -32605,6 +32953,9 @@
       <c r="CK116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CL116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -32880,6 +33231,9 @@
       <c r="CK117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CL117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -33155,6 +33509,9 @@
       <c r="CK118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CL118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -33430,6 +33787,9 @@
       <c r="CK119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CL119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -33705,6 +34065,9 @@
       <c r="CK120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CL120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -33980,6 +34343,9 @@
       <c r="CK121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CL121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -34255,6 +34621,9 @@
       <c r="CK122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CL122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -34530,6 +34899,9 @@
       <c r="CK123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CL123" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -34805,6 +35177,9 @@
       <c r="CK124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CL124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -35080,6 +35455,9 @@
       <c r="CK125" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CL125" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -35355,6 +35733,9 @@
       <c r="CK126" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CL126" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -35630,6 +36011,9 @@
       <c r="CK127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CL127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -35905,6 +36289,9 @@
       <c r="CK128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CL128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -36180,6 +36567,9 @@
       <c r="CK129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CL129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -36455,6 +36845,9 @@
       <c r="CK130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CL130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -36730,6 +37123,9 @@
       <c r="CK131" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CL131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -37005,6 +37401,9 @@
       <c r="CK132" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CL132" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -37280,6 +37679,9 @@
       <c r="CK133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CL133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -37555,6 +37957,9 @@
       <c r="CK134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="CL134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -37830,6 +38235,9 @@
       <c r="CK135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CL135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -38105,6 +38513,9 @@
       <c r="CK136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CL136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -38380,6 +38791,9 @@
       <c r="CK137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CL137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -38655,6 +39069,9 @@
       <c r="CK138" s="3" t="n">
         <v>23.29</v>
       </c>
+      <c r="CL138" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -38930,6 +39347,9 @@
       <c r="CK139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CL139" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -39205,6 +39625,9 @@
       <c r="CK140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CL140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -39480,6 +39903,9 @@
       <c r="CK141" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CL141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -39755,6 +40181,9 @@
       <c r="CK142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CL142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -40030,6 +40459,9 @@
       <c r="CK143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CL143" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -40305,6 +40737,9 @@
       <c r="CK144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CL144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -40580,6 +41015,9 @@
       <c r="CK145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CL145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -40855,6 +41293,9 @@
       <c r="CK146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CL146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -41130,6 +41571,9 @@
       <c r="CK147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CL147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -41405,6 +41849,9 @@
       <c r="CK148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CL148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -41680,6 +42127,9 @@
       <c r="CK149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CL149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -41955,6 +42405,9 @@
       <c r="CK150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CL150" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -42230,6 +42683,9 @@
       <c r="CK151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CL151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -42505,6 +42961,9 @@
       <c r="CK152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CL152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -42780,6 +43239,9 @@
       <c r="CK153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CL153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -43055,6 +43517,9 @@
       <c r="CK154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CL154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -43330,6 +43795,9 @@
       <c r="CK155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CL155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -43605,6 +44073,9 @@
       <c r="CK156" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CL156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -43880,6 +44351,9 @@
       <c r="CK157" s="3" t="n">
         <v>22.8</v>
       </c>
+      <c r="CL157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -44155,6 +44629,9 @@
       <c r="CK158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CL158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -44430,6 +44907,9 @@
       <c r="CK159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CL159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -44705,6 +45185,9 @@
       <c r="CK160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CL160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -44980,6 +45463,9 @@
       <c r="CK161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CL161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -45255,6 +45741,9 @@
       <c r="CK162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CL162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -45530,6 +46019,9 @@
       <c r="CK163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CL163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -45805,6 +46297,9 @@
       <c r="CK164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CL164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -45981,9 +46476,12 @@
       <c r="CK165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CL165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CK165"/>
+  <autoFilter ref="A1:CL165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-15 18:10 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CL$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CM$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CL165"/>
+  <dimension ref="A1:CM165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -533,6 +533,7 @@
     <col width="16" customWidth="1" min="88" max="88"/>
     <col width="16" customWidth="1" min="89" max="89"/>
     <col width="16" customWidth="1" min="90" max="90"/>
+    <col width="16" customWidth="1" min="91" max="91"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -986,6 +987,11 @@
           <t>2026-09-15 10:09</t>
         </is>
       </c>
+      <c r="CM1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-15 13:10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1264,6 +1270,9 @@
       <c r="CL2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CM2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1542,6 +1551,9 @@
       <c r="CL3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CM3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1820,6 +1832,9 @@
       <c r="CL4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CM4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2098,6 +2113,9 @@
       <c r="CL5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CM5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2376,6 +2394,9 @@
       <c r="CL6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CM6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2654,6 +2675,9 @@
       <c r="CL7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CM7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2932,6 +2956,9 @@
       <c r="CL8" s="3" t="n">
         <v>20.49</v>
       </c>
+      <c r="CM8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3210,6 +3237,9 @@
       <c r="CL9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CM9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3488,6 +3518,9 @@
       <c r="CL10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CM10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3766,6 +3799,9 @@
       <c r="CL11" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CM11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4044,6 +4080,9 @@
       <c r="CL12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CM12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4322,6 +4361,9 @@
       <c r="CL13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CM13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4600,6 +4642,9 @@
       <c r="CL14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CM14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4878,6 +4923,9 @@
       <c r="CL15" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="CM15" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5156,6 +5204,9 @@
       <c r="CL16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CM16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5434,6 +5485,9 @@
       <c r="CL17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CM17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5712,6 +5766,9 @@
       <c r="CL18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CM18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -5990,6 +6047,9 @@
       <c r="CL19" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="CM19" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -6268,6 +6328,9 @@
       <c r="CL20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CM20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -6546,6 +6609,9 @@
       <c r="CL21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="CM21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -6824,6 +6890,9 @@
       <c r="CL22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CM22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -7102,6 +7171,9 @@
       <c r="CL23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CM23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -7380,6 +7452,9 @@
       <c r="CL24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CM24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -7658,6 +7733,9 @@
       <c r="CL25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CM25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -7936,6 +8014,9 @@
       <c r="CL26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="CM26" s="3" t="n">
+        <v>20.8</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -8214,6 +8295,9 @@
       <c r="CL27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CM27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -8492,6 +8576,9 @@
       <c r="CL28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CM28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -8770,6 +8857,9 @@
       <c r="CL29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CM29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -9048,6 +9138,9 @@
       <c r="CL30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CM30" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -9326,6 +9419,9 @@
       <c r="CL31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CM31" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -9604,6 +9700,9 @@
       <c r="CL32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CM32" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -9882,6 +9981,9 @@
       <c r="CL33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CM33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -10160,6 +10262,9 @@
       <c r="CL34" s="3" t="n">
         <v>21.33</v>
       </c>
+      <c r="CM34" s="3" t="n">
+        <v>21.33</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -10438,6 +10543,9 @@
       <c r="CL35" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CM35" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -10716,6 +10824,9 @@
       <c r="CL36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CM36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -10994,6 +11105,9 @@
       <c r="CL37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CM37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -11272,6 +11386,9 @@
       <c r="CL38" s="3" t="n">
         <v>21.46</v>
       </c>
+      <c r="CM38" s="3" t="n">
+        <v>21.51</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -11550,6 +11667,9 @@
       <c r="CL39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CM39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -11828,6 +11948,9 @@
       <c r="CL40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CM40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -12106,6 +12229,9 @@
       <c r="CL41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CM41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -12384,6 +12510,9 @@
       <c r="CL42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CM42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -12662,6 +12791,9 @@
       <c r="CL43" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CM43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -12940,6 +13072,9 @@
       <c r="CL44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CM44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -13218,6 +13353,9 @@
       <c r="CL45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="CM45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -13496,6 +13634,9 @@
       <c r="CL46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="CM46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -13774,6 +13915,9 @@
       <c r="CL47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CM47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -14052,6 +14196,9 @@
       <c r="CL48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CM48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -14330,6 +14477,9 @@
       <c r="CL49" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CM49" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -14608,6 +14758,9 @@
       <c r="CL50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CM50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -14886,6 +15039,9 @@
       <c r="CL51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CM51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -15164,6 +15320,9 @@
       <c r="CL52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CM52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -15442,6 +15601,9 @@
       <c r="CL53" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CM53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -15720,6 +15882,9 @@
       <c r="CL54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CM54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -15998,6 +16163,9 @@
       <c r="CL55" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CM55" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -16276,6 +16444,9 @@
       <c r="CL56" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CM56" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -16554,6 +16725,9 @@
       <c r="CL57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CM57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -16832,6 +17006,9 @@
       <c r="CL58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CM58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -17110,6 +17287,9 @@
       <c r="CL59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CM59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -17388,6 +17568,9 @@
       <c r="CL60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CM60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -17666,6 +17849,9 @@
       <c r="CL61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CM61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -17944,6 +18130,9 @@
       <c r="CL62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CM62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -18222,6 +18411,9 @@
       <c r="CL63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CM63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -18500,6 +18692,9 @@
       <c r="CL64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CM64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -18778,6 +18973,9 @@
       <c r="CL65" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CM65" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -19056,6 +19254,9 @@
       <c r="CL66" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CM66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -19334,6 +19535,9 @@
       <c r="CL67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CM67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -19612,6 +19816,9 @@
       <c r="CL68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CM68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -19890,6 +20097,9 @@
       <c r="CL69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CM69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -20168,6 +20378,9 @@
       <c r="CL70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CM70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -20446,6 +20659,9 @@
       <c r="CL71" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CM71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -20724,6 +20940,9 @@
       <c r="CL72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CM72" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -21002,6 +21221,9 @@
       <c r="CL73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CM73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -21280,6 +21502,9 @@
       <c r="CL74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CM74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -21558,6 +21783,9 @@
       <c r="CL75" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CM75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -21836,6 +22064,9 @@
       <c r="CL76" s="3" t="n">
         <v>21.67</v>
       </c>
+      <c r="CM76" s="3" t="n">
+        <v>21.67</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -22114,6 +22345,9 @@
       <c r="CL77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CM77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -22392,6 +22626,9 @@
       <c r="CL78" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CM78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -22670,6 +22907,9 @@
       <c r="CL79" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CM79" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -22948,6 +23188,9 @@
       <c r="CL80" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CM80" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -23226,6 +23469,9 @@
       <c r="CL81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CM81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -23504,6 +23750,9 @@
       <c r="CL82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CM82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -23782,6 +24031,9 @@
       <c r="CL83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CM83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -24060,6 +24312,9 @@
       <c r="CL84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CM84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -24338,6 +24593,9 @@
       <c r="CL85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CM85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -24616,6 +24874,9 @@
       <c r="CL86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="CM86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -24894,6 +25155,9 @@
       <c r="CL87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CM87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -25172,6 +25436,9 @@
       <c r="CL88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CM88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -25450,6 +25717,9 @@
       <c r="CL89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CM89" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -25728,6 +25998,9 @@
       <c r="CL90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CM90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -26006,6 +26279,9 @@
       <c r="CL91" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CM91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -26284,6 +26560,9 @@
       <c r="CL92" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CM92" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -26562,6 +26841,9 @@
       <c r="CL93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CM93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -26840,6 +27122,9 @@
       <c r="CL94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CM94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -27118,6 +27403,9 @@
       <c r="CL95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="CM95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -27396,6 +27684,9 @@
       <c r="CL96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CM96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -27674,6 +27965,9 @@
       <c r="CL97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CM97" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -27952,6 +28246,9 @@
       <c r="CL98" s="3" t="n">
         <v>20.95</v>
       </c>
+      <c r="CM98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -28230,6 +28527,9 @@
       <c r="CL99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CM99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -28508,6 +28808,9 @@
       <c r="CL100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CM100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -28786,6 +29089,9 @@
       <c r="CL101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CM101" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -29064,6 +29370,9 @@
       <c r="CL102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CM102" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -29342,6 +29651,9 @@
       <c r="CL103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CM103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -29620,6 +29932,9 @@
       <c r="CL104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CM104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -29898,6 +30213,9 @@
       <c r="CL105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CM105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -30176,6 +30494,9 @@
       <c r="CL106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CM106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -30454,6 +30775,9 @@
       <c r="CL107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CM107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -30732,6 +31056,9 @@
       <c r="CL108" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CM108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -31010,6 +31337,9 @@
       <c r="CL109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CM109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -31288,6 +31618,9 @@
       <c r="CL110" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CM110" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -31566,6 +31899,9 @@
       <c r="CL111" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CM111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -31844,6 +32180,9 @@
       <c r="CL112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CM112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -32122,6 +32461,9 @@
       <c r="CL113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CM113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -32400,6 +32742,9 @@
       <c r="CL114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CM114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -32678,6 +33023,9 @@
       <c r="CL115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CM115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -32956,6 +33304,9 @@
       <c r="CL116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CM116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -33234,6 +33585,9 @@
       <c r="CL117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CM117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -33512,6 +33866,9 @@
       <c r="CL118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CM118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -33790,6 +34147,9 @@
       <c r="CL119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CM119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -34068,6 +34428,9 @@
       <c r="CL120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CM120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -34346,6 +34709,9 @@
       <c r="CL121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CM121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -34624,6 +34990,9 @@
       <c r="CL122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CM122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -34902,6 +35271,9 @@
       <c r="CL123" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="CM123" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -35180,6 +35552,9 @@
       <c r="CL124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CM124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -35458,6 +35833,9 @@
       <c r="CL125" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CM125" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -35736,6 +36114,9 @@
       <c r="CL126" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CM126" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -36014,6 +36395,9 @@
       <c r="CL127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CM127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -36292,6 +36676,9 @@
       <c r="CL128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CM128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -36570,6 +36957,9 @@
       <c r="CL129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CM129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -36848,6 +37238,9 @@
       <c r="CL130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CM130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -37126,6 +37519,9 @@
       <c r="CL131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="CM131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -37404,6 +37800,9 @@
       <c r="CL132" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CM132" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -37682,6 +38081,9 @@
       <c r="CL133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CM133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -37960,6 +38362,9 @@
       <c r="CL134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="CM134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -38238,6 +38643,9 @@
       <c r="CL135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CM135" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -38516,6 +38924,9 @@
       <c r="CL136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CM136" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -38794,6 +39205,9 @@
       <c r="CL137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CM137" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -39072,6 +39486,9 @@
       <c r="CL138" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CM138" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -39350,6 +39767,9 @@
       <c r="CL139" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CM139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -39628,6 +40048,9 @@
       <c r="CL140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CM140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -39906,6 +40329,9 @@
       <c r="CL141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CM141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -40184,6 +40610,9 @@
       <c r="CL142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CM142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -40462,6 +40891,9 @@
       <c r="CL143" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CM143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -40740,6 +41172,9 @@
       <c r="CL144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CM144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -41018,6 +41453,9 @@
       <c r="CL145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CM145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -41296,6 +41734,9 @@
       <c r="CL146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CM146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -41574,6 +42015,9 @@
       <c r="CL147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CM147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -41852,6 +42296,9 @@
       <c r="CL148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CM148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -42130,6 +42577,9 @@
       <c r="CL149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CM149" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -42408,6 +42858,9 @@
       <c r="CL150" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CM150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -42686,6 +43139,9 @@
       <c r="CL151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CM151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -42964,6 +43420,9 @@
       <c r="CL152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CM152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -43242,6 +43701,9 @@
       <c r="CL153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CM153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -43520,6 +43982,9 @@
       <c r="CL154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CM154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -43798,6 +44263,9 @@
       <c r="CL155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CM155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -44076,6 +44544,9 @@
       <c r="CL156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CM156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -44354,6 +44825,9 @@
       <c r="CL157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CM157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -44632,6 +45106,9 @@
       <c r="CL158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CM158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -44910,6 +45387,9 @@
       <c r="CL159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CM159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -45188,6 +45668,9 @@
       <c r="CL160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CM160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -45466,6 +45949,9 @@
       <c r="CL161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CM161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -45744,6 +46230,9 @@
       <c r="CL162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CM162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -46022,6 +46511,9 @@
       <c r="CL163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CM163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -46300,6 +46792,9 @@
       <c r="CL164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CM164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -46479,9 +46974,12 @@
       <c r="CL165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CM165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CL165"/>
+  <autoFilter ref="A1:CM165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-15 21:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CM$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CN$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CM165"/>
+  <dimension ref="A1:CN165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -534,6 +534,7 @@
     <col width="16" customWidth="1" min="89" max="89"/>
     <col width="16" customWidth="1" min="90" max="90"/>
     <col width="16" customWidth="1" min="91" max="91"/>
+    <col width="16" customWidth="1" min="92" max="92"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -992,6 +993,11 @@
           <t>2026-09-15 13:10</t>
         </is>
       </c>
+      <c r="CN1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-15 16:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1273,6 +1279,9 @@
       <c r="CM2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CN2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1554,6 +1563,9 @@
       <c r="CM3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CN3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1835,6 +1847,9 @@
       <c r="CM4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CN4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2116,6 +2131,9 @@
       <c r="CM5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CN5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2397,6 +2415,9 @@
       <c r="CM6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CN6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2678,6 +2699,9 @@
       <c r="CM7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CN7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2959,6 +2983,9 @@
       <c r="CM8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CN8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3240,6 +3267,9 @@
       <c r="CM9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CN9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3521,6 +3551,9 @@
       <c r="CM10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CN10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3802,6 +3835,9 @@
       <c r="CM11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CN11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4083,6 +4119,9 @@
       <c r="CM12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CN12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4364,6 +4403,9 @@
       <c r="CM13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CN13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4645,6 +4687,9 @@
       <c r="CM14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CN14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4926,6 +4971,9 @@
       <c r="CM15" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="CN15" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5207,6 +5255,9 @@
       <c r="CM16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CN16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5488,6 +5539,9 @@
       <c r="CM17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CN17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5769,6 +5823,9 @@
       <c r="CM18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CN18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -6050,6 +6107,9 @@
       <c r="CM19" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="CN19" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -6331,6 +6391,9 @@
       <c r="CM20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CN20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -6612,6 +6675,9 @@
       <c r="CM21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="CN21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -6893,6 +6959,9 @@
       <c r="CM22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CN22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -7174,6 +7243,9 @@
       <c r="CM23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CN23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -7455,6 +7527,9 @@
       <c r="CM24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CN24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -7736,6 +7811,9 @@
       <c r="CM25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CN25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -8017,6 +8095,9 @@
       <c r="CM26" s="3" t="n">
         <v>20.8</v>
       </c>
+      <c r="CN26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -8298,6 +8379,9 @@
       <c r="CM27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CN27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -8579,6 +8663,9 @@
       <c r="CM28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CN28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -8860,6 +8947,9 @@
       <c r="CM29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CN29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -9141,6 +9231,9 @@
       <c r="CM30" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CN30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -9422,6 +9515,9 @@
       <c r="CM31" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CN31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -9703,6 +9799,9 @@
       <c r="CM32" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CN32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -9984,6 +10083,9 @@
       <c r="CM33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CN33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -10265,6 +10367,9 @@
       <c r="CM34" s="3" t="n">
         <v>21.33</v>
       </c>
+      <c r="CN34" s="3" t="n">
+        <v>21.33</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -10546,6 +10651,9 @@
       <c r="CM35" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CN35" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -10827,6 +10935,9 @@
       <c r="CM36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CN36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -11108,6 +11219,9 @@
       <c r="CM37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CN37" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -11389,6 +11503,9 @@
       <c r="CM38" s="3" t="n">
         <v>21.51</v>
       </c>
+      <c r="CN38" s="3" t="n">
+        <v>21.51</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -11670,6 +11787,9 @@
       <c r="CM39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CN39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -11951,6 +12071,9 @@
       <c r="CM40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CN40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -12232,6 +12355,9 @@
       <c r="CM41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CN41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -12513,6 +12639,9 @@
       <c r="CM42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CN42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -12794,6 +12923,9 @@
       <c r="CM43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CN43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -13075,6 +13207,9 @@
       <c r="CM44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CN44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -13356,6 +13491,9 @@
       <c r="CM45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="CN45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -13637,6 +13775,9 @@
       <c r="CM46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="CN46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -13918,6 +14059,9 @@
       <c r="CM47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CN47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -14199,6 +14343,9 @@
       <c r="CM48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CN48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -14480,6 +14627,9 @@
       <c r="CM49" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CN49" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -14761,6 +14911,9 @@
       <c r="CM50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CN50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -15042,6 +15195,9 @@
       <c r="CM51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CN51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -15323,6 +15479,9 @@
       <c r="CM52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CN52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -15604,6 +15763,9 @@
       <c r="CM53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="CN53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -15885,6 +16047,9 @@
       <c r="CM54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CN54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -16166,6 +16331,9 @@
       <c r="CM55" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CN55" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -16447,6 +16615,9 @@
       <c r="CM56" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CN56" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -16728,6 +16899,9 @@
       <c r="CM57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CN57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -17009,6 +17183,9 @@
       <c r="CM58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CN58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -17290,6 +17467,9 @@
       <c r="CM59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CN59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -17571,6 +17751,9 @@
       <c r="CM60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CN60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -17852,6 +18035,9 @@
       <c r="CM61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CN61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -18133,6 +18319,9 @@
       <c r="CM62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CN62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -18414,6 +18603,9 @@
       <c r="CM63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CN63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -18695,6 +18887,9 @@
       <c r="CM64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CN64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -18976,6 +19171,9 @@
       <c r="CM65" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CN65" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -19257,6 +19455,9 @@
       <c r="CM66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CN66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -19538,6 +19739,9 @@
       <c r="CM67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CN67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -19819,6 +20023,9 @@
       <c r="CM68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CN68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -20100,6 +20307,9 @@
       <c r="CM69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CN69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -20381,6 +20591,9 @@
       <c r="CM70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CN70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -20662,6 +20875,9 @@
       <c r="CM71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CN71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -20943,6 +21159,9 @@
       <c r="CM72" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CN72" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -21224,6 +21443,9 @@
       <c r="CM73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CN73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -21505,6 +21727,9 @@
       <c r="CM74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CN74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -21786,6 +22011,9 @@
       <c r="CM75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CN75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -22067,6 +22295,9 @@
       <c r="CM76" s="3" t="n">
         <v>21.67</v>
       </c>
+      <c r="CN76" s="3" t="n">
+        <v>21.67</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -22348,6 +22579,9 @@
       <c r="CM77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CN77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -22629,6 +22863,9 @@
       <c r="CM78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CN78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -22910,6 +23147,9 @@
       <c r="CM79" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CN79" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -23191,6 +23431,9 @@
       <c r="CM80" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CN80" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -23472,6 +23715,9 @@
       <c r="CM81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CN81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -23753,6 +23999,9 @@
       <c r="CM82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CN82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -24034,6 +24283,9 @@
       <c r="CM83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CN83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -24315,6 +24567,9 @@
       <c r="CM84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CN84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -24596,6 +24851,9 @@
       <c r="CM85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CN85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -24877,6 +25135,9 @@
       <c r="CM86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="CN86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -25158,6 +25419,9 @@
       <c r="CM87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CN87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -25439,6 +25703,9 @@
       <c r="CM88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CN88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -25720,6 +25987,9 @@
       <c r="CM89" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CN89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -26001,6 +26271,9 @@
       <c r="CM90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CN90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -26282,6 +26555,9 @@
       <c r="CM91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CN91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -26563,6 +26839,9 @@
       <c r="CM92" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CN92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -26844,6 +27123,9 @@
       <c r="CM93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CN93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -27125,6 +27407,9 @@
       <c r="CM94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CN94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -27406,6 +27691,9 @@
       <c r="CM95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="CN95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -27687,6 +27975,9 @@
       <c r="CM96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CN96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -27968,6 +28259,9 @@
       <c r="CM97" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CN97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -28249,6 +28543,9 @@
       <c r="CM98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CN98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -28530,6 +28827,9 @@
       <c r="CM99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CN99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -28811,6 +29111,9 @@
       <c r="CM100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CN100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -29092,6 +29395,9 @@
       <c r="CM101" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CN101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -29373,6 +29679,9 @@
       <c r="CM102" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CN102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -29654,6 +29963,9 @@
       <c r="CM103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CN103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -29935,6 +30247,9 @@
       <c r="CM104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CN104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -30216,6 +30531,9 @@
       <c r="CM105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CN105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -30497,6 +30815,9 @@
       <c r="CM106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CN106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -30778,6 +31099,9 @@
       <c r="CM107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CN107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -31059,6 +31383,9 @@
       <c r="CM108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CN108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -31340,6 +31667,9 @@
       <c r="CM109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CN109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -31621,6 +31951,9 @@
       <c r="CM110" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CN110" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -31902,6 +32235,9 @@
       <c r="CM111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="CN111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -32183,6 +32519,9 @@
       <c r="CM112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CN112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -32464,6 +32803,9 @@
       <c r="CM113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CN113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -32745,6 +33087,9 @@
       <c r="CM114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CN114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -33026,6 +33371,9 @@
       <c r="CM115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CN115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -33307,6 +33655,9 @@
       <c r="CM116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CN116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -33588,6 +33939,9 @@
       <c r="CM117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CN117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -33869,6 +34223,9 @@
       <c r="CM118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CN118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -34150,6 +34507,9 @@
       <c r="CM119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CN119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -34431,6 +34791,9 @@
       <c r="CM120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CN120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -34712,6 +35075,9 @@
       <c r="CM121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CN121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -34993,6 +35359,9 @@
       <c r="CM122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CN122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -35274,6 +35643,9 @@
       <c r="CM123" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="CN123" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -35555,6 +35927,9 @@
       <c r="CM124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CN124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -35836,6 +36211,9 @@
       <c r="CM125" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CN125" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -36117,6 +36495,9 @@
       <c r="CM126" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CN126" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -36398,6 +36779,9 @@
       <c r="CM127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CN127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -36679,6 +37063,9 @@
       <c r="CM128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CN128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -36960,6 +37347,9 @@
       <c r="CM129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CN129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -37241,6 +37631,9 @@
       <c r="CM130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CN130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -37522,6 +37915,9 @@
       <c r="CM131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="CN131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -37803,6 +38199,9 @@
       <c r="CM132" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CN132" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -38084,6 +38483,9 @@
       <c r="CM133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CN133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -38365,6 +38767,9 @@
       <c r="CM134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="CN134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -38646,6 +39051,9 @@
       <c r="CM135" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CN135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -38927,6 +39335,9 @@
       <c r="CM136" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CN136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -39208,6 +39619,9 @@
       <c r="CM137" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CN137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -39489,6 +39903,9 @@
       <c r="CM138" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CN138" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -39770,6 +40187,9 @@
       <c r="CM139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CN139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -40051,6 +40471,9 @@
       <c r="CM140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CN140" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -40332,6 +40755,9 @@
       <c r="CM141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CN141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -40613,6 +41039,9 @@
       <c r="CM142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CN142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -40894,6 +41323,9 @@
       <c r="CM143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CN143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -41175,6 +41607,9 @@
       <c r="CM144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CN144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -41456,6 +41891,9 @@
       <c r="CM145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CN145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -41737,6 +42175,9 @@
       <c r="CM146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CN146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -42018,6 +42459,9 @@
       <c r="CM147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CN147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -42299,6 +42743,9 @@
       <c r="CM148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CN148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -42580,6 +43027,9 @@
       <c r="CM149" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CN149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -42861,6 +43311,9 @@
       <c r="CM150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CN150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -43142,6 +43595,9 @@
       <c r="CM151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CN151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -43423,6 +43879,9 @@
       <c r="CM152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CN152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -43704,6 +44163,9 @@
       <c r="CM153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CN153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -43985,6 +44447,9 @@
       <c r="CM154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CN154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -44266,6 +44731,9 @@
       <c r="CM155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CN155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -44547,6 +45015,9 @@
       <c r="CM156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CN156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -44828,6 +45299,9 @@
       <c r="CM157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CN157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -45109,6 +45583,9 @@
       <c r="CM158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CN158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -45390,6 +45867,9 @@
       <c r="CM159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CN159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -45671,6 +46151,9 @@
       <c r="CM160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CN160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -45952,6 +46435,9 @@
       <c r="CM161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CN161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -46233,6 +46719,9 @@
       <c r="CM162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CN162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -46514,6 +47003,9 @@
       <c r="CM163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CN163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -46795,6 +47287,9 @@
       <c r="CM164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CN164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -46977,9 +47472,12 @@
       <c r="CM165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CN165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CM165"/>
+  <autoFilter ref="A1:CN165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-16 00:12 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CN$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CO$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CN165"/>
+  <dimension ref="A1:CO165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -535,6 +535,7 @@
     <col width="16" customWidth="1" min="90" max="90"/>
     <col width="16" customWidth="1" min="91" max="91"/>
     <col width="16" customWidth="1" min="92" max="92"/>
+    <col width="16" customWidth="1" min="93" max="93"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -998,6 +999,11 @@
           <t>2026-09-15 16:09</t>
         </is>
       </c>
+      <c r="CO1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-15 19:12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1282,6 +1288,9 @@
       <c r="CN2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CO2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1566,6 +1575,9 @@
       <c r="CN3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CO3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1850,6 +1862,9 @@
       <c r="CN4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CO4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2134,6 +2149,9 @@
       <c r="CN5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CO5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2418,6 +2436,9 @@
       <c r="CN6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CO6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2702,6 +2723,9 @@
       <c r="CN7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CO7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2986,6 +3010,9 @@
       <c r="CN8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CO8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3270,6 +3297,9 @@
       <c r="CN9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CO9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3554,6 +3584,9 @@
       <c r="CN10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CO10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3838,6 +3871,9 @@
       <c r="CN11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CO11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4122,6 +4158,9 @@
       <c r="CN12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CO12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4406,6 +4445,9 @@
       <c r="CN13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CO13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4690,6 +4732,9 @@
       <c r="CN14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CO14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -4974,6 +5019,9 @@
       <c r="CN15" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="CO15" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5258,6 +5306,9 @@
       <c r="CN16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CO16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5542,6 +5593,9 @@
       <c r="CN17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CO17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5826,6 +5880,9 @@
       <c r="CN18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CO18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -6110,6 +6167,9 @@
       <c r="CN19" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="CO19" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -6394,6 +6454,9 @@
       <c r="CN20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CO20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -6678,6 +6741,9 @@
       <c r="CN21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="CO21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -6962,6 +7028,9 @@
       <c r="CN22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CO22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -7246,6 +7315,9 @@
       <c r="CN23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CO23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -7530,6 +7602,9 @@
       <c r="CN24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CO24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -7814,6 +7889,9 @@
       <c r="CN25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CO25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -8098,6 +8176,9 @@
       <c r="CN26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CO26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -8382,6 +8463,9 @@
       <c r="CN27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CO27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -8666,6 +8750,9 @@
       <c r="CN28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CO28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -8950,6 +9037,9 @@
       <c r="CN29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CO29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -9234,6 +9324,9 @@
       <c r="CN30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CO30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -9518,6 +9611,9 @@
       <c r="CN31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CO31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -9802,6 +9898,9 @@
       <c r="CN32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CO32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -10086,6 +10185,9 @@
       <c r="CN33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CO33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -10370,6 +10472,9 @@
       <c r="CN34" s="3" t="n">
         <v>21.33</v>
       </c>
+      <c r="CO34" s="3" t="n">
+        <v>21.33</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -10654,6 +10759,9 @@
       <c r="CN35" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CO35" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -10938,6 +11046,9 @@
       <c r="CN36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CO36" s="3" t="n">
+        <v>20.68</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -11222,6 +11333,9 @@
       <c r="CN37" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CO37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -11506,6 +11620,9 @@
       <c r="CN38" s="3" t="n">
         <v>21.51</v>
       </c>
+      <c r="CO38" s="3" t="n">
+        <v>21.51</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -11790,6 +11907,9 @@
       <c r="CN39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CO39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -12074,6 +12194,9 @@
       <c r="CN40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CO40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -12358,6 +12481,9 @@
       <c r="CN41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CO41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -12642,6 +12768,9 @@
       <c r="CN42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CO42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -12926,6 +13055,9 @@
       <c r="CN43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CO43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -13210,6 +13342,9 @@
       <c r="CN44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CO44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -13494,6 +13629,9 @@
       <c r="CN45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="CO45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -13778,6 +13916,9 @@
       <c r="CN46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="CO46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -14062,6 +14203,9 @@
       <c r="CN47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CO47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -14346,6 +14490,9 @@
       <c r="CN48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CO48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -14630,6 +14777,9 @@
       <c r="CN49" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CO49" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -14914,6 +15064,9 @@
       <c r="CN50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CO50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -15198,6 +15351,9 @@
       <c r="CN51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CO51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -15482,6 +15638,9 @@
       <c r="CN52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CO52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -15766,6 +15925,9 @@
       <c r="CN53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="CO53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -16050,6 +16212,9 @@
       <c r="CN54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CO54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -16334,6 +16499,9 @@
       <c r="CN55" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CO55" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -16618,6 +16786,9 @@
       <c r="CN56" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CO56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -16902,6 +17073,9 @@
       <c r="CN57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CO57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -17186,6 +17360,9 @@
       <c r="CN58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CO58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -17470,6 +17647,9 @@
       <c r="CN59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CO59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -17754,6 +17934,9 @@
       <c r="CN60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CO60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -18038,6 +18221,9 @@
       <c r="CN61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CO61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -18322,6 +18508,9 @@
       <c r="CN62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CO62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -18606,6 +18795,9 @@
       <c r="CN63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CO63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -18890,6 +19082,9 @@
       <c r="CN64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CO64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -19174,6 +19369,9 @@
       <c r="CN65" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CO65" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -19458,6 +19656,9 @@
       <c r="CN66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CO66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -19742,6 +19943,9 @@
       <c r="CN67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CO67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -20026,6 +20230,9 @@
       <c r="CN68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CO68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -20310,6 +20517,9 @@
       <c r="CN69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CO69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -20594,6 +20804,9 @@
       <c r="CN70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CO70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -20878,6 +21091,9 @@
       <c r="CN71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CO71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -21162,6 +21378,9 @@
       <c r="CN72" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CO72" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -21446,6 +21665,9 @@
       <c r="CN73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CO73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -21730,6 +21952,9 @@
       <c r="CN74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CO74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -22014,6 +22239,9 @@
       <c r="CN75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CO75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -22298,6 +22526,9 @@
       <c r="CN76" s="3" t="n">
         <v>21.67</v>
       </c>
+      <c r="CO76" s="3" t="n">
+        <v>21.67</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -22582,6 +22813,9 @@
       <c r="CN77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CO77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -22866,6 +23100,9 @@
       <c r="CN78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CO78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -23150,6 +23387,9 @@
       <c r="CN79" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CO79" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -23434,6 +23674,9 @@
       <c r="CN80" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CO80" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -23718,6 +23961,9 @@
       <c r="CN81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CO81" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -24002,6 +24248,9 @@
       <c r="CN82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CO82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -24286,6 +24535,9 @@
       <c r="CN83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CO83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -24570,6 +24822,9 @@
       <c r="CN84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CO84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -24854,6 +25109,9 @@
       <c r="CN85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CO85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -25138,6 +25396,9 @@
       <c r="CN86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="CO86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -25422,6 +25683,9 @@
       <c r="CN87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CO87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -25706,6 +25970,9 @@
       <c r="CN88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CO88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -25990,6 +26257,9 @@
       <c r="CN89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CO89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -26274,6 +26544,9 @@
       <c r="CN90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CO90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -26558,6 +26831,9 @@
       <c r="CN91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CO91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -26842,6 +27118,9 @@
       <c r="CN92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CO92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -27126,6 +27405,9 @@
       <c r="CN93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CO93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -27410,6 +27692,9 @@
       <c r="CN94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CO94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -27694,6 +27979,9 @@
       <c r="CN95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="CO95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -27978,6 +28266,9 @@
       <c r="CN96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CO96" s="3" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -28262,6 +28553,9 @@
       <c r="CN97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CO97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -28546,6 +28840,9 @@
       <c r="CN98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CO98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -28830,6 +29127,9 @@
       <c r="CN99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CO99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -29114,6 +29414,9 @@
       <c r="CN100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CO100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -29398,6 +29701,9 @@
       <c r="CN101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CO101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -29682,6 +29988,9 @@
       <c r="CN102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="CO102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -29966,6 +30275,9 @@
       <c r="CN103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CO103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -30250,6 +30562,9 @@
       <c r="CN104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CO104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -30534,6 +30849,9 @@
       <c r="CN105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CO105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -30818,6 +31136,9 @@
       <c r="CN106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CO106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -31102,6 +31423,9 @@
       <c r="CN107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CO107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -31386,6 +31710,9 @@
       <c r="CN108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CO108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -31670,6 +31997,9 @@
       <c r="CN109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CO109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -31954,6 +32284,9 @@
       <c r="CN110" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CO110" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -32238,6 +32571,9 @@
       <c r="CN111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="CO111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -32522,6 +32858,9 @@
       <c r="CN112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CO112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -32806,6 +33145,9 @@
       <c r="CN113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CO113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -33090,6 +33432,9 @@
       <c r="CN114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CO114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -33374,6 +33719,9 @@
       <c r="CN115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CO115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -33658,6 +34006,9 @@
       <c r="CN116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CO116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -33942,6 +34293,9 @@
       <c r="CN117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CO117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -34226,6 +34580,9 @@
       <c r="CN118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CO118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -34510,6 +34867,9 @@
       <c r="CN119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CO119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -34794,6 +35154,9 @@
       <c r="CN120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CO120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -35078,6 +35441,9 @@
       <c r="CN121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CO121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -35362,6 +35728,9 @@
       <c r="CN122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CO122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -35646,6 +36015,9 @@
       <c r="CN123" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="CO123" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -35930,6 +36302,9 @@
       <c r="CN124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CO124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -36214,6 +36589,9 @@
       <c r="CN125" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CO125" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -36498,6 +36876,9 @@
       <c r="CN126" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CO126" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -36782,6 +37163,9 @@
       <c r="CN127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CO127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -37066,6 +37450,9 @@
       <c r="CN128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CO128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -37350,6 +37737,9 @@
       <c r="CN129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CO129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -37634,6 +38024,9 @@
       <c r="CN130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CO130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -37918,6 +38311,9 @@
       <c r="CN131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="CO131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -38202,6 +38598,9 @@
       <c r="CN132" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CO132" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -38486,6 +38885,9 @@
       <c r="CN133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CO133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -38770,6 +39172,9 @@
       <c r="CN134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="CO134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -39054,6 +39459,9 @@
       <c r="CN135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CO135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -39338,6 +39746,9 @@
       <c r="CN136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CO136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -39622,6 +40033,9 @@
       <c r="CN137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CO137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -39906,6 +40320,9 @@
       <c r="CN138" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CO138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -40190,6 +40607,9 @@
       <c r="CN139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CO139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -40474,6 +40894,9 @@
       <c r="CN140" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CO140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -40758,6 +41181,9 @@
       <c r="CN141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CO141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -41042,6 +41468,9 @@
       <c r="CN142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CO142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -41326,6 +41755,9 @@
       <c r="CN143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CO143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -41610,6 +42042,9 @@
       <c r="CN144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CO144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -41894,6 +42329,9 @@
       <c r="CN145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CO145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -42178,6 +42616,9 @@
       <c r="CN146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CO146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -42462,6 +42903,9 @@
       <c r="CN147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CO147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -42746,6 +43190,9 @@
       <c r="CN148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CO148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -43030,6 +43477,9 @@
       <c r="CN149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CO149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -43314,6 +43764,9 @@
       <c r="CN150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CO150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -43598,6 +44051,9 @@
       <c r="CN151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CO151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -43882,6 +44338,9 @@
       <c r="CN152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CO152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -44166,6 +44625,9 @@
       <c r="CN153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CO153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -44450,6 +44912,9 @@
       <c r="CN154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CO154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -44734,6 +45199,9 @@
       <c r="CN155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CO155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -45018,6 +45486,9 @@
       <c r="CN156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CO156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -45302,6 +45773,9 @@
       <c r="CN157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CO157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -45586,6 +46060,9 @@
       <c r="CN158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CO158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -45870,6 +46347,9 @@
       <c r="CN159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CO159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -46154,6 +46634,9 @@
       <c r="CN160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CO160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -46438,6 +46921,9 @@
       <c r="CN161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CO161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -46722,6 +47208,9 @@
       <c r="CN162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CO162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -47006,6 +47495,9 @@
       <c r="CN163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CO163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -47290,6 +47782,9 @@
       <c r="CN164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CO164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -47475,9 +47970,12 @@
       <c r="CN165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CO165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CN165"/>
+  <autoFilter ref="A1:CO165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-16 03:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CO$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CP$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CO165"/>
+  <dimension ref="A1:CP165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -536,6 +536,7 @@
     <col width="16" customWidth="1" min="91" max="91"/>
     <col width="16" customWidth="1" min="92" max="92"/>
     <col width="16" customWidth="1" min="93" max="93"/>
+    <col width="16" customWidth="1" min="94" max="94"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1004,6 +1005,11 @@
           <t>2026-09-15 19:12</t>
         </is>
       </c>
+      <c r="CP1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-15 22:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1291,6 +1297,9 @@
       <c r="CO2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CP2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1578,6 +1587,9 @@
       <c r="CO3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CP3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1865,6 +1877,9 @@
       <c r="CO4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CP4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2152,6 +2167,9 @@
       <c r="CO5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CP5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2439,6 +2457,9 @@
       <c r="CO6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CP6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2726,6 +2747,9 @@
       <c r="CO7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CP7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3013,6 +3037,9 @@
       <c r="CO8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CP8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3300,6 +3327,9 @@
       <c r="CO9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CP9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3587,6 +3617,9 @@
       <c r="CO10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CP10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3874,6 +3907,9 @@
       <c r="CO11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CP11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4161,6 +4197,9 @@
       <c r="CO12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CP12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4448,6 +4487,9 @@
       <c r="CO13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CP13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4735,6 +4777,9 @@
       <c r="CO14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CP14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5022,6 +5067,9 @@
       <c r="CO15" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="CP15" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5309,6 +5357,9 @@
       <c r="CO16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CP16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5596,6 +5647,9 @@
       <c r="CO17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CP17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5883,6 +5937,9 @@
       <c r="CO18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CP18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -6170,6 +6227,9 @@
       <c r="CO19" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="CP19" s="3" t="n">
+        <v>20.85</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -6457,6 +6517,9 @@
       <c r="CO20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CP20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -6744,6 +6807,9 @@
       <c r="CO21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="CP21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -7031,6 +7097,9 @@
       <c r="CO22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CP22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -7318,6 +7387,9 @@
       <c r="CO23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CP23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -7605,6 +7677,9 @@
       <c r="CO24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CP24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -7892,6 +7967,9 @@
       <c r="CO25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CP25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -8179,6 +8257,9 @@
       <c r="CO26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CP26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -8466,6 +8547,9 @@
       <c r="CO27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CP27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -8753,6 +8837,9 @@
       <c r="CO28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CP28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -9040,6 +9127,9 @@
       <c r="CO29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CP29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -9327,6 +9417,9 @@
       <c r="CO30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CP30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -9614,6 +9707,9 @@
       <c r="CO31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CP31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -9901,6 +9997,9 @@
       <c r="CO32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CP32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -10188,6 +10287,9 @@
       <c r="CO33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CP33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -10475,6 +10577,9 @@
       <c r="CO34" s="3" t="n">
         <v>21.33</v>
       </c>
+      <c r="CP34" s="3" t="n">
+        <v>21.33</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -10762,6 +10867,9 @@
       <c r="CO35" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CP35" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -11049,6 +11157,9 @@
       <c r="CO36" s="3" t="n">
         <v>20.68</v>
       </c>
+      <c r="CP36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -11336,6 +11447,9 @@
       <c r="CO37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CP37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -11623,6 +11737,9 @@
       <c r="CO38" s="3" t="n">
         <v>21.51</v>
       </c>
+      <c r="CP38" s="3" t="n">
+        <v>21.51</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -11910,6 +12027,9 @@
       <c r="CO39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CP39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -12197,6 +12317,9 @@
       <c r="CO40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CP40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -12484,6 +12607,9 @@
       <c r="CO41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CP41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -12771,6 +12897,9 @@
       <c r="CO42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CP42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -13058,6 +13187,9 @@
       <c r="CO43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CP43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -13345,6 +13477,9 @@
       <c r="CO44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CP44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -13632,6 +13767,9 @@
       <c r="CO45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="CP45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -13919,6 +14057,9 @@
       <c r="CO46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="CP46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -14206,6 +14347,9 @@
       <c r="CO47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CP47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -14493,6 +14637,9 @@
       <c r="CO48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CP48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -14780,6 +14927,9 @@
       <c r="CO49" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CP49" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -15067,6 +15217,9 @@
       <c r="CO50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CP50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -15354,6 +15507,9 @@
       <c r="CO51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CP51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -15641,6 +15797,9 @@
       <c r="CO52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CP52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -15928,6 +16087,9 @@
       <c r="CO53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="CP53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -16215,6 +16377,9 @@
       <c r="CO54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CP54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -16502,6 +16667,9 @@
       <c r="CO55" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CP55" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -16789,6 +16957,9 @@
       <c r="CO56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CP56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -17076,6 +17247,9 @@
       <c r="CO57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CP57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -17363,6 +17537,9 @@
       <c r="CO58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CP58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -17650,6 +17827,9 @@
       <c r="CO59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CP59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -17937,6 +18117,9 @@
       <c r="CO60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CP60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -18224,6 +18407,9 @@
       <c r="CO61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CP61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -18511,6 +18697,9 @@
       <c r="CO62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CP62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -18798,6 +18987,9 @@
       <c r="CO63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CP63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -19085,6 +19277,9 @@
       <c r="CO64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CP64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -19372,6 +19567,9 @@
       <c r="CO65" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CP65" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -19659,6 +19857,9 @@
       <c r="CO66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CP66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -19946,6 +20147,9 @@
       <c r="CO67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CP67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -20233,6 +20437,9 @@
       <c r="CO68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CP68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -20520,6 +20727,9 @@
       <c r="CO69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CP69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -20807,6 +21017,9 @@
       <c r="CO70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CP70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -21094,6 +21307,9 @@
       <c r="CO71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CP71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -21381,6 +21597,9 @@
       <c r="CO72" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CP72" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -21668,6 +21887,9 @@
       <c r="CO73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CP73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -21955,6 +22177,9 @@
       <c r="CO74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CP74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -22242,6 +22467,9 @@
       <c r="CO75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CP75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -22529,6 +22757,9 @@
       <c r="CO76" s="3" t="n">
         <v>21.67</v>
       </c>
+      <c r="CP76" s="3" t="n">
+        <v>21.67</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -22816,6 +23047,9 @@
       <c r="CO77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CP77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -23103,6 +23337,9 @@
       <c r="CO78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CP78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -23390,6 +23627,9 @@
       <c r="CO79" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CP79" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -23677,6 +23917,9 @@
       <c r="CO80" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CP80" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -23964,6 +24207,9 @@
       <c r="CO81" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CP81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -24251,6 +24497,9 @@
       <c r="CO82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CP82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -24538,6 +24787,9 @@
       <c r="CO83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CP83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -24825,6 +25077,9 @@
       <c r="CO84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CP84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -25112,6 +25367,9 @@
       <c r="CO85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CP85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -25399,6 +25657,9 @@
       <c r="CO86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="CP86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -25686,6 +25947,9 @@
       <c r="CO87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CP87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -25973,6 +26237,9 @@
       <c r="CO88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CP88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -26260,6 +26527,9 @@
       <c r="CO89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CP89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -26547,6 +26817,9 @@
       <c r="CO90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CP90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -26834,6 +27107,9 @@
       <c r="CO91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CP91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -27121,6 +27397,9 @@
       <c r="CO92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CP92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -27408,6 +27687,9 @@
       <c r="CO93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CP93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -27695,6 +27977,9 @@
       <c r="CO94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CP94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -27982,6 +28267,9 @@
       <c r="CO95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="CP95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -28269,6 +28557,9 @@
       <c r="CO96" s="3" t="n">
         <v>21</v>
       </c>
+      <c r="CP96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -28556,6 +28847,9 @@
       <c r="CO97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CP97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -28843,6 +29137,9 @@
       <c r="CO98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CP98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -29130,6 +29427,9 @@
       <c r="CO99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CP99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -29417,6 +29717,9 @@
       <c r="CO100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CP100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -29704,6 +30007,9 @@
       <c r="CO101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CP101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -29991,6 +30297,9 @@
       <c r="CO102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="CP102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -30278,6 +30587,9 @@
       <c r="CO103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CP103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -30565,6 +30877,9 @@
       <c r="CO104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CP104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -30852,6 +31167,9 @@
       <c r="CO105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CP105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -31139,6 +31457,9 @@
       <c r="CO106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CP106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -31426,6 +31747,9 @@
       <c r="CO107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CP107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -31713,6 +32037,9 @@
       <c r="CO108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CP108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -32000,6 +32327,9 @@
       <c r="CO109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CP109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -32287,6 +32617,9 @@
       <c r="CO110" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CP110" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -32574,6 +32907,9 @@
       <c r="CO111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="CP111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -32861,6 +33197,9 @@
       <c r="CO112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CP112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -33148,6 +33487,9 @@
       <c r="CO113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CP113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -33435,6 +33777,9 @@
       <c r="CO114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CP114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -33722,6 +34067,9 @@
       <c r="CO115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CP115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -34009,6 +34357,9 @@
       <c r="CO116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CP116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -34296,6 +34647,9 @@
       <c r="CO117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CP117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -34583,6 +34937,9 @@
       <c r="CO118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CP118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -34870,6 +35227,9 @@
       <c r="CO119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CP119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -35157,6 +35517,9 @@
       <c r="CO120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CP120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -35444,6 +35807,9 @@
       <c r="CO121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CP121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -35731,6 +36097,9 @@
       <c r="CO122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CP122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -36018,6 +36387,9 @@
       <c r="CO123" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="CP123" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -36305,6 +36677,9 @@
       <c r="CO124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CP124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -36592,6 +36967,9 @@
       <c r="CO125" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CP125" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -36879,6 +37257,9 @@
       <c r="CO126" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CP126" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -37166,6 +37547,9 @@
       <c r="CO127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CP127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -37453,6 +37837,9 @@
       <c r="CO128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CP128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -37740,6 +38127,9 @@
       <c r="CO129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CP129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -38027,6 +38417,9 @@
       <c r="CO130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CP130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -38314,6 +38707,9 @@
       <c r="CO131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="CP131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -38601,6 +38997,9 @@
       <c r="CO132" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CP132" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -38888,6 +39287,9 @@
       <c r="CO133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CP133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -39175,6 +39577,9 @@
       <c r="CO134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="CP134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -39462,6 +39867,9 @@
       <c r="CO135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CP135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -39749,6 +40157,9 @@
       <c r="CO136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CP136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -40036,6 +40447,9 @@
       <c r="CO137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CP137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -40323,6 +40737,9 @@
       <c r="CO138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="CP138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -40610,6 +41027,9 @@
       <c r="CO139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CP139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -40897,6 +41317,9 @@
       <c r="CO140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CP140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -41184,6 +41607,9 @@
       <c r="CO141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CP141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -41471,6 +41897,9 @@
       <c r="CO142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CP142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -41758,6 +42187,9 @@
       <c r="CO143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CP143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -42045,6 +42477,9 @@
       <c r="CO144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CP144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -42332,6 +42767,9 @@
       <c r="CO145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CP145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -42619,6 +43057,9 @@
       <c r="CO146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CP146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -42906,6 +43347,9 @@
       <c r="CO147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CP147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -43193,6 +43637,9 @@
       <c r="CO148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CP148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -43480,6 +43927,9 @@
       <c r="CO149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CP149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -43767,6 +44217,9 @@
       <c r="CO150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CP150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -44054,6 +44507,9 @@
       <c r="CO151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CP151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -44341,6 +44797,9 @@
       <c r="CO152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CP152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -44628,6 +45087,9 @@
       <c r="CO153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CP153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -44915,6 +45377,9 @@
       <c r="CO154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CP154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -45202,6 +45667,9 @@
       <c r="CO155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CP155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -45489,6 +45957,9 @@
       <c r="CO156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CP156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -45776,6 +46247,9 @@
       <c r="CO157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CP157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -46063,6 +46537,9 @@
       <c r="CO158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CP158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -46350,6 +46827,9 @@
       <c r="CO159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CP159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -46637,6 +47117,9 @@
       <c r="CO160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CP160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -46924,6 +47407,9 @@
       <c r="CO161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CP161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -47211,6 +47697,9 @@
       <c r="CO162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CP162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -47498,6 +47987,9 @@
       <c r="CO163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CP163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -47785,6 +48277,9 @@
       <c r="CO164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CP164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -47973,9 +48468,12 @@
       <c r="CO165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CP165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CO165"/>
+  <autoFilter ref="A1:CP165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-16 06:12 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CP$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CQ$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CP165"/>
+  <dimension ref="A1:CQ165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -537,6 +537,7 @@
     <col width="16" customWidth="1" min="92" max="92"/>
     <col width="16" customWidth="1" min="93" max="93"/>
     <col width="16" customWidth="1" min="94" max="94"/>
+    <col width="16" customWidth="1" min="95" max="95"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1010,6 +1011,11 @@
           <t>2026-09-15 22:09</t>
         </is>
       </c>
+      <c r="CQ1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-16 01:12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1300,6 +1306,9 @@
       <c r="CP2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CQ2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1590,6 +1599,9 @@
       <c r="CP3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CQ3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1880,6 +1892,9 @@
       <c r="CP4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CQ4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2170,6 +2185,9 @@
       <c r="CP5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CQ5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2460,6 +2478,9 @@
       <c r="CP6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CQ6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2750,6 +2771,9 @@
       <c r="CP7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CQ7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3040,6 +3064,9 @@
       <c r="CP8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CQ8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3330,6 +3357,9 @@
       <c r="CP9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CQ9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3620,6 +3650,9 @@
       <c r="CP10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CQ10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3910,6 +3943,9 @@
       <c r="CP11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CQ11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4200,6 +4236,9 @@
       <c r="CP12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CQ12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4490,6 +4529,9 @@
       <c r="CP13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CQ13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4780,6 +4822,9 @@
       <c r="CP14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CQ14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5070,6 +5115,9 @@
       <c r="CP15" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="CQ15" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5360,6 +5408,9 @@
       <c r="CP16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CQ16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5650,6 +5701,9 @@
       <c r="CP17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CQ17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5940,6 +5994,9 @@
       <c r="CP18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CQ18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -6230,6 +6287,9 @@
       <c r="CP19" s="3" t="n">
         <v>20.85</v>
       </c>
+      <c r="CQ19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -6520,6 +6580,9 @@
       <c r="CP20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CQ20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -6810,6 +6873,9 @@
       <c r="CP21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="CQ21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -7100,6 +7166,9 @@
       <c r="CP22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CQ22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -7390,6 +7459,9 @@
       <c r="CP23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CQ23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -7680,6 +7752,9 @@
       <c r="CP24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CQ24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -7970,6 +8045,9 @@
       <c r="CP25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CQ25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -8260,6 +8338,9 @@
       <c r="CP26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CQ26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -8550,6 +8631,9 @@
       <c r="CP27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CQ27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -8840,6 +8924,9 @@
       <c r="CP28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CQ28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -9130,6 +9217,9 @@
       <c r="CP29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CQ29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -9420,6 +9510,9 @@
       <c r="CP30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CQ30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -9710,6 +9803,9 @@
       <c r="CP31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CQ31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -10000,6 +10096,9 @@
       <c r="CP32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CQ32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -10290,6 +10389,9 @@
       <c r="CP33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CQ33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -10580,6 +10682,9 @@
       <c r="CP34" s="3" t="n">
         <v>21.33</v>
       </c>
+      <c r="CQ34" s="3" t="n">
+        <v>21.33</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -10870,6 +10975,9 @@
       <c r="CP35" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CQ35" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -11160,6 +11268,9 @@
       <c r="CP36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CQ36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -11450,6 +11561,9 @@
       <c r="CP37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CQ37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -11740,6 +11854,9 @@
       <c r="CP38" s="3" t="n">
         <v>21.51</v>
       </c>
+      <c r="CQ38" s="3" t="n">
+        <v>21.51</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -12030,6 +12147,9 @@
       <c r="CP39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CQ39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -12320,6 +12440,9 @@
       <c r="CP40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CQ40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -12610,6 +12733,9 @@
       <c r="CP41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CQ41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -12900,6 +13026,9 @@
       <c r="CP42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CQ42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -13190,6 +13319,9 @@
       <c r="CP43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CQ43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -13480,6 +13612,9 @@
       <c r="CP44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CQ44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -13770,6 +13905,9 @@
       <c r="CP45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="CQ45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -14060,6 +14198,9 @@
       <c r="CP46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="CQ46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -14350,6 +14491,9 @@
       <c r="CP47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CQ47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -14640,6 +14784,9 @@
       <c r="CP48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CQ48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -14930,6 +15077,9 @@
       <c r="CP49" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CQ49" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -15220,6 +15370,9 @@
       <c r="CP50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CQ50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -15510,6 +15663,9 @@
       <c r="CP51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CQ51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -15800,6 +15956,9 @@
       <c r="CP52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CQ52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -16090,6 +16249,9 @@
       <c r="CP53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="CQ53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -16380,6 +16542,9 @@
       <c r="CP54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CQ54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -16670,6 +16835,9 @@
       <c r="CP55" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CQ55" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -16960,6 +17128,9 @@
       <c r="CP56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CQ56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -17250,6 +17421,9 @@
       <c r="CP57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CQ57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -17540,6 +17714,9 @@
       <c r="CP58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CQ58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -17830,6 +18007,9 @@
       <c r="CP59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CQ59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -18120,6 +18300,9 @@
       <c r="CP60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CQ60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -18410,6 +18593,9 @@
       <c r="CP61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CQ61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -18700,6 +18886,9 @@
       <c r="CP62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CQ62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -18990,6 +19179,9 @@
       <c r="CP63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CQ63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -19280,6 +19472,9 @@
       <c r="CP64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CQ64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -19570,6 +19765,9 @@
       <c r="CP65" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CQ65" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -19860,6 +20058,9 @@
       <c r="CP66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CQ66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -20150,6 +20351,9 @@
       <c r="CP67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CQ67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -20440,6 +20644,9 @@
       <c r="CP68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CQ68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -20730,6 +20937,9 @@
       <c r="CP69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CQ69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -21020,6 +21230,9 @@
       <c r="CP70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CQ70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -21310,6 +21523,9 @@
       <c r="CP71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CQ71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -21600,6 +21816,9 @@
       <c r="CP72" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CQ72" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -21890,6 +22109,9 @@
       <c r="CP73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CQ73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -22180,6 +22402,9 @@
       <c r="CP74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CQ74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -22470,6 +22695,9 @@
       <c r="CP75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CQ75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -22760,6 +22988,9 @@
       <c r="CP76" s="3" t="n">
         <v>21.67</v>
       </c>
+      <c r="CQ76" s="3" t="n">
+        <v>21.67</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -23050,6 +23281,9 @@
       <c r="CP77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CQ77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -23340,6 +23574,9 @@
       <c r="CP78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CQ78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -23630,6 +23867,9 @@
       <c r="CP79" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CQ79" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -23920,6 +24160,9 @@
       <c r="CP80" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CQ80" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -24210,6 +24453,9 @@
       <c r="CP81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CQ81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -24500,6 +24746,9 @@
       <c r="CP82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CQ82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -24790,6 +25039,9 @@
       <c r="CP83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CQ83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -25080,6 +25332,9 @@
       <c r="CP84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CQ84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -25370,6 +25625,9 @@
       <c r="CP85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CQ85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -25660,6 +25918,9 @@
       <c r="CP86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="CQ86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -25950,6 +26211,9 @@
       <c r="CP87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CQ87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -26240,6 +26504,9 @@
       <c r="CP88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CQ88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -26530,6 +26797,9 @@
       <c r="CP89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CQ89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -26820,6 +27090,9 @@
       <c r="CP90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CQ90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -27110,6 +27383,9 @@
       <c r="CP91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CQ91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -27400,6 +27676,9 @@
       <c r="CP92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CQ92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -27690,6 +27969,9 @@
       <c r="CP93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CQ93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -27980,6 +28262,9 @@
       <c r="CP94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CQ94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -28270,6 +28555,9 @@
       <c r="CP95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="CQ95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -28560,6 +28848,9 @@
       <c r="CP96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="CQ96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -28850,6 +29141,9 @@
       <c r="CP97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CQ97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -29140,6 +29434,9 @@
       <c r="CP98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CQ98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -29430,6 +29727,9 @@
       <c r="CP99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CQ99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -29720,6 +30020,9 @@
       <c r="CP100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CQ100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -30010,6 +30313,9 @@
       <c r="CP101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CQ101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -30300,6 +30606,9 @@
       <c r="CP102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="CQ102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -30590,6 +30899,9 @@
       <c r="CP103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CQ103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -30880,6 +31192,9 @@
       <c r="CP104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CQ104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -31170,6 +31485,9 @@
       <c r="CP105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CQ105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -31460,6 +31778,9 @@
       <c r="CP106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CQ106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -31750,6 +32071,9 @@
       <c r="CP107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CQ107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -32040,6 +32364,9 @@
       <c r="CP108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CQ108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -32330,6 +32657,9 @@
       <c r="CP109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CQ109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -32620,6 +32950,9 @@
       <c r="CP110" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CQ110" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -32910,6 +33243,9 @@
       <c r="CP111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="CQ111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -33200,6 +33536,9 @@
       <c r="CP112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CQ112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -33490,6 +33829,9 @@
       <c r="CP113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CQ113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -33780,6 +34122,9 @@
       <c r="CP114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CQ114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -34070,6 +34415,9 @@
       <c r="CP115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CQ115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -34360,6 +34708,9 @@
       <c r="CP116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CQ116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -34650,6 +35001,9 @@
       <c r="CP117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CQ117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -34940,6 +35294,9 @@
       <c r="CP118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CQ118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -35230,6 +35587,9 @@
       <c r="CP119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CQ119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -35520,6 +35880,9 @@
       <c r="CP120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CQ120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -35810,6 +36173,9 @@
       <c r="CP121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CQ121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -36100,6 +36466,9 @@
       <c r="CP122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CQ122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -36390,6 +36759,9 @@
       <c r="CP123" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="CQ123" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -36680,6 +37052,9 @@
       <c r="CP124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CQ124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -36970,6 +37345,9 @@
       <c r="CP125" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CQ125" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -37260,6 +37638,9 @@
       <c r="CP126" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CQ126" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -37550,6 +37931,9 @@
       <c r="CP127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CQ127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -37840,6 +38224,9 @@
       <c r="CP128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CQ128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -38130,6 +38517,9 @@
       <c r="CP129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CQ129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -38420,6 +38810,9 @@
       <c r="CP130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CQ130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -38710,6 +39103,9 @@
       <c r="CP131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="CQ131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -39000,6 +39396,9 @@
       <c r="CP132" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CQ132" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -39290,6 +39689,9 @@
       <c r="CP133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CQ133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -39580,6 +39982,9 @@
       <c r="CP134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="CQ134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -39870,6 +40275,9 @@
       <c r="CP135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CQ135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -40160,6 +40568,9 @@
       <c r="CP136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CQ136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -40450,6 +40861,9 @@
       <c r="CP137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CQ137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -40740,6 +41154,9 @@
       <c r="CP138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="CQ138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -41030,6 +41447,9 @@
       <c r="CP139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CQ139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -41320,6 +41740,9 @@
       <c r="CP140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CQ140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -41610,6 +42033,9 @@
       <c r="CP141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CQ141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -41900,6 +42326,9 @@
       <c r="CP142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CQ142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -42190,6 +42619,9 @@
       <c r="CP143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CQ143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -42480,6 +42912,9 @@
       <c r="CP144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CQ144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -42770,6 +43205,9 @@
       <c r="CP145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CQ145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -43060,6 +43498,9 @@
       <c r="CP146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CQ146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -43350,6 +43791,9 @@
       <c r="CP147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CQ147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -43640,6 +44084,9 @@
       <c r="CP148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CQ148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -43930,6 +44377,9 @@
       <c r="CP149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CQ149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -44220,6 +44670,9 @@
       <c r="CP150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CQ150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -44510,6 +44963,9 @@
       <c r="CP151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CQ151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -44800,6 +45256,9 @@
       <c r="CP152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CQ152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -45090,6 +45549,9 @@
       <c r="CP153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CQ153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -45380,6 +45842,9 @@
       <c r="CP154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CQ154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -45670,6 +46135,9 @@
       <c r="CP155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CQ155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -45960,6 +46428,9 @@
       <c r="CP156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CQ156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -46250,6 +46721,9 @@
       <c r="CP157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CQ157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -46540,6 +47014,9 @@
       <c r="CP158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CQ158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -46830,6 +47307,9 @@
       <c r="CP159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CQ159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -47120,6 +47600,9 @@
       <c r="CP160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CQ160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -47410,6 +47893,9 @@
       <c r="CP161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CQ161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -47700,6 +48186,9 @@
       <c r="CP162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CQ162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -47990,6 +48479,9 @@
       <c r="CP163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CQ163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -48280,6 +48772,9 @@
       <c r="CP164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CQ164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -48471,9 +48966,12 @@
       <c r="CP165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CQ165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CP165"/>
+  <autoFilter ref="A1:CQ165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-16 09:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CQ$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CR$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ165"/>
+  <dimension ref="A1:CR165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -538,6 +538,7 @@
     <col width="16" customWidth="1" min="93" max="93"/>
     <col width="16" customWidth="1" min="94" max="94"/>
     <col width="16" customWidth="1" min="95" max="95"/>
+    <col width="16" customWidth="1" min="96" max="96"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1016,6 +1017,11 @@
           <t>2026-09-16 01:12</t>
         </is>
       </c>
+      <c r="CR1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-16 04:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1309,6 +1315,9 @@
       <c r="CQ2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CR2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1602,6 +1611,9 @@
       <c r="CQ3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CR3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1895,6 +1907,9 @@
       <c r="CQ4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CR4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2188,6 +2203,9 @@
       <c r="CQ5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CR5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2481,6 +2499,9 @@
       <c r="CQ6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CR6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2774,6 +2795,9 @@
       <c r="CQ7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CR7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3067,6 +3091,9 @@
       <c r="CQ8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CR8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3360,6 +3387,9 @@
       <c r="CQ9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CR9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3653,6 +3683,9 @@
       <c r="CQ10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CR10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3946,6 +3979,9 @@
       <c r="CQ11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CR11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4239,6 +4275,9 @@
       <c r="CQ12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CR12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4532,6 +4571,9 @@
       <c r="CQ13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CR13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4825,6 +4867,9 @@
       <c r="CQ14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CR14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5118,6 +5163,9 @@
       <c r="CQ15" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="CR15" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5411,6 +5459,9 @@
       <c r="CQ16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CR16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5704,6 +5755,9 @@
       <c r="CQ17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CR17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -5997,6 +6051,9 @@
       <c r="CQ18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CR18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -6290,6 +6347,9 @@
       <c r="CQ19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="CR19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -6583,6 +6643,9 @@
       <c r="CQ20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CR20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -6876,6 +6939,9 @@
       <c r="CQ21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="CR21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -7169,6 +7235,9 @@
       <c r="CQ22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CR22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -7462,6 +7531,9 @@
       <c r="CQ23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CR23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -7755,6 +7827,9 @@
       <c r="CQ24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CR24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -8048,6 +8123,9 @@
       <c r="CQ25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CR25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -8341,6 +8419,9 @@
       <c r="CQ26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CR26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -8634,6 +8715,9 @@
       <c r="CQ27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CR27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -8927,6 +9011,9 @@
       <c r="CQ28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CR28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -9220,6 +9307,9 @@
       <c r="CQ29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CR29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -9513,6 +9603,9 @@
       <c r="CQ30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CR30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -9806,6 +9899,9 @@
       <c r="CQ31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CR31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -10099,6 +10195,9 @@
       <c r="CQ32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CR32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -10392,6 +10491,9 @@
       <c r="CQ33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CR33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -10685,6 +10787,9 @@
       <c r="CQ34" s="3" t="n">
         <v>21.33</v>
       </c>
+      <c r="CR34" s="3" t="n">
+        <v>21.33</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -10978,6 +11083,9 @@
       <c r="CQ35" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CR35" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -11271,6 +11379,9 @@
       <c r="CQ36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CR36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -11564,6 +11675,9 @@
       <c r="CQ37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CR37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -11857,6 +11971,9 @@
       <c r="CQ38" s="3" t="n">
         <v>21.51</v>
       </c>
+      <c r="CR38" s="3" t="n">
+        <v>21.51</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -12150,6 +12267,9 @@
       <c r="CQ39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CR39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -12443,6 +12563,9 @@
       <c r="CQ40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CR40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -12736,6 +12859,9 @@
       <c r="CQ41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CR41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -13029,6 +13155,9 @@
       <c r="CQ42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CR42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -13322,6 +13451,9 @@
       <c r="CQ43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CR43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -13615,6 +13747,9 @@
       <c r="CQ44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CR44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -13908,6 +14043,9 @@
       <c r="CQ45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="CR45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -14201,6 +14339,9 @@
       <c r="CQ46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="CR46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -14494,6 +14635,9 @@
       <c r="CQ47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CR47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -14787,6 +14931,9 @@
       <c r="CQ48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CR48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -15080,6 +15227,9 @@
       <c r="CQ49" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CR49" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -15373,6 +15523,9 @@
       <c r="CQ50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CR50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -15666,6 +15819,9 @@
       <c r="CQ51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CR51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -15959,6 +16115,9 @@
       <c r="CQ52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CR52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -16252,6 +16411,9 @@
       <c r="CQ53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="CR53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -16545,6 +16707,9 @@
       <c r="CQ54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CR54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -16838,6 +17003,9 @@
       <c r="CQ55" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CR55" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -17131,6 +17299,9 @@
       <c r="CQ56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CR56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -17424,6 +17595,9 @@
       <c r="CQ57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CR57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -17717,6 +17891,9 @@
       <c r="CQ58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CR58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -18010,6 +18187,9 @@
       <c r="CQ59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CR59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -18303,6 +18483,9 @@
       <c r="CQ60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CR60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -18596,6 +18779,9 @@
       <c r="CQ61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CR61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -18889,6 +19075,9 @@
       <c r="CQ62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CR62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -19182,6 +19371,9 @@
       <c r="CQ63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CR63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -19475,6 +19667,9 @@
       <c r="CQ64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CR64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -19768,6 +19963,9 @@
       <c r="CQ65" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CR65" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -20061,6 +20259,9 @@
       <c r="CQ66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CR66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -20354,6 +20555,9 @@
       <c r="CQ67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CR67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -20647,6 +20851,9 @@
       <c r="CQ68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CR68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -20940,6 +21147,9 @@
       <c r="CQ69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CR69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -21233,6 +21443,9 @@
       <c r="CQ70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CR70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -21526,6 +21739,9 @@
       <c r="CQ71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CR71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -21819,6 +22035,9 @@
       <c r="CQ72" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CR72" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -22112,6 +22331,9 @@
       <c r="CQ73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CR73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -22405,6 +22627,9 @@
       <c r="CQ74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CR74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -22698,6 +22923,9 @@
       <c r="CQ75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CR75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -22991,6 +23219,9 @@
       <c r="CQ76" s="3" t="n">
         <v>21.67</v>
       </c>
+      <c r="CR76" s="3" t="n">
+        <v>21.67</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -23284,6 +23515,9 @@
       <c r="CQ77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CR77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -23577,6 +23811,9 @@
       <c r="CQ78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CR78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -23870,6 +24107,9 @@
       <c r="CQ79" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CR79" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -24163,6 +24403,9 @@
       <c r="CQ80" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CR80" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -24456,6 +24699,9 @@
       <c r="CQ81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CR81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -24749,6 +24995,9 @@
       <c r="CQ82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CR82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -25042,6 +25291,9 @@
       <c r="CQ83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CR83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -25335,6 +25587,9 @@
       <c r="CQ84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CR84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -25628,6 +25883,9 @@
       <c r="CQ85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CR85" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -25921,6 +26179,9 @@
       <c r="CQ86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="CR86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -26214,6 +26475,9 @@
       <c r="CQ87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CR87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -26507,6 +26771,9 @@
       <c r="CQ88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CR88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -26800,6 +27067,9 @@
       <c r="CQ89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CR89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -27093,6 +27363,9 @@
       <c r="CQ90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CR90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -27386,6 +27659,9 @@
       <c r="CQ91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CR91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -27679,6 +27955,9 @@
       <c r="CQ92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CR92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -27972,6 +28251,9 @@
       <c r="CQ93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CR93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -28265,6 +28547,9 @@
       <c r="CQ94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CR94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -28558,6 +28843,9 @@
       <c r="CQ95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="CR95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -28851,6 +29139,9 @@
       <c r="CQ96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="CR96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -29144,6 +29435,9 @@
       <c r="CQ97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CR97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -29437,6 +29731,9 @@
       <c r="CQ98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CR98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -29730,6 +30027,9 @@
       <c r="CQ99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CR99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -30023,6 +30323,9 @@
       <c r="CQ100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CR100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -30316,6 +30619,9 @@
       <c r="CQ101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CR101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -30609,6 +30915,9 @@
       <c r="CQ102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="CR102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -30902,6 +31211,9 @@
       <c r="CQ103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CR103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -31195,6 +31507,9 @@
       <c r="CQ104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CR104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -31488,6 +31803,9 @@
       <c r="CQ105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CR105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -31781,6 +32099,9 @@
       <c r="CQ106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CR106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -32074,6 +32395,9 @@
       <c r="CQ107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CR107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -32367,6 +32691,9 @@
       <c r="CQ108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CR108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -32660,6 +32987,9 @@
       <c r="CQ109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CR109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -32953,6 +33283,9 @@
       <c r="CQ110" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CR110" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -33246,6 +33579,9 @@
       <c r="CQ111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="CR111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -33539,6 +33875,9 @@
       <c r="CQ112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CR112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -33832,6 +34171,9 @@
       <c r="CQ113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CR113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -34125,6 +34467,9 @@
       <c r="CQ114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CR114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -34418,6 +34763,9 @@
       <c r="CQ115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CR115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -34711,6 +35059,9 @@
       <c r="CQ116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CR116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -35004,6 +35355,9 @@
       <c r="CQ117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CR117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -35297,6 +35651,9 @@
       <c r="CQ118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CR118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -35590,6 +35947,9 @@
       <c r="CQ119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CR119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -35883,6 +36243,9 @@
       <c r="CQ120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CR120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -36176,6 +36539,9 @@
       <c r="CQ121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CR121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -36469,6 +36835,9 @@
       <c r="CQ122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CR122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -36762,6 +37131,9 @@
       <c r="CQ123" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="CR123" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -37055,6 +37427,9 @@
       <c r="CQ124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CR124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -37348,6 +37723,9 @@
       <c r="CQ125" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CR125" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -37641,6 +38019,9 @@
       <c r="CQ126" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CR126" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -37934,6 +38315,9 @@
       <c r="CQ127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CR127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -38227,6 +38611,9 @@
       <c r="CQ128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CR128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -38520,6 +38907,9 @@
       <c r="CQ129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CR129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -38813,6 +39203,9 @@
       <c r="CQ130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CR130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -39106,6 +39499,9 @@
       <c r="CQ131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="CR131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -39399,6 +39795,9 @@
       <c r="CQ132" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CR132" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -39692,6 +40091,9 @@
       <c r="CQ133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CR133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -39985,6 +40387,9 @@
       <c r="CQ134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="CR134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -40278,6 +40683,9 @@
       <c r="CQ135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CR135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -40571,6 +40979,9 @@
       <c r="CQ136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CR136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -40864,6 +41275,9 @@
       <c r="CQ137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CR137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -41157,6 +41571,9 @@
       <c r="CQ138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="CR138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -41450,6 +41867,9 @@
       <c r="CQ139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CR139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -41743,6 +42163,9 @@
       <c r="CQ140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CR140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -42036,6 +42459,9 @@
       <c r="CQ141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CR141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -42329,6 +42755,9 @@
       <c r="CQ142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CR142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -42622,6 +43051,9 @@
       <c r="CQ143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CR143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -42915,6 +43347,9 @@
       <c r="CQ144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CR144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -43208,6 +43643,9 @@
       <c r="CQ145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CR145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -43501,6 +43939,9 @@
       <c r="CQ146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CR146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -43794,6 +44235,9 @@
       <c r="CQ147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CR147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -44087,6 +44531,9 @@
       <c r="CQ148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CR148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -44380,6 +44827,9 @@
       <c r="CQ149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CR149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -44673,6 +45123,9 @@
       <c r="CQ150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CR150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -44966,6 +45419,9 @@
       <c r="CQ151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CR151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -45259,6 +45715,9 @@
       <c r="CQ152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CR152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -45552,6 +46011,9 @@
       <c r="CQ153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CR153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -45845,6 +46307,9 @@
       <c r="CQ154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CR154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -46138,6 +46603,9 @@
       <c r="CQ155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CR155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -46431,6 +46899,9 @@
       <c r="CQ156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CR156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -46724,6 +47195,9 @@
       <c r="CQ157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CR157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -47017,6 +47491,9 @@
       <c r="CQ158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CR158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -47310,6 +47787,9 @@
       <c r="CQ159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CR159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -47603,6 +48083,9 @@
       <c r="CQ160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CR160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -47896,6 +48379,9 @@
       <c r="CQ161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CR161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -48189,6 +48675,9 @@
       <c r="CQ162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CR162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -48482,6 +48971,9 @@
       <c r="CQ163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CR163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -48775,6 +49267,9 @@
       <c r="CQ164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CR164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -48969,9 +49464,12 @@
       <c r="CQ165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CR165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CQ165"/>
+  <autoFilter ref="A1:CR165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-16 12:12 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CR$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CS$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CR165"/>
+  <dimension ref="A1:CS165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -539,6 +539,7 @@
     <col width="16" customWidth="1" min="94" max="94"/>
     <col width="16" customWidth="1" min="95" max="95"/>
     <col width="16" customWidth="1" min="96" max="96"/>
+    <col width="16" customWidth="1" min="97" max="97"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1022,6 +1023,11 @@
           <t>2026-09-16 04:09</t>
         </is>
       </c>
+      <c r="CS1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1318,6 +1324,9 @@
       <c r="CR2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CS2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1614,6 +1623,9 @@
       <c r="CR3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CS3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1910,6 +1922,9 @@
       <c r="CR4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CS4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2206,6 +2221,9 @@
       <c r="CR5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CS5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2502,6 +2520,9 @@
       <c r="CR6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CS6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2798,6 +2819,9 @@
       <c r="CR7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CS7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3094,6 +3118,9 @@
       <c r="CR8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CS8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3390,6 +3417,9 @@
       <c r="CR9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CS9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3686,6 +3716,9 @@
       <c r="CR10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CS10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3982,6 +4015,9 @@
       <c r="CR11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CS11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4278,6 +4314,9 @@
       <c r="CR12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CS12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4574,6 +4613,9 @@
       <c r="CR13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CS13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4870,6 +4912,9 @@
       <c r="CR14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CS14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5166,6 +5211,9 @@
       <c r="CR15" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="CS15" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5462,6 +5510,9 @@
       <c r="CR16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CS16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5758,6 +5809,9 @@
       <c r="CR17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CS17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -6054,6 +6108,9 @@
       <c r="CR18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CS18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -6350,6 +6407,9 @@
       <c r="CR19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="CS19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -6646,6 +6706,9 @@
       <c r="CR20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CS20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -6942,6 +7005,9 @@
       <c r="CR21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="CS21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -7238,6 +7304,9 @@
       <c r="CR22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CS22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -7534,6 +7603,9 @@
       <c r="CR23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CS23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -7830,6 +7902,9 @@
       <c r="CR24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CS24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -8126,6 +8201,9 @@
       <c r="CR25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CS25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -8422,6 +8500,9 @@
       <c r="CR26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CS26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -8718,6 +8799,9 @@
       <c r="CR27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CS27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -9014,6 +9098,9 @@
       <c r="CR28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CS28" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -9310,6 +9397,9 @@
       <c r="CR29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CS29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -9606,6 +9696,9 @@
       <c r="CR30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CS30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -9902,6 +9995,9 @@
       <c r="CR31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CS31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -10198,6 +10294,9 @@
       <c r="CR32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CS32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -10494,6 +10593,9 @@
       <c r="CR33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CS33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -10790,6 +10892,9 @@
       <c r="CR34" s="3" t="n">
         <v>21.33</v>
       </c>
+      <c r="CS34" s="3" t="n">
+        <v>21.33</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -11086,6 +11191,9 @@
       <c r="CR35" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CS35" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -11382,6 +11490,9 @@
       <c r="CR36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CS36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -11678,6 +11789,9 @@
       <c r="CR37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CS37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -11974,6 +12088,9 @@
       <c r="CR38" s="3" t="n">
         <v>21.51</v>
       </c>
+      <c r="CS38" s="3" t="n">
+        <v>21.51</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -12270,6 +12387,9 @@
       <c r="CR39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CS39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -12566,6 +12686,9 @@
       <c r="CR40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CS40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -12862,6 +12985,9 @@
       <c r="CR41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CS41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -13158,6 +13284,9 @@
       <c r="CR42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CS42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -13454,6 +13583,9 @@
       <c r="CR43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CS43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -13750,6 +13882,9 @@
       <c r="CR44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CS44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -14046,6 +14181,9 @@
       <c r="CR45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="CS45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -14342,6 +14480,9 @@
       <c r="CR46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="CS46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -14638,6 +14779,9 @@
       <c r="CR47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CS47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -14934,6 +15078,9 @@
       <c r="CR48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CS48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -15230,6 +15377,9 @@
       <c r="CR49" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CS49" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -15526,6 +15676,9 @@
       <c r="CR50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CS50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -15822,6 +15975,9 @@
       <c r="CR51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CS51" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -16118,6 +16274,9 @@
       <c r="CR52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CS52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -16414,6 +16573,9 @@
       <c r="CR53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="CS53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -16710,6 +16872,9 @@
       <c r="CR54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CS54" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -17006,6 +17171,9 @@
       <c r="CR55" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CS55" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -17302,6 +17470,9 @@
       <c r="CR56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CS56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -17598,6 +17769,9 @@
       <c r="CR57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CS57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -17894,6 +18068,9 @@
       <c r="CR58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CS58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -18190,6 +18367,9 @@
       <c r="CR59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CS59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -18486,6 +18666,9 @@
       <c r="CR60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CS60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -18782,6 +18965,9 @@
       <c r="CR61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CS61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -19078,6 +19264,9 @@
       <c r="CR62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CS62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -19374,6 +19563,9 @@
       <c r="CR63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CS63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -19670,6 +19862,9 @@
       <c r="CR64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CS64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -19966,6 +20161,9 @@
       <c r="CR65" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CS65" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -20262,6 +20460,9 @@
       <c r="CR66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CS66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -20558,6 +20759,9 @@
       <c r="CR67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CS67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -20854,6 +21058,9 @@
       <c r="CR68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CS68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -21150,6 +21357,9 @@
       <c r="CR69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CS69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -21446,6 +21656,9 @@
       <c r="CR70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CS70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -21742,6 +21955,9 @@
       <c r="CR71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CS71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -22038,6 +22254,9 @@
       <c r="CR72" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CS72" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -22334,6 +22553,9 @@
       <c r="CR73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CS73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -22630,6 +22852,9 @@
       <c r="CR74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CS74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -22926,6 +23151,9 @@
       <c r="CR75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CS75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -23222,6 +23450,9 @@
       <c r="CR76" s="3" t="n">
         <v>21.67</v>
       </c>
+      <c r="CS76" s="3" t="n">
+        <v>21.67</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -23518,6 +23749,9 @@
       <c r="CR77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CS77" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -23814,6 +24048,9 @@
       <c r="CR78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CS78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -24110,6 +24347,9 @@
       <c r="CR79" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CS79" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -24406,6 +24646,9 @@
       <c r="CR80" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CS80" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -24702,6 +24945,9 @@
       <c r="CR81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CS81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -24998,6 +25244,9 @@
       <c r="CR82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CS82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -25294,6 +25543,9 @@
       <c r="CR83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CS83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -25590,6 +25842,9 @@
       <c r="CR84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CS84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -25886,6 +26141,9 @@
       <c r="CR85" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CS85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -26182,6 +26440,9 @@
       <c r="CR86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="CS86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -26478,6 +26739,9 @@
       <c r="CR87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CS87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -26774,6 +27038,9 @@
       <c r="CR88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CS88" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -27070,6 +27337,9 @@
       <c r="CR89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CS89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -27366,6 +27636,9 @@
       <c r="CR90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CS90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -27662,6 +27935,9 @@
       <c r="CR91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CS91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -27958,6 +28234,9 @@
       <c r="CR92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CS92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -28254,6 +28533,9 @@
       <c r="CR93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CS93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -28550,6 +28832,9 @@
       <c r="CR94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CS94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -28846,6 +29131,9 @@
       <c r="CR95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="CS95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -29142,6 +29430,9 @@
       <c r="CR96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="CS96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -29438,6 +29729,9 @@
       <c r="CR97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CS97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -29734,6 +30028,9 @@
       <c r="CR98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CS98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -30030,6 +30327,9 @@
       <c r="CR99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CS99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -30326,6 +30626,9 @@
       <c r="CR100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CS100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -30622,6 +30925,9 @@
       <c r="CR101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CS101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -30918,6 +31224,9 @@
       <c r="CR102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="CS102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -31214,6 +31523,9 @@
       <c r="CR103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CS103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -31510,6 +31822,9 @@
       <c r="CR104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CS104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -31806,6 +32121,9 @@
       <c r="CR105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CS105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -32102,6 +32420,9 @@
       <c r="CR106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CS106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -32398,6 +32719,9 @@
       <c r="CR107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CS107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -32694,6 +33018,9 @@
       <c r="CR108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CS108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -32990,6 +33317,9 @@
       <c r="CR109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CS109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -33286,6 +33616,9 @@
       <c r="CR110" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CS110" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -33582,6 +33915,9 @@
       <c r="CR111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="CS111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -33878,6 +34214,9 @@
       <c r="CR112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CS112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -34174,6 +34513,9 @@
       <c r="CR113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CS113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -34470,6 +34812,9 @@
       <c r="CR114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CS114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -34766,6 +35111,9 @@
       <c r="CR115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CS115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -35062,6 +35410,9 @@
       <c r="CR116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CS116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -35358,6 +35709,9 @@
       <c r="CR117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CS117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -35654,6 +36008,9 @@
       <c r="CR118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CS118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -35950,6 +36307,9 @@
       <c r="CR119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CS119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -36246,6 +36606,9 @@
       <c r="CR120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CS120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -36542,6 +36905,9 @@
       <c r="CR121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CS121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -36838,6 +37204,9 @@
       <c r="CR122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CS122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -37134,6 +37503,9 @@
       <c r="CR123" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="CS123" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -37430,6 +37802,9 @@
       <c r="CR124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CS124" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -37726,6 +38101,9 @@
       <c r="CR125" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CS125" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -38022,6 +38400,9 @@
       <c r="CR126" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CS126" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -38318,6 +38699,9 @@
       <c r="CR127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CS127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -38614,6 +38998,9 @@
       <c r="CR128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CS128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -38910,6 +39297,9 @@
       <c r="CR129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CS129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -39206,6 +39596,9 @@
       <c r="CR130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CS130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -39502,6 +39895,9 @@
       <c r="CR131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="CS131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -39798,6 +40194,9 @@
       <c r="CR132" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CS132" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -40094,6 +40493,9 @@
       <c r="CR133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CS133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -40390,6 +40792,9 @@
       <c r="CR134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="CS134" s="3" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -40686,6 +41091,9 @@
       <c r="CR135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CS135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -40982,6 +41390,9 @@
       <c r="CR136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CS136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -41278,6 +41689,9 @@
       <c r="CR137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CS137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -41574,6 +41988,9 @@
       <c r="CR138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="CS138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -41870,6 +42287,9 @@
       <c r="CR139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CS139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -42166,6 +42586,9 @@
       <c r="CR140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CS140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -42462,6 +42885,9 @@
       <c r="CR141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CS141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -42758,6 +43184,9 @@
       <c r="CR142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CS142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -43054,6 +43483,9 @@
       <c r="CR143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CS143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -43350,6 +43782,9 @@
       <c r="CR144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CS144" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -43646,6 +44081,9 @@
       <c r="CR145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CS145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -43942,6 +44380,9 @@
       <c r="CR146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CS146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -44238,6 +44679,9 @@
       <c r="CR147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CS147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -44534,6 +44978,9 @@
       <c r="CR148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CS148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -44830,6 +45277,9 @@
       <c r="CR149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CS149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -45126,6 +45576,9 @@
       <c r="CR150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CS150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -45422,6 +45875,9 @@
       <c r="CR151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CS151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -45718,6 +46174,9 @@
       <c r="CR152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CS152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -46014,6 +46473,9 @@
       <c r="CR153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CS153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -46310,6 +46772,9 @@
       <c r="CR154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CS154" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -46606,6 +47071,9 @@
       <c r="CR155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CS155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -46902,6 +47370,9 @@
       <c r="CR156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CS156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -47198,6 +47669,9 @@
       <c r="CR157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CS157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -47494,6 +47968,9 @@
       <c r="CR158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CS158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -47790,6 +48267,9 @@
       <c r="CR159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CS159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -48086,6 +48566,9 @@
       <c r="CR160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CS160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -48382,6 +48865,9 @@
       <c r="CR161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CS161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -48678,6 +49164,9 @@
       <c r="CR162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CS162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -48974,6 +49463,9 @@
       <c r="CR163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CS163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -49270,6 +49762,9 @@
       <c r="CR164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CS164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -49467,9 +49962,12 @@
       <c r="CR165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CS165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CR165"/>
+  <autoFilter ref="A1:CS165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-16 15:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CS$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CT$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CS165"/>
+  <dimension ref="A1:CT165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -540,6 +540,7 @@
     <col width="16" customWidth="1" min="95" max="95"/>
     <col width="16" customWidth="1" min="96" max="96"/>
     <col width="16" customWidth="1" min="97" max="97"/>
+    <col width="16" customWidth="1" min="98" max="98"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1028,6 +1029,11 @@
           <t>2026-09-16 07:12</t>
         </is>
       </c>
+      <c r="CT1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-16 10:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1327,6 +1333,9 @@
       <c r="CS2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CT2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1626,6 +1635,9 @@
       <c r="CS3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CT3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1925,6 +1937,9 @@
       <c r="CS4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CT4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2224,6 +2239,9 @@
       <c r="CS5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CT5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2523,6 +2541,9 @@
       <c r="CS6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CT6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2822,6 +2843,9 @@
       <c r="CS7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CT7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3121,6 +3145,9 @@
       <c r="CS8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CT8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3420,6 +3447,9 @@
       <c r="CS9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CT9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3719,6 +3749,9 @@
       <c r="CS10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CT10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4018,6 +4051,9 @@
       <c r="CS11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CT11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4317,6 +4353,9 @@
       <c r="CS12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CT12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4616,6 +4655,9 @@
       <c r="CS13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CT13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4915,6 +4957,9 @@
       <c r="CS14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CT14" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5214,6 +5259,9 @@
       <c r="CS15" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="CT15" s="3" t="n">
+        <v>20.54</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5513,6 +5561,9 @@
       <c r="CS16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CT16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5812,6 +5863,9 @@
       <c r="CS17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CT17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -6111,6 +6165,9 @@
       <c r="CS18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CT18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -6410,6 +6467,9 @@
       <c r="CS19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="CT19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -6709,6 +6769,9 @@
       <c r="CS20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CT20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -7008,6 +7071,9 @@
       <c r="CS21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="CT21" s="3" t="n">
+        <v>20.48</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -7307,6 +7373,9 @@
       <c r="CS22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CT22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -7606,6 +7675,9 @@
       <c r="CS23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CT23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -7905,6 +7977,9 @@
       <c r="CS24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CT24" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -8204,6 +8279,9 @@
       <c r="CS25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CT25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -8503,6 +8581,9 @@
       <c r="CS26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CT26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -8802,6 +8883,9 @@
       <c r="CS27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CT27" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -9101,6 +9185,9 @@
       <c r="CS28" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CT28" s="3" t="n">
+        <v>21.84</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -9400,6 +9487,9 @@
       <c r="CS29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CT29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -9699,6 +9789,9 @@
       <c r="CS30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CT30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -9998,6 +10091,9 @@
       <c r="CS31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CT31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -10297,6 +10393,9 @@
       <c r="CS32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CT32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -10596,6 +10695,9 @@
       <c r="CS33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CT33" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -10895,6 +10997,9 @@
       <c r="CS34" s="3" t="n">
         <v>21.33</v>
       </c>
+      <c r="CT34" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -11194,6 +11299,9 @@
       <c r="CS35" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CT35" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -11493,6 +11601,9 @@
       <c r="CS36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CT36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -11792,6 +11903,9 @@
       <c r="CS37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CT37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -12091,6 +12205,9 @@
       <c r="CS38" s="3" t="n">
         <v>21.51</v>
       </c>
+      <c r="CT38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -12390,6 +12507,9 @@
       <c r="CS39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CT39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -12689,6 +12809,9 @@
       <c r="CS40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CT40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -12988,6 +13111,9 @@
       <c r="CS41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CT41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -13287,6 +13413,9 @@
       <c r="CS42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CT42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -13586,6 +13715,9 @@
       <c r="CS43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CT43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -13885,6 +14017,9 @@
       <c r="CS44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CT44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -14184,6 +14319,9 @@
       <c r="CS45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="CT45" s="3" t="n">
+        <v>20.69</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -14483,6 +14621,9 @@
       <c r="CS46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="CT46" s="3" t="n">
+        <v>21.15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -14782,6 +14923,9 @@
       <c r="CS47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CT47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -15081,6 +15225,9 @@
       <c r="CS48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CT48" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -15380,6 +15527,9 @@
       <c r="CS49" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CT49" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -15679,6 +15829,9 @@
       <c r="CS50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CT50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -15978,6 +16131,9 @@
       <c r="CS51" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CT51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -16277,6 +16433,9 @@
       <c r="CS52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CT52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -16576,6 +16735,9 @@
       <c r="CS53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="CT53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -16875,6 +17037,9 @@
       <c r="CS54" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CT54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -17174,6 +17339,9 @@
       <c r="CS55" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CT55" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -17473,6 +17641,9 @@
       <c r="CS56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CT56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -17772,6 +17943,9 @@
       <c r="CS57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CT57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -18071,6 +18245,9 @@
       <c r="CS58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CT58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -18370,6 +18547,9 @@
       <c r="CS59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CT59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -18669,6 +18849,9 @@
       <c r="CS60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CT60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -18968,6 +19151,9 @@
       <c r="CS61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CT61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -19267,6 +19453,9 @@
       <c r="CS62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CT62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -19566,6 +19755,9 @@
       <c r="CS63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CT63" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -19865,6 +20057,9 @@
       <c r="CS64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CT64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -20164,6 +20359,9 @@
       <c r="CS65" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CT65" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -20463,6 +20661,9 @@
       <c r="CS66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CT66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -20762,6 +20963,9 @@
       <c r="CS67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CT67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -21061,6 +21265,9 @@
       <c r="CS68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CT68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -21360,6 +21567,9 @@
       <c r="CS69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CT69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -21659,6 +21869,9 @@
       <c r="CS70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CT70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -21958,6 +22171,9 @@
       <c r="CS71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CT71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -22257,6 +22473,9 @@
       <c r="CS72" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CT72" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -22556,6 +22775,9 @@
       <c r="CS73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CT73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -22855,6 +23077,9 @@
       <c r="CS74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CT74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -23154,6 +23379,9 @@
       <c r="CS75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CT75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -23453,6 +23681,9 @@
       <c r="CS76" s="3" t="n">
         <v>21.67</v>
       </c>
+      <c r="CT76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -23752,6 +23983,9 @@
       <c r="CS77" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CT77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -24051,6 +24285,9 @@
       <c r="CS78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CT78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -24350,6 +24587,9 @@
       <c r="CS79" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CT79" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -24649,6 +24889,9 @@
       <c r="CS80" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CT80" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -24948,6 +25191,9 @@
       <c r="CS81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CT81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -25247,6 +25493,9 @@
       <c r="CS82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CT82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -25546,6 +25795,9 @@
       <c r="CS83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CT83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -25845,6 +26097,9 @@
       <c r="CS84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CT84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -26144,6 +26399,9 @@
       <c r="CS85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="CT85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -26443,6 +26701,9 @@
       <c r="CS86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="CT86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -26742,6 +27003,9 @@
       <c r="CS87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CT87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -27041,6 +27305,9 @@
       <c r="CS88" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CT88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -27340,6 +27607,9 @@
       <c r="CS89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CT89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -27639,6 +27909,9 @@
       <c r="CS90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CT90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -27938,6 +28211,9 @@
       <c r="CS91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CT91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -28237,6 +28513,9 @@
       <c r="CS92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CT92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -28536,6 +28815,9 @@
       <c r="CS93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CT93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -28835,6 +29117,9 @@
       <c r="CS94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CT94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -29134,6 +29419,9 @@
       <c r="CS95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="CT95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -29433,6 +29721,9 @@
       <c r="CS96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="CT96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -29732,6 +30023,9 @@
       <c r="CS97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CT97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -30031,6 +30325,9 @@
       <c r="CS98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CT98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -30330,6 +30627,9 @@
       <c r="CS99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CT99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -30629,6 +30929,9 @@
       <c r="CS100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CT100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -30928,6 +31231,9 @@
       <c r="CS101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CT101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -31227,6 +31533,9 @@
       <c r="CS102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="CT102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -31526,6 +31835,9 @@
       <c r="CS103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CT103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -31825,6 +32137,9 @@
       <c r="CS104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CT104" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -32124,6 +32439,9 @@
       <c r="CS105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CT105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -32423,6 +32741,9 @@
       <c r="CS106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CT106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -32722,6 +33043,9 @@
       <c r="CS107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CT107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -33021,6 +33345,9 @@
       <c r="CS108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CT108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -33320,6 +33647,9 @@
       <c r="CS109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CT109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -33619,6 +33949,9 @@
       <c r="CS110" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CT110" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -33918,6 +34251,9 @@
       <c r="CS111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="CT111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -34217,6 +34553,9 @@
       <c r="CS112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CT112" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -34516,6 +34855,9 @@
       <c r="CS113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CT113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -34815,6 +35157,9 @@
       <c r="CS114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CT114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -35114,6 +35459,9 @@
       <c r="CS115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CT115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -35413,6 +35761,9 @@
       <c r="CS116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CT116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -35712,6 +36063,9 @@
       <c r="CS117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CT117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -36011,6 +36365,9 @@
       <c r="CS118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CT118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -36310,6 +36667,9 @@
       <c r="CS119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CT119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -36609,6 +36969,9 @@
       <c r="CS120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CT120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -36908,6 +37271,9 @@
       <c r="CS121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CT121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -37207,6 +37573,9 @@
       <c r="CS122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CT122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -37506,6 +37875,9 @@
       <c r="CS123" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="CT123" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -37805,6 +38177,9 @@
       <c r="CS124" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CT124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -38104,6 +38479,9 @@
       <c r="CS125" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CT125" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -38403,6 +38781,9 @@
       <c r="CS126" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CT126" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -38702,6 +39083,9 @@
       <c r="CS127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CT127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -39001,6 +39385,9 @@
       <c r="CS128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CT128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -39300,6 +39687,9 @@
       <c r="CS129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CT129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -39599,6 +39989,9 @@
       <c r="CS130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CT130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -39898,6 +40291,9 @@
       <c r="CS131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="CT131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -40197,6 +40593,9 @@
       <c r="CS132" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CT132" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -40496,6 +40895,9 @@
       <c r="CS133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CT133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -40795,6 +41197,9 @@
       <c r="CS134" s="3" t="n">
         <v>21.7</v>
       </c>
+      <c r="CT134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -41094,6 +41499,9 @@
       <c r="CS135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CT135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -41393,6 +41801,9 @@
       <c r="CS136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CT136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -41692,6 +42103,9 @@
       <c r="CS137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CT137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -41991,6 +42405,9 @@
       <c r="CS138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="CT138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -42290,6 +42707,9 @@
       <c r="CS139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CT139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -42589,6 +43009,9 @@
       <c r="CS140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CT140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -42888,6 +43311,9 @@
       <c r="CS141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CT141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -43187,6 +43613,9 @@
       <c r="CS142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CT142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -43486,6 +43915,9 @@
       <c r="CS143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CT143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -43785,6 +44217,9 @@
       <c r="CS144" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CT144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -44084,6 +44519,9 @@
       <c r="CS145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CT145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -44383,6 +44821,9 @@
       <c r="CS146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CT146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -44682,6 +45123,9 @@
       <c r="CS147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CT147" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -44981,6 +45425,9 @@
       <c r="CS148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CT148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -45280,6 +45727,9 @@
       <c r="CS149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CT149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -45579,6 +46029,9 @@
       <c r="CS150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CT150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -45878,6 +46331,9 @@
       <c r="CS151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CT151" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -46177,6 +46633,9 @@
       <c r="CS152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CT152" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -46476,6 +46935,9 @@
       <c r="CS153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CT153" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -46775,6 +47237,9 @@
       <c r="CS154" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CT154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -47074,6 +47539,9 @@
       <c r="CS155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CT155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -47373,6 +47841,9 @@
       <c r="CS156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CT156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -47672,6 +48143,9 @@
       <c r="CS157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CT157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -47971,6 +48445,9 @@
       <c r="CS158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CT158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -48270,6 +48747,9 @@
       <c r="CS159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CT159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -48569,6 +49049,9 @@
       <c r="CS160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CT160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -48868,6 +49351,9 @@
       <c r="CS161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CT161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -49167,6 +49653,9 @@
       <c r="CS162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CT162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -49466,6 +49955,9 @@
       <c r="CS163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CT163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -49765,6 +50257,9 @@
       <c r="CS164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CT164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -49965,9 +50460,12 @@
       <c r="CS165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CT165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CS165"/>
+  <autoFilter ref="A1:CT165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-16 18:11 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CT$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CU$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CT165"/>
+  <dimension ref="A1:CU165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -541,6 +541,7 @@
     <col width="16" customWidth="1" min="96" max="96"/>
     <col width="16" customWidth="1" min="97" max="97"/>
     <col width="16" customWidth="1" min="98" max="98"/>
+    <col width="16" customWidth="1" min="99" max="99"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1034,6 +1035,11 @@
           <t>2026-09-16 10:09</t>
         </is>
       </c>
+      <c r="CU1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-16 13:11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1336,6 +1342,9 @@
       <c r="CT2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CU2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1638,6 +1647,9 @@
       <c r="CT3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CU3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1940,6 +1952,9 @@
       <c r="CT4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CU4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2242,6 +2257,9 @@
       <c r="CT5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CU5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2544,6 +2562,9 @@
       <c r="CT6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CU6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2846,6 +2867,9 @@
       <c r="CT7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CU7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3148,6 +3172,9 @@
       <c r="CT8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CU8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3450,6 +3477,9 @@
       <c r="CT9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CU9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3752,6 +3782,9 @@
       <c r="CT10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CU10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4054,6 +4087,9 @@
       <c r="CT11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CU11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4356,6 +4392,9 @@
       <c r="CT12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CU12" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4658,6 +4697,9 @@
       <c r="CT13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CU13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -4960,6 +5002,9 @@
       <c r="CT14" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CU14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5262,6 +5307,9 @@
       <c r="CT15" s="3" t="n">
         <v>20.54</v>
       </c>
+      <c r="CU15" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5564,6 +5612,9 @@
       <c r="CT16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CU16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5866,6 +5917,9 @@
       <c r="CT17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CU17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -6168,6 +6222,9 @@
       <c r="CT18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CU18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -6470,6 +6527,9 @@
       <c r="CT19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="CU19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -6772,6 +6832,9 @@
       <c r="CT20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CU20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -7074,6 +7137,9 @@
       <c r="CT21" s="3" t="n">
         <v>20.48</v>
       </c>
+      <c r="CU21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -7376,6 +7442,9 @@
       <c r="CT22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CU22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -7678,6 +7747,9 @@
       <c r="CT23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CU23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -7980,6 +8052,9 @@
       <c r="CT24" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CU24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -8282,6 +8357,9 @@
       <c r="CT25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CU25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -8584,6 +8662,9 @@
       <c r="CT26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CU26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -8886,6 +8967,9 @@
       <c r="CT27" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CU27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -9188,6 +9272,9 @@
       <c r="CT28" s="3" t="n">
         <v>21.84</v>
       </c>
+      <c r="CU28" s="3" t="n">
+        <v>21.84</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -9490,6 +9577,9 @@
       <c r="CT29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CU29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -9792,6 +9882,9 @@
       <c r="CT30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CU30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -10094,6 +10187,9 @@
       <c r="CT31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CU31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -10396,6 +10492,9 @@
       <c r="CT32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CU32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -10698,6 +10797,9 @@
       <c r="CT33" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CU33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -11000,6 +11102,9 @@
       <c r="CT34" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CU34" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -11302,6 +11407,9 @@
       <c r="CT35" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CU35" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -11604,6 +11712,9 @@
       <c r="CT36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CU36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -11906,6 +12017,9 @@
       <c r="CT37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CU37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -12208,6 +12322,9 @@
       <c r="CT38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CU38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -12510,6 +12627,9 @@
       <c r="CT39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CU39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -12812,6 +12932,9 @@
       <c r="CT40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CU40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -13114,6 +13237,9 @@
       <c r="CT41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CU41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -13416,6 +13542,9 @@
       <c r="CT42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CU42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -13718,6 +13847,9 @@
       <c r="CT43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CU43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -14020,6 +14152,9 @@
       <c r="CT44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CU44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -14322,6 +14457,9 @@
       <c r="CT45" s="3" t="n">
         <v>20.69</v>
       </c>
+      <c r="CU45" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -14624,6 +14762,9 @@
       <c r="CT46" s="3" t="n">
         <v>21.15</v>
       </c>
+      <c r="CU46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -14926,6 +15067,9 @@
       <c r="CT47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CU47" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -15228,6 +15372,9 @@
       <c r="CT48" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CU48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -15530,6 +15677,9 @@
       <c r="CT49" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CU49" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -15832,6 +15982,9 @@
       <c r="CT50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CU50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -16134,6 +16287,9 @@
       <c r="CT51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CU51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -16436,6 +16592,9 @@
       <c r="CT52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CU52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -16738,6 +16897,9 @@
       <c r="CT53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="CU53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -17040,6 +17202,9 @@
       <c r="CT54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CU54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -17342,6 +17507,9 @@
       <c r="CT55" s="3" t="n">
         <v>21.8</v>
       </c>
+      <c r="CU55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -17644,6 +17812,9 @@
       <c r="CT56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CU56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -17946,6 +18117,9 @@
       <c r="CT57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CU57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -18248,6 +18422,9 @@
       <c r="CT58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CU58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -18550,6 +18727,9 @@
       <c r="CT59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CU59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -18852,6 +19032,9 @@
       <c r="CT60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CU60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -19154,6 +19337,9 @@
       <c r="CT61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CU61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -19456,6 +19642,9 @@
       <c r="CT62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CU62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -19758,6 +19947,9 @@
       <c r="CT63" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CU63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -20060,6 +20252,9 @@
       <c r="CT64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CU64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -20362,6 +20557,9 @@
       <c r="CT65" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CU65" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -20664,6 +20862,9 @@
       <c r="CT66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CU66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -20966,6 +21167,9 @@
       <c r="CT67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CU67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -21268,6 +21472,9 @@
       <c r="CT68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CU68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -21570,6 +21777,9 @@
       <c r="CT69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CU69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -21872,6 +22082,9 @@
       <c r="CT70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CU70" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -22174,6 +22387,9 @@
       <c r="CT71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CU71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -22476,6 +22692,9 @@
       <c r="CT72" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CU72" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -22778,6 +22997,9 @@
       <c r="CT73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CU73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -23080,6 +23302,9 @@
       <c r="CT74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CU74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -23382,6 +23607,9 @@
       <c r="CT75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CU75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -23684,6 +23912,9 @@
       <c r="CT76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CU76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -23986,6 +24217,9 @@
       <c r="CT77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="CU77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -24288,6 +24522,9 @@
       <c r="CT78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CU78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -24590,6 +24827,9 @@
       <c r="CT79" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CU79" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -24892,6 +25132,9 @@
       <c r="CT80" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CU80" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -25194,6 +25437,9 @@
       <c r="CT81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CU81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -25496,6 +25742,9 @@
       <c r="CT82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CU82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -25798,6 +26047,9 @@
       <c r="CT83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CU83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -26100,6 +26352,9 @@
       <c r="CT84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CU84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -26402,6 +26657,9 @@
       <c r="CT85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="CU85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -26704,6 +26962,9 @@
       <c r="CT86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="CU86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -27006,6 +27267,9 @@
       <c r="CT87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CU87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -27308,6 +27572,9 @@
       <c r="CT88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CU88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -27610,6 +27877,9 @@
       <c r="CT89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CU89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -27912,6 +28182,9 @@
       <c r="CT90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CU90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -28214,6 +28487,9 @@
       <c r="CT91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CU91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -28516,6 +28792,9 @@
       <c r="CT92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CU92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -28818,6 +29097,9 @@
       <c r="CT93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CU93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -29120,6 +29402,9 @@
       <c r="CT94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CU94" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -29422,6 +29707,9 @@
       <c r="CT95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="CU95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -29724,6 +30012,9 @@
       <c r="CT96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="CU96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -30026,6 +30317,9 @@
       <c r="CT97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CU97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -30328,6 +30622,9 @@
       <c r="CT98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CU98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -30630,6 +30927,9 @@
       <c r="CT99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CU99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -30932,6 +31232,9 @@
       <c r="CT100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CU100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -31234,6 +31537,9 @@
       <c r="CT101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CU101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -31536,6 +31842,9 @@
       <c r="CT102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="CU102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -31838,6 +32147,9 @@
       <c r="CT103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CU103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -32140,6 +32452,9 @@
       <c r="CT104" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CU104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -32442,6 +32757,9 @@
       <c r="CT105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CU105" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -32744,6 +33062,9 @@
       <c r="CT106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CU106" s="3" t="n">
+        <v>21.28</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -33046,6 +33367,9 @@
       <c r="CT107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CU107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -33348,6 +33672,9 @@
       <c r="CT108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CU108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -33650,6 +33977,9 @@
       <c r="CT109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CU109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -33952,6 +34282,9 @@
       <c r="CT110" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CU110" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -34254,6 +34587,9 @@
       <c r="CT111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="CU111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -34556,6 +34892,9 @@
       <c r="CT112" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CU112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -34858,6 +35197,9 @@
       <c r="CT113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CU113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -35160,6 +35502,9 @@
       <c r="CT114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CU114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -35462,6 +35807,9 @@
       <c r="CT115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CU115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -35764,6 +36112,9 @@
       <c r="CT116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CU116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -36066,6 +36417,9 @@
       <c r="CT117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CU117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -36368,6 +36722,9 @@
       <c r="CT118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CU118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -36670,6 +37027,9 @@
       <c r="CT119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CU119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -36972,6 +37332,9 @@
       <c r="CT120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CU120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -37274,6 +37637,9 @@
       <c r="CT121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CU121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -37576,6 +37942,9 @@
       <c r="CT122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CU122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -37878,6 +38247,9 @@
       <c r="CT123" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="CU123" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -38180,6 +38552,9 @@
       <c r="CT124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="CU124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -38482,6 +38857,9 @@
       <c r="CT125" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CU125" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -38784,6 +39162,9 @@
       <c r="CT126" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CU126" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -39086,6 +39467,9 @@
       <c r="CT127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CU127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -39388,6 +39772,9 @@
       <c r="CT128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CU128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -39690,6 +40077,9 @@
       <c r="CT129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CU129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -39992,6 +40382,9 @@
       <c r="CT130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CU130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -40294,6 +40687,9 @@
       <c r="CT131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="CU131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -40596,6 +40992,9 @@
       <c r="CT132" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CU132" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -40898,6 +41297,9 @@
       <c r="CT133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CU133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -41200,6 +41602,9 @@
       <c r="CT134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="CU134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -41502,6 +41907,9 @@
       <c r="CT135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CU135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -41804,6 +42212,9 @@
       <c r="CT136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CU136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -42106,6 +42517,9 @@
       <c r="CT137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CU137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -42408,6 +42822,9 @@
       <c r="CT138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="CU138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -42710,6 +43127,9 @@
       <c r="CT139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CU139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -43012,6 +43432,9 @@
       <c r="CT140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CU140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -43314,6 +43737,9 @@
       <c r="CT141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CU141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -43616,6 +44042,9 @@
       <c r="CT142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CU142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -43918,6 +44347,9 @@
       <c r="CT143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CU143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -44220,6 +44652,9 @@
       <c r="CT144" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CU144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -44522,6 +44957,9 @@
       <c r="CT145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CU145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -44824,6 +45262,9 @@
       <c r="CT146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CU146" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -45126,6 +45567,9 @@
       <c r="CT147" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CU147" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -45428,6 +45872,9 @@
       <c r="CT148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CU148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -45730,6 +46177,9 @@
       <c r="CT149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CU149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -46032,6 +46482,9 @@
       <c r="CT150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CU150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -46334,6 +46787,9 @@
       <c r="CT151" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CU151" s="3" t="n">
+        <v>23.39</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -46636,6 +47092,9 @@
       <c r="CT152" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CU152" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -46938,6 +47397,9 @@
       <c r="CT153" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CU153" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -47240,6 +47702,9 @@
       <c r="CT154" s="3" t="n">
         <v>23.7</v>
       </c>
+      <c r="CU154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -47542,6 +48007,9 @@
       <c r="CT155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CU155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -47844,6 +48312,9 @@
       <c r="CT156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CU156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -48146,6 +48617,9 @@
       <c r="CT157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CU157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -48448,6 +48922,9 @@
       <c r="CT158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CU158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -48750,6 +49227,9 @@
       <c r="CT159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CU159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -49052,6 +49532,9 @@
       <c r="CT160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CU160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -49354,6 +49837,9 @@
       <c r="CT161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CU161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -49656,6 +50142,9 @@
       <c r="CT162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CU162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -49958,6 +50447,9 @@
       <c r="CT163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CU163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -50260,6 +50752,9 @@
       <c r="CT164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CU164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -50463,9 +50958,12 @@
       <c r="CT165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CU165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CT165"/>
+  <autoFilter ref="A1:CU165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-16 21:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CU$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CV$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CU165"/>
+  <dimension ref="A1:CV165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -542,6 +542,7 @@
     <col width="16" customWidth="1" min="97" max="97"/>
     <col width="16" customWidth="1" min="98" max="98"/>
     <col width="16" customWidth="1" min="99" max="99"/>
+    <col width="16" customWidth="1" min="100" max="100"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1040,6 +1041,11 @@
           <t>2026-09-16 13:11</t>
         </is>
       </c>
+      <c r="CV1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-16 16:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1345,6 +1351,9 @@
       <c r="CU2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CV2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1650,6 +1659,9 @@
       <c r="CU3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CV3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1955,6 +1967,9 @@
       <c r="CU4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CV4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2260,6 +2275,9 @@
       <c r="CU5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CV5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2565,6 +2583,9 @@
       <c r="CU6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CV6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2870,6 +2891,9 @@
       <c r="CU7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CV7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3175,6 +3199,9 @@
       <c r="CU8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CV8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3480,6 +3507,9 @@
       <c r="CU9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CV9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3785,6 +3815,9 @@
       <c r="CU10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CV10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4090,6 +4123,9 @@
       <c r="CU11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CV11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4395,6 +4431,9 @@
       <c r="CU12" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CV12" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4700,6 +4739,9 @@
       <c r="CU13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CV13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5005,6 +5047,9 @@
       <c r="CU14" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CV14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5310,6 +5355,9 @@
       <c r="CU15" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CV15" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5615,6 +5663,9 @@
       <c r="CU16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CV16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5920,6 +5971,9 @@
       <c r="CU17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CV17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -6225,6 +6279,9 @@
       <c r="CU18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CV18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -6530,6 +6587,9 @@
       <c r="CU19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="CV19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -6835,6 +6895,9 @@
       <c r="CU20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CV20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -7140,6 +7203,9 @@
       <c r="CU21" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CV21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -7445,6 +7511,9 @@
       <c r="CU22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CV22" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -7750,6 +7819,9 @@
       <c r="CU23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CV23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -8055,6 +8127,9 @@
       <c r="CU24" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CV24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -8360,6 +8435,9 @@
       <c r="CU25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CV25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -8665,6 +8743,9 @@
       <c r="CU26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CV26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -8970,6 +9051,9 @@
       <c r="CU27" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CV27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -9275,6 +9359,9 @@
       <c r="CU28" s="3" t="n">
         <v>21.84</v>
       </c>
+      <c r="CV28" s="3" t="n">
+        <v>21.84</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -9580,6 +9667,9 @@
       <c r="CU29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CV29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -9885,6 +9975,9 @@
       <c r="CU30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CV30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -10190,6 +10283,9 @@
       <c r="CU31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CV31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -10495,6 +10591,9 @@
       <c r="CU32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CV32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -10800,6 +10899,9 @@
       <c r="CU33" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CV33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -11105,6 +11207,9 @@
       <c r="CU34" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CV34" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -11410,6 +11515,9 @@
       <c r="CU35" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CV35" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -11715,6 +11823,9 @@
       <c r="CU36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CV36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -12020,6 +12131,9 @@
       <c r="CU37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CV37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -12325,6 +12439,9 @@
       <c r="CU38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CV38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -12630,6 +12747,9 @@
       <c r="CU39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CV39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -12935,6 +13055,9 @@
       <c r="CU40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CV40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -13240,6 +13363,9 @@
       <c r="CU41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CV41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -13545,6 +13671,9 @@
       <c r="CU42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CV42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -13850,6 +13979,9 @@
       <c r="CU43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CV43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -14155,6 +14287,9 @@
       <c r="CU44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CV44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -14460,6 +14595,9 @@
       <c r="CU45" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CV45" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -14765,6 +14903,9 @@
       <c r="CU46" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="CV46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -15070,6 +15211,9 @@
       <c r="CU47" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CV47" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -15375,6 +15519,9 @@
       <c r="CU48" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CV48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -15680,6 +15827,9 @@
       <c r="CU49" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CV49" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -15985,6 +16135,9 @@
       <c r="CU50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CV50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -16290,6 +16443,9 @@
       <c r="CU51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CV51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -16595,6 +16751,9 @@
       <c r="CU52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CV52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -16900,6 +17059,9 @@
       <c r="CU53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="CV53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -17205,6 +17367,9 @@
       <c r="CU54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CV54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -17510,6 +17675,9 @@
       <c r="CU55" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CV55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -17815,6 +17983,9 @@
       <c r="CU56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CV56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -18120,6 +18291,9 @@
       <c r="CU57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CV57" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -18425,6 +18599,9 @@
       <c r="CU58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CV58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -18730,6 +18907,9 @@
       <c r="CU59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CV59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -19035,6 +19215,9 @@
       <c r="CU60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CV60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -19340,6 +19523,9 @@
       <c r="CU61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CV61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -19645,6 +19831,9 @@
       <c r="CU62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CV62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -19950,6 +20139,9 @@
       <c r="CU63" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="CV63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -20255,6 +20447,9 @@
       <c r="CU64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CV64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -20560,6 +20755,9 @@
       <c r="CU65" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CV65" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -20865,6 +21063,9 @@
       <c r="CU66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CV66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -21170,6 +21371,9 @@
       <c r="CU67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CV67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -21475,6 +21679,9 @@
       <c r="CU68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CV68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -21780,6 +21987,9 @@
       <c r="CU69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CV69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -22085,6 +22295,9 @@
       <c r="CU70" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CV70" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -22390,6 +22603,9 @@
       <c r="CU71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CV71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -22695,6 +22911,9 @@
       <c r="CU72" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CV72" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -23000,6 +23219,9 @@
       <c r="CU73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CV73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -23305,6 +23527,9 @@
       <c r="CU74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CV74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -23610,6 +23835,9 @@
       <c r="CU75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CV75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -23915,6 +24143,9 @@
       <c r="CU76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CV76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -24220,6 +24451,9 @@
       <c r="CU77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="CV77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -24525,6 +24759,9 @@
       <c r="CU78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CV78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -24830,6 +25067,9 @@
       <c r="CU79" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CV79" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -25135,6 +25375,9 @@
       <c r="CU80" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CV80" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -25440,6 +25683,9 @@
       <c r="CU81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CV81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -25745,6 +25991,9 @@
       <c r="CU82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CV82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -26050,6 +26299,9 @@
       <c r="CU83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CV83" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -26355,6 +26607,9 @@
       <c r="CU84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CV84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -26660,6 +26915,9 @@
       <c r="CU85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="CV85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -26965,6 +27223,9 @@
       <c r="CU86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="CV86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -27270,6 +27531,9 @@
       <c r="CU87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CV87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -27575,6 +27839,9 @@
       <c r="CU88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CV88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -27880,6 +28147,9 @@
       <c r="CU89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CV89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -28185,6 +28455,9 @@
       <c r="CU90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CV90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -28490,6 +28763,9 @@
       <c r="CU91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CV91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -28795,6 +29071,9 @@
       <c r="CU92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CV92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -29100,6 +29379,9 @@
       <c r="CU93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CV93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -29405,6 +29687,9 @@
       <c r="CU94" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CV94" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -29710,6 +29995,9 @@
       <c r="CU95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="CV95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -30015,6 +30303,9 @@
       <c r="CU96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="CV96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -30320,6 +30611,9 @@
       <c r="CU97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CV97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -30625,6 +30919,9 @@
       <c r="CU98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CV98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -30930,6 +31227,9 @@
       <c r="CU99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CV99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -31235,6 +31535,9 @@
       <c r="CU100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CV100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -31540,6 +31843,9 @@
       <c r="CU101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CV101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -31845,6 +32151,9 @@
       <c r="CU102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="CV102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -32150,6 +32459,9 @@
       <c r="CU103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CV103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -32455,6 +32767,9 @@
       <c r="CU104" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CV104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -32760,6 +33075,9 @@
       <c r="CU105" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CV105" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -33065,6 +33383,9 @@
       <c r="CU106" s="3" t="n">
         <v>21.28</v>
       </c>
+      <c r="CV106" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -33370,6 +33691,9 @@
       <c r="CU107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CV107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -33675,6 +33999,9 @@
       <c r="CU108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CV108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -33980,6 +34307,9 @@
       <c r="CU109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CV109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -34285,6 +34615,9 @@
       <c r="CU110" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CV110" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -34590,6 +34923,9 @@
       <c r="CU111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="CV111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -34895,6 +35231,9 @@
       <c r="CU112" s="3" t="n">
         <v>23.8</v>
       </c>
+      <c r="CV112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -35200,6 +35539,9 @@
       <c r="CU113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CV113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -35505,6 +35847,9 @@
       <c r="CU114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CV114" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -35810,6 +36155,9 @@
       <c r="CU115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CV115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -36115,6 +36463,9 @@
       <c r="CU116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CV116" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -36420,6 +36771,9 @@
       <c r="CU117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CV117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -36725,6 +37079,9 @@
       <c r="CU118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CV118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -37030,6 +37387,9 @@
       <c r="CU119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CV119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -37335,6 +37695,9 @@
       <c r="CU120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CV120" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -37640,6 +38003,9 @@
       <c r="CU121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CV121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -37945,6 +38311,9 @@
       <c r="CU122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CV122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -38250,6 +38619,9 @@
       <c r="CU123" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="CV123" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -38555,6 +38927,9 @@
       <c r="CU124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="CV124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -38860,6 +39235,9 @@
       <c r="CU125" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CV125" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -39165,6 +39543,9 @@
       <c r="CU126" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CV126" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -39470,6 +39851,9 @@
       <c r="CU127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CV127" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -39775,6 +40159,9 @@
       <c r="CU128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CV128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -40080,6 +40467,9 @@
       <c r="CU129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CV129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -40385,6 +40775,9 @@
       <c r="CU130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CV130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -40690,6 +41083,9 @@
       <c r="CU131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="CV131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -40995,6 +41391,9 @@
       <c r="CU132" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CV132" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -41300,6 +41699,9 @@
       <c r="CU133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CV133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -41605,6 +42007,9 @@
       <c r="CU134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="CV134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -41910,6 +42315,9 @@
       <c r="CU135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CV135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -42215,6 +42623,9 @@
       <c r="CU136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CV136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -42520,6 +42931,9 @@
       <c r="CU137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CV137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -42825,6 +43239,9 @@
       <c r="CU138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="CV138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -43130,6 +43547,9 @@
       <c r="CU139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CV139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -43435,6 +43855,9 @@
       <c r="CU140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CV140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -43740,6 +44163,9 @@
       <c r="CU141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CV141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -44045,6 +44471,9 @@
       <c r="CU142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CV142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -44350,6 +44779,9 @@
       <c r="CU143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CV143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -44655,6 +45087,9 @@
       <c r="CU144" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CV144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -44960,6 +45395,9 @@
       <c r="CU145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CV145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -45265,6 +45703,9 @@
       <c r="CU146" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CV146" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -45570,6 +46011,9 @@
       <c r="CU147" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CV147" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -45875,6 +46319,9 @@
       <c r="CU148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CV148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -46180,6 +46627,9 @@
       <c r="CU149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CV149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -46485,6 +46935,9 @@
       <c r="CU150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CV150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -46790,6 +47243,9 @@
       <c r="CU151" s="3" t="n">
         <v>23.39</v>
       </c>
+      <c r="CV151" s="3" t="n">
+        <v>23.39</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -47095,6 +47551,9 @@
       <c r="CU152" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CV152" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -47400,6 +47859,9 @@
       <c r="CU153" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CV153" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -47705,6 +48167,9 @@
       <c r="CU154" s="3" t="n">
         <v>23.7</v>
       </c>
+      <c r="CV154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -48010,6 +48475,9 @@
       <c r="CU155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CV155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -48315,6 +48783,9 @@
       <c r="CU156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CV156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -48620,6 +49091,9 @@
       <c r="CU157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CV157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -48925,6 +49399,9 @@
       <c r="CU158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CV158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -49230,6 +49707,9 @@
       <c r="CU159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CV159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -49535,6 +50015,9 @@
       <c r="CU160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CV160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -49840,6 +50323,9 @@
       <c r="CU161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CV161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -50145,6 +50631,9 @@
       <c r="CU162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CV162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -50450,6 +50939,9 @@
       <c r="CU163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CV163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -50755,6 +51247,9 @@
       <c r="CU164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CV164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -50961,9 +51456,12 @@
       <c r="CU165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CV165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CU165"/>
+  <autoFilter ref="A1:CV165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-17 00:12 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CV$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CW$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CV165"/>
+  <dimension ref="A1:CW165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -543,6 +543,7 @@
     <col width="16" customWidth="1" min="98" max="98"/>
     <col width="16" customWidth="1" min="99" max="99"/>
     <col width="16" customWidth="1" min="100" max="100"/>
+    <col width="16" customWidth="1" min="101" max="101"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1046,6 +1047,11 @@
           <t>2026-09-16 16:09</t>
         </is>
       </c>
+      <c r="CW1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-16 19:12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1354,6 +1360,9 @@
       <c r="CV2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CW2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1662,6 +1671,9 @@
       <c r="CV3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CW3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1970,6 +1982,9 @@
       <c r="CV4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CW4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2278,6 +2293,9 @@
       <c r="CV5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CW5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2586,6 +2604,9 @@
       <c r="CV6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CW6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2894,6 +2915,9 @@
       <c r="CV7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CW7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3202,6 +3226,9 @@
       <c r="CV8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CW8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3510,6 +3537,9 @@
       <c r="CV9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CW9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3818,6 +3848,9 @@
       <c r="CV10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CW10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4126,6 +4159,9 @@
       <c r="CV11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CW11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4434,6 +4470,9 @@
       <c r="CV12" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW12" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4742,6 +4781,9 @@
       <c r="CV13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CW13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5050,6 +5092,9 @@
       <c r="CV14" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CW14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5358,6 +5403,9 @@
       <c r="CV15" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CW15" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5666,6 +5714,9 @@
       <c r="CV16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CW16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -5974,6 +6025,9 @@
       <c r="CV17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CW17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -6282,6 +6336,9 @@
       <c r="CV18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CW18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -6590,6 +6647,9 @@
       <c r="CV19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="CW19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -6898,6 +6958,9 @@
       <c r="CV20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CW20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -7206,6 +7269,9 @@
       <c r="CV21" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CW21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -7514,6 +7580,9 @@
       <c r="CV22" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW22" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -7822,6 +7891,9 @@
       <c r="CV23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CW23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -8130,6 +8202,9 @@
       <c r="CV24" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CW24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -8438,6 +8513,9 @@
       <c r="CV25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CW25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -8746,6 +8824,9 @@
       <c r="CV26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CW26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -9054,6 +9135,9 @@
       <c r="CV27" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CW27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -9362,6 +9446,9 @@
       <c r="CV28" s="3" t="n">
         <v>21.84</v>
       </c>
+      <c r="CW28" s="3" t="n">
+        <v>21.84</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -9670,6 +9757,9 @@
       <c r="CV29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CW29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -9978,6 +10068,9 @@
       <c r="CV30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -10286,6 +10379,9 @@
       <c r="CV31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CW31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -10594,6 +10690,9 @@
       <c r="CV32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CW32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -10902,6 +11001,9 @@
       <c r="CV33" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -11210,6 +11312,9 @@
       <c r="CV34" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CW34" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -11518,6 +11623,9 @@
       <c r="CV35" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CW35" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -11826,6 +11934,9 @@
       <c r="CV36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CW36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -12134,6 +12245,9 @@
       <c r="CV37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CW37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -12442,6 +12556,9 @@
       <c r="CV38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CW38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -12750,6 +12867,9 @@
       <c r="CV39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CW39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -13058,6 +13178,9 @@
       <c r="CV40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -13366,6 +13489,9 @@
       <c r="CV41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CW41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -13674,6 +13800,9 @@
       <c r="CV42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CW42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -13982,6 +14111,9 @@
       <c r="CV43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CW43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -14290,6 +14422,9 @@
       <c r="CV44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -14598,6 +14733,9 @@
       <c r="CV45" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CW45" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -14906,6 +15044,9 @@
       <c r="CV46" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="CW46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -15214,6 +15355,9 @@
       <c r="CV47" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CW47" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -15522,6 +15666,9 @@
       <c r="CV48" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CW48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -15830,6 +15977,9 @@
       <c r="CV49" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CW49" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -16138,6 +16288,9 @@
       <c r="CV50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CW50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -16446,6 +16599,9 @@
       <c r="CV51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CW51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -16754,6 +16910,9 @@
       <c r="CV52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CW52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -17062,6 +17221,9 @@
       <c r="CV53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="CW53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -17370,6 +17532,9 @@
       <c r="CV54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -17678,6 +17843,9 @@
       <c r="CV55" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CW55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -17986,6 +18154,9 @@
       <c r="CV56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -18294,6 +18465,9 @@
       <c r="CV57" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CW57" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -18602,6 +18776,9 @@
       <c r="CV58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CW58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -18910,6 +19087,9 @@
       <c r="CV59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CW59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -19218,6 +19398,9 @@
       <c r="CV60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CW60" s="3" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -19526,6 +19709,9 @@
       <c r="CV61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CW61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -19834,6 +20020,9 @@
       <c r="CV62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CW62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -20142,6 +20331,9 @@
       <c r="CV63" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="CW63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -20450,6 +20642,9 @@
       <c r="CV64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CW64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -20758,6 +20953,9 @@
       <c r="CV65" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CW65" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -21066,6 +21264,9 @@
       <c r="CV66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -21374,6 +21575,9 @@
       <c r="CV67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CW67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -21682,6 +21886,9 @@
       <c r="CV68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CW68" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -21990,6 +22197,9 @@
       <c r="CV69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CW69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -22298,6 +22508,9 @@
       <c r="CV70" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW70" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -22606,6 +22819,9 @@
       <c r="CV71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -22914,6 +23130,9 @@
       <c r="CV72" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CW72" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -23222,6 +23441,9 @@
       <c r="CV73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CW73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -23530,6 +23752,9 @@
       <c r="CV74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CW74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -23838,6 +24063,9 @@
       <c r="CV75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -24146,6 +24374,9 @@
       <c r="CV76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -24454,6 +24685,9 @@
       <c r="CV77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="CW77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -24762,6 +24996,9 @@
       <c r="CV78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CW78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -25070,6 +25307,9 @@
       <c r="CV79" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CW79" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -25378,6 +25618,9 @@
       <c r="CV80" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CW80" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -25686,6 +25929,9 @@
       <c r="CV81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -25994,6 +26240,9 @@
       <c r="CV82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CW82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -26302,6 +26551,9 @@
       <c r="CV83" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CW83" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -26610,6 +26862,9 @@
       <c r="CV84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CW84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -26918,6 +27173,9 @@
       <c r="CV85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="CW85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -27226,6 +27484,9 @@
       <c r="CV86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="CW86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -27534,6 +27795,9 @@
       <c r="CV87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CW87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -27842,6 +28106,9 @@
       <c r="CV88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -28150,6 +28417,9 @@
       <c r="CV89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CW89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -28458,6 +28728,9 @@
       <c r="CV90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -28766,6 +29039,9 @@
       <c r="CV91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -29074,6 +29350,9 @@
       <c r="CV92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -29382,6 +29661,9 @@
       <c r="CV93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CW93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -29690,6 +29972,9 @@
       <c r="CV94" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CW94" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -29998,6 +30283,9 @@
       <c r="CV95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="CW95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -30306,6 +30594,9 @@
       <c r="CV96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="CW96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -30614,6 +30905,9 @@
       <c r="CV97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CW97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -30922,6 +31216,9 @@
       <c r="CV98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CW98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -31230,6 +31527,9 @@
       <c r="CV99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CW99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -31538,6 +31838,9 @@
       <c r="CV100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CW100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -31846,6 +32149,9 @@
       <c r="CV101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -32154,6 +32460,9 @@
       <c r="CV102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="CW102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -32462,6 +32771,9 @@
       <c r="CV103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CW103" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -32770,6 +33082,9 @@
       <c r="CV104" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -33078,6 +33393,9 @@
       <c r="CV105" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW105" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -33386,6 +33704,9 @@
       <c r="CV106" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW106" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -33694,6 +34015,9 @@
       <c r="CV107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CW107" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -34002,6 +34326,9 @@
       <c r="CV108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CW108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -34310,6 +34637,9 @@
       <c r="CV109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -34618,6 +34948,9 @@
       <c r="CV110" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CW110" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -34926,6 +35259,9 @@
       <c r="CV111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="CW111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -35234,6 +35570,9 @@
       <c r="CV112" s="3" t="n">
         <v>23.8</v>
       </c>
+      <c r="CW112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -35542,6 +35881,9 @@
       <c r="CV113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CW113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -35850,6 +36192,9 @@
       <c r="CV114" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CW114" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -36158,6 +36503,9 @@
       <c r="CV115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CW115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -36466,6 +36814,9 @@
       <c r="CV116" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CW116" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -36774,6 +37125,9 @@
       <c r="CV117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CW117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -37082,6 +37436,9 @@
       <c r="CV118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CW118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -37390,6 +37747,9 @@
       <c r="CV119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CW119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -37698,6 +38058,9 @@
       <c r="CV120" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CW120" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -38006,6 +38369,9 @@
       <c r="CV121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CW121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -38314,6 +38680,9 @@
       <c r="CV122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CW122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -38622,6 +38991,9 @@
       <c r="CV123" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="CW123" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -38930,6 +39302,9 @@
       <c r="CV124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="CW124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -39238,6 +39613,9 @@
       <c r="CV125" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW125" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -39546,6 +39924,9 @@
       <c r="CV126" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW126" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -39854,6 +40235,9 @@
       <c r="CV127" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CW127" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -40162,6 +40546,9 @@
       <c r="CV128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CW128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -40470,6 +40857,9 @@
       <c r="CV129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CW129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -40778,6 +41168,9 @@
       <c r="CV130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CW130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -41086,6 +41479,9 @@
       <c r="CV131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="CW131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -41394,6 +41790,9 @@
       <c r="CV132" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW132" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -41702,6 +42101,9 @@
       <c r="CV133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CW133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -42010,6 +42412,9 @@
       <c r="CV134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="CW134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -42318,6 +42723,9 @@
       <c r="CV135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CW135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -42626,6 +43034,9 @@
       <c r="CV136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CW136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -42934,6 +43345,9 @@
       <c r="CV137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CW137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -43242,6 +43656,9 @@
       <c r="CV138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="CW138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -43550,6 +43967,9 @@
       <c r="CV139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CW139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -43858,6 +44278,9 @@
       <c r="CV140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CW140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -44166,6 +44589,9 @@
       <c r="CV141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CW141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -44474,6 +44900,9 @@
       <c r="CV142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CW142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -44782,6 +45211,9 @@
       <c r="CV143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CW143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -45090,6 +45522,9 @@
       <c r="CV144" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CW144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -45398,6 +45833,9 @@
       <c r="CV145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CW145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -45706,6 +46144,9 @@
       <c r="CV146" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CW146" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -46014,6 +46455,9 @@
       <c r="CV147" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CW147" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -46322,6 +46766,9 @@
       <c r="CV148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CW148" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -46630,6 +47077,9 @@
       <c r="CV149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CW149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -46938,6 +47388,9 @@
       <c r="CV150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CW150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -47246,6 +47699,9 @@
       <c r="CV151" s="3" t="n">
         <v>23.39</v>
       </c>
+      <c r="CW151" s="3" t="n">
+        <v>23.39</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -47554,6 +48010,9 @@
       <c r="CV152" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CW152" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -47862,6 +48321,9 @@
       <c r="CV153" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CW153" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -48170,6 +48632,9 @@
       <c r="CV154" s="3" t="n">
         <v>23.7</v>
       </c>
+      <c r="CW154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -48478,6 +48943,9 @@
       <c r="CV155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CW155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -48786,6 +49254,9 @@
       <c r="CV156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CW156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -49094,6 +49565,9 @@
       <c r="CV157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CW157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -49402,6 +49876,9 @@
       <c r="CV158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CW158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -49710,6 +50187,9 @@
       <c r="CV159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CW159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -50018,6 +50498,9 @@
       <c r="CV160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CW160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -50326,6 +50809,9 @@
       <c r="CV161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CW161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -50634,6 +51120,9 @@
       <c r="CV162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CW162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -50942,6 +51431,9 @@
       <c r="CV163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CW163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -51250,6 +51742,9 @@
       <c r="CV164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CW164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -51459,9 +51954,12 @@
       <c r="CV165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CW165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CV165"/>
+  <autoFilter ref="A1:CW165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-17 03:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CW$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CX$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CW165"/>
+  <dimension ref="A1:CX165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -544,6 +544,7 @@
     <col width="16" customWidth="1" min="99" max="99"/>
     <col width="16" customWidth="1" min="100" max="100"/>
     <col width="16" customWidth="1" min="101" max="101"/>
+    <col width="16" customWidth="1" min="102" max="102"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1052,6 +1053,11 @@
           <t>2026-09-16 19:12</t>
         </is>
       </c>
+      <c r="CX1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-16 22:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1363,6 +1369,9 @@
       <c r="CW2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CX2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1674,6 +1683,9 @@
       <c r="CW3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CX3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1985,6 +1997,9 @@
       <c r="CW4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CX4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2296,6 +2311,9 @@
       <c r="CW5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CX5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2607,6 +2625,9 @@
       <c r="CW6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CX6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2918,6 +2939,9 @@
       <c r="CW7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CX7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3229,6 +3253,9 @@
       <c r="CW8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CX8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3540,6 +3567,9 @@
       <c r="CW9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CX9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3851,6 +3881,9 @@
       <c r="CW10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CX10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4162,6 +4195,9 @@
       <c r="CW11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CX11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4473,6 +4509,9 @@
       <c r="CW12" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX12" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4784,6 +4823,9 @@
       <c r="CW13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CX13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5095,6 +5137,9 @@
       <c r="CW14" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CX14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5406,6 +5451,9 @@
       <c r="CW15" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CX15" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5717,6 +5765,9 @@
       <c r="CW16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CX16" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6028,6 +6079,9 @@
       <c r="CW17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CX17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -6339,6 +6393,9 @@
       <c r="CW18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CX18" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -6650,6 +6707,9 @@
       <c r="CW19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="CX19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -6961,6 +7021,9 @@
       <c r="CW20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CX20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -7272,6 +7335,9 @@
       <c r="CW21" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CX21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -7583,6 +7649,9 @@
       <c r="CW22" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CX22" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -7894,6 +7963,9 @@
       <c r="CW23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CX23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -8205,6 +8277,9 @@
       <c r="CW24" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CX24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -8516,6 +8591,9 @@
       <c r="CW25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CX25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -8827,6 +8905,9 @@
       <c r="CW26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CX26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -9138,6 +9219,9 @@
       <c r="CW27" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CX27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -9449,6 +9533,9 @@
       <c r="CW28" s="3" t="n">
         <v>21.84</v>
       </c>
+      <c r="CX28" s="3" t="n">
+        <v>21.84</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -9760,6 +9847,9 @@
       <c r="CW29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CX29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -10071,6 +10161,9 @@
       <c r="CW30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -10382,6 +10475,9 @@
       <c r="CW31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CX31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -10693,6 +10789,9 @@
       <c r="CW32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CX32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -11004,6 +11103,9 @@
       <c r="CW33" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -11315,6 +11417,9 @@
       <c r="CW34" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CX34" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -11626,6 +11731,9 @@
       <c r="CW35" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CX35" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -11937,6 +12045,9 @@
       <c r="CW36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CX36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -12248,6 +12359,9 @@
       <c r="CW37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CX37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -12559,6 +12673,9 @@
       <c r="CW38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CX38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -12870,6 +12987,9 @@
       <c r="CW39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CX39" s="3" t="n">
+        <v>20.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -13181,6 +13301,9 @@
       <c r="CW40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -13492,6 +13615,9 @@
       <c r="CW41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CX41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -13803,6 +13929,9 @@
       <c r="CW42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CX42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -14114,6 +14243,9 @@
       <c r="CW43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CX43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -14425,6 +14557,9 @@
       <c r="CW44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -14736,6 +14871,9 @@
       <c r="CW45" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CX45" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -15047,6 +15185,9 @@
       <c r="CW46" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="CX46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -15358,6 +15499,9 @@
       <c r="CW47" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CX47" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -15669,6 +15813,9 @@
       <c r="CW48" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CX48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -15980,6 +16127,9 @@
       <c r="CW49" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CX49" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -16291,6 +16441,9 @@
       <c r="CW50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CX50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -16602,6 +16755,9 @@
       <c r="CW51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CX51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -16913,6 +17069,9 @@
       <c r="CW52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CX52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -17224,6 +17383,9 @@
       <c r="CW53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="CX53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -17535,6 +17697,9 @@
       <c r="CW54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -17846,6 +18011,9 @@
       <c r="CW55" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CX55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -18157,6 +18325,9 @@
       <c r="CW56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -18468,6 +18639,9 @@
       <c r="CW57" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CX57" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -18779,6 +18953,9 @@
       <c r="CW58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CX58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -19090,6 +19267,9 @@
       <c r="CW59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CX59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -19401,6 +19581,9 @@
       <c r="CW60" s="3" t="n">
         <v>20.9</v>
       </c>
+      <c r="CX60" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -19712,6 +19895,9 @@
       <c r="CW61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CX61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -20023,6 +20209,9 @@
       <c r="CW62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CX62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -20334,6 +20523,9 @@
       <c r="CW63" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="CX63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -20645,6 +20837,9 @@
       <c r="CW64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CX64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -20956,6 +21151,9 @@
       <c r="CW65" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CX65" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -21267,6 +21465,9 @@
       <c r="CW66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -21578,6 +21779,9 @@
       <c r="CW67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CX67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -21889,6 +22093,9 @@
       <c r="CW68" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CX68" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -22200,6 +22407,9 @@
       <c r="CW69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CX69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -22511,6 +22721,9 @@
       <c r="CW70" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX70" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -22822,6 +23035,9 @@
       <c r="CW71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -23133,6 +23349,9 @@
       <c r="CW72" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CX72" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -23444,6 +23663,9 @@
       <c r="CW73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CX73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -23755,6 +23977,9 @@
       <c r="CW74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CX74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -24066,6 +24291,9 @@
       <c r="CW75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -24377,6 +24605,9 @@
       <c r="CW76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -24688,6 +24919,9 @@
       <c r="CW77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="CX77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -24999,6 +25233,9 @@
       <c r="CW78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CX78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -25310,6 +25547,9 @@
       <c r="CW79" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CX79" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -25621,6 +25861,9 @@
       <c r="CW80" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CX80" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -25932,6 +26175,9 @@
       <c r="CW81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -26243,6 +26489,9 @@
       <c r="CW82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CX82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -26554,6 +26803,9 @@
       <c r="CW83" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX83" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -26865,6 +27117,9 @@
       <c r="CW84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CX84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -27176,6 +27431,9 @@
       <c r="CW85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="CX85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -27487,6 +27745,9 @@
       <c r="CW86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="CX86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -27798,6 +28059,9 @@
       <c r="CW87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CX87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -28109,6 +28373,9 @@
       <c r="CW88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -28420,6 +28687,9 @@
       <c r="CW89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CX89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -28731,6 +29001,9 @@
       <c r="CW90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -29042,6 +29315,9 @@
       <c r="CW91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -29353,6 +29629,9 @@
       <c r="CW92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -29664,6 +29943,9 @@
       <c r="CW93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CX93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -29975,6 +30257,9 @@
       <c r="CW94" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CX94" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -30286,6 +30571,9 @@
       <c r="CW95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="CX95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -30597,6 +30885,9 @@
       <c r="CW96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="CX96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -30908,6 +31199,9 @@
       <c r="CW97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CX97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -31219,6 +31513,9 @@
       <c r="CW98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CX98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -31530,6 +31827,9 @@
       <c r="CW99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CX99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -31841,6 +32141,9 @@
       <c r="CW100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CX100" s="3" t="n">
+        <v>21.19</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -32152,6 +32455,9 @@
       <c r="CW101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -32463,6 +32769,9 @@
       <c r="CW102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="CX102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -32774,6 +33083,9 @@
       <c r="CW103" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CX103" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -33085,6 +33397,9 @@
       <c r="CW104" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -33396,6 +33711,9 @@
       <c r="CW105" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX105" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -33707,6 +34025,9 @@
       <c r="CW106" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX106" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -34018,6 +34339,9 @@
       <c r="CW107" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CX107" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -34329,6 +34653,9 @@
       <c r="CW108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CX108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -34640,6 +34967,9 @@
       <c r="CW109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -34951,6 +35281,9 @@
       <c r="CW110" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CX110" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -35262,6 +35595,9 @@
       <c r="CW111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="CX111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -35573,6 +35909,9 @@
       <c r="CW112" s="3" t="n">
         <v>23.8</v>
       </c>
+      <c r="CX112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -35884,6 +36223,9 @@
       <c r="CW113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CX113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -36195,6 +36537,9 @@
       <c r="CW114" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX114" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -36506,6 +36851,9 @@
       <c r="CW115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CX115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -36817,6 +37165,9 @@
       <c r="CW116" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CX116" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -37128,6 +37479,9 @@
       <c r="CW117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CX117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -37439,6 +37793,9 @@
       <c r="CW118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CX118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -37750,6 +38107,9 @@
       <c r="CW119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CX119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -38061,6 +38421,9 @@
       <c r="CW120" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX120" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -38372,6 +38735,9 @@
       <c r="CW121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CX121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -38683,6 +39049,9 @@
       <c r="CW122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CX122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -38994,6 +39363,9 @@
       <c r="CW123" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="CX123" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -39305,6 +39677,9 @@
       <c r="CW124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="CX124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -39616,6 +39991,9 @@
       <c r="CW125" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX125" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -39927,6 +40305,9 @@
       <c r="CW126" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX126" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -40238,6 +40619,9 @@
       <c r="CW127" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="CX127" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -40549,6 +40933,9 @@
       <c r="CW128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CX128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -40860,6 +41247,9 @@
       <c r="CW129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CX129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -41171,6 +41561,9 @@
       <c r="CW130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CX130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -41482,6 +41875,9 @@
       <c r="CW131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="CX131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -41793,6 +42189,9 @@
       <c r="CW132" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="CX132" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -42104,6 +42503,9 @@
       <c r="CW133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CX133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -42415,6 +42817,9 @@
       <c r="CW134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="CX134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -42726,6 +43131,9 @@
       <c r="CW135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CX135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -43037,6 +43445,9 @@
       <c r="CW136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CX136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -43348,6 +43759,9 @@
       <c r="CW137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CX137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -43659,6 +44073,9 @@
       <c r="CW138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="CX138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -43970,6 +44387,9 @@
       <c r="CW139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CX139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -44281,6 +44701,9 @@
       <c r="CW140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CX140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -44592,6 +45015,9 @@
       <c r="CW141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CX141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -44903,6 +45329,9 @@
       <c r="CW142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CX142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -45214,6 +45643,9 @@
       <c r="CW143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CX143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -45525,6 +45957,9 @@
       <c r="CW144" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CX144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -45836,6 +46271,9 @@
       <c r="CW145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CX145" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -46147,6 +46585,9 @@
       <c r="CW146" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CX146" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -46458,6 +46899,9 @@
       <c r="CW147" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CX147" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -46769,6 +47213,9 @@
       <c r="CW148" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CX148" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -47080,6 +47527,9 @@
       <c r="CW149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CX149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -47391,6 +47841,9 @@
       <c r="CW150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CX150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -47702,6 +48155,9 @@
       <c r="CW151" s="3" t="n">
         <v>23.39</v>
       </c>
+      <c r="CX151" s="3" t="n">
+        <v>23.39</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -48013,6 +48469,9 @@
       <c r="CW152" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CX152" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -48324,6 +48783,9 @@
       <c r="CW153" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CX153" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -48635,6 +49097,9 @@
       <c r="CW154" s="3" t="n">
         <v>23.7</v>
       </c>
+      <c r="CX154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -48946,6 +49411,9 @@
       <c r="CW155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CX155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -49257,6 +49725,9 @@
       <c r="CW156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CX156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -49568,6 +50039,9 @@
       <c r="CW157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CX157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -49879,6 +50353,9 @@
       <c r="CW158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CX158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -50190,6 +50667,9 @@
       <c r="CW159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CX159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -50501,6 +50981,9 @@
       <c r="CW160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CX160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -50812,6 +51295,9 @@
       <c r="CW161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CX161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -51123,6 +51609,9 @@
       <c r="CW162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CX162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -51434,6 +51923,9 @@
       <c r="CW163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CX163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -51745,6 +52237,9 @@
       <c r="CW164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CX164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -51957,9 +52452,12 @@
       <c r="CW165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CX165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CW165"/>
+  <autoFilter ref="A1:CX165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-17 06:12 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CX$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CY$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CX165"/>
+  <dimension ref="A1:CY165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -545,6 +545,7 @@
     <col width="16" customWidth="1" min="100" max="100"/>
     <col width="16" customWidth="1" min="101" max="101"/>
     <col width="16" customWidth="1" min="102" max="102"/>
+    <col width="16" customWidth="1" min="103" max="103"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1058,6 +1059,11 @@
           <t>2026-09-16 22:09</t>
         </is>
       </c>
+      <c r="CY1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-17 01:12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1372,6 +1378,9 @@
       <c r="CX2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CY2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1686,6 +1695,9 @@
       <c r="CX3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CY3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2000,6 +2012,9 @@
       <c r="CX4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CY4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2314,6 +2329,9 @@
       <c r="CX5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CY5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2628,6 +2646,9 @@
       <c r="CX6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CY6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2942,6 +2963,9 @@
       <c r="CX7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CY7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3256,6 +3280,9 @@
       <c r="CX8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CY8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3570,6 +3597,9 @@
       <c r="CX9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CY9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3884,6 +3914,9 @@
       <c r="CX10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CY10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4198,6 +4231,9 @@
       <c r="CX11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CY11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4512,6 +4548,9 @@
       <c r="CX12" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY12" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4826,6 +4865,9 @@
       <c r="CX13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CY13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5140,6 +5182,9 @@
       <c r="CX14" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CY14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5454,6 +5499,9 @@
       <c r="CX15" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CY15" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5768,6 +5816,9 @@
       <c r="CX16" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CY16" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6082,6 +6133,9 @@
       <c r="CX17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CY17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -6396,6 +6450,9 @@
       <c r="CX18" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CY18" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -6710,6 +6767,9 @@
       <c r="CX19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="CY19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -7024,6 +7084,9 @@
       <c r="CX20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CY20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -7338,6 +7401,9 @@
       <c r="CX21" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CY21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -7652,6 +7718,9 @@
       <c r="CX22" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CY22" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -7966,6 +8035,9 @@
       <c r="CX23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CY23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -8280,6 +8352,9 @@
       <c r="CX24" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CY24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -8594,6 +8669,9 @@
       <c r="CX25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CY25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -8908,6 +8986,9 @@
       <c r="CX26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CY26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -9222,6 +9303,9 @@
       <c r="CX27" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CY27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -9536,6 +9620,9 @@
       <c r="CX28" s="3" t="n">
         <v>21.84</v>
       </c>
+      <c r="CY28" s="3" t="n">
+        <v>21.84</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -9850,6 +9937,9 @@
       <c r="CX29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CY29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -10164,6 +10254,9 @@
       <c r="CX30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -10478,6 +10571,9 @@
       <c r="CX31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CY31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -10792,6 +10888,9 @@
       <c r="CX32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CY32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -11106,6 +11205,9 @@
       <c r="CX33" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -11420,6 +11522,9 @@
       <c r="CX34" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CY34" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -11734,6 +11839,9 @@
       <c r="CX35" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CY35" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -12048,6 +12156,9 @@
       <c r="CX36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CY36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -12362,6 +12473,9 @@
       <c r="CX37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CY37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -12676,6 +12790,9 @@
       <c r="CX38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CY38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -12990,6 +13107,9 @@
       <c r="CX39" s="3" t="n">
         <v>20.98</v>
       </c>
+      <c r="CY39" s="3" t="n">
+        <v>21.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -13304,6 +13424,9 @@
       <c r="CX40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -13618,6 +13741,9 @@
       <c r="CX41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CY41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -13932,6 +14058,9 @@
       <c r="CX42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CY42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -14246,6 +14375,9 @@
       <c r="CX43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CY43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -14560,6 +14692,9 @@
       <c r="CX44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -14874,6 +15009,9 @@
       <c r="CX45" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CY45" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -15188,6 +15326,9 @@
       <c r="CX46" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="CY46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -15502,6 +15643,9 @@
       <c r="CX47" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CY47" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -15816,6 +15960,9 @@
       <c r="CX48" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CY48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -16130,6 +16277,9 @@
       <c r="CX49" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CY49" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -16444,6 +16594,9 @@
       <c r="CX50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CY50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -16758,6 +16911,9 @@
       <c r="CX51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CY51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -17072,6 +17228,9 @@
       <c r="CX52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CY52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -17386,6 +17545,9 @@
       <c r="CX53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="CY53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -17700,6 +17862,9 @@
       <c r="CX54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -18014,6 +18179,9 @@
       <c r="CX55" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CY55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -18328,6 +18496,9 @@
       <c r="CX56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -18642,6 +18813,9 @@
       <c r="CX57" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CY57" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -18956,6 +19130,9 @@
       <c r="CX58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CY58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -19270,6 +19447,9 @@
       <c r="CX59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CY59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -19584,6 +19764,9 @@
       <c r="CX60" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CY60" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -19898,6 +20081,9 @@
       <c r="CX61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CY61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -20212,6 +20398,9 @@
       <c r="CX62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CY62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -20526,6 +20715,9 @@
       <c r="CX63" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="CY63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -20840,6 +21032,9 @@
       <c r="CX64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CY64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -21154,6 +21349,9 @@
       <c r="CX65" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CY65" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -21468,6 +21666,9 @@
       <c r="CX66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -21782,6 +21983,9 @@
       <c r="CX67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CY67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -22096,6 +22300,9 @@
       <c r="CX68" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CY68" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -22410,6 +22617,9 @@
       <c r="CX69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CY69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -22724,6 +22934,9 @@
       <c r="CX70" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY70" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -23038,6 +23251,9 @@
       <c r="CX71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -23352,6 +23568,9 @@
       <c r="CX72" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CY72" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -23666,6 +23885,9 @@
       <c r="CX73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CY73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -23980,6 +24202,9 @@
       <c r="CX74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CY74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -24294,6 +24519,9 @@
       <c r="CX75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -24608,6 +24836,9 @@
       <c r="CX76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -24922,6 +25153,9 @@
       <c r="CX77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="CY77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -25236,6 +25470,9 @@
       <c r="CX78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CY78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -25550,6 +25787,9 @@
       <c r="CX79" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CY79" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -25864,6 +26104,9 @@
       <c r="CX80" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CY80" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -26178,6 +26421,9 @@
       <c r="CX81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -26492,6 +26738,9 @@
       <c r="CX82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CY82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -26806,6 +27055,9 @@
       <c r="CX83" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY83" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -27120,6 +27372,9 @@
       <c r="CX84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CY84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -27434,6 +27689,9 @@
       <c r="CX85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="CY85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -27748,6 +28006,9 @@
       <c r="CX86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="CY86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -28062,6 +28323,9 @@
       <c r="CX87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CY87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -28376,6 +28640,9 @@
       <c r="CX88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -28690,6 +28957,9 @@
       <c r="CX89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CY89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -29004,6 +29274,9 @@
       <c r="CX90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -29318,6 +29591,9 @@
       <c r="CX91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -29632,6 +29908,9 @@
       <c r="CX92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -29946,6 +30225,9 @@
       <c r="CX93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CY93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -30260,6 +30542,9 @@
       <c r="CX94" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CY94" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -30574,6 +30859,9 @@
       <c r="CX95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="CY95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -30888,6 +31176,9 @@
       <c r="CX96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="CY96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -31202,6 +31493,9 @@
       <c r="CX97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CY97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -31516,6 +31810,9 @@
       <c r="CX98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CY98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -31830,6 +32127,9 @@
       <c r="CX99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CY99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -32144,6 +32444,9 @@
       <c r="CX100" s="3" t="n">
         <v>21.19</v>
       </c>
+      <c r="CY100" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -32458,6 +32761,9 @@
       <c r="CX101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -32772,6 +33078,9 @@
       <c r="CX102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="CY102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -33086,6 +33395,9 @@
       <c r="CX103" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY103" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -33400,6 +33712,9 @@
       <c r="CX104" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -33714,6 +34029,9 @@
       <c r="CX105" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY105" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -34028,6 +34346,9 @@
       <c r="CX106" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY106" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -34342,6 +34663,9 @@
       <c r="CX107" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CY107" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -34656,6 +34980,9 @@
       <c r="CX108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CY108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -34970,6 +35297,9 @@
       <c r="CX109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -35284,6 +35614,9 @@
       <c r="CX110" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CY110" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -35598,6 +35931,9 @@
       <c r="CX111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="CY111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -35912,6 +36248,9 @@
       <c r="CX112" s="3" t="n">
         <v>23.8</v>
       </c>
+      <c r="CY112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -36226,6 +36565,9 @@
       <c r="CX113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CY113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -36540,6 +36882,9 @@
       <c r="CX114" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY114" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -36854,6 +37199,9 @@
       <c r="CX115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CY115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -37168,6 +37516,9 @@
       <c r="CX116" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CY116" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -37482,6 +37833,9 @@
       <c r="CX117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CY117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -37796,6 +38150,9 @@
       <c r="CX118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CY118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -38110,6 +38467,9 @@
       <c r="CX119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CY119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -38424,6 +38784,9 @@
       <c r="CX120" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY120" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -38738,6 +39101,9 @@
       <c r="CX121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CY121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -39052,6 +39418,9 @@
       <c r="CX122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CY122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -39366,6 +39735,9 @@
       <c r="CX123" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="CY123" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -39680,6 +40052,9 @@
       <c r="CX124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="CY124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -39994,6 +40369,9 @@
       <c r="CX125" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY125" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -40308,6 +40686,9 @@
       <c r="CX126" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY126" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -40622,6 +41003,9 @@
       <c r="CX127" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="CY127" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -40936,6 +41320,9 @@
       <c r="CX128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CY128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -41250,6 +41637,9 @@
       <c r="CX129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CY129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -41564,6 +41954,9 @@
       <c r="CX130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CY130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -41878,6 +42271,9 @@
       <c r="CX131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="CY131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -42192,6 +42588,9 @@
       <c r="CX132" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="CY132" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -42506,6 +42905,9 @@
       <c r="CX133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CY133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -42820,6 +43222,9 @@
       <c r="CX134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="CY134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -43134,6 +43539,9 @@
       <c r="CX135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CY135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -43448,6 +43856,9 @@
       <c r="CX136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CY136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -43762,6 +44173,9 @@
       <c r="CX137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CY137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -44076,6 +44490,9 @@
       <c r="CX138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="CY138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -44390,6 +44807,9 @@
       <c r="CX139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CY139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -44704,6 +45124,9 @@
       <c r="CX140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CY140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -45018,6 +45441,9 @@
       <c r="CX141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CY141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -45332,6 +45758,9 @@
       <c r="CX142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CY142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -45646,6 +46075,9 @@
       <c r="CX143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CY143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -45960,6 +46392,9 @@
       <c r="CX144" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CY144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -46274,6 +46709,9 @@
       <c r="CX145" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CY145" s="3" t="n">
+        <v>23.19</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -46588,6 +47026,9 @@
       <c r="CX146" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CY146" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -46902,6 +47343,9 @@
       <c r="CX147" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CY147" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -47216,6 +47660,9 @@
       <c r="CX148" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CY148" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -47530,6 +47977,9 @@
       <c r="CX149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CY149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -47844,6 +48294,9 @@
       <c r="CX150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CY150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -48158,6 +48611,9 @@
       <c r="CX151" s="3" t="n">
         <v>23.39</v>
       </c>
+      <c r="CY151" s="3" t="n">
+        <v>23.39</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -48472,6 +48928,9 @@
       <c r="CX152" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CY152" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -48786,6 +49245,9 @@
       <c r="CX153" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CY153" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -49100,6 +49562,9 @@
       <c r="CX154" s="3" t="n">
         <v>23.7</v>
       </c>
+      <c r="CY154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -49414,6 +49879,9 @@
       <c r="CX155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CY155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -49728,6 +50196,9 @@
       <c r="CX156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CY156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -50042,6 +50513,9 @@
       <c r="CX157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CY157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -50356,6 +50830,9 @@
       <c r="CX158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CY158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -50670,6 +51147,9 @@
       <c r="CX159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CY159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -50984,6 +51464,9 @@
       <c r="CX160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CY160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -51298,6 +51781,9 @@
       <c r="CX161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CY161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -51612,6 +52098,9 @@
       <c r="CX162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CY162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -51926,6 +52415,9 @@
       <c r="CX163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CY163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -52240,6 +52732,9 @@
       <c r="CX164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CY164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -52455,9 +52950,12 @@
       <c r="CX165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CY165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CX165"/>
+  <autoFilter ref="A1:CY165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-17 09:10 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CY$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CZ$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CY165"/>
+  <dimension ref="A1:CZ165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -546,6 +546,7 @@
     <col width="16" customWidth="1" min="101" max="101"/>
     <col width="16" customWidth="1" min="102" max="102"/>
     <col width="16" customWidth="1" min="103" max="103"/>
+    <col width="16" customWidth="1" min="104" max="104"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1064,6 +1065,11 @@
           <t>2026-09-17 01:12</t>
         </is>
       </c>
+      <c r="CZ1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-17 04:10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1381,6 +1387,9 @@
       <c r="CY2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="CZ2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1698,6 +1707,9 @@
       <c r="CY3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="CZ3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2015,6 +2027,9 @@
       <c r="CY4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="CZ4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2332,6 +2347,9 @@
       <c r="CY5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CZ5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2649,6 +2667,9 @@
       <c r="CY6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="CZ6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2966,6 +2987,9 @@
       <c r="CY7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="CZ7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3283,6 +3307,9 @@
       <c r="CY8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CZ8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3600,6 +3627,9 @@
       <c r="CY9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="CZ9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3917,6 +3947,9 @@
       <c r="CY10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="CZ10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4234,6 +4267,9 @@
       <c r="CY11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CZ11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4551,6 +4587,9 @@
       <c r="CY12" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ12" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4868,6 +4907,9 @@
       <c r="CY13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="CZ13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5185,6 +5227,9 @@
       <c r="CY14" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CZ14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5502,6 +5547,9 @@
       <c r="CY15" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CZ15" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5819,6 +5867,9 @@
       <c r="CY16" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CZ16" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6136,6 +6187,9 @@
       <c r="CY17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CZ17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -6453,6 +6507,9 @@
       <c r="CY18" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CZ18" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -6770,6 +6827,9 @@
       <c r="CY19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="CZ19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -7087,6 +7147,9 @@
       <c r="CY20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CZ20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -7404,6 +7467,9 @@
       <c r="CY21" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CZ21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -7721,6 +7787,9 @@
       <c r="CY22" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="CZ22" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -8038,6 +8107,9 @@
       <c r="CY23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="CZ23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -8355,6 +8427,9 @@
       <c r="CY24" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CZ24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -8672,6 +8747,9 @@
       <c r="CY25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CZ25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -8989,6 +9067,9 @@
       <c r="CY26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CZ26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -9306,6 +9387,9 @@
       <c r="CY27" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CZ27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -9623,6 +9707,9 @@
       <c r="CY28" s="3" t="n">
         <v>21.84</v>
       </c>
+      <c r="CZ28" s="3" t="n">
+        <v>21.84</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -9940,6 +10027,9 @@
       <c r="CY29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="CZ29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -10257,6 +10347,9 @@
       <c r="CY30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -10574,6 +10667,9 @@
       <c r="CY31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CZ31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -10891,6 +10987,9 @@
       <c r="CY32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CZ32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -11208,6 +11307,9 @@
       <c r="CY33" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -11525,6 +11627,9 @@
       <c r="CY34" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CZ34" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -11842,6 +11947,9 @@
       <c r="CY35" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CZ35" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -12159,6 +12267,9 @@
       <c r="CY36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CZ36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -12476,6 +12587,9 @@
       <c r="CY37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="CZ37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -12793,6 +12907,9 @@
       <c r="CY38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CZ38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -13110,6 +13227,9 @@
       <c r="CY39" s="3" t="n">
         <v>21.98</v>
       </c>
+      <c r="CZ39" s="3" t="n">
+        <v>21.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -13427,6 +13547,9 @@
       <c r="CY40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -13744,6 +13867,9 @@
       <c r="CY41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CZ41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -14061,6 +14187,9 @@
       <c r="CY42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CZ42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -14378,6 +14507,9 @@
       <c r="CY43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CZ43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -14695,6 +14827,9 @@
       <c r="CY44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -15012,6 +15147,9 @@
       <c r="CY45" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CZ45" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -15329,6 +15467,9 @@
       <c r="CY46" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="CZ46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -15646,6 +15787,9 @@
       <c r="CY47" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CZ47" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -15963,6 +16107,9 @@
       <c r="CY48" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CZ48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -16280,6 +16427,9 @@
       <c r="CY49" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CZ49" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -16597,6 +16747,9 @@
       <c r="CY50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="CZ50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -16914,6 +17067,9 @@
       <c r="CY51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CZ51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -17231,6 +17387,9 @@
       <c r="CY52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CZ52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -17548,6 +17707,9 @@
       <c r="CY53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="CZ53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -17865,6 +18027,9 @@
       <c r="CY54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -18182,6 +18347,9 @@
       <c r="CY55" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CZ55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -18499,6 +18667,9 @@
       <c r="CY56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -18816,6 +18987,9 @@
       <c r="CY57" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CZ57" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -19133,6 +19307,9 @@
       <c r="CY58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="CZ58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -19450,6 +19627,9 @@
       <c r="CY59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CZ59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -19767,6 +19947,9 @@
       <c r="CY60" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CZ60" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -20084,6 +20267,9 @@
       <c r="CY61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CZ61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -20401,6 +20587,9 @@
       <c r="CY62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CZ62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -20718,6 +20907,9 @@
       <c r="CY63" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="CZ63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -21035,6 +21227,9 @@
       <c r="CY64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CZ64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -21352,6 +21547,9 @@
       <c r="CY65" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="CZ65" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -21669,6 +21867,9 @@
       <c r="CY66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -21986,6 +22187,9 @@
       <c r="CY67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CZ67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -22303,6 +22507,9 @@
       <c r="CY68" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CZ68" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -22620,6 +22827,9 @@
       <c r="CY69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CZ69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -22937,6 +23147,9 @@
       <c r="CY70" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ70" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -23254,6 +23467,9 @@
       <c r="CY71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -23571,6 +23787,9 @@
       <c r="CY72" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CZ72" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -23888,6 +24107,9 @@
       <c r="CY73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CZ73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -24205,6 +24427,9 @@
       <c r="CY74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CZ74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -24522,6 +24747,9 @@
       <c r="CY75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -24839,6 +25067,9 @@
       <c r="CY76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -25156,6 +25387,9 @@
       <c r="CY77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="CZ77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -25473,6 +25707,9 @@
       <c r="CY78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="CZ78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -25790,6 +26027,9 @@
       <c r="CY79" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CZ79" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -26107,6 +26347,9 @@
       <c r="CY80" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="CZ80" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -26424,6 +26667,9 @@
       <c r="CY81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -26741,6 +26987,9 @@
       <c r="CY82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CZ82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -27058,6 +27307,9 @@
       <c r="CY83" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ83" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -27375,6 +27627,9 @@
       <c r="CY84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CZ84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -27692,6 +27947,9 @@
       <c r="CY85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="CZ85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -28009,6 +28267,9 @@
       <c r="CY86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="CZ86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -28326,6 +28587,9 @@
       <c r="CY87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="CZ87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -28643,6 +28907,9 @@
       <c r="CY88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -28960,6 +29227,9 @@
       <c r="CY89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CZ89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -29277,6 +29547,9 @@
       <c r="CY90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -29594,6 +29867,9 @@
       <c r="CY91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -29911,6 +30187,9 @@
       <c r="CY92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -30228,6 +30507,9 @@
       <c r="CY93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="CZ93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -30545,6 +30827,9 @@
       <c r="CY94" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CZ94" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -30862,6 +31147,9 @@
       <c r="CY95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="CZ95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -31179,6 +31467,9 @@
       <c r="CY96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="CZ96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -31496,6 +31787,9 @@
       <c r="CY97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CZ97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -31813,6 +32107,9 @@
       <c r="CY98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CZ98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -32130,6 +32427,9 @@
       <c r="CY99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CZ99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -32447,6 +32747,9 @@
       <c r="CY100" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="CZ100" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -32764,6 +33067,9 @@
       <c r="CY101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -33081,6 +33387,9 @@
       <c r="CY102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="CZ102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -33398,6 +33707,9 @@
       <c r="CY103" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ103" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -33715,6 +34027,9 @@
       <c r="CY104" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -34032,6 +34347,9 @@
       <c r="CY105" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ105" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -34349,6 +34667,9 @@
       <c r="CY106" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ106" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -34666,6 +34987,9 @@
       <c r="CY107" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="CZ107" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -34983,6 +35307,9 @@
       <c r="CY108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="CZ108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -35300,6 +35627,9 @@
       <c r="CY109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -35617,6 +35947,9 @@
       <c r="CY110" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="CZ110" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -35934,6 +36267,9 @@
       <c r="CY111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="CZ111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -36251,6 +36587,9 @@
       <c r="CY112" s="3" t="n">
         <v>23.8</v>
       </c>
+      <c r="CZ112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -36568,6 +36907,9 @@
       <c r="CY113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="CZ113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -36885,6 +37227,9 @@
       <c r="CY114" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ114" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -37202,6 +37547,9 @@
       <c r="CY115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="CZ115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -37519,6 +37867,9 @@
       <c r="CY116" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="CZ116" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -37836,6 +38187,9 @@
       <c r="CY117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CZ117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -38153,6 +38507,9 @@
       <c r="CY118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CZ118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -38470,6 +38827,9 @@
       <c r="CY119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="CZ119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -38787,6 +39147,9 @@
       <c r="CY120" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ120" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -39104,6 +39467,9 @@
       <c r="CY121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="CZ121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -39421,6 +39787,9 @@
       <c r="CY122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="CZ122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -39738,6 +40107,9 @@
       <c r="CY123" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="CZ123" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -40055,6 +40427,9 @@
       <c r="CY124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="CZ124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -40372,6 +40747,9 @@
       <c r="CY125" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ125" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -40689,6 +41067,9 @@
       <c r="CY126" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ126" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -41006,6 +41387,9 @@
       <c r="CY127" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="CZ127" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -41323,6 +41707,9 @@
       <c r="CY128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="CZ128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -41640,6 +42027,9 @@
       <c r="CY129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="CZ129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -41957,6 +42347,9 @@
       <c r="CY130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CZ130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -42274,6 +42667,9 @@
       <c r="CY131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="CZ131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -42591,6 +42987,9 @@
       <c r="CY132" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="CZ132" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -42908,6 +43307,9 @@
       <c r="CY133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="CZ133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -43225,6 +43627,9 @@
       <c r="CY134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="CZ134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -43542,6 +43947,9 @@
       <c r="CY135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CZ135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -43859,6 +44267,9 @@
       <c r="CY136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CZ136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -44176,6 +44587,9 @@
       <c r="CY137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="CZ137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -44493,6 +44907,9 @@
       <c r="CY138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="CZ138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -44810,6 +45227,9 @@
       <c r="CY139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CZ139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -45127,6 +45547,9 @@
       <c r="CY140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CZ140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -45444,6 +45867,9 @@
       <c r="CY141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CZ141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -45761,6 +46187,9 @@
       <c r="CY142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="CZ142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -46078,6 +46507,9 @@
       <c r="CY143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CZ143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -46395,6 +46827,9 @@
       <c r="CY144" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CZ144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -46712,6 +47147,9 @@
       <c r="CY145" s="3" t="n">
         <v>23.19</v>
       </c>
+      <c r="CZ145" s="3" t="n">
+        <v>23.19</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -47029,6 +47467,9 @@
       <c r="CY146" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CZ146" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -47346,6 +47787,9 @@
       <c r="CY147" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CZ147" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -47663,6 +48107,9 @@
       <c r="CY148" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CZ148" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -47980,6 +48427,9 @@
       <c r="CY149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CZ149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -48297,6 +48747,9 @@
       <c r="CY150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CZ150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -48614,6 +49067,9 @@
       <c r="CY151" s="3" t="n">
         <v>23.39</v>
       </c>
+      <c r="CZ151" s="3" t="n">
+        <v>23.39</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -48931,6 +49387,9 @@
       <c r="CY152" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CZ152" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -49248,6 +49707,9 @@
       <c r="CY153" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CZ153" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -49565,6 +50027,9 @@
       <c r="CY154" s="3" t="n">
         <v>23.7</v>
       </c>
+      <c r="CZ154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -49882,6 +50347,9 @@
       <c r="CY155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="CZ155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -50199,6 +50667,9 @@
       <c r="CY156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CZ156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -50516,6 +50987,9 @@
       <c r="CY157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="CZ157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -50833,6 +51307,9 @@
       <c r="CY158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CZ158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -51150,6 +51627,9 @@
       <c r="CY159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CZ159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -51467,6 +51947,9 @@
       <c r="CY160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CZ160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -51784,6 +52267,9 @@
       <c r="CY161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="CZ161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -52101,6 +52587,9 @@
       <c r="CY162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="CZ162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -52418,6 +52907,9 @@
       <c r="CY163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="CZ163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -52735,6 +53227,9 @@
       <c r="CY164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="CZ164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -52953,9 +53448,12 @@
       <c r="CY165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="CZ165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CY165"/>
+  <autoFilter ref="A1:CZ165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-17 12:12 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$CZ$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DA$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CZ165"/>
+  <dimension ref="A1:DA165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -547,6 +547,7 @@
     <col width="16" customWidth="1" min="102" max="102"/>
     <col width="16" customWidth="1" min="103" max="103"/>
     <col width="16" customWidth="1" min="104" max="104"/>
+    <col width="16" customWidth="1" min="105" max="105"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1070,6 +1071,11 @@
           <t>2026-09-17 04:10</t>
         </is>
       </c>
+      <c r="DA1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1390,6 +1396,9 @@
       <c r="CZ2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="DA2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1710,6 +1719,9 @@
       <c r="CZ3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="DA3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2030,6 +2042,9 @@
       <c r="CZ4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="DA4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2350,6 +2365,9 @@
       <c r="CZ5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DA5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2670,6 +2688,9 @@
       <c r="CZ6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DA6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2990,6 +3011,9 @@
       <c r="CZ7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="DA7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3310,6 +3334,9 @@
       <c r="CZ8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DA8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3630,6 +3657,9 @@
       <c r="CZ9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="DA9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3950,6 +3980,9 @@
       <c r="CZ10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DA10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4270,6 +4303,9 @@
       <c r="CZ11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DA11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4590,6 +4626,9 @@
       <c r="CZ12" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA12" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4910,6 +4949,9 @@
       <c r="CZ13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="DA13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5230,6 +5272,9 @@
       <c r="CZ14" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DA14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5550,6 +5595,9 @@
       <c r="CZ15" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DA15" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5870,6 +5918,9 @@
       <c r="CZ16" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DA16" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6190,6 +6241,9 @@
       <c r="CZ17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DA17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -6510,6 +6564,9 @@
       <c r="CZ18" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DA18" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -6830,6 +6887,9 @@
       <c r="CZ19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="DA19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -7150,6 +7210,9 @@
       <c r="CZ20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DA20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -7470,6 +7533,9 @@
       <c r="CZ21" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DA21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -7790,6 +7856,9 @@
       <c r="CZ22" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DA22" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -8110,6 +8179,9 @@
       <c r="CZ23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="DA23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -8430,6 +8502,9 @@
       <c r="CZ24" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DA24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -8750,6 +8825,9 @@
       <c r="CZ25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DA25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -9070,6 +9148,9 @@
       <c r="CZ26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DA26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -9390,6 +9471,9 @@
       <c r="CZ27" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DA27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -9710,6 +9794,9 @@
       <c r="CZ28" s="3" t="n">
         <v>21.84</v>
       </c>
+      <c r="DA28" s="3" t="n">
+        <v>21.84</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -10030,6 +10117,9 @@
       <c r="CZ29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="DA29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -10350,6 +10440,9 @@
       <c r="CZ30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -10670,6 +10763,9 @@
       <c r="CZ31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DA31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -10990,6 +11086,9 @@
       <c r="CZ32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DA32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -11310,6 +11409,9 @@
       <c r="CZ33" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -11630,6 +11732,9 @@
       <c r="CZ34" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DA34" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -11950,6 +12055,9 @@
       <c r="CZ35" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="DA35" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -12270,6 +12378,9 @@
       <c r="CZ36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DA36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -12590,6 +12701,9 @@
       <c r="CZ37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DA37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -12910,6 +13024,9 @@
       <c r="CZ38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DA38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -13230,6 +13347,9 @@
       <c r="CZ39" s="3" t="n">
         <v>21.98</v>
       </c>
+      <c r="DA39" s="3" t="n">
+        <v>21.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -13550,6 +13670,9 @@
       <c r="CZ40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -13870,6 +13993,9 @@
       <c r="CZ41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DA41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -14190,6 +14316,9 @@
       <c r="CZ42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DA42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -14510,6 +14639,9 @@
       <c r="CZ43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DA43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -14830,6 +14962,9 @@
       <c r="CZ44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -15150,6 +15285,9 @@
       <c r="CZ45" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DA45" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -15470,6 +15608,9 @@
       <c r="CZ46" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="DA46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -15790,6 +15931,9 @@
       <c r="CZ47" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DA47" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -16110,6 +16254,9 @@
       <c r="CZ48" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DA48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -16430,6 +16577,9 @@
       <c r="CZ49" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DA49" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -16750,6 +16900,9 @@
       <c r="CZ50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="DA50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -17070,6 +17223,9 @@
       <c r="CZ51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DA51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -17390,6 +17546,9 @@
       <c r="CZ52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DA52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -17710,6 +17869,9 @@
       <c r="CZ53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="DA53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -18030,6 +18192,9 @@
       <c r="CZ54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -18350,6 +18515,9 @@
       <c r="CZ55" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DA55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -18670,6 +18838,9 @@
       <c r="CZ56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -18990,6 +19161,9 @@
       <c r="CZ57" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DA57" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -19310,6 +19484,9 @@
       <c r="CZ58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="DA58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -19630,6 +19807,9 @@
       <c r="CZ59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="DA59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -19950,6 +20130,9 @@
       <c r="CZ60" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DA60" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -20270,6 +20453,9 @@
       <c r="CZ61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DA61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -20590,6 +20776,9 @@
       <c r="CZ62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DA62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -20910,6 +21099,9 @@
       <c r="CZ63" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DA63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -21230,6 +21422,9 @@
       <c r="CZ64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DA64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -21550,6 +21745,9 @@
       <c r="CZ65" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="DA65" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -21870,6 +22068,9 @@
       <c r="CZ66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -22190,6 +22391,9 @@
       <c r="CZ67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DA67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -22510,6 +22714,9 @@
       <c r="CZ68" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DA68" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -22830,6 +23037,9 @@
       <c r="CZ69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DA69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -23150,6 +23360,9 @@
       <c r="CZ70" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA70" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -23470,6 +23683,9 @@
       <c r="CZ71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -23790,6 +24006,9 @@
       <c r="CZ72" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DA72" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -24110,6 +24329,9 @@
       <c r="CZ73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DA73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -24430,6 +24652,9 @@
       <c r="CZ74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DA74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -24750,6 +24975,9 @@
       <c r="CZ75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -25070,6 +25298,9 @@
       <c r="CZ76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -25390,6 +25621,9 @@
       <c r="CZ77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="DA77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -25710,6 +25944,9 @@
       <c r="CZ78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DA78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -26030,6 +26267,9 @@
       <c r="CZ79" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DA79" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -26350,6 +26590,9 @@
       <c r="CZ80" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DA80" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -26670,6 +26913,9 @@
       <c r="CZ81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -26990,6 +27236,9 @@
       <c r="CZ82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DA82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -27310,6 +27559,9 @@
       <c r="CZ83" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA83" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -27630,6 +27882,9 @@
       <c r="CZ84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DA84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -27950,6 +28205,9 @@
       <c r="CZ85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="DA85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -28270,6 +28528,9 @@
       <c r="CZ86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="DA86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -28590,6 +28851,9 @@
       <c r="CZ87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DA87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -28910,6 +29174,9 @@
       <c r="CZ88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -29230,6 +29497,9 @@
       <c r="CZ89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DA89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -29550,6 +29820,9 @@
       <c r="CZ90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -29870,6 +30143,9 @@
       <c r="CZ91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -30190,6 +30466,9 @@
       <c r="CZ92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -30510,6 +30789,9 @@
       <c r="CZ93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DA93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -30830,6 +31112,9 @@
       <c r="CZ94" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DA94" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -31150,6 +31435,9 @@
       <c r="CZ95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DA95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -31470,6 +31758,9 @@
       <c r="CZ96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="DA96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -31790,6 +32081,9 @@
       <c r="CZ97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DA97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -32110,6 +32404,9 @@
       <c r="CZ98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DA98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -32430,6 +32727,9 @@
       <c r="CZ99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DA99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -32750,6 +33050,9 @@
       <c r="CZ100" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DA100" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -33070,6 +33373,9 @@
       <c r="CZ101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -33390,6 +33696,9 @@
       <c r="CZ102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="DA102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -33710,6 +34019,9 @@
       <c r="CZ103" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA103" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -34030,6 +34342,9 @@
       <c r="CZ104" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -34350,6 +34665,9 @@
       <c r="CZ105" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA105" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -34670,6 +34988,9 @@
       <c r="CZ106" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA106" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -34990,6 +35311,9 @@
       <c r="CZ107" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DA107" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -35310,6 +35634,9 @@
       <c r="CZ108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DA108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -35630,6 +35957,9 @@
       <c r="CZ109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -35950,6 +36280,9 @@
       <c r="CZ110" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="DA110" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -36270,6 +36603,9 @@
       <c r="CZ111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DA111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -36590,6 +36926,9 @@
       <c r="CZ112" s="3" t="n">
         <v>23.8</v>
       </c>
+      <c r="DA112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -36910,6 +37249,9 @@
       <c r="CZ113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DA113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -37230,6 +37572,9 @@
       <c r="CZ114" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA114" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -37550,6 +37895,9 @@
       <c r="CZ115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DA115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -37870,6 +38218,9 @@
       <c r="CZ116" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DA116" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -38190,6 +38541,9 @@
       <c r="CZ117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DA117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -38510,6 +38864,9 @@
       <c r="CZ118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DA118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -38830,6 +39187,9 @@
       <c r="CZ119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="DA119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -39150,6 +39510,9 @@
       <c r="CZ120" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA120" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -39470,6 +39833,9 @@
       <c r="CZ121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DA121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -39790,6 +40156,9 @@
       <c r="CZ122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DA122" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -40110,6 +40479,9 @@
       <c r="CZ123" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DA123" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -40430,6 +40802,9 @@
       <c r="CZ124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="DA124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -40750,6 +41125,9 @@
       <c r="CZ125" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA125" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -41070,6 +41448,9 @@
       <c r="CZ126" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA126" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -41390,6 +41771,9 @@
       <c r="CZ127" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DA127" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -41710,6 +42094,9 @@
       <c r="CZ128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="DA128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -42030,6 +42417,9 @@
       <c r="CZ129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DA129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -42350,6 +42740,9 @@
       <c r="CZ130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DA130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -42670,6 +43063,9 @@
       <c r="CZ131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="DA131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -42990,6 +43386,9 @@
       <c r="CZ132" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DA132" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -43310,6 +43709,9 @@
       <c r="CZ133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DA133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -43630,6 +44032,9 @@
       <c r="CZ134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="DA134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -43950,6 +44355,9 @@
       <c r="CZ135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DA135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -44270,6 +44678,9 @@
       <c r="CZ136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DA136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -44590,6 +45001,9 @@
       <c r="CZ137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DA137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -44910,6 +45324,9 @@
       <c r="CZ138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DA138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -45230,6 +45647,9 @@
       <c r="CZ139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DA139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -45550,6 +45970,9 @@
       <c r="CZ140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DA140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -45870,6 +46293,9 @@
       <c r="CZ141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DA141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -46190,6 +46616,9 @@
       <c r="CZ142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DA142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -46510,6 +46939,9 @@
       <c r="CZ143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DA143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -46830,6 +47262,9 @@
       <c r="CZ144" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DA144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -47150,6 +47585,9 @@
       <c r="CZ145" s="3" t="n">
         <v>23.19</v>
       </c>
+      <c r="DA145" s="3" t="n">
+        <v>23.19</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -47470,6 +47908,9 @@
       <c r="CZ146" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DA146" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -47790,6 +48231,9 @@
       <c r="CZ147" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DA147" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -48110,6 +48554,9 @@
       <c r="CZ148" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DA148" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -48430,6 +48877,9 @@
       <c r="CZ149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DA149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -48750,6 +49200,9 @@
       <c r="CZ150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DA150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -49070,6 +49523,9 @@
       <c r="CZ151" s="3" t="n">
         <v>23.39</v>
       </c>
+      <c r="DA151" s="3" t="n">
+        <v>23.39</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -49390,6 +49846,9 @@
       <c r="CZ152" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DA152" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -49710,6 +50169,9 @@
       <c r="CZ153" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DA153" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -50030,6 +50492,9 @@
       <c r="CZ154" s="3" t="n">
         <v>23.7</v>
       </c>
+      <c r="DA154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -50350,6 +50815,9 @@
       <c r="CZ155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DA155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -50670,6 +51138,9 @@
       <c r="CZ156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DA156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -50990,6 +51461,9 @@
       <c r="CZ157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DA157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -51310,6 +51784,9 @@
       <c r="CZ158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DA158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -51630,6 +52107,9 @@
       <c r="CZ159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DA159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -51950,6 +52430,9 @@
       <c r="CZ160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DA160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -52270,6 +52753,9 @@
       <c r="CZ161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DA161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -52590,6 +53076,9 @@
       <c r="CZ162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DA162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -52910,6 +53399,9 @@
       <c r="CZ163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DA163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -53230,6 +53722,9 @@
       <c r="CZ164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="DA164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -53451,9 +53946,12 @@
       <c r="CZ165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="DA165" s="3" t="n">
+        <v>20.59</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CZ165"/>
+  <autoFilter ref="A1:DA165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-17 15:10 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DA$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DB$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DA165"/>
+  <dimension ref="A1:DB165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -548,6 +548,7 @@
     <col width="16" customWidth="1" min="103" max="103"/>
     <col width="16" customWidth="1" min="104" max="104"/>
     <col width="16" customWidth="1" min="105" max="105"/>
+    <col width="16" customWidth="1" min="106" max="106"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1076,6 +1077,11 @@
           <t>2026-09-17 07:12</t>
         </is>
       </c>
+      <c r="DB1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-17 10:10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1399,6 +1405,9 @@
       <c r="DA2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="DB2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1722,6 +1731,9 @@
       <c r="DA3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="DB3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2045,6 +2057,9 @@
       <c r="DA4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="DB4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2368,6 +2383,9 @@
       <c r="DA5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DB5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2691,6 +2709,9 @@
       <c r="DA6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DB6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3014,6 +3035,9 @@
       <c r="DA7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="DB7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3337,6 +3361,9 @@
       <c r="DA8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DB8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3660,6 +3687,9 @@
       <c r="DA9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="DB9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3983,6 +4013,9 @@
       <c r="DA10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DB10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4306,6 +4339,9 @@
       <c r="DA11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DB11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4629,6 +4665,9 @@
       <c r="DA12" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB12" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4952,6 +4991,9 @@
       <c r="DA13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="DB13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5275,6 +5317,9 @@
       <c r="DA14" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DB14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5598,6 +5643,9 @@
       <c r="DA15" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DB15" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5921,6 +5969,9 @@
       <c r="DA16" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DB16" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6244,6 +6295,9 @@
       <c r="DA17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DB17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -6567,6 +6621,9 @@
       <c r="DA18" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DB18" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -6890,6 +6947,9 @@
       <c r="DA19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="DB19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -7213,6 +7273,9 @@
       <c r="DA20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DB20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -7536,6 +7599,9 @@
       <c r="DA21" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DB21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -7859,6 +7925,9 @@
       <c r="DA22" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DB22" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -8182,6 +8251,9 @@
       <c r="DA23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="DB23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -8505,6 +8577,9 @@
       <c r="DA24" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DB24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -8828,6 +8903,9 @@
       <c r="DA25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DB25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -9151,6 +9229,9 @@
       <c r="DA26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DB26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -9474,6 +9555,9 @@
       <c r="DA27" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DB27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -9797,6 +9881,9 @@
       <c r="DA28" s="3" t="n">
         <v>21.84</v>
       </c>
+      <c r="DB28" s="3" t="n">
+        <v>21.84</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -10120,6 +10207,9 @@
       <c r="DA29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="DB29" s="3" t="n">
+        <v>20.89</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -10443,6 +10533,9 @@
       <c r="DA30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -10766,6 +10859,9 @@
       <c r="DA31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DB31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -11089,6 +11185,9 @@
       <c r="DA32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DB32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -11412,6 +11511,9 @@
       <c r="DA33" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -11735,6 +11837,9 @@
       <c r="DA34" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DB34" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -12058,6 +12163,9 @@
       <c r="DA35" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="DB35" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -12381,6 +12489,9 @@
       <c r="DA36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DB36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -12704,6 +12815,9 @@
       <c r="DA37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DB37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -13027,6 +13141,9 @@
       <c r="DA38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DB38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -13350,6 +13467,9 @@
       <c r="DA39" s="3" t="n">
         <v>21.98</v>
       </c>
+      <c r="DB39" s="3" t="n">
+        <v>21.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -13673,6 +13793,9 @@
       <c r="DA40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -13996,6 +14119,9 @@
       <c r="DA41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DB41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -14319,6 +14445,9 @@
       <c r="DA42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DB42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -14642,6 +14771,9 @@
       <c r="DA43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DB43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -14965,6 +15097,9 @@
       <c r="DA44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -15288,6 +15423,9 @@
       <c r="DA45" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DB45" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -15611,6 +15749,9 @@
       <c r="DA46" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="DB46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -15934,6 +16075,9 @@
       <c r="DA47" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DB47" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -16257,6 +16401,9 @@
       <c r="DA48" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DB48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -16580,6 +16727,9 @@
       <c r="DA49" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DB49" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -16903,6 +17053,9 @@
       <c r="DA50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="DB50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -17226,6 +17379,9 @@
       <c r="DA51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DB51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -17549,6 +17705,9 @@
       <c r="DA52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DB52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -17872,6 +18031,9 @@
       <c r="DA53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="DB53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -18195,6 +18357,9 @@
       <c r="DA54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -18518,6 +18683,9 @@
       <c r="DA55" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DB55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -18841,6 +19009,9 @@
       <c r="DA56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -19164,6 +19335,9 @@
       <c r="DA57" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DB57" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -19487,6 +19661,9 @@
       <c r="DA58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="DB58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -19810,6 +19987,9 @@
       <c r="DA59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="DB59" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -20133,6 +20313,9 @@
       <c r="DA60" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DB60" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -20456,6 +20639,9 @@
       <c r="DA61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DB61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -20779,6 +20965,9 @@
       <c r="DA62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DB62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -21102,6 +21291,9 @@
       <c r="DA63" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DB63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -21425,6 +21617,9 @@
       <c r="DA64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DB64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -21748,6 +21943,9 @@
       <c r="DA65" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="DB65" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -22071,6 +22269,9 @@
       <c r="DA66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -22394,6 +22595,9 @@
       <c r="DA67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DB67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -22717,6 +22921,9 @@
       <c r="DA68" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DB68" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -23040,6 +23247,9 @@
       <c r="DA69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DB69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -23363,6 +23573,9 @@
       <c r="DA70" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB70" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -23686,6 +23899,9 @@
       <c r="DA71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -24009,6 +24225,9 @@
       <c r="DA72" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DB72" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -24332,6 +24551,9 @@
       <c r="DA73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DB73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -24655,6 +24877,9 @@
       <c r="DA74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DB74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -24978,6 +25203,9 @@
       <c r="DA75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -25301,6 +25529,9 @@
       <c r="DA76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -25624,6 +25855,9 @@
       <c r="DA77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="DB77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -25947,6 +26181,9 @@
       <c r="DA78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DB78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -26270,6 +26507,9 @@
       <c r="DA79" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DB79" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -26593,6 +26833,9 @@
       <c r="DA80" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DB80" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -26916,6 +27159,9 @@
       <c r="DA81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -27239,6 +27485,9 @@
       <c r="DA82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DB82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -27562,6 +27811,9 @@
       <c r="DA83" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB83" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -27885,6 +28137,9 @@
       <c r="DA84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DB84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -28208,6 +28463,9 @@
       <c r="DA85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="DB85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -28531,6 +28789,9 @@
       <c r="DA86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="DB86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -28854,6 +29115,9 @@
       <c r="DA87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DB87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -29177,6 +29441,9 @@
       <c r="DA88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -29500,6 +29767,9 @@
       <c r="DA89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DB89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -29823,6 +30093,9 @@
       <c r="DA90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -30146,6 +30419,9 @@
       <c r="DA91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -30469,6 +30745,9 @@
       <c r="DA92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -30792,6 +31071,9 @@
       <c r="DA93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DB93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -31115,6 +31397,9 @@
       <c r="DA94" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DB94" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -31438,6 +31723,9 @@
       <c r="DA95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DB95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -31761,6 +32049,9 @@
       <c r="DA96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="DB96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -32084,6 +32375,9 @@
       <c r="DA97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DB97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -32407,6 +32701,9 @@
       <c r="DA98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DB98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -32730,6 +33027,9 @@
       <c r="DA99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DB99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -33053,6 +33353,9 @@
       <c r="DA100" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DB100" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -33376,6 +33679,9 @@
       <c r="DA101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -33699,6 +34005,9 @@
       <c r="DA102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="DB102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -34022,6 +34331,9 @@
       <c r="DA103" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB103" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -34345,6 +34657,9 @@
       <c r="DA104" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -34668,6 +34983,9 @@
       <c r="DA105" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB105" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -34991,6 +35309,9 @@
       <c r="DA106" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB106" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -35314,6 +35635,9 @@
       <c r="DA107" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DB107" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -35637,6 +35961,9 @@
       <c r="DA108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DB108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -35960,6 +36287,9 @@
       <c r="DA109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -36283,6 +36613,9 @@
       <c r="DA110" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="DB110" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -36606,6 +36939,9 @@
       <c r="DA111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DB111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -36929,6 +37265,9 @@
       <c r="DA112" s="3" t="n">
         <v>23.8</v>
       </c>
+      <c r="DB112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -37252,6 +37591,9 @@
       <c r="DA113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DB113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -37575,6 +37917,9 @@
       <c r="DA114" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB114" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -37898,6 +38243,9 @@
       <c r="DA115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DB115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -38221,6 +38569,9 @@
       <c r="DA116" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DB116" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -38544,6 +38895,9 @@
       <c r="DA117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DB117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -38867,6 +39221,9 @@
       <c r="DA118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DB118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -39190,6 +39547,9 @@
       <c r="DA119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="DB119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -39513,6 +39873,9 @@
       <c r="DA120" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB120" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -39836,6 +40199,9 @@
       <c r="DA121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DB121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -40159,6 +40525,9 @@
       <c r="DA122" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DB122" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -40482,6 +40851,9 @@
       <c r="DA123" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DB123" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -40805,6 +41177,9 @@
       <c r="DA124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="DB124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -41128,6 +41503,9 @@
       <c r="DA125" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB125" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -41451,6 +41829,9 @@
       <c r="DA126" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB126" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -41774,6 +42155,9 @@
       <c r="DA127" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DB127" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -42097,6 +42481,9 @@
       <c r="DA128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="DB128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -42420,6 +42807,9 @@
       <c r="DA129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DB129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -42743,6 +43133,9 @@
       <c r="DA130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DB130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -43066,6 +43459,9 @@
       <c r="DA131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="DB131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -43389,6 +43785,9 @@
       <c r="DA132" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DB132" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -43712,6 +44111,9 @@
       <c r="DA133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DB133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -44035,6 +44437,9 @@
       <c r="DA134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="DB134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -44358,6 +44763,9 @@
       <c r="DA135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DB135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -44681,6 +45089,9 @@
       <c r="DA136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DB136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -45004,6 +45415,9 @@
       <c r="DA137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DB137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -45327,6 +45741,9 @@
       <c r="DA138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DB138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -45650,6 +46067,9 @@
       <c r="DA139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DB139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -45973,6 +46393,9 @@
       <c r="DA140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DB140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -46296,6 +46719,9 @@
       <c r="DA141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DB141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -46619,6 +47045,9 @@
       <c r="DA142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DB142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -46942,6 +47371,9 @@
       <c r="DA143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DB143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -47265,6 +47697,9 @@
       <c r="DA144" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DB144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -47588,6 +48023,9 @@
       <c r="DA145" s="3" t="n">
         <v>23.19</v>
       </c>
+      <c r="DB145" s="3" t="n">
+        <v>23.19</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -47911,6 +48349,9 @@
       <c r="DA146" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DB146" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -48234,6 +48675,9 @@
       <c r="DA147" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DB147" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -48557,6 +49001,9 @@
       <c r="DA148" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DB148" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -48880,6 +49327,9 @@
       <c r="DA149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DB149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -49203,6 +49653,9 @@
       <c r="DA150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DB150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -49526,6 +49979,9 @@
       <c r="DA151" s="3" t="n">
         <v>23.39</v>
       </c>
+      <c r="DB151" s="3" t="n">
+        <v>23.39</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -49849,6 +50305,9 @@
       <c r="DA152" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DB152" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -50172,6 +50631,9 @@
       <c r="DA153" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DB153" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -50495,6 +50957,9 @@
       <c r="DA154" s="3" t="n">
         <v>23.7</v>
       </c>
+      <c r="DB154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -50818,6 +51283,9 @@
       <c r="DA155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DB155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -51141,6 +51609,9 @@
       <c r="DA156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DB156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -51464,6 +51935,9 @@
       <c r="DA157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DB157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -51787,6 +52261,9 @@
       <c r="DA158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DB158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -52110,6 +52587,9 @@
       <c r="DA159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DB159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -52433,6 +52913,9 @@
       <c r="DA160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DB160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -52756,6 +53239,9 @@
       <c r="DA161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DB161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -53079,6 +53565,9 @@
       <c r="DA162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DB162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -53402,6 +53891,9 @@
       <c r="DA163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DB163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -53725,6 +54217,9 @@
       <c r="DA164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="DB164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -53949,9 +54444,12 @@
       <c r="DA165" s="3" t="n">
         <v>20.59</v>
       </c>
+      <c r="DB165" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:DA165"/>
+  <autoFilter ref="A1:DB165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-17 18:11 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DB$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DC$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DB165"/>
+  <dimension ref="A1:DC165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -549,6 +549,7 @@
     <col width="16" customWidth="1" min="104" max="104"/>
     <col width="16" customWidth="1" min="105" max="105"/>
     <col width="16" customWidth="1" min="106" max="106"/>
+    <col width="16" customWidth="1" min="107" max="107"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1082,6 +1083,11 @@
           <t>2026-09-17 10:10</t>
         </is>
       </c>
+      <c r="DC1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-17 13:11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1408,6 +1414,9 @@
       <c r="DB2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="DC2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1734,6 +1743,9 @@
       <c r="DB3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="DC3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2060,6 +2072,9 @@
       <c r="DB4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="DC4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2386,6 +2401,9 @@
       <c r="DB5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DC5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2712,6 +2730,9 @@
       <c r="DB6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DC6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3038,6 +3059,9 @@
       <c r="DB7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="DC7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3364,6 +3388,9 @@
       <c r="DB8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DC8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3690,6 +3717,9 @@
       <c r="DB9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="DC9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4016,6 +4046,9 @@
       <c r="DB10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DC10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4342,6 +4375,9 @@
       <c r="DB11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DC11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4668,6 +4704,9 @@
       <c r="DB12" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC12" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -4994,6 +5033,9 @@
       <c r="DB13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="DC13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5320,6 +5362,9 @@
       <c r="DB14" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DC14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5646,6 +5691,9 @@
       <c r="DB15" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DC15" s="3" t="n">
+        <v>21.41</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -5972,6 +6020,9 @@
       <c r="DB16" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DC16" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6298,6 +6349,9 @@
       <c r="DB17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DC17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -6624,6 +6678,9 @@
       <c r="DB18" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DC18" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -6950,6 +7007,9 @@
       <c r="DB19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="DC19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -7276,6 +7336,9 @@
       <c r="DB20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DC20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -7602,6 +7665,9 @@
       <c r="DB21" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DC21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -7928,6 +7994,9 @@
       <c r="DB22" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DC22" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -8254,6 +8323,9 @@
       <c r="DB23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="DC23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -8580,6 +8652,9 @@
       <c r="DB24" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DC24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -8906,6 +8981,9 @@
       <c r="DB25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DC25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -9232,6 +9310,9 @@
       <c r="DB26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DC26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -9558,6 +9639,9 @@
       <c r="DB27" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DC27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -9884,6 +9968,9 @@
       <c r="DB28" s="3" t="n">
         <v>21.84</v>
       </c>
+      <c r="DC28" s="3" t="n">
+        <v>21.84</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -10210,6 +10297,9 @@
       <c r="DB29" s="3" t="n">
         <v>20.89</v>
       </c>
+      <c r="DC29" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -10536,6 +10626,9 @@
       <c r="DB30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -10862,6 +10955,9 @@
       <c r="DB31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DC31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -11188,6 +11284,9 @@
       <c r="DB32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DC32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -11514,6 +11613,9 @@
       <c r="DB33" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -11840,6 +11942,9 @@
       <c r="DB34" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DC34" s="3" t="n">
+        <v>21.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -12166,6 +12271,9 @@
       <c r="DB35" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="DC35" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -12492,6 +12600,9 @@
       <c r="DB36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DC36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -12818,6 +12929,9 @@
       <c r="DB37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DC37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -13144,6 +13258,9 @@
       <c r="DB38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DC38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -13470,6 +13587,9 @@
       <c r="DB39" s="3" t="n">
         <v>21.98</v>
       </c>
+      <c r="DC39" s="3" t="n">
+        <v>21.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -13796,6 +13916,9 @@
       <c r="DB40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -14122,6 +14245,9 @@
       <c r="DB41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DC41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -14448,6 +14574,9 @@
       <c r="DB42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DC42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -14774,6 +14903,9 @@
       <c r="DB43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DC43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -15100,6 +15232,9 @@
       <c r="DB44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -15426,6 +15561,9 @@
       <c r="DB45" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DC45" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -15752,6 +15890,9 @@
       <c r="DB46" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="DC46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -16078,6 +16219,9 @@
       <c r="DB47" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DC47" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -16404,6 +16548,9 @@
       <c r="DB48" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DC48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -16730,6 +16877,9 @@
       <c r="DB49" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DC49" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -17056,6 +17206,9 @@
       <c r="DB50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="DC50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -17382,6 +17535,9 @@
       <c r="DB51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DC51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -17708,6 +17864,9 @@
       <c r="DB52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DC52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -18034,6 +18193,9 @@
       <c r="DB53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="DC53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -18360,6 +18522,9 @@
       <c r="DB54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -18686,6 +18851,9 @@
       <c r="DB55" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DC55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -19012,6 +19180,9 @@
       <c r="DB56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -19338,6 +19509,9 @@
       <c r="DB57" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DC57" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -19664,6 +19838,9 @@
       <c r="DB58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="DC58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -19990,6 +20167,9 @@
       <c r="DB59" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="DC59" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -20316,6 +20496,9 @@
       <c r="DB60" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DC60" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -20642,6 +20825,9 @@
       <c r="DB61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DC61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -20968,6 +21154,9 @@
       <c r="DB62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DC62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -21294,6 +21483,9 @@
       <c r="DB63" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DC63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -21620,6 +21812,9 @@
       <c r="DB64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DC64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -21946,6 +22141,9 @@
       <c r="DB65" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="DC65" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -22272,6 +22470,9 @@
       <c r="DB66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -22598,6 +22799,9 @@
       <c r="DB67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DC67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -22924,6 +23128,9 @@
       <c r="DB68" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DC68" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -23250,6 +23457,9 @@
       <c r="DB69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DC69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -23576,6 +23786,9 @@
       <c r="DB70" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC70" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -23902,6 +24115,9 @@
       <c r="DB71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -24228,6 +24444,9 @@
       <c r="DB72" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DC72" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -24554,6 +24773,9 @@
       <c r="DB73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DC73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -24880,6 +25102,9 @@
       <c r="DB74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DC74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -25206,6 +25431,9 @@
       <c r="DB75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -25532,6 +25760,9 @@
       <c r="DB76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -25858,6 +26089,9 @@
       <c r="DB77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="DC77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -26184,6 +26418,9 @@
       <c r="DB78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DC78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -26510,6 +26747,9 @@
       <c r="DB79" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DC79" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -26836,6 +27076,9 @@
       <c r="DB80" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DC80" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -27162,6 +27405,9 @@
       <c r="DB81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -27488,6 +27734,9 @@
       <c r="DB82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DC82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -27814,6 +28063,9 @@
       <c r="DB83" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC83" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -28140,6 +28392,9 @@
       <c r="DB84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DC84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -28466,6 +28721,9 @@
       <c r="DB85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="DC85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -28792,6 +29050,9 @@
       <c r="DB86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="DC86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -29118,6 +29379,9 @@
       <c r="DB87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DC87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -29444,6 +29708,9 @@
       <c r="DB88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -29770,6 +30037,9 @@
       <c r="DB89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DC89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -30096,6 +30366,9 @@
       <c r="DB90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -30422,6 +30695,9 @@
       <c r="DB91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -30748,6 +31024,9 @@
       <c r="DB92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -31074,6 +31353,9 @@
       <c r="DB93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DC93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -31400,6 +31682,9 @@
       <c r="DB94" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DC94" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -31726,6 +32011,9 @@
       <c r="DB95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DC95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -32052,6 +32340,9 @@
       <c r="DB96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="DC96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -32378,6 +32669,9 @@
       <c r="DB97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DC97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -32704,6 +32998,9 @@
       <c r="DB98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DC98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -33030,6 +33327,9 @@
       <c r="DB99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DC99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -33356,6 +33656,9 @@
       <c r="DB100" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DC100" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -33682,6 +33985,9 @@
       <c r="DB101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -34008,6 +34314,9 @@
       <c r="DB102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="DC102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -34334,6 +34643,9 @@
       <c r="DB103" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC103" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -34660,6 +34972,9 @@
       <c r="DB104" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -34986,6 +35301,9 @@
       <c r="DB105" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC105" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -35312,6 +35630,9 @@
       <c r="DB106" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC106" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -35638,6 +35959,9 @@
       <c r="DB107" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DC107" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -35964,6 +36288,9 @@
       <c r="DB108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DC108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -36290,6 +36617,9 @@
       <c r="DB109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -36616,6 +36946,9 @@
       <c r="DB110" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="DC110" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -36942,6 +37275,9 @@
       <c r="DB111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DC111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -37268,6 +37604,9 @@
       <c r="DB112" s="3" t="n">
         <v>23.8</v>
       </c>
+      <c r="DC112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -37594,6 +37933,9 @@
       <c r="DB113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DC113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -37920,6 +38262,9 @@
       <c r="DB114" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC114" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -38246,6 +38591,9 @@
       <c r="DB115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DC115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -38572,6 +38920,9 @@
       <c r="DB116" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DC116" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -38898,6 +39249,9 @@
       <c r="DB117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DC117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -39224,6 +39578,9 @@
       <c r="DB118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DC118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -39550,6 +39907,9 @@
       <c r="DB119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="DC119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -39876,6 +40236,9 @@
       <c r="DB120" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC120" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -40202,6 +40565,9 @@
       <c r="DB121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DC121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -40528,6 +40894,9 @@
       <c r="DB122" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC122" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -40854,6 +41223,9 @@
       <c r="DB123" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DC123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -41180,6 +41552,9 @@
       <c r="DB124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="DC124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -41506,6 +41881,9 @@
       <c r="DB125" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC125" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -41832,6 +42210,9 @@
       <c r="DB126" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC126" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -42158,6 +42539,9 @@
       <c r="DB127" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DC127" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -42484,6 +42868,9 @@
       <c r="DB128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="DC128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -42810,6 +43197,9 @@
       <c r="DB129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DC129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -43136,6 +43526,9 @@
       <c r="DB130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DC130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -43462,6 +43855,9 @@
       <c r="DB131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="DC131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -43788,6 +44184,9 @@
       <c r="DB132" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DC132" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -44114,6 +44513,9 @@
       <c r="DB133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DC133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -44440,6 +44842,9 @@
       <c r="DB134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="DC134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -44766,6 +45171,9 @@
       <c r="DB135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DC135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -45092,6 +45500,9 @@
       <c r="DB136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DC136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -45418,6 +45829,9 @@
       <c r="DB137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DC137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -45744,6 +46158,9 @@
       <c r="DB138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DC138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -46070,6 +46487,9 @@
       <c r="DB139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DC139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -46396,6 +46816,9 @@
       <c r="DB140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DC140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -46722,6 +47145,9 @@
       <c r="DB141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DC141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -47048,6 +47474,9 @@
       <c r="DB142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DC142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -47374,6 +47803,9 @@
       <c r="DB143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DC143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -47700,6 +48132,9 @@
       <c r="DB144" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DC144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -48026,6 +48461,9 @@
       <c r="DB145" s="3" t="n">
         <v>23.19</v>
       </c>
+      <c r="DC145" s="3" t="n">
+        <v>23.19</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -48352,6 +48790,9 @@
       <c r="DB146" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DC146" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -48678,6 +49119,9 @@
       <c r="DB147" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DC147" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -49004,6 +49448,9 @@
       <c r="DB148" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DC148" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -49330,6 +49777,9 @@
       <c r="DB149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DC149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -49656,6 +50106,9 @@
       <c r="DB150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DC150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -49982,6 +50435,9 @@
       <c r="DB151" s="3" t="n">
         <v>23.39</v>
       </c>
+      <c r="DC151" s="3" t="n">
+        <v>23.39</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -50308,6 +50764,9 @@
       <c r="DB152" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DC152" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -50634,6 +51093,9 @@
       <c r="DB153" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DC153" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -50960,6 +51422,9 @@
       <c r="DB154" s="3" t="n">
         <v>23.7</v>
       </c>
+      <c r="DC154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -51286,6 +51751,9 @@
       <c r="DB155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DC155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -51612,6 +52080,9 @@
       <c r="DB156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DC156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -51938,6 +52409,9 @@
       <c r="DB157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DC157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -52264,6 +52738,9 @@
       <c r="DB158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DC158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -52590,6 +53067,9 @@
       <c r="DB159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DC159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -52916,6 +53396,9 @@
       <c r="DB160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DC160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -53242,6 +53725,9 @@
       <c r="DB161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DC161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -53568,6 +54054,9 @@
       <c r="DB162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DC162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -53894,6 +54383,9 @@
       <c r="DB163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DC163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -54220,6 +54712,9 @@
       <c r="DB164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="DC164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -54447,9 +54942,12 @@
       <c r="DB165" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DC165" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:DB165"/>
+  <autoFilter ref="A1:DC165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-17 21:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DC$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DD$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DC165"/>
+  <dimension ref="A1:DD165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -550,6 +550,7 @@
     <col width="16" customWidth="1" min="105" max="105"/>
     <col width="16" customWidth="1" min="106" max="106"/>
     <col width="16" customWidth="1" min="107" max="107"/>
+    <col width="16" customWidth="1" min="108" max="108"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1088,6 +1089,11 @@
           <t>2026-09-17 13:11</t>
         </is>
       </c>
+      <c r="DD1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-17 16:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1417,6 +1423,9 @@
       <c r="DC2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="DD2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1746,6 +1755,9 @@
       <c r="DC3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="DD3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2075,6 +2087,9 @@
       <c r="DC4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="DD4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2404,6 +2419,9 @@
       <c r="DC5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DD5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2733,6 +2751,9 @@
       <c r="DC6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DD6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3062,6 +3083,9 @@
       <c r="DC7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="DD7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3391,6 +3415,9 @@
       <c r="DC8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DD8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3720,6 +3747,9 @@
       <c r="DC9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="DD9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4049,6 +4079,9 @@
       <c r="DC10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DD10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4378,6 +4411,9 @@
       <c r="DC11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DD11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4707,6 +4743,9 @@
       <c r="DC12" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD12" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -5036,6 +5075,9 @@
       <c r="DC13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="DD13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5365,6 +5407,9 @@
       <c r="DC14" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DD14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5694,6 +5739,9 @@
       <c r="DC15" s="3" t="n">
         <v>21.41</v>
       </c>
+      <c r="DD15" s="3" t="n">
+        <v>21.41</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -6023,6 +6071,9 @@
       <c r="DC16" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DD16" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6352,6 +6403,9 @@
       <c r="DC17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DD17" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -6681,6 +6735,9 @@
       <c r="DC18" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DD18" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -7010,6 +7067,9 @@
       <c r="DC19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="DD19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -7339,6 +7399,9 @@
       <c r="DC20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DD20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -7668,6 +7731,9 @@
       <c r="DC21" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DD21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -7997,6 +8063,9 @@
       <c r="DC22" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DD22" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -8326,6 +8395,9 @@
       <c r="DC23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="DD23" s="3" t="n">
+        <v>21.09</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -8655,6 +8727,9 @@
       <c r="DC24" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DD24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -8984,6 +9059,9 @@
       <c r="DC25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DD25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -9313,6 +9391,9 @@
       <c r="DC26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DD26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -9642,6 +9723,9 @@
       <c r="DC27" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DD27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -9971,6 +10055,9 @@
       <c r="DC28" s="3" t="n">
         <v>21.84</v>
       </c>
+      <c r="DD28" s="3" t="n">
+        <v>21.84</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -10300,6 +10387,9 @@
       <c r="DC29" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DD29" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -10629,6 +10719,9 @@
       <c r="DC30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -10958,6 +11051,9 @@
       <c r="DC31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DD31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -11287,6 +11383,9 @@
       <c r="DC32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DD32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -11616,6 +11715,9 @@
       <c r="DC33" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -11945,6 +12047,9 @@
       <c r="DC34" s="3" t="n">
         <v>21.77</v>
       </c>
+      <c r="DD34" s="3" t="n">
+        <v>21.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -12274,6 +12379,9 @@
       <c r="DC35" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="DD35" s="3" t="n">
+        <v>20.79</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -12603,6 +12711,9 @@
       <c r="DC36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DD36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -12932,6 +13043,9 @@
       <c r="DC37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DD37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -13261,6 +13375,9 @@
       <c r="DC38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DD38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -13590,6 +13707,9 @@
       <c r="DC39" s="3" t="n">
         <v>21.98</v>
       </c>
+      <c r="DD39" s="3" t="n">
+        <v>21.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -13919,6 +14039,9 @@
       <c r="DC40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -14248,6 +14371,9 @@
       <c r="DC41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DD41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -14577,6 +14703,9 @@
       <c r="DC42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DD42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -14906,6 +15035,9 @@
       <c r="DC43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DD43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -15235,6 +15367,9 @@
       <c r="DC44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -15564,6 +15699,9 @@
       <c r="DC45" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DD45" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -15893,6 +16031,9 @@
       <c r="DC46" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="DD46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -16222,6 +16363,9 @@
       <c r="DC47" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DD47" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -16551,6 +16695,9 @@
       <c r="DC48" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DD48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -16880,6 +17027,9 @@
       <c r="DC49" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DD49" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -17209,6 +17359,9 @@
       <c r="DC50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="DD50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -17538,6 +17691,9 @@
       <c r="DC51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DD51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -17867,6 +18023,9 @@
       <c r="DC52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DD52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -18196,6 +18355,9 @@
       <c r="DC53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="DD53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -18525,6 +18687,9 @@
       <c r="DC54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -18854,6 +19019,9 @@
       <c r="DC55" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DD55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -19183,6 +19351,9 @@
       <c r="DC56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -19512,6 +19683,9 @@
       <c r="DC57" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DD57" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -19841,6 +20015,9 @@
       <c r="DC58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="DD58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -20170,6 +20347,9 @@
       <c r="DC59" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DD59" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -20499,6 +20679,9 @@
       <c r="DC60" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DD60" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -20828,6 +21011,9 @@
       <c r="DC61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DD61" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -21157,6 +21343,9 @@
       <c r="DC62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DD62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -21486,6 +21675,9 @@
       <c r="DC63" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DD63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -21815,6 +22007,9 @@
       <c r="DC64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DD64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -22144,6 +22339,9 @@
       <c r="DC65" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="DD65" s="3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -22473,6 +22671,9 @@
       <c r="DC66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -22802,6 +23003,9 @@
       <c r="DC67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DD67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -23131,6 +23335,9 @@
       <c r="DC68" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DD68" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -23460,6 +23667,9 @@
       <c r="DC69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DD69" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -23789,6 +23999,9 @@
       <c r="DC70" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD70" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -24118,6 +24331,9 @@
       <c r="DC71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -24447,6 +24663,9 @@
       <c r="DC72" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DD72" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -24776,6 +24995,9 @@
       <c r="DC73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DD73" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -25105,6 +25327,9 @@
       <c r="DC74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DD74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -25434,6 +25659,9 @@
       <c r="DC75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -25763,6 +25991,9 @@
       <c r="DC76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -26092,6 +26323,9 @@
       <c r="DC77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="DD77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -26421,6 +26655,9 @@
       <c r="DC78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DD78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -26750,6 +26987,9 @@
       <c r="DC79" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DD79" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -27079,6 +27319,9 @@
       <c r="DC80" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DD80" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -27408,6 +27651,9 @@
       <c r="DC81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -27737,6 +27983,9 @@
       <c r="DC82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DD82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -28066,6 +28315,9 @@
       <c r="DC83" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD83" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -28395,6 +28647,9 @@
       <c r="DC84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DD84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -28724,6 +28979,9 @@
       <c r="DC85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="DD85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -29053,6 +29311,9 @@
       <c r="DC86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="DD86" s="3" t="n">
+        <v>21.37</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -29382,6 +29643,9 @@
       <c r="DC87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DD87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -29711,6 +29975,9 @@
       <c r="DC88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -30040,6 +30307,9 @@
       <c r="DC89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DD89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -30369,6 +30639,9 @@
       <c r="DC90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -30698,6 +30971,9 @@
       <c r="DC91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -31027,6 +31303,9 @@
       <c r="DC92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -31356,6 +31635,9 @@
       <c r="DC93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DD93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -31685,6 +31967,9 @@
       <c r="DC94" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DD94" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -32014,6 +32299,9 @@
       <c r="DC95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DD95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -32343,6 +32631,9 @@
       <c r="DC96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="DD96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -32672,6 +32963,9 @@
       <c r="DC97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DD97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -33001,6 +33295,9 @@
       <c r="DC98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DD98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -33330,6 +33627,9 @@
       <c r="DC99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DD99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -33659,6 +33959,9 @@
       <c r="DC100" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DD100" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -33988,6 +34291,9 @@
       <c r="DC101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -34317,6 +34623,9 @@
       <c r="DC102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="DD102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -34646,6 +34955,9 @@
       <c r="DC103" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD103" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -34975,6 +35287,9 @@
       <c r="DC104" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -35304,6 +35619,9 @@
       <c r="DC105" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD105" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -35633,6 +35951,9 @@
       <c r="DC106" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD106" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -35962,6 +36283,9 @@
       <c r="DC107" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DD107" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -36291,6 +36615,9 @@
       <c r="DC108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DD108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -36620,6 +36947,9 @@
       <c r="DC109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DD109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -36949,6 +37279,9 @@
       <c r="DC110" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="DD110" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -37278,6 +37611,9 @@
       <c r="DC111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DD111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -37607,6 +37943,9 @@
       <c r="DC112" s="3" t="n">
         <v>23.8</v>
       </c>
+      <c r="DD112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -37936,6 +38275,9 @@
       <c r="DC113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DD113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -38265,6 +38607,9 @@
       <c r="DC114" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD114" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -38594,6 +38939,9 @@
       <c r="DC115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DD115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -38923,6 +39271,9 @@
       <c r="DC116" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DD116" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -39252,6 +39603,9 @@
       <c r="DC117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DD117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -39581,6 +39935,9 @@
       <c r="DC118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DD118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -39910,6 +40267,9 @@
       <c r="DC119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="DD119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -40239,6 +40599,9 @@
       <c r="DC120" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD120" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -40568,6 +40931,9 @@
       <c r="DC121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DD121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -40897,6 +41263,9 @@
       <c r="DC122" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD122" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -41226,6 +41595,9 @@
       <c r="DC123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DD123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -41555,6 +41927,9 @@
       <c r="DC124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="DD124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -41884,6 +42259,9 @@
       <c r="DC125" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DD125" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -42213,6 +42591,9 @@
       <c r="DC126" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DD126" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -42542,6 +42923,9 @@
       <c r="DC127" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DD127" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -42871,6 +43255,9 @@
       <c r="DC128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="DD128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -43200,6 +43587,9 @@
       <c r="DC129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DD129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -43529,6 +43919,9 @@
       <c r="DC130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DD130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -43858,6 +44251,9 @@
       <c r="DC131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="DD131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -44187,6 +44583,9 @@
       <c r="DC132" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DD132" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -44516,6 +44915,9 @@
       <c r="DC133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DD133" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -44845,6 +45247,9 @@
       <c r="DC134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="DD134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -45174,6 +45579,9 @@
       <c r="DC135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DD135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -45503,6 +45911,9 @@
       <c r="DC136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DD136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -45832,6 +46243,9 @@
       <c r="DC137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DD137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -46161,6 +46575,9 @@
       <c r="DC138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DD138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -46490,6 +46907,9 @@
       <c r="DC139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DD139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -46819,6 +47239,9 @@
       <c r="DC140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DD140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -47148,6 +47571,9 @@
       <c r="DC141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DD141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -47477,6 +47903,9 @@
       <c r="DC142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DD142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -47806,6 +48235,9 @@
       <c r="DC143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DD143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -48135,6 +48567,9 @@
       <c r="DC144" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DD144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -48464,6 +48899,9 @@
       <c r="DC145" s="3" t="n">
         <v>23.19</v>
       </c>
+      <c r="DD145" s="3" t="n">
+        <v>23.19</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -48793,6 +49231,9 @@
       <c r="DC146" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DD146" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -49122,6 +49563,9 @@
       <c r="DC147" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DD147" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -49451,6 +49895,9 @@
       <c r="DC148" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DD148" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -49780,6 +50227,9 @@
       <c r="DC149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DD149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -50109,6 +50559,9 @@
       <c r="DC150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DD150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -50438,6 +50891,9 @@
       <c r="DC151" s="3" t="n">
         <v>23.39</v>
       </c>
+      <c r="DD151" s="3" t="n">
+        <v>23.39</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -50767,6 +51223,9 @@
       <c r="DC152" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DD152" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -51096,6 +51555,9 @@
       <c r="DC153" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DD153" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -51425,6 +51887,9 @@
       <c r="DC154" s="3" t="n">
         <v>23.7</v>
       </c>
+      <c r="DD154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -51754,6 +52219,9 @@
       <c r="DC155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DD155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -52083,6 +52551,9 @@
       <c r="DC156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DD156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -52412,6 +52883,9 @@
       <c r="DC157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DD157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -52741,6 +53215,9 @@
       <c r="DC158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DD158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -53070,6 +53547,9 @@
       <c r="DC159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DD159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -53399,6 +53879,9 @@
       <c r="DC160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DD160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -53728,6 +54211,9 @@
       <c r="DC161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DD161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -54057,6 +54543,9 @@
       <c r="DC162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DD162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -54386,6 +54875,9 @@
       <c r="DC163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DD163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -54715,6 +55207,9 @@
       <c r="DC164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="DD164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -54945,9 +55440,12 @@
       <c r="DC165" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DD165" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:DC165"/>
+  <autoFilter ref="A1:DD165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-18 00:12 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DD$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DE$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DD165"/>
+  <dimension ref="A1:DE165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -551,6 +551,7 @@
     <col width="16" customWidth="1" min="106" max="106"/>
     <col width="16" customWidth="1" min="107" max="107"/>
     <col width="16" customWidth="1" min="108" max="108"/>
+    <col width="16" customWidth="1" min="109" max="109"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1094,6 +1095,11 @@
           <t>2026-09-17 16:09</t>
         </is>
       </c>
+      <c r="DE1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-17 19:12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1426,6 +1432,9 @@
       <c r="DD2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="DE2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1758,6 +1767,9 @@
       <c r="DD3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="DE3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2090,6 +2102,9 @@
       <c r="DD4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="DE4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2422,6 +2437,9 @@
       <c r="DD5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DE5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2754,6 +2772,9 @@
       <c r="DD6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DE6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3086,6 +3107,9 @@
       <c r="DD7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="DE7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3418,6 +3442,9 @@
       <c r="DD8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DE8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3750,6 +3777,9 @@
       <c r="DD9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="DE9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4082,6 +4112,9 @@
       <c r="DD10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DE10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4414,6 +4447,9 @@
       <c r="DD11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DE11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4746,6 +4782,9 @@
       <c r="DD12" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE12" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -5078,6 +5117,9 @@
       <c r="DD13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="DE13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5410,6 +5452,9 @@
       <c r="DD14" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DE14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5742,6 +5787,9 @@
       <c r="DD15" s="3" t="n">
         <v>21.41</v>
       </c>
+      <c r="DE15" s="3" t="n">
+        <v>21.41</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -6074,6 +6122,9 @@
       <c r="DD16" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DE16" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6406,6 +6457,9 @@
       <c r="DD17" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DE17" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -6738,6 +6792,9 @@
       <c r="DD18" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DE18" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -7070,6 +7127,9 @@
       <c r="DD19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="DE19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -7402,6 +7462,9 @@
       <c r="DD20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DE20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -7734,6 +7797,9 @@
       <c r="DD21" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DE21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -8066,6 +8132,9 @@
       <c r="DD22" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DE22" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -8398,6 +8467,9 @@
       <c r="DD23" s="3" t="n">
         <v>21.09</v>
       </c>
+      <c r="DE23" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -8730,6 +8802,9 @@
       <c r="DD24" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DE24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -9062,6 +9137,9 @@
       <c r="DD25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DE25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -9394,6 +9472,9 @@
       <c r="DD26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DE26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -9726,6 +9807,9 @@
       <c r="DD27" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DE27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -10058,6 +10142,9 @@
       <c r="DD28" s="3" t="n">
         <v>21.84</v>
       </c>
+      <c r="DE28" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -10390,6 +10477,9 @@
       <c r="DD29" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DE29" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -10722,6 +10812,9 @@
       <c r="DD30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -11054,6 +11147,9 @@
       <c r="DD31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DE31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -11386,6 +11482,9 @@
       <c r="DD32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DE32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -11718,6 +11817,9 @@
       <c r="DD33" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -12050,6 +12152,9 @@
       <c r="DD34" s="3" t="n">
         <v>21.77</v>
       </c>
+      <c r="DE34" s="3" t="n">
+        <v>21.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -12382,6 +12487,9 @@
       <c r="DD35" s="3" t="n">
         <v>20.79</v>
       </c>
+      <c r="DE35" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -12714,6 +12822,9 @@
       <c r="DD36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DE36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -13046,6 +13157,9 @@
       <c r="DD37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DE37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -13378,6 +13492,9 @@
       <c r="DD38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DE38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -13710,6 +13827,9 @@
       <c r="DD39" s="3" t="n">
         <v>21.98</v>
       </c>
+      <c r="DE39" s="3" t="n">
+        <v>21.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -14042,6 +14162,9 @@
       <c r="DD40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -14374,6 +14497,9 @@
       <c r="DD41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DE41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -14706,6 +14832,9 @@
       <c r="DD42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DE42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -15038,6 +15167,9 @@
       <c r="DD43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DE43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -15370,6 +15502,9 @@
       <c r="DD44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -15702,6 +15837,9 @@
       <c r="DD45" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DE45" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -16034,6 +16172,9 @@
       <c r="DD46" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="DE46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -16366,6 +16507,9 @@
       <c r="DD47" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DE47" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -16698,6 +16842,9 @@
       <c r="DD48" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DE48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -17030,6 +17177,9 @@
       <c r="DD49" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DE49" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -17362,6 +17512,9 @@
       <c r="DD50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="DE50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -17694,6 +17847,9 @@
       <c r="DD51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DE51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -18026,6 +18182,9 @@
       <c r="DD52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DE52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -18358,6 +18517,9 @@
       <c r="DD53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="DE53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -18690,6 +18852,9 @@
       <c r="DD54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -19022,6 +19187,9 @@
       <c r="DD55" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DE55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -19354,6 +19522,9 @@
       <c r="DD56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -19686,6 +19857,9 @@
       <c r="DD57" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DE57" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -20018,6 +20192,9 @@
       <c r="DD58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="DE58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -20350,6 +20527,9 @@
       <c r="DD59" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DE59" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -20682,6 +20862,9 @@
       <c r="DD60" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DE60" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -21014,6 +21197,9 @@
       <c r="DD61" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DE61" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -21346,6 +21532,9 @@
       <c r="DD62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DE62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -21678,6 +21867,9 @@
       <c r="DD63" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DE63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -22010,6 +22202,9 @@
       <c r="DD64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DE64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -22342,6 +22537,9 @@
       <c r="DD65" s="3" t="n">
         <v>22.29</v>
       </c>
+      <c r="DE65" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -22674,6 +22872,9 @@
       <c r="DD66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -23006,6 +23207,9 @@
       <c r="DD67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DE67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -23338,6 +23542,9 @@
       <c r="DD68" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DE68" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -23670,6 +23877,9 @@
       <c r="DD69" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DE69" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -24002,6 +24212,9 @@
       <c r="DD70" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE70" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -24334,6 +24547,9 @@
       <c r="DD71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -24666,6 +24882,9 @@
       <c r="DD72" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DE72" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -24998,6 +25217,9 @@
       <c r="DD73" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DE73" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -25330,6 +25552,9 @@
       <c r="DD74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DE74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -25662,6 +25887,9 @@
       <c r="DD75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -25994,6 +26222,9 @@
       <c r="DD76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -26326,6 +26557,9 @@
       <c r="DD77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="DE77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -26658,6 +26892,9 @@
       <c r="DD78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DE78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -26990,6 +27227,9 @@
       <c r="DD79" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DE79" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -27322,6 +27562,9 @@
       <c r="DD80" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DE80" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -27654,6 +27897,9 @@
       <c r="DD81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -27986,6 +28232,9 @@
       <c r="DD82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DE82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -28318,6 +28567,9 @@
       <c r="DD83" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE83" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -28650,6 +28902,9 @@
       <c r="DD84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DE84" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -28982,6 +29237,9 @@
       <c r="DD85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="DE85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -29314,6 +29572,9 @@
       <c r="DD86" s="3" t="n">
         <v>21.37</v>
       </c>
+      <c r="DE86" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -29646,6 +29907,9 @@
       <c r="DD87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DE87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -29978,6 +30242,9 @@
       <c r="DD88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -30310,6 +30577,9 @@
       <c r="DD89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DE89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -30642,6 +30912,9 @@
       <c r="DD90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -30974,6 +31247,9 @@
       <c r="DD91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -31306,6 +31582,9 @@
       <c r="DD92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -31638,6 +31917,9 @@
       <c r="DD93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DE93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -31970,6 +32252,9 @@
       <c r="DD94" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DE94" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -32302,6 +32587,9 @@
       <c r="DD95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DE95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -32634,6 +32922,9 @@
       <c r="DD96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="DE96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -32966,6 +33257,9 @@
       <c r="DD97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DE97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -33298,6 +33592,9 @@
       <c r="DD98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DE98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -33630,6 +33927,9 @@
       <c r="DD99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DE99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -33962,6 +34262,9 @@
       <c r="DD100" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DE100" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -34294,6 +34597,9 @@
       <c r="DD101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -34626,6 +34932,9 @@
       <c r="DD102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="DE102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -34958,6 +35267,9 @@
       <c r="DD103" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE103" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -35290,6 +35602,9 @@
       <c r="DD104" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -35622,6 +35937,9 @@
       <c r="DD105" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE105" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -35954,6 +36272,9 @@
       <c r="DD106" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE106" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -36286,6 +36607,9 @@
       <c r="DD107" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DE107" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -36618,6 +36942,9 @@
       <c r="DD108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DE108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -36950,6 +37277,9 @@
       <c r="DD109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DE109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -37282,6 +37612,9 @@
       <c r="DD110" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DE110" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -37614,6 +37947,9 @@
       <c r="DD111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DE111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -37946,6 +38282,9 @@
       <c r="DD112" s="3" t="n">
         <v>23.8</v>
       </c>
+      <c r="DE112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -38278,6 +38617,9 @@
       <c r="DD113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DE113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -38610,6 +38952,9 @@
       <c r="DD114" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE114" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -38942,6 +39287,9 @@
       <c r="DD115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DE115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -39274,6 +39622,9 @@
       <c r="DD116" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DE116" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -39606,6 +39957,9 @@
       <c r="DD117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DE117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -39938,6 +40292,9 @@
       <c r="DD118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DE118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -40270,6 +40627,9 @@
       <c r="DD119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="DE119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -40602,6 +40962,9 @@
       <c r="DD120" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE120" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -40934,6 +41297,9 @@
       <c r="DD121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DE121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -41266,6 +41632,9 @@
       <c r="DD122" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE122" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -41598,6 +41967,9 @@
       <c r="DD123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DE123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -41930,6 +42302,9 @@
       <c r="DD124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="DE124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -42262,6 +42637,9 @@
       <c r="DD125" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DE125" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -42594,6 +42972,9 @@
       <c r="DD126" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DE126" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -42926,6 +43307,9 @@
       <c r="DD127" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DE127" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -43258,6 +43642,9 @@
       <c r="DD128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="DE128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -43590,6 +43977,9 @@
       <c r="DD129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DE129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -43922,6 +44312,9 @@
       <c r="DD130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DE130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -44254,6 +44647,9 @@
       <c r="DD131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="DE131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -44586,6 +44982,9 @@
       <c r="DD132" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DE132" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -44918,6 +45317,9 @@
       <c r="DD133" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DE133" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -45250,6 +45652,9 @@
       <c r="DD134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="DE134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -45582,6 +45987,9 @@
       <c r="DD135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DE135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -45914,6 +46322,9 @@
       <c r="DD136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DE136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -46246,6 +46657,9 @@
       <c r="DD137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DE137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -46578,6 +46992,9 @@
       <c r="DD138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DE138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -46910,6 +47327,9 @@
       <c r="DD139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DE139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -47242,6 +47662,9 @@
       <c r="DD140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DE140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -47574,6 +47997,9 @@
       <c r="DD141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DE141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -47906,6 +48332,9 @@
       <c r="DD142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DE142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -48238,6 +48667,9 @@
       <c r="DD143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DE143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -48570,6 +49002,9 @@
       <c r="DD144" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DE144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -48902,6 +49337,9 @@
       <c r="DD145" s="3" t="n">
         <v>23.19</v>
       </c>
+      <c r="DE145" s="3" t="n">
+        <v>23.19</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -49234,6 +49672,9 @@
       <c r="DD146" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DE146" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -49566,6 +50007,9 @@
       <c r="DD147" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DE147" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -49898,6 +50342,9 @@
       <c r="DD148" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DE148" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -50230,6 +50677,9 @@
       <c r="DD149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DE149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -50562,6 +51012,9 @@
       <c r="DD150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DE150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -50894,6 +51347,9 @@
       <c r="DD151" s="3" t="n">
         <v>23.39</v>
       </c>
+      <c r="DE151" s="3" t="n">
+        <v>23.39</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -51226,6 +51682,9 @@
       <c r="DD152" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DE152" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -51558,6 +52017,9 @@
       <c r="DD153" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DE153" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -51890,6 +52352,9 @@
       <c r="DD154" s="3" t="n">
         <v>23.7</v>
       </c>
+      <c r="DE154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -52222,6 +52687,9 @@
       <c r="DD155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DE155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -52554,6 +53022,9 @@
       <c r="DD156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DE156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -52886,6 +53357,9 @@
       <c r="DD157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DE157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -53218,6 +53692,9 @@
       <c r="DD158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DE158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -53550,6 +54027,9 @@
       <c r="DD159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DE159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -53882,6 +54362,9 @@
       <c r="DD160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DE160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -54214,6 +54697,9 @@
       <c r="DD161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DE161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -54546,6 +55032,9 @@
       <c r="DD162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DE162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -54878,6 +55367,9 @@
       <c r="DD163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DE163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -55210,6 +55702,9 @@
       <c r="DD164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="DE164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -55443,9 +55938,12 @@
       <c r="DD165" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DE165" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:DD165"/>
+  <autoFilter ref="A1:DE165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-18 03:10 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DE$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DF$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DE165"/>
+  <dimension ref="A1:DF165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -552,6 +552,7 @@
     <col width="16" customWidth="1" min="107" max="107"/>
     <col width="16" customWidth="1" min="108" max="108"/>
     <col width="16" customWidth="1" min="109" max="109"/>
+    <col width="16" customWidth="1" min="110" max="110"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1100,6 +1101,11 @@
           <t>2026-09-17 19:12</t>
         </is>
       </c>
+      <c r="DF1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-17 22:10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1435,6 +1441,9 @@
       <c r="DE2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="DF2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1770,6 +1779,9 @@
       <c r="DE3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="DF3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2105,6 +2117,9 @@
       <c r="DE4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="DF4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2440,6 +2455,9 @@
       <c r="DE5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DF5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2775,6 +2793,9 @@
       <c r="DE6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DF6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3110,6 +3131,9 @@
       <c r="DE7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="DF7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3445,6 +3469,9 @@
       <c r="DE8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DF8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3780,6 +3807,9 @@
       <c r="DE9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="DF9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4115,6 +4145,9 @@
       <c r="DE10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DF10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4450,6 +4483,9 @@
       <c r="DE11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DF11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4785,6 +4821,9 @@
       <c r="DE12" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF12" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -5120,6 +5159,9 @@
       <c r="DE13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="DF13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5455,6 +5497,9 @@
       <c r="DE14" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DF14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5790,6 +5835,9 @@
       <c r="DE15" s="3" t="n">
         <v>21.41</v>
       </c>
+      <c r="DF15" s="3" t="n">
+        <v>21.41</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -6125,6 +6173,9 @@
       <c r="DE16" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DF16" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6460,6 +6511,9 @@
       <c r="DE17" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DF17" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -6795,6 +6849,9 @@
       <c r="DE18" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DF18" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -7130,6 +7187,9 @@
       <c r="DE19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="DF19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -7465,6 +7525,9 @@
       <c r="DE20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DF20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -7800,6 +7863,9 @@
       <c r="DE21" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DF21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -8135,6 +8201,9 @@
       <c r="DE22" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DF22" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -8470,6 +8539,9 @@
       <c r="DE23" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DF23" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -8805,6 +8877,9 @@
       <c r="DE24" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DF24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -9140,6 +9215,9 @@
       <c r="DE25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DF25" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -9475,6 +9553,9 @@
       <c r="DE26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DF26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -9810,6 +9891,9 @@
       <c r="DE27" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DF27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -10145,6 +10229,9 @@
       <c r="DE28" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DF28" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -10480,6 +10567,9 @@
       <c r="DE29" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DF29" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -10815,6 +10905,9 @@
       <c r="DE30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -11150,6 +11243,9 @@
       <c r="DE31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DF31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -11485,6 +11581,9 @@
       <c r="DE32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DF32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -11820,6 +11919,9 @@
       <c r="DE33" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -12155,6 +12257,9 @@
       <c r="DE34" s="3" t="n">
         <v>21.77</v>
       </c>
+      <c r="DF34" s="3" t="n">
+        <v>21.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -12490,6 +12595,9 @@
       <c r="DE35" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DF35" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -12825,6 +12933,9 @@
       <c r="DE36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DF36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -13160,6 +13271,9 @@
       <c r="DE37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DF37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -13495,6 +13609,9 @@
       <c r="DE38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DF38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -13830,6 +13947,9 @@
       <c r="DE39" s="3" t="n">
         <v>21.98</v>
       </c>
+      <c r="DF39" s="3" t="n">
+        <v>21.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -14165,6 +14285,9 @@
       <c r="DE40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -14500,6 +14623,9 @@
       <c r="DE41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DF41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -14835,6 +14961,9 @@
       <c r="DE42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DF42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -15170,6 +15299,9 @@
       <c r="DE43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DF43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -15505,6 +15637,9 @@
       <c r="DE44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -15840,6 +15975,9 @@
       <c r="DE45" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DF45" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -16175,6 +16313,9 @@
       <c r="DE46" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="DF46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -16510,6 +16651,9 @@
       <c r="DE47" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DF47" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -16845,6 +16989,9 @@
       <c r="DE48" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DF48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -17180,6 +17327,9 @@
       <c r="DE49" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DF49" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -17515,6 +17665,9 @@
       <c r="DE50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="DF50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -17850,6 +18003,9 @@
       <c r="DE51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DF51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -18185,6 +18341,9 @@
       <c r="DE52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DF52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -18520,6 +18679,9 @@
       <c r="DE53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="DF53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -18855,6 +19017,9 @@
       <c r="DE54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -19190,6 +19355,9 @@
       <c r="DE55" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DF55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -19525,6 +19693,9 @@
       <c r="DE56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -19860,6 +20031,9 @@
       <c r="DE57" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DF57" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -20195,6 +20369,9 @@
       <c r="DE58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="DF58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -20530,6 +20707,9 @@
       <c r="DE59" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DF59" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -20865,6 +21045,9 @@
       <c r="DE60" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DF60" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -21200,6 +21383,9 @@
       <c r="DE61" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DF61" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -21535,6 +21721,9 @@
       <c r="DE62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DF62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -21870,6 +22059,9 @@
       <c r="DE63" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DF63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -22205,6 +22397,9 @@
       <c r="DE64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DF64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -22540,6 +22735,9 @@
       <c r="DE65" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF65" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -22875,6 +23073,9 @@
       <c r="DE66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -23210,6 +23411,9 @@
       <c r="DE67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DF67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -23545,6 +23749,9 @@
       <c r="DE68" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DF68" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -23880,6 +24087,9 @@
       <c r="DE69" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DF69" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -24215,6 +24425,9 @@
       <c r="DE70" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF70" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -24550,6 +24763,9 @@
       <c r="DE71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -24885,6 +25101,9 @@
       <c r="DE72" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DF72" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -25220,6 +25439,9 @@
       <c r="DE73" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DF73" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -25555,6 +25777,9 @@
       <c r="DE74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DF74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -25890,6 +26115,9 @@
       <c r="DE75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -26225,6 +26453,9 @@
       <c r="DE76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -26560,6 +26791,9 @@
       <c r="DE77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="DF77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -26895,6 +27129,9 @@
       <c r="DE78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DF78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -27230,6 +27467,9 @@
       <c r="DE79" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DF79" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -27565,6 +27805,9 @@
       <c r="DE80" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DF80" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -27900,6 +28143,9 @@
       <c r="DE81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -28235,6 +28481,9 @@
       <c r="DE82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DF82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -28570,6 +28819,9 @@
       <c r="DE83" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF83" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -28905,6 +29157,9 @@
       <c r="DE84" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DF84" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -29240,6 +29495,9 @@
       <c r="DE85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="DF85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -29575,6 +29833,9 @@
       <c r="DE86" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DF86" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -29910,6 +30171,9 @@
       <c r="DE87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DF87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -30245,6 +30509,9 @@
       <c r="DE88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -30580,6 +30847,9 @@
       <c r="DE89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DF89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -30915,6 +31185,9 @@
       <c r="DE90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -31250,6 +31523,9 @@
       <c r="DE91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -31585,6 +31861,9 @@
       <c r="DE92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -31920,6 +32199,9 @@
       <c r="DE93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DF93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -32255,6 +32537,9 @@
       <c r="DE94" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DF94" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -32590,6 +32875,9 @@
       <c r="DE95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DF95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -32925,6 +33213,9 @@
       <c r="DE96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="DF96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -33260,6 +33551,9 @@
       <c r="DE97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DF97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -33595,6 +33889,9 @@
       <c r="DE98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DF98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -33930,6 +34227,9 @@
       <c r="DE99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DF99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -34265,6 +34565,9 @@
       <c r="DE100" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DF100" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -34600,6 +34903,9 @@
       <c r="DE101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -34935,6 +35241,9 @@
       <c r="DE102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="DF102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -35270,6 +35579,9 @@
       <c r="DE103" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF103" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -35605,6 +35917,9 @@
       <c r="DE104" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -35940,6 +36255,9 @@
       <c r="DE105" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF105" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -36275,6 +36593,9 @@
       <c r="DE106" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF106" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -36610,6 +36931,9 @@
       <c r="DE107" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DF107" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -36945,6 +37269,9 @@
       <c r="DE108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DF108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -37280,6 +37607,9 @@
       <c r="DE109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DF109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -37615,6 +37945,9 @@
       <c r="DE110" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DF110" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -37950,6 +38283,9 @@
       <c r="DE111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DF111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -38285,6 +38621,9 @@
       <c r="DE112" s="3" t="n">
         <v>23.8</v>
       </c>
+      <c r="DF112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -38620,6 +38959,9 @@
       <c r="DE113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DF113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -38955,6 +39297,9 @@
       <c r="DE114" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF114" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -39290,6 +39635,9 @@
       <c r="DE115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DF115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -39625,6 +39973,9 @@
       <c r="DE116" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DF116" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -39960,6 +40311,9 @@
       <c r="DE117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DF117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -40295,6 +40649,9 @@
       <c r="DE118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DF118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -40630,6 +40987,9 @@
       <c r="DE119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="DF119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -40965,6 +41325,9 @@
       <c r="DE120" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF120" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -41300,6 +41663,9 @@
       <c r="DE121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DF121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -41635,6 +42001,9 @@
       <c r="DE122" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF122" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -41970,6 +42339,9 @@
       <c r="DE123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DF123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -42305,6 +42677,9 @@
       <c r="DE124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="DF124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -42640,6 +43015,9 @@
       <c r="DE125" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DF125" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -42975,6 +43353,9 @@
       <c r="DE126" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DF126" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -43310,6 +43691,9 @@
       <c r="DE127" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DF127" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -43645,6 +44029,9 @@
       <c r="DE128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="DF128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -43980,6 +44367,9 @@
       <c r="DE129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DF129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -44315,6 +44705,9 @@
       <c r="DE130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DF130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -44650,6 +45043,9 @@
       <c r="DE131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="DF131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -44985,6 +45381,9 @@
       <c r="DE132" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DF132" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -45320,6 +45719,9 @@
       <c r="DE133" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DF133" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -45655,6 +46057,9 @@
       <c r="DE134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="DF134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -45990,6 +46395,9 @@
       <c r="DE135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DF135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -46325,6 +46733,9 @@
       <c r="DE136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DF136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -46660,6 +47071,9 @@
       <c r="DE137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DF137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -46995,6 +47409,9 @@
       <c r="DE138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DF138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -47330,6 +47747,9 @@
       <c r="DE139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DF139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -47665,6 +48085,9 @@
       <c r="DE140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DF140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -48000,6 +48423,9 @@
       <c r="DE141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DF141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -48335,6 +48761,9 @@
       <c r="DE142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DF142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -48670,6 +49099,9 @@
       <c r="DE143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DF143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -49005,6 +49437,9 @@
       <c r="DE144" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DF144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -49340,6 +49775,9 @@
       <c r="DE145" s="3" t="n">
         <v>23.19</v>
       </c>
+      <c r="DF145" s="3" t="n">
+        <v>23.19</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -49675,6 +50113,9 @@
       <c r="DE146" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DF146" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -50010,6 +50451,9 @@
       <c r="DE147" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DF147" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -50345,6 +50789,9 @@
       <c r="DE148" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DF148" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -50680,6 +51127,9 @@
       <c r="DE149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DF149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -51015,6 +51465,9 @@
       <c r="DE150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DF150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -51350,6 +51803,9 @@
       <c r="DE151" s="3" t="n">
         <v>23.39</v>
       </c>
+      <c r="DF151" s="3" t="n">
+        <v>23.39</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -51685,6 +52141,9 @@
       <c r="DE152" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DF152" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -52020,6 +52479,9 @@
       <c r="DE153" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DF153" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -52355,6 +52817,9 @@
       <c r="DE154" s="3" t="n">
         <v>23.7</v>
       </c>
+      <c r="DF154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -52690,6 +53155,9 @@
       <c r="DE155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DF155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -53025,6 +53493,9 @@
       <c r="DE156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DF156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -53360,6 +53831,9 @@
       <c r="DE157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DF157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -53695,6 +54169,9 @@
       <c r="DE158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DF158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -54030,6 +54507,9 @@
       <c r="DE159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DF159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -54365,6 +54845,9 @@
       <c r="DE160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DF160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -54700,6 +55183,9 @@
       <c r="DE161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DF161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -55035,6 +55521,9 @@
       <c r="DE162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DF162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -55370,6 +55859,9 @@
       <c r="DE163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DF163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -55705,6 +56197,9 @@
       <c r="DE164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="DF164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -55941,9 +56436,12 @@
       <c r="DE165" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DF165" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:DE165"/>
+  <autoFilter ref="A1:DF165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-18 06:12 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DF$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DG$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DF165"/>
+  <dimension ref="A1:DG165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -553,6 +553,7 @@
     <col width="16" customWidth="1" min="108" max="108"/>
     <col width="16" customWidth="1" min="109" max="109"/>
     <col width="16" customWidth="1" min="110" max="110"/>
+    <col width="16" customWidth="1" min="111" max="111"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1106,6 +1107,11 @@
           <t>2026-09-17 22:10</t>
         </is>
       </c>
+      <c r="DG1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-18 01:12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1444,6 +1450,9 @@
       <c r="DF2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="DG2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1782,6 +1791,9 @@
       <c r="DF3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="DG3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2120,6 +2132,9 @@
       <c r="DF4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="DG4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2458,6 +2473,9 @@
       <c r="DF5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DG5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2796,6 +2814,9 @@
       <c r="DF6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DG6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3134,6 +3155,9 @@
       <c r="DF7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="DG7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3472,6 +3496,9 @@
       <c r="DF8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DG8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3810,6 +3837,9 @@
       <c r="DF9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="DG9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4148,6 +4178,9 @@
       <c r="DF10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DG10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4486,6 +4519,9 @@
       <c r="DF11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DG11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4824,6 +4860,9 @@
       <c r="DF12" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG12" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -5162,6 +5201,9 @@
       <c r="DF13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="DG13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5500,6 +5542,9 @@
       <c r="DF14" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DG14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5838,6 +5883,9 @@
       <c r="DF15" s="3" t="n">
         <v>21.41</v>
       </c>
+      <c r="DG15" s="3" t="n">
+        <v>21.41</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -6176,6 +6224,9 @@
       <c r="DF16" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DG16" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6514,6 +6565,9 @@
       <c r="DF17" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DG17" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -6852,6 +6906,9 @@
       <c r="DF18" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DG18" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -7190,6 +7247,9 @@
       <c r="DF19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="DG19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -7528,6 +7588,9 @@
       <c r="DF20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DG20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -7866,6 +7929,9 @@
       <c r="DF21" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DG21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -8204,6 +8270,9 @@
       <c r="DF22" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DG22" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -8542,6 +8611,9 @@
       <c r="DF23" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DG23" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -8880,6 +8952,9 @@
       <c r="DF24" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DG24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -9218,6 +9293,9 @@
       <c r="DF25" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DG25" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -9556,6 +9634,9 @@
       <c r="DF26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DG26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -9894,6 +9975,9 @@
       <c r="DF27" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DG27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -10232,6 +10316,9 @@
       <c r="DF28" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DG28" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -10570,6 +10657,9 @@
       <c r="DF29" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DG29" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -10908,6 +10998,9 @@
       <c r="DF30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -11246,6 +11339,9 @@
       <c r="DF31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DG31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -11584,6 +11680,9 @@
       <c r="DF32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DG32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -11922,6 +12021,9 @@
       <c r="DF33" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -12260,6 +12362,9 @@
       <c r="DF34" s="3" t="n">
         <v>21.77</v>
       </c>
+      <c r="DG34" s="3" t="n">
+        <v>21.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -12598,6 +12703,9 @@
       <c r="DF35" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DG35" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -12936,6 +13044,9 @@
       <c r="DF36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DG36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -13274,6 +13385,9 @@
       <c r="DF37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DG37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -13612,6 +13726,9 @@
       <c r="DF38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DG38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -13950,6 +14067,9 @@
       <c r="DF39" s="3" t="n">
         <v>21.98</v>
       </c>
+      <c r="DG39" s="3" t="n">
+        <v>21.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -14288,6 +14408,9 @@
       <c r="DF40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -14626,6 +14749,9 @@
       <c r="DF41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DG41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -14964,6 +15090,9 @@
       <c r="DF42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DG42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -15302,6 +15431,9 @@
       <c r="DF43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DG43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -15640,6 +15772,9 @@
       <c r="DF44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -15978,6 +16113,9 @@
       <c r="DF45" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DG45" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -16316,6 +16454,9 @@
       <c r="DF46" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="DG46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -16654,6 +16795,9 @@
       <c r="DF47" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DG47" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -16992,6 +17136,9 @@
       <c r="DF48" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DG48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -17330,6 +17477,9 @@
       <c r="DF49" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DG49" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -17668,6 +17818,9 @@
       <c r="DF50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="DG50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -18006,6 +18159,9 @@
       <c r="DF51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DG51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -18344,6 +18500,9 @@
       <c r="DF52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DG52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -18682,6 +18841,9 @@
       <c r="DF53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="DG53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -19020,6 +19182,9 @@
       <c r="DF54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -19358,6 +19523,9 @@
       <c r="DF55" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DG55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -19696,6 +19864,9 @@
       <c r="DF56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -20034,6 +20205,9 @@
       <c r="DF57" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DG57" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -20372,6 +20546,9 @@
       <c r="DF58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="DG58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -20710,6 +20887,9 @@
       <c r="DF59" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DG59" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -21048,6 +21228,9 @@
       <c r="DF60" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DG60" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -21386,6 +21569,9 @@
       <c r="DF61" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DG61" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -21724,6 +21910,9 @@
       <c r="DF62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DG62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -22062,6 +22251,9 @@
       <c r="DF63" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DG63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -22400,6 +22592,9 @@
       <c r="DF64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DG64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -22738,6 +22933,9 @@
       <c r="DF65" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG65" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -23076,6 +23274,9 @@
       <c r="DF66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -23414,6 +23615,9 @@
       <c r="DF67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DG67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -23752,6 +23956,9 @@
       <c r="DF68" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DG68" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -24090,6 +24297,9 @@
       <c r="DF69" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DG69" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -24428,6 +24638,9 @@
       <c r="DF70" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG70" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -24766,6 +24979,9 @@
       <c r="DF71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -25104,6 +25320,9 @@
       <c r="DF72" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DG72" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -25442,6 +25661,9 @@
       <c r="DF73" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DG73" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -25780,6 +26002,9 @@
       <c r="DF74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DG74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -26118,6 +26343,9 @@
       <c r="DF75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -26456,6 +26684,9 @@
       <c r="DF76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -26794,6 +27025,9 @@
       <c r="DF77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="DG77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -27132,6 +27366,9 @@
       <c r="DF78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DG78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -27470,6 +27707,9 @@
       <c r="DF79" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DG79" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -27808,6 +28048,9 @@
       <c r="DF80" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DG80" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -28146,6 +28389,9 @@
       <c r="DF81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -28484,6 +28730,9 @@
       <c r="DF82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DG82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -28822,6 +29071,9 @@
       <c r="DF83" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG83" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -29160,6 +29412,9 @@
       <c r="DF84" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DG84" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -29498,6 +29753,9 @@
       <c r="DF85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="DG85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -29836,6 +30094,9 @@
       <c r="DF86" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DG86" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -30174,6 +30435,9 @@
       <c r="DF87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DG87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -30512,6 +30776,9 @@
       <c r="DF88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -30850,6 +31117,9 @@
       <c r="DF89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DG89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -31188,6 +31458,9 @@
       <c r="DF90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -31526,6 +31799,9 @@
       <c r="DF91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -31864,6 +32140,9 @@
       <c r="DF92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -32202,6 +32481,9 @@
       <c r="DF93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DG93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -32540,6 +32822,9 @@
       <c r="DF94" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DG94" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -32878,6 +33163,9 @@
       <c r="DF95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DG95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -33216,6 +33504,9 @@
       <c r="DF96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="DG96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -33554,6 +33845,9 @@
       <c r="DF97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DG97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -33892,6 +34186,9 @@
       <c r="DF98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DG98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -34230,6 +34527,9 @@
       <c r="DF99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DG99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -34568,6 +34868,9 @@
       <c r="DF100" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DG100" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -34906,6 +35209,9 @@
       <c r="DF101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -35244,6 +35550,9 @@
       <c r="DF102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="DG102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -35582,6 +35891,9 @@
       <c r="DF103" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG103" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -35920,6 +36232,9 @@
       <c r="DF104" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -36258,6 +36573,9 @@
       <c r="DF105" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG105" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -36596,6 +36914,9 @@
       <c r="DF106" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG106" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -36934,6 +37255,9 @@
       <c r="DF107" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DG107" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -37272,6 +37596,9 @@
       <c r="DF108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DG108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -37610,6 +37937,9 @@
       <c r="DF109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DG109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -37948,6 +38278,9 @@
       <c r="DF110" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DG110" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -38286,6 +38619,9 @@
       <c r="DF111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DG111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -38624,6 +38960,9 @@
       <c r="DF112" s="3" t="n">
         <v>23.8</v>
       </c>
+      <c r="DG112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -38962,6 +39301,9 @@
       <c r="DF113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DG113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -39300,6 +39642,9 @@
       <c r="DF114" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG114" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -39638,6 +39983,9 @@
       <c r="DF115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DG115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -39976,6 +40324,9 @@
       <c r="DF116" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DG116" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -40314,6 +40665,9 @@
       <c r="DF117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DG117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -40652,6 +41006,9 @@
       <c r="DF118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DG118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -40990,6 +41347,9 @@
       <c r="DF119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="DG119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -41328,6 +41688,9 @@
       <c r="DF120" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG120" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -41666,6 +42029,9 @@
       <c r="DF121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DG121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -42004,6 +42370,9 @@
       <c r="DF122" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG122" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -42342,6 +42711,9 @@
       <c r="DF123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DG123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -42680,6 +43052,9 @@
       <c r="DF124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="DG124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -43018,6 +43393,9 @@
       <c r="DF125" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DG125" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -43356,6 +43734,9 @@
       <c r="DF126" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DG126" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -43694,6 +44075,9 @@
       <c r="DF127" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DG127" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -44032,6 +44416,9 @@
       <c r="DF128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="DG128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -44370,6 +44757,9 @@
       <c r="DF129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DG129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -44708,6 +45098,9 @@
       <c r="DF130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DG130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -45046,6 +45439,9 @@
       <c r="DF131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="DG131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -45384,6 +45780,9 @@
       <c r="DF132" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DG132" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -45722,6 +46121,9 @@
       <c r="DF133" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DG133" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -46060,6 +46462,9 @@
       <c r="DF134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="DG134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -46398,6 +46803,9 @@
       <c r="DF135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DG135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -46736,6 +47144,9 @@
       <c r="DF136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DG136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -47074,6 +47485,9 @@
       <c r="DF137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DG137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -47412,6 +47826,9 @@
       <c r="DF138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DG138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -47750,6 +48167,9 @@
       <c r="DF139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DG139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -48088,6 +48508,9 @@
       <c r="DF140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DG140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -48426,6 +48849,9 @@
       <c r="DF141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DG141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -48764,6 +49190,9 @@
       <c r="DF142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DG142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -49102,6 +49531,9 @@
       <c r="DF143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DG143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -49440,6 +49872,9 @@
       <c r="DF144" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DG144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -49778,6 +50213,9 @@
       <c r="DF145" s="3" t="n">
         <v>23.19</v>
       </c>
+      <c r="DG145" s="3" t="n">
+        <v>23.19</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -50116,6 +50554,9 @@
       <c r="DF146" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DG146" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -50454,6 +50895,9 @@
       <c r="DF147" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DG147" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -50792,6 +51236,9 @@
       <c r="DF148" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DG148" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -51130,6 +51577,9 @@
       <c r="DF149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DG149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -51468,6 +51918,9 @@
       <c r="DF150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DG150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -51806,6 +52259,9 @@
       <c r="DF151" s="3" t="n">
         <v>23.39</v>
       </c>
+      <c r="DG151" s="3" t="n">
+        <v>23.39</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -52144,6 +52600,9 @@
       <c r="DF152" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DG152" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -52482,6 +52941,9 @@
       <c r="DF153" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DG153" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -52820,6 +53282,9 @@
       <c r="DF154" s="3" t="n">
         <v>23.7</v>
       </c>
+      <c r="DG154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -53158,6 +53623,9 @@
       <c r="DF155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DG155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -53496,6 +53964,9 @@
       <c r="DF156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DG156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -53834,6 +54305,9 @@
       <c r="DF157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DG157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -54172,6 +54646,9 @@
       <c r="DF158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DG158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -54510,6 +54987,9 @@
       <c r="DF159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DG159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -54848,6 +55328,9 @@
       <c r="DF160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DG160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -55186,6 +55669,9 @@
       <c r="DF161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DG161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -55524,6 +56010,9 @@
       <c r="DF162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DG162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -55862,6 +56351,9 @@
       <c r="DF163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DG163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -56200,6 +56692,9 @@
       <c r="DF164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="DG164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -56439,9 +56934,12 @@
       <c r="DF165" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DG165" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:DF165"/>
+  <autoFilter ref="A1:DG165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-18 09:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DG$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DH$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DG165"/>
+  <dimension ref="A1:DH165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -554,6 +554,7 @@
     <col width="16" customWidth="1" min="109" max="109"/>
     <col width="16" customWidth="1" min="110" max="110"/>
     <col width="16" customWidth="1" min="111" max="111"/>
+    <col width="16" customWidth="1" min="112" max="112"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1112,6 +1113,11 @@
           <t>2026-09-18 01:12</t>
         </is>
       </c>
+      <c r="DH1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-18 04:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1453,6 +1459,9 @@
       <c r="DG2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="DH2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1794,6 +1803,9 @@
       <c r="DG3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="DH3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2135,6 +2147,9 @@
       <c r="DG4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="DH4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2476,6 +2491,9 @@
       <c r="DG5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DH5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2817,6 +2835,9 @@
       <c r="DG6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DH6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3158,6 +3179,9 @@
       <c r="DG7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="DH7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3499,6 +3523,9 @@
       <c r="DG8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DH8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3840,6 +3867,9 @@
       <c r="DG9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="DH9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4181,6 +4211,9 @@
       <c r="DG10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DH10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4522,6 +4555,9 @@
       <c r="DG11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DH11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4863,6 +4899,9 @@
       <c r="DG12" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH12" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -5204,6 +5243,9 @@
       <c r="DG13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="DH13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5545,6 +5587,9 @@
       <c r="DG14" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DH14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5886,6 +5931,9 @@
       <c r="DG15" s="3" t="n">
         <v>21.41</v>
       </c>
+      <c r="DH15" s="3" t="n">
+        <v>21.41</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -6227,6 +6275,9 @@
       <c r="DG16" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DH16" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6568,6 +6619,9 @@
       <c r="DG17" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DH17" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -6909,6 +6963,9 @@
       <c r="DG18" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DH18" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -7250,6 +7307,9 @@
       <c r="DG19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="DH19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -7591,6 +7651,9 @@
       <c r="DG20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DH20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -7932,6 +7995,9 @@
       <c r="DG21" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DH21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -8273,6 +8339,9 @@
       <c r="DG22" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DH22" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -8614,6 +8683,9 @@
       <c r="DG23" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DH23" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -8955,6 +9027,9 @@
       <c r="DG24" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DH24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -9296,6 +9371,9 @@
       <c r="DG25" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DH25" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -9637,6 +9715,9 @@
       <c r="DG26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DH26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -9978,6 +10059,9 @@
       <c r="DG27" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DH27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -10319,6 +10403,9 @@
       <c r="DG28" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DH28" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -10660,6 +10747,9 @@
       <c r="DG29" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DH29" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -11001,6 +11091,9 @@
       <c r="DG30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -11342,6 +11435,9 @@
       <c r="DG31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DH31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -11683,6 +11779,9 @@
       <c r="DG32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DH32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -12024,6 +12123,9 @@
       <c r="DG33" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -12365,6 +12467,9 @@
       <c r="DG34" s="3" t="n">
         <v>21.77</v>
       </c>
+      <c r="DH34" s="3" t="n">
+        <v>21.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -12706,6 +12811,9 @@
       <c r="DG35" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DH35" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -13047,6 +13155,9 @@
       <c r="DG36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DH36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -13388,6 +13499,9 @@
       <c r="DG37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DH37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -13729,6 +13843,9 @@
       <c r="DG38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DH38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -14070,6 +14187,9 @@
       <c r="DG39" s="3" t="n">
         <v>21.98</v>
       </c>
+      <c r="DH39" s="3" t="n">
+        <v>21.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -14411,6 +14531,9 @@
       <c r="DG40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -14752,6 +14875,9 @@
       <c r="DG41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DH41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -15093,6 +15219,9 @@
       <c r="DG42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DH42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -15434,6 +15563,9 @@
       <c r="DG43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DH43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -15775,6 +15907,9 @@
       <c r="DG44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -16116,6 +16251,9 @@
       <c r="DG45" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DH45" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -16457,6 +16595,9 @@
       <c r="DG46" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="DH46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -16798,6 +16939,9 @@
       <c r="DG47" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DH47" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -17139,6 +17283,9 @@
       <c r="DG48" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DH48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -17480,6 +17627,9 @@
       <c r="DG49" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DH49" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -17821,6 +17971,9 @@
       <c r="DG50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="DH50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -18162,6 +18315,9 @@
       <c r="DG51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DH51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -18503,6 +18659,9 @@
       <c r="DG52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DH52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -18844,6 +19003,9 @@
       <c r="DG53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="DH53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -19185,6 +19347,9 @@
       <c r="DG54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -19526,6 +19691,9 @@
       <c r="DG55" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DH55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -19867,6 +20035,9 @@
       <c r="DG56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -20208,6 +20379,9 @@
       <c r="DG57" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DH57" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -20549,6 +20723,9 @@
       <c r="DG58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="DH58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -20890,6 +21067,9 @@
       <c r="DG59" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DH59" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -21231,6 +21411,9 @@
       <c r="DG60" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DH60" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -21572,6 +21755,9 @@
       <c r="DG61" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DH61" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -21913,6 +22099,9 @@
       <c r="DG62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DH62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -22254,6 +22443,9 @@
       <c r="DG63" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DH63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -22595,6 +22787,9 @@
       <c r="DG64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DH64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -22936,6 +23131,9 @@
       <c r="DG65" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH65" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -23277,6 +23475,9 @@
       <c r="DG66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -23618,6 +23819,9 @@
       <c r="DG67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DH67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -23959,6 +24163,9 @@
       <c r="DG68" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DH68" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -24300,6 +24507,9 @@
       <c r="DG69" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DH69" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -24641,6 +24851,9 @@
       <c r="DG70" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH70" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -24982,6 +25195,9 @@
       <c r="DG71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -25323,6 +25539,9 @@
       <c r="DG72" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DH72" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -25664,6 +25883,9 @@
       <c r="DG73" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DH73" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -26005,6 +26227,9 @@
       <c r="DG74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DH74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -26346,6 +26571,9 @@
       <c r="DG75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -26687,6 +26915,9 @@
       <c r="DG76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -27028,6 +27259,9 @@
       <c r="DG77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="DH77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -27369,6 +27603,9 @@
       <c r="DG78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DH78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -27710,6 +27947,9 @@
       <c r="DG79" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DH79" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -28051,6 +28291,9 @@
       <c r="DG80" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DH80" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -28392,6 +28635,9 @@
       <c r="DG81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -28733,6 +28979,9 @@
       <c r="DG82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DH82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -29074,6 +29323,9 @@
       <c r="DG83" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH83" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -29415,6 +29667,9 @@
       <c r="DG84" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DH84" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -29756,6 +30011,9 @@
       <c r="DG85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="DH85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -30097,6 +30355,9 @@
       <c r="DG86" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DH86" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -30438,6 +30699,9 @@
       <c r="DG87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DH87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -30779,6 +31043,9 @@
       <c r="DG88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -31120,6 +31387,9 @@
       <c r="DG89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DH89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -31461,6 +31731,9 @@
       <c r="DG90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -31802,6 +32075,9 @@
       <c r="DG91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -32143,6 +32419,9 @@
       <c r="DG92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -32484,6 +32763,9 @@
       <c r="DG93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DH93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -32825,6 +33107,9 @@
       <c r="DG94" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DH94" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -33166,6 +33451,9 @@
       <c r="DG95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DH95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -33507,6 +33795,9 @@
       <c r="DG96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="DH96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -33848,6 +34139,9 @@
       <c r="DG97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DH97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -34189,6 +34483,9 @@
       <c r="DG98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DH98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -34530,6 +34827,9 @@
       <c r="DG99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DH99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -34871,6 +35171,9 @@
       <c r="DG100" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DH100" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -35212,6 +35515,9 @@
       <c r="DG101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -35553,6 +35859,9 @@
       <c r="DG102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="DH102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -35894,6 +36203,9 @@
       <c r="DG103" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH103" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -36235,6 +36547,9 @@
       <c r="DG104" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -36576,6 +36891,9 @@
       <c r="DG105" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH105" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -36917,6 +37235,9 @@
       <c r="DG106" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH106" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -37258,6 +37579,9 @@
       <c r="DG107" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DH107" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -37599,6 +37923,9 @@
       <c r="DG108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DH108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -37940,6 +38267,9 @@
       <c r="DG109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DH109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -38281,6 +38611,9 @@
       <c r="DG110" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DH110" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -38622,6 +38955,9 @@
       <c r="DG111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DH111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -38963,6 +39299,9 @@
       <c r="DG112" s="3" t="n">
         <v>23.8</v>
       </c>
+      <c r="DH112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -39304,6 +39643,9 @@
       <c r="DG113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DH113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -39645,6 +39987,9 @@
       <c r="DG114" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH114" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -39986,6 +40331,9 @@
       <c r="DG115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DH115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -40327,6 +40675,9 @@
       <c r="DG116" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DH116" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -40668,6 +41019,9 @@
       <c r="DG117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DH117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -41009,6 +41363,9 @@
       <c r="DG118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DH118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -41350,6 +41707,9 @@
       <c r="DG119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="DH119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -41691,6 +42051,9 @@
       <c r="DG120" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH120" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -42032,6 +42395,9 @@
       <c r="DG121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DH121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -42373,6 +42739,9 @@
       <c r="DG122" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH122" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -42714,6 +43083,9 @@
       <c r="DG123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DH123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -43055,6 +43427,9 @@
       <c r="DG124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="DH124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -43396,6 +43771,9 @@
       <c r="DG125" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DH125" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -43737,6 +44115,9 @@
       <c r="DG126" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DH126" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -44078,6 +44459,9 @@
       <c r="DG127" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DH127" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -44419,6 +44803,9 @@
       <c r="DG128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="DH128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -44760,6 +45147,9 @@
       <c r="DG129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DH129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -45101,6 +45491,9 @@
       <c r="DG130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DH130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -45442,6 +45835,9 @@
       <c r="DG131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="DH131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -45783,6 +46179,9 @@
       <c r="DG132" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DH132" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -46124,6 +46523,9 @@
       <c r="DG133" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DH133" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -46465,6 +46867,9 @@
       <c r="DG134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="DH134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -46806,6 +47211,9 @@
       <c r="DG135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DH135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -47147,6 +47555,9 @@
       <c r="DG136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DH136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -47488,6 +47899,9 @@
       <c r="DG137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DH137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -47829,6 +48243,9 @@
       <c r="DG138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DH138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -48170,6 +48587,9 @@
       <c r="DG139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DH139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -48511,6 +48931,9 @@
       <c r="DG140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DH140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -48852,6 +49275,9 @@
       <c r="DG141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DH141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -49193,6 +49619,9 @@
       <c r="DG142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DH142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -49534,6 +49963,9 @@
       <c r="DG143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DH143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -49875,6 +50307,9 @@
       <c r="DG144" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DH144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -50216,6 +50651,9 @@
       <c r="DG145" s="3" t="n">
         <v>23.19</v>
       </c>
+      <c r="DH145" s="3" t="n">
+        <v>23.19</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -50557,6 +50995,9 @@
       <c r="DG146" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DH146" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -50898,6 +51339,9 @@
       <c r="DG147" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DH147" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -51239,6 +51683,9 @@
       <c r="DG148" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DH148" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -51580,6 +52027,9 @@
       <c r="DG149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DH149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -51921,6 +52371,9 @@
       <c r="DG150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DH150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -52262,6 +52715,9 @@
       <c r="DG151" s="3" t="n">
         <v>23.39</v>
       </c>
+      <c r="DH151" s="3" t="n">
+        <v>23.39</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -52603,6 +53059,9 @@
       <c r="DG152" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DH152" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -52944,6 +53403,9 @@
       <c r="DG153" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DH153" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -53285,6 +53747,9 @@
       <c r="DG154" s="3" t="n">
         <v>23.7</v>
       </c>
+      <c r="DH154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -53626,6 +54091,9 @@
       <c r="DG155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DH155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -53967,6 +54435,9 @@
       <c r="DG156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DH156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -54308,6 +54779,9 @@
       <c r="DG157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DH157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -54649,6 +55123,9 @@
       <c r="DG158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DH158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -54990,6 +55467,9 @@
       <c r="DG159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DH159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -55331,6 +55811,9 @@
       <c r="DG160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DH160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -55672,6 +56155,9 @@
       <c r="DG161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DH161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -56013,6 +56499,9 @@
       <c r="DG162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DH162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -56354,6 +56843,9 @@
       <c r="DG163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DH163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -56695,6 +57187,9 @@
       <c r="DG164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="DH164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -56937,9 +57432,12 @@
       <c r="DG165" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DH165" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:DG165"/>
+  <autoFilter ref="A1:DH165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-18 12:12 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DH$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DI$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DH165"/>
+  <dimension ref="A1:DI165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -555,6 +555,7 @@
     <col width="16" customWidth="1" min="110" max="110"/>
     <col width="16" customWidth="1" min="111" max="111"/>
     <col width="16" customWidth="1" min="112" max="112"/>
+    <col width="16" customWidth="1" min="113" max="113"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1118,6 +1119,11 @@
           <t>2026-09-18 04:09</t>
         </is>
       </c>
+      <c r="DI1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-18 07:11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1462,6 +1468,9 @@
       <c r="DH2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="DI2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1806,6 +1815,9 @@
       <c r="DH3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="DI3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2150,6 +2162,9 @@
       <c r="DH4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="DI4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2494,6 +2509,9 @@
       <c r="DH5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DI5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2838,6 +2856,9 @@
       <c r="DH6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DI6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3182,6 +3203,9 @@
       <c r="DH7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="DI7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3526,6 +3550,9 @@
       <c r="DH8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DI8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3870,6 +3897,9 @@
       <c r="DH9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="DI9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4214,6 +4244,9 @@
       <c r="DH10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DI10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4558,6 +4591,9 @@
       <c r="DH11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DI11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4902,6 +4938,9 @@
       <c r="DH12" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI12" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -5246,6 +5285,9 @@
       <c r="DH13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="DI13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5590,6 +5632,9 @@
       <c r="DH14" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DI14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5934,6 +5979,9 @@
       <c r="DH15" s="3" t="n">
         <v>21.41</v>
       </c>
+      <c r="DI15" s="3" t="n">
+        <v>21.41</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -6278,6 +6326,9 @@
       <c r="DH16" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DI16" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6622,6 +6673,9 @@
       <c r="DH17" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DI17" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -6966,6 +7020,9 @@
       <c r="DH18" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DI18" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -7310,6 +7367,9 @@
       <c r="DH19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="DI19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -7654,6 +7714,9 @@
       <c r="DH20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DI20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -7998,6 +8061,9 @@
       <c r="DH21" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DI21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -8342,6 +8408,9 @@
       <c r="DH22" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DI22" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -8686,6 +8755,9 @@
       <c r="DH23" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DI23" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -9030,6 +9102,9 @@
       <c r="DH24" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DI24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -9374,6 +9449,9 @@
       <c r="DH25" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DI25" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -9718,6 +9796,9 @@
       <c r="DH26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DI26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -10062,6 +10143,9 @@
       <c r="DH27" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DI27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -10406,6 +10490,9 @@
       <c r="DH28" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DI28" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -10750,6 +10837,9 @@
       <c r="DH29" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DI29" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -11094,6 +11184,9 @@
       <c r="DH30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -11438,6 +11531,9 @@
       <c r="DH31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DI31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -11782,6 +11878,9 @@
       <c r="DH32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DI32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -12126,6 +12225,9 @@
       <c r="DH33" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -12470,6 +12572,9 @@
       <c r="DH34" s="3" t="n">
         <v>21.77</v>
       </c>
+      <c r="DI34" s="3" t="n">
+        <v>21.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -12814,6 +12919,9 @@
       <c r="DH35" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DI35" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -13158,6 +13266,9 @@
       <c r="DH36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DI36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -13502,6 +13613,9 @@
       <c r="DH37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DI37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -13846,6 +13960,9 @@
       <c r="DH38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DI38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -14190,6 +14307,9 @@
       <c r="DH39" s="3" t="n">
         <v>21.98</v>
       </c>
+      <c r="DI39" s="3" t="n">
+        <v>21.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -14534,6 +14654,9 @@
       <c r="DH40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -14878,6 +15001,9 @@
       <c r="DH41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DI41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -15222,6 +15348,9 @@
       <c r="DH42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DI42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -15566,6 +15695,9 @@
       <c r="DH43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DI43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -15910,6 +16042,9 @@
       <c r="DH44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -16254,6 +16389,9 @@
       <c r="DH45" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DI45" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -16598,6 +16736,9 @@
       <c r="DH46" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="DI46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -16942,6 +17083,9 @@
       <c r="DH47" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DI47" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -17286,6 +17430,9 @@
       <c r="DH48" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DI48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -17630,6 +17777,9 @@
       <c r="DH49" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DI49" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -17974,6 +18124,9 @@
       <c r="DH50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="DI50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -18318,6 +18471,9 @@
       <c r="DH51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DI51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -18662,6 +18818,9 @@
       <c r="DH52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DI52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -19006,6 +19165,9 @@
       <c r="DH53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="DI53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -19350,6 +19512,9 @@
       <c r="DH54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -19694,6 +19859,9 @@
       <c r="DH55" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DI55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -20038,6 +20206,9 @@
       <c r="DH56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -20382,6 +20553,9 @@
       <c r="DH57" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DI57" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -20726,6 +20900,9 @@
       <c r="DH58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="DI58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -21070,6 +21247,9 @@
       <c r="DH59" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DI59" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -21414,6 +21594,9 @@
       <c r="DH60" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DI60" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -21758,6 +21941,9 @@
       <c r="DH61" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DI61" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -22102,6 +22288,9 @@
       <c r="DH62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DI62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -22446,6 +22635,9 @@
       <c r="DH63" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DI63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -22790,6 +22982,9 @@
       <c r="DH64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DI64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -23134,6 +23329,9 @@
       <c r="DH65" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI65" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -23478,6 +23676,9 @@
       <c r="DH66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -23822,6 +24023,9 @@
       <c r="DH67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DI67" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -24166,6 +24370,9 @@
       <c r="DH68" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DI68" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -24510,6 +24717,9 @@
       <c r="DH69" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DI69" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -24854,6 +25064,9 @@
       <c r="DH70" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI70" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -25198,6 +25411,9 @@
       <c r="DH71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -25542,6 +25758,9 @@
       <c r="DH72" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DI72" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -25886,6 +26105,9 @@
       <c r="DH73" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DI73" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -26230,6 +26452,9 @@
       <c r="DH74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DI74" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -26574,6 +26799,9 @@
       <c r="DH75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -26918,6 +27146,9 @@
       <c r="DH76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -27262,6 +27493,9 @@
       <c r="DH77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="DI77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -27606,6 +27840,9 @@
       <c r="DH78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DI78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -27950,6 +28187,9 @@
       <c r="DH79" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DI79" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -28294,6 +28534,9 @@
       <c r="DH80" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DI80" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -28638,6 +28881,9 @@
       <c r="DH81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -28982,6 +29228,9 @@
       <c r="DH82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DI82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -29326,6 +29575,9 @@
       <c r="DH83" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI83" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -29670,6 +29922,9 @@
       <c r="DH84" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DI84" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -30014,6 +30269,9 @@
       <c r="DH85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="DI85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -30358,6 +30616,9 @@
       <c r="DH86" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DI86" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -30702,6 +30963,9 @@
       <c r="DH87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DI87" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -31046,6 +31310,9 @@
       <c r="DH88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -31390,6 +31657,9 @@
       <c r="DH89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DI89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -31734,6 +32004,9 @@
       <c r="DH90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -32078,6 +32351,9 @@
       <c r="DH91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -32422,6 +32698,9 @@
       <c r="DH92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -32766,6 +33045,9 @@
       <c r="DH93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DI93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -33110,6 +33392,9 @@
       <c r="DH94" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DI94" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -33454,6 +33739,9 @@
       <c r="DH95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DI95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -33798,6 +34086,9 @@
       <c r="DH96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="DI96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -34142,6 +34433,9 @@
       <c r="DH97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DI97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -34486,6 +34780,9 @@
       <c r="DH98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DI98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -34830,6 +35127,9 @@
       <c r="DH99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DI99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -35174,6 +35474,9 @@
       <c r="DH100" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DI100" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -35518,6 +35821,9 @@
       <c r="DH101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -35862,6 +36168,9 @@
       <c r="DH102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="DI102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -36206,6 +36515,9 @@
       <c r="DH103" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI103" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -36550,6 +36862,9 @@
       <c r="DH104" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -36894,6 +37209,9 @@
       <c r="DH105" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI105" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -37238,6 +37556,9 @@
       <c r="DH106" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI106" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -37582,6 +37903,9 @@
       <c r="DH107" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DI107" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -37926,6 +38250,9 @@
       <c r="DH108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DI108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -38270,6 +38597,9 @@
       <c r="DH109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DI109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -38614,6 +38944,9 @@
       <c r="DH110" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DI110" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -38958,6 +39291,9 @@
       <c r="DH111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DI111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -39302,6 +39638,9 @@
       <c r="DH112" s="3" t="n">
         <v>23.8</v>
       </c>
+      <c r="DI112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -39646,6 +39985,9 @@
       <c r="DH113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DI113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -39990,6 +40332,9 @@
       <c r="DH114" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI114" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -40334,6 +40679,9 @@
       <c r="DH115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DI115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -40678,6 +41026,9 @@
       <c r="DH116" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DI116" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -41022,6 +41373,9 @@
       <c r="DH117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DI117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -41366,6 +41720,9 @@
       <c r="DH118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DI118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -41710,6 +42067,9 @@
       <c r="DH119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="DI119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -42054,6 +42414,9 @@
       <c r="DH120" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI120" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -42398,6 +42761,9 @@
       <c r="DH121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DI121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -42742,6 +43108,9 @@
       <c r="DH122" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI122" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -43086,6 +43455,9 @@
       <c r="DH123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DI123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -43430,6 +43802,9 @@
       <c r="DH124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="DI124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -43774,6 +44149,9 @@
       <c r="DH125" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DI125" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -44118,6 +44496,9 @@
       <c r="DH126" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DI126" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -44462,6 +44843,9 @@
       <c r="DH127" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DI127" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -44806,6 +45190,9 @@
       <c r="DH128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="DI128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -45150,6 +45537,9 @@
       <c r="DH129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DI129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -45494,6 +45884,9 @@
       <c r="DH130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DI130" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -45838,6 +46231,9 @@
       <c r="DH131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="DI131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -46182,6 +46578,9 @@
       <c r="DH132" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DI132" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -46526,6 +46925,9 @@
       <c r="DH133" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DI133" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -46870,6 +47272,9 @@
       <c r="DH134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="DI134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -47214,6 +47619,9 @@
       <c r="DH135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DI135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -47558,6 +47966,9 @@
       <c r="DH136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DI136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -47902,6 +48313,9 @@
       <c r="DH137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DI137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -48246,6 +48660,9 @@
       <c r="DH138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DI138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -48590,6 +49007,9 @@
       <c r="DH139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DI139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -48934,6 +49354,9 @@
       <c r="DH140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DI140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -49278,6 +49701,9 @@
       <c r="DH141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DI141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -49622,6 +50048,9 @@
       <c r="DH142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DI142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -49966,6 +50395,9 @@
       <c r="DH143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DI143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -50310,6 +50742,9 @@
       <c r="DH144" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DI144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -50654,6 +51089,9 @@
       <c r="DH145" s="3" t="n">
         <v>23.19</v>
       </c>
+      <c r="DI145" s="3" t="n">
+        <v>23.19</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -50998,6 +51436,9 @@
       <c r="DH146" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DI146" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -51342,6 +51783,9 @@
       <c r="DH147" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DI147" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -51686,6 +52130,9 @@
       <c r="DH148" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DI148" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -52030,6 +52477,9 @@
       <c r="DH149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DI149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -52374,6 +52824,9 @@
       <c r="DH150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DI150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -52718,6 +53171,9 @@
       <c r="DH151" s="3" t="n">
         <v>23.39</v>
       </c>
+      <c r="DI151" s="3" t="n">
+        <v>23.39</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -53062,6 +53518,9 @@
       <c r="DH152" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DI152" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -53406,6 +53865,9 @@
       <c r="DH153" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DI153" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -53750,6 +54212,9 @@
       <c r="DH154" s="3" t="n">
         <v>23.7</v>
       </c>
+      <c r="DI154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -54094,6 +54559,9 @@
       <c r="DH155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DI155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -54438,6 +54906,9 @@
       <c r="DH156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DI156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -54782,6 +55253,9 @@
       <c r="DH157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DI157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -55126,6 +55600,9 @@
       <c r="DH158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DI158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -55470,6 +55947,9 @@
       <c r="DH159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DI159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -55814,6 +56294,9 @@
       <c r="DH160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DI160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -56158,6 +56641,9 @@
       <c r="DH161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DI161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -56502,6 +56988,9 @@
       <c r="DH162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DI162" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -56846,6 +57335,9 @@
       <c r="DH163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DI163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -57190,6 +57682,9 @@
       <c r="DH164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="DI164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -57435,9 +57930,12 @@
       <c r="DH165" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DI165" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:DH165"/>
+  <autoFilter ref="A1:DI165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-18 15:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DI$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DJ$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DI165"/>
+  <dimension ref="A1:DJ165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -556,6 +556,7 @@
     <col width="16" customWidth="1" min="111" max="111"/>
     <col width="16" customWidth="1" min="112" max="112"/>
     <col width="16" customWidth="1" min="113" max="113"/>
+    <col width="16" customWidth="1" min="114" max="114"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1124,6 +1125,11 @@
           <t>2026-09-18 07:11</t>
         </is>
       </c>
+      <c r="DJ1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-18 10:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1471,6 +1477,9 @@
       <c r="DI2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="DJ2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1818,6 +1827,9 @@
       <c r="DI3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="DJ3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2165,6 +2177,9 @@
       <c r="DI4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="DJ4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2512,6 +2527,9 @@
       <c r="DI5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DJ5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2859,6 +2877,9 @@
       <c r="DI6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DJ6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3206,6 +3227,9 @@
       <c r="DI7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="DJ7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3553,6 +3577,9 @@
       <c r="DI8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DJ8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3900,6 +3927,9 @@
       <c r="DI9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="DJ9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4247,6 +4277,9 @@
       <c r="DI10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DJ10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4594,6 +4627,9 @@
       <c r="DI11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DJ11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4941,6 +4977,9 @@
       <c r="DI12" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ12" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -5288,6 +5327,9 @@
       <c r="DI13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="DJ13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5635,6 +5677,9 @@
       <c r="DI14" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DJ14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -5982,6 +6027,9 @@
       <c r="DI15" s="3" t="n">
         <v>21.41</v>
       </c>
+      <c r="DJ15" s="3" t="n">
+        <v>21.41</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -6329,6 +6377,9 @@
       <c r="DI16" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DJ16" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6676,6 +6727,9 @@
       <c r="DI17" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DJ17" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -7023,6 +7077,9 @@
       <c r="DI18" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DJ18" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -7370,6 +7427,9 @@
       <c r="DI19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="DJ19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -7717,6 +7777,9 @@
       <c r="DI20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DJ20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -8064,6 +8127,9 @@
       <c r="DI21" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DJ21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -8411,6 +8477,9 @@
       <c r="DI22" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DJ22" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -8758,6 +8827,9 @@
       <c r="DI23" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DJ23" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -9105,6 +9177,9 @@
       <c r="DI24" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DJ24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -9452,6 +9527,9 @@
       <c r="DI25" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DJ25" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -9799,6 +9877,9 @@
       <c r="DI26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DJ26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -10146,6 +10227,9 @@
       <c r="DI27" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DJ27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -10493,6 +10577,9 @@
       <c r="DI28" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DJ28" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -10840,6 +10927,9 @@
       <c r="DI29" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DJ29" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -11187,6 +11277,9 @@
       <c r="DI30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -11534,6 +11627,9 @@
       <c r="DI31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DJ31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -11881,6 +11977,9 @@
       <c r="DI32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DJ32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -12228,6 +12327,9 @@
       <c r="DI33" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -12575,6 +12677,9 @@
       <c r="DI34" s="3" t="n">
         <v>21.77</v>
       </c>
+      <c r="DJ34" s="3" t="n">
+        <v>21.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -12922,6 +13027,9 @@
       <c r="DI35" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DJ35" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -13269,6 +13377,9 @@
       <c r="DI36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DJ36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -13616,6 +13727,9 @@
       <c r="DI37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DJ37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -13963,6 +14077,9 @@
       <c r="DI38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DJ38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -14310,6 +14427,9 @@
       <c r="DI39" s="3" t="n">
         <v>21.98</v>
       </c>
+      <c r="DJ39" s="3" t="n">
+        <v>21.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -14657,6 +14777,9 @@
       <c r="DI40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -15004,6 +15127,9 @@
       <c r="DI41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DJ41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -15351,6 +15477,9 @@
       <c r="DI42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DJ42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -15698,6 +15827,9 @@
       <c r="DI43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DJ43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -16045,6 +16177,9 @@
       <c r="DI44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -16392,6 +16527,9 @@
       <c r="DI45" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DJ45" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -16739,6 +16877,9 @@
       <c r="DI46" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="DJ46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -17086,6 +17227,9 @@
       <c r="DI47" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DJ47" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -17433,6 +17577,9 @@
       <c r="DI48" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DJ48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -17780,6 +17927,9 @@
       <c r="DI49" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DJ49" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -18127,6 +18277,9 @@
       <c r="DI50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="DJ50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -18474,6 +18627,9 @@
       <c r="DI51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DJ51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -18821,6 +18977,9 @@
       <c r="DI52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DJ52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -19168,6 +19327,9 @@
       <c r="DI53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="DJ53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -19515,6 +19677,9 @@
       <c r="DI54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -19862,6 +20027,9 @@
       <c r="DI55" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DJ55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -20209,6 +20377,9 @@
       <c r="DI56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -20556,6 +20727,9 @@
       <c r="DI57" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DJ57" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -20903,6 +21077,9 @@
       <c r="DI58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="DJ58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -21250,6 +21427,9 @@
       <c r="DI59" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DJ59" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -21597,6 +21777,9 @@
       <c r="DI60" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DJ60" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -21944,6 +22127,9 @@
       <c r="DI61" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DJ61" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -22291,6 +22477,9 @@
       <c r="DI62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DJ62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -22638,6 +22827,9 @@
       <c r="DI63" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DJ63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -22985,6 +23177,9 @@
       <c r="DI64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DJ64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -23332,6 +23527,9 @@
       <c r="DI65" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ65" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -23679,6 +23877,9 @@
       <c r="DI66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -24026,6 +24227,9 @@
       <c r="DI67" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DJ67" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -24373,6 +24577,9 @@
       <c r="DI68" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DJ68" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -24720,6 +24927,9 @@
       <c r="DI69" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DJ69" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -25067,6 +25277,9 @@
       <c r="DI70" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ70" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -25414,6 +25627,9 @@
       <c r="DI71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -25761,6 +25977,9 @@
       <c r="DI72" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DJ72" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -26108,6 +26327,9 @@
       <c r="DI73" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DJ73" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -26455,6 +26677,9 @@
       <c r="DI74" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DJ74" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -26802,6 +27027,9 @@
       <c r="DI75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -27149,6 +27377,9 @@
       <c r="DI76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -27496,6 +27727,9 @@
       <c r="DI77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="DJ77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -27843,6 +28077,9 @@
       <c r="DI78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DJ78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -28190,6 +28427,9 @@
       <c r="DI79" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DJ79" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -28537,6 +28777,9 @@
       <c r="DI80" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DJ80" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -28884,6 +29127,9 @@
       <c r="DI81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -29231,6 +29477,9 @@
       <c r="DI82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DJ82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -29578,6 +29827,9 @@
       <c r="DI83" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ83" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -29925,6 +30177,9 @@
       <c r="DI84" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DJ84" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -30272,6 +30527,9 @@
       <c r="DI85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="DJ85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -30619,6 +30877,9 @@
       <c r="DI86" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DJ86" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -30966,6 +31227,9 @@
       <c r="DI87" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DJ87" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -31313,6 +31577,9 @@
       <c r="DI88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -31660,6 +31927,9 @@
       <c r="DI89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DJ89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -32007,6 +32277,9 @@
       <c r="DI90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -32354,6 +32627,9 @@
       <c r="DI91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -32701,6 +32977,9 @@
       <c r="DI92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -33048,6 +33327,9 @@
       <c r="DI93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DJ93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -33395,6 +33677,9 @@
       <c r="DI94" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DJ94" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -33742,6 +34027,9 @@
       <c r="DI95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DJ95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -34089,6 +34377,9 @@
       <c r="DI96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="DJ96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -34436,6 +34727,9 @@
       <c r="DI97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DJ97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -34783,6 +35077,9 @@
       <c r="DI98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DJ98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -35130,6 +35427,9 @@
       <c r="DI99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DJ99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -35477,6 +35777,9 @@
       <c r="DI100" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DJ100" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -35824,6 +36127,9 @@
       <c r="DI101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -36171,6 +36477,9 @@
       <c r="DI102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="DJ102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -36518,6 +36827,9 @@
       <c r="DI103" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ103" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -36865,6 +37177,9 @@
       <c r="DI104" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -37212,6 +37527,9 @@
       <c r="DI105" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ105" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -37559,6 +37877,9 @@
       <c r="DI106" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ106" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -37906,6 +38227,9 @@
       <c r="DI107" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DJ107" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -38253,6 +38577,9 @@
       <c r="DI108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DJ108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -38600,6 +38927,9 @@
       <c r="DI109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DJ109" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -38947,6 +39277,9 @@
       <c r="DI110" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DJ110" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -39294,6 +39627,9 @@
       <c r="DI111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DJ111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -39641,6 +39977,9 @@
       <c r="DI112" s="3" t="n">
         <v>23.8</v>
       </c>
+      <c r="DJ112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -39988,6 +40327,9 @@
       <c r="DI113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DJ113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -40335,6 +40677,9 @@
       <c r="DI114" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ114" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -40682,6 +41027,9 @@
       <c r="DI115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DJ115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -41029,6 +41377,9 @@
       <c r="DI116" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DJ116" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -41376,6 +41727,9 @@
       <c r="DI117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DJ117" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -41723,6 +42077,9 @@
       <c r="DI118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DJ118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -42070,6 +42427,9 @@
       <c r="DI119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="DJ119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -42417,6 +42777,9 @@
       <c r="DI120" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ120" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -42764,6 +43127,9 @@
       <c r="DI121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DJ121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -43111,6 +43477,9 @@
       <c r="DI122" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ122" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -43458,6 +43827,9 @@
       <c r="DI123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DJ123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -43805,6 +44177,9 @@
       <c r="DI124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="DJ124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -44152,6 +44527,9 @@
       <c r="DI125" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DJ125" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -44499,6 +44877,9 @@
       <c r="DI126" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DJ126" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -44846,6 +45227,9 @@
       <c r="DI127" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DJ127" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -45193,6 +45577,9 @@
       <c r="DI128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="DJ128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -45540,6 +45927,9 @@
       <c r="DI129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DJ129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -45887,6 +46277,9 @@
       <c r="DI130" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DJ130" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -46234,6 +46627,9 @@
       <c r="DI131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="DJ131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -46581,6 +46977,9 @@
       <c r="DI132" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DJ132" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -46928,6 +47327,9 @@
       <c r="DI133" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DJ133" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -47275,6 +47677,9 @@
       <c r="DI134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="DJ134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -47622,6 +48027,9 @@
       <c r="DI135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DJ135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -47969,6 +48377,9 @@
       <c r="DI136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DJ136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -48316,6 +48727,9 @@
       <c r="DI137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DJ137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -48663,6 +49077,9 @@
       <c r="DI138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DJ138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -49010,6 +49427,9 @@
       <c r="DI139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DJ139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -49357,6 +49777,9 @@
       <c r="DI140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DJ140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -49704,6 +50127,9 @@
       <c r="DI141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DJ141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -50051,6 +50477,9 @@
       <c r="DI142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DJ142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -50398,6 +50827,9 @@
       <c r="DI143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DJ143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -50745,6 +51177,9 @@
       <c r="DI144" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DJ144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -51092,6 +51527,9 @@
       <c r="DI145" s="3" t="n">
         <v>23.19</v>
       </c>
+      <c r="DJ145" s="3" t="n">
+        <v>23.19</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -51439,6 +51877,9 @@
       <c r="DI146" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DJ146" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -51786,6 +52227,9 @@
       <c r="DI147" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DJ147" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -52133,6 +52577,9 @@
       <c r="DI148" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DJ148" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -52480,6 +52927,9 @@
       <c r="DI149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DJ149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -52827,6 +53277,9 @@
       <c r="DI150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DJ150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -53174,6 +53627,9 @@
       <c r="DI151" s="3" t="n">
         <v>23.39</v>
       </c>
+      <c r="DJ151" s="3" t="n">
+        <v>23.39</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -53521,6 +53977,9 @@
       <c r="DI152" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DJ152" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -53868,6 +54327,9 @@
       <c r="DI153" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DJ153" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -54215,6 +54677,9 @@
       <c r="DI154" s="3" t="n">
         <v>23.7</v>
       </c>
+      <c r="DJ154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -54562,6 +55027,9 @@
       <c r="DI155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DJ155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -54909,6 +55377,9 @@
       <c r="DI156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DJ156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -55256,6 +55727,9 @@
       <c r="DI157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DJ157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -55603,6 +56077,9 @@
       <c r="DI158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DJ158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -55950,6 +56427,9 @@
       <c r="DI159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DJ159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -56297,6 +56777,9 @@
       <c r="DI160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DJ160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -56644,6 +57127,9 @@
       <c r="DI161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DJ161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -56991,6 +57477,9 @@
       <c r="DI162" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DJ162" s="3" t="n">
+        <v>24.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -57338,6 +57827,9 @@
       <c r="DI163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DJ163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -57685,6 +58177,9 @@
       <c r="DI164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="DJ164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -57933,9 +58428,12 @@
       <c r="DI165" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DJ165" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:DI165"/>
+  <autoFilter ref="A1:DJ165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-18 18:10 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DJ$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DK$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DJ165"/>
+  <dimension ref="A1:DK165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -557,6 +557,7 @@
     <col width="16" customWidth="1" min="112" max="112"/>
     <col width="16" customWidth="1" min="113" max="113"/>
     <col width="16" customWidth="1" min="114" max="114"/>
+    <col width="16" customWidth="1" min="115" max="115"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1130,6 +1131,11 @@
           <t>2026-09-18 10:09</t>
         </is>
       </c>
+      <c r="DK1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-18 13:10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1480,6 +1486,9 @@
       <c r="DJ2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="DK2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1830,6 +1839,9 @@
       <c r="DJ3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="DK3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2180,6 +2192,9 @@
       <c r="DJ4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="DK4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2530,6 +2545,9 @@
       <c r="DJ5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DK5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2880,6 +2898,9 @@
       <c r="DJ6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DK6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3230,6 +3251,9 @@
       <c r="DJ7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="DK7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3580,6 +3604,9 @@
       <c r="DJ8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DK8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3930,6 +3957,9 @@
       <c r="DJ9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="DK9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4280,6 +4310,9 @@
       <c r="DJ10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DK10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4630,6 +4663,9 @@
       <c r="DJ11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DK11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4980,6 +5016,9 @@
       <c r="DJ12" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK12" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -5330,6 +5369,9 @@
       <c r="DJ13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="DK13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5680,6 +5722,9 @@
       <c r="DJ14" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DK14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -6030,6 +6075,9 @@
       <c r="DJ15" s="3" t="n">
         <v>21.41</v>
       </c>
+      <c r="DK15" s="3" t="n">
+        <v>21.41</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -6380,6 +6428,9 @@
       <c r="DJ16" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DK16" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6730,6 +6781,9 @@
       <c r="DJ17" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DK17" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -7080,6 +7134,9 @@
       <c r="DJ18" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DK18" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -7430,6 +7487,9 @@
       <c r="DJ19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="DK19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -7780,6 +7840,9 @@
       <c r="DJ20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DK20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -8130,6 +8193,9 @@
       <c r="DJ21" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DK21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -8480,6 +8546,9 @@
       <c r="DJ22" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DK22" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -8830,6 +8899,9 @@
       <c r="DJ23" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DK23" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -9180,6 +9252,9 @@
       <c r="DJ24" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DK24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -9530,6 +9605,9 @@
       <c r="DJ25" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DK25" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -9880,6 +9958,9 @@
       <c r="DJ26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DK26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -10230,6 +10311,9 @@
       <c r="DJ27" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DK27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -10580,6 +10664,9 @@
       <c r="DJ28" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DK28" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -10930,6 +11017,9 @@
       <c r="DJ29" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DK29" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -11280,6 +11370,9 @@
       <c r="DJ30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -11630,6 +11723,9 @@
       <c r="DJ31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DK31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -11980,6 +12076,9 @@
       <c r="DJ32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DK32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -12330,6 +12429,9 @@
       <c r="DJ33" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -12680,6 +12782,9 @@
       <c r="DJ34" s="3" t="n">
         <v>21.77</v>
       </c>
+      <c r="DK34" s="3" t="n">
+        <v>21.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -13030,6 +13135,9 @@
       <c r="DJ35" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DK35" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -13380,6 +13488,9 @@
       <c r="DJ36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DK36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -13730,6 +13841,9 @@
       <c r="DJ37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DK37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -14080,6 +14194,9 @@
       <c r="DJ38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DK38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -14430,6 +14547,9 @@
       <c r="DJ39" s="3" t="n">
         <v>21.98</v>
       </c>
+      <c r="DK39" s="3" t="n">
+        <v>21.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -14780,6 +14900,9 @@
       <c r="DJ40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -15130,6 +15253,9 @@
       <c r="DJ41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DK41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -15480,6 +15606,9 @@
       <c r="DJ42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DK42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -15830,6 +15959,9 @@
       <c r="DJ43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DK43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -16180,6 +16312,9 @@
       <c r="DJ44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -16530,6 +16665,9 @@
       <c r="DJ45" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DK45" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -16880,6 +17018,9 @@
       <c r="DJ46" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="DK46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -17230,6 +17371,9 @@
       <c r="DJ47" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DK47" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -17580,6 +17724,9 @@
       <c r="DJ48" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DK48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -17930,6 +18077,9 @@
       <c r="DJ49" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DK49" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -18280,6 +18430,9 @@
       <c r="DJ50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="DK50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -18630,6 +18783,9 @@
       <c r="DJ51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DK51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -18980,6 +19136,9 @@
       <c r="DJ52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DK52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -19330,6 +19489,9 @@
       <c r="DJ53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="DK53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -19680,6 +19842,9 @@
       <c r="DJ54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -20030,6 +20195,9 @@
       <c r="DJ55" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DK55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -20380,6 +20548,9 @@
       <c r="DJ56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -20730,6 +20901,9 @@
       <c r="DJ57" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DK57" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -21080,6 +21254,9 @@
       <c r="DJ58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="DK58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -21430,6 +21607,9 @@
       <c r="DJ59" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DK59" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -21780,6 +21960,9 @@
       <c r="DJ60" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DK60" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -22130,6 +22313,9 @@
       <c r="DJ61" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DK61" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -22480,6 +22666,9 @@
       <c r="DJ62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DK62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -22830,6 +23019,9 @@
       <c r="DJ63" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DK63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -23180,6 +23372,9 @@
       <c r="DJ64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DK64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -23530,6 +23725,9 @@
       <c r="DJ65" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK65" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -23880,6 +24078,9 @@
       <c r="DJ66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -24230,6 +24431,9 @@
       <c r="DJ67" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK67" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -24580,6 +24784,9 @@
       <c r="DJ68" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DK68" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -24930,6 +25137,9 @@
       <c r="DJ69" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DK69" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -25280,6 +25490,9 @@
       <c r="DJ70" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK70" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -25630,6 +25843,9 @@
       <c r="DJ71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -25980,6 +26196,9 @@
       <c r="DJ72" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DK72" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -26330,6 +26549,9 @@
       <c r="DJ73" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DK73" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -26680,6 +26902,9 @@
       <c r="DJ74" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK74" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -27030,6 +27255,9 @@
       <c r="DJ75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -27380,6 +27608,9 @@
       <c r="DJ76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -27730,6 +27961,9 @@
       <c r="DJ77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="DK77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -28080,6 +28314,9 @@
       <c r="DJ78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DK78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -28430,6 +28667,9 @@
       <c r="DJ79" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK79" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -28780,6 +29020,9 @@
       <c r="DJ80" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK80" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -29130,6 +29373,9 @@
       <c r="DJ81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -29480,6 +29726,9 @@
       <c r="DJ82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DK82" s="3" t="n">
+        <v>21.29</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -29830,6 +30079,9 @@
       <c r="DJ83" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK83" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -30180,6 +30432,9 @@
       <c r="DJ84" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DK84" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -30530,6 +30785,9 @@
       <c r="DJ85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="DK85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -30880,6 +31138,9 @@
       <c r="DJ86" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DK86" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -31230,6 +31491,9 @@
       <c r="DJ87" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK87" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -31580,6 +31844,9 @@
       <c r="DJ88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -31930,6 +32197,9 @@
       <c r="DJ89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DK89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -32280,6 +32550,9 @@
       <c r="DJ90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -32630,6 +32903,9 @@
       <c r="DJ91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -32980,6 +33256,9 @@
       <c r="DJ92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -33330,6 +33609,9 @@
       <c r="DJ93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DK93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -33680,6 +33962,9 @@
       <c r="DJ94" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DK94" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -34030,6 +34315,9 @@
       <c r="DJ95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DK95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -34380,6 +34668,9 @@
       <c r="DJ96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="DK96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -34730,6 +35021,9 @@
       <c r="DJ97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DK97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -35080,6 +35374,9 @@
       <c r="DJ98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DK98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -35430,6 +35727,9 @@
       <c r="DJ99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DK99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -35780,6 +36080,9 @@
       <c r="DJ100" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DK100" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -36130,6 +36433,9 @@
       <c r="DJ101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -36480,6 +36786,9 @@
       <c r="DJ102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="DK102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -36830,6 +37139,9 @@
       <c r="DJ103" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK103" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -37180,6 +37492,9 @@
       <c r="DJ104" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -37530,6 +37845,9 @@
       <c r="DJ105" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK105" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -37880,6 +38198,9 @@
       <c r="DJ106" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK106" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -38230,6 +38551,9 @@
       <c r="DJ107" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DK107" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -38580,6 +38904,9 @@
       <c r="DJ108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DK108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -38930,6 +39257,9 @@
       <c r="DJ109" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DK109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -39280,6 +39610,9 @@
       <c r="DJ110" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DK110" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -39630,6 +39963,9 @@
       <c r="DJ111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DK111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -39980,6 +40316,9 @@
       <c r="DJ112" s="3" t="n">
         <v>23.8</v>
       </c>
+      <c r="DK112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -40330,6 +40669,9 @@
       <c r="DJ113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DK113" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -40680,6 +41022,9 @@
       <c r="DJ114" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK114" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -41030,6 +41375,9 @@
       <c r="DJ115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DK115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -41380,6 +41728,9 @@
       <c r="DJ116" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DK116" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -41730,6 +42081,9 @@
       <c r="DJ117" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DK117" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -42080,6 +42434,9 @@
       <c r="DJ118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DK118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -42430,6 +42787,9 @@
       <c r="DJ119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="DK119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -42780,6 +43140,9 @@
       <c r="DJ120" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK120" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -43130,6 +43493,9 @@
       <c r="DJ121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DK121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -43480,6 +43846,9 @@
       <c r="DJ122" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK122" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -43830,6 +44199,9 @@
       <c r="DJ123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DK123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -44180,6 +44552,9 @@
       <c r="DJ124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="DK124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -44530,6 +44905,9 @@
       <c r="DJ125" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DK125" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -44880,6 +45258,9 @@
       <c r="DJ126" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DK126" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -45230,6 +45611,9 @@
       <c r="DJ127" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DK127" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -45580,6 +45964,9 @@
       <c r="DJ128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="DK128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -45930,6 +46317,9 @@
       <c r="DJ129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DK129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -46280,6 +46670,9 @@
       <c r="DJ130" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DK130" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -46630,6 +47023,9 @@
       <c r="DJ131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="DK131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -46980,6 +47376,9 @@
       <c r="DJ132" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DK132" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -47330,6 +47729,9 @@
       <c r="DJ133" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DK133" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -47680,6 +48082,9 @@
       <c r="DJ134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="DK134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -48030,6 +48435,9 @@
       <c r="DJ135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DK135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -48380,6 +48788,9 @@
       <c r="DJ136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DK136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -48730,6 +49141,9 @@
       <c r="DJ137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DK137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -49080,6 +49494,9 @@
       <c r="DJ138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DK138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -49430,6 +49847,9 @@
       <c r="DJ139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DK139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -49780,6 +50200,9 @@
       <c r="DJ140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DK140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -50130,6 +50553,9 @@
       <c r="DJ141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DK141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -50480,6 +50906,9 @@
       <c r="DJ142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DK142" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -50830,6 +51259,9 @@
       <c r="DJ143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DK143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -51180,6 +51612,9 @@
       <c r="DJ144" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DK144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -51530,6 +51965,9 @@
       <c r="DJ145" s="3" t="n">
         <v>23.19</v>
       </c>
+      <c r="DK145" s="3" t="n">
+        <v>23.19</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -51880,6 +52318,9 @@
       <c r="DJ146" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DK146" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -52230,6 +52671,9 @@
       <c r="DJ147" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DK147" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -52580,6 +53024,9 @@
       <c r="DJ148" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DK148" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -52930,6 +53377,9 @@
       <c r="DJ149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DK149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -53280,6 +53730,9 @@
       <c r="DJ150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DK150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -53630,6 +54083,9 @@
       <c r="DJ151" s="3" t="n">
         <v>23.39</v>
       </c>
+      <c r="DK151" s="3" t="n">
+        <v>23.39</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -53980,6 +54436,9 @@
       <c r="DJ152" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DK152" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -54330,6 +54789,9 @@
       <c r="DJ153" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DK153" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -54680,6 +55142,9 @@
       <c r="DJ154" s="3" t="n">
         <v>23.7</v>
       </c>
+      <c r="DK154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -55030,6 +55495,9 @@
       <c r="DJ155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DK155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -55380,6 +55848,9 @@
       <c r="DJ156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DK156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -55730,6 +56201,9 @@
       <c r="DJ157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DK157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -56080,6 +56554,9 @@
       <c r="DJ158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DK158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -56430,6 +56907,9 @@
       <c r="DJ159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DK159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -56780,6 +57260,9 @@
       <c r="DJ160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DK160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -57130,6 +57613,9 @@
       <c r="DJ161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DK161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -57480,6 +57966,9 @@
       <c r="DJ162" s="3" t="n">
         <v>24.49</v>
       </c>
+      <c r="DK162" s="3" t="n">
+        <v>24.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -57830,6 +58319,9 @@
       <c r="DJ163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DK163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -58180,6 +58672,9 @@
       <c r="DJ164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="DK164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -58431,9 +58926,12 @@
       <c r="DJ165" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DK165" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:DJ165"/>
+  <autoFilter ref="A1:DK165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-18 21:08 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DK$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DL$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DK165"/>
+  <dimension ref="A1:DL165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -558,6 +558,7 @@
     <col width="16" customWidth="1" min="113" max="113"/>
     <col width="16" customWidth="1" min="114" max="114"/>
     <col width="16" customWidth="1" min="115" max="115"/>
+    <col width="16" customWidth="1" min="116" max="116"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1136,6 +1137,11 @@
           <t>2026-09-18 13:10</t>
         </is>
       </c>
+      <c r="DL1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-18 16:08</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1489,6 +1495,9 @@
       <c r="DK2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="DL2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1842,6 +1851,9 @@
       <c r="DK3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="DL3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2195,6 +2207,9 @@
       <c r="DK4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="DL4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2548,6 +2563,9 @@
       <c r="DK5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DL5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2901,6 +2919,9 @@
       <c r="DK6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DL6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3254,6 +3275,9 @@
       <c r="DK7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="DL7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3607,6 +3631,9 @@
       <c r="DK8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DL8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3960,6 +3987,9 @@
       <c r="DK9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="DL9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4313,6 +4343,9 @@
       <c r="DK10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DL10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4666,6 +4699,9 @@
       <c r="DK11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DL11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -5019,6 +5055,9 @@
       <c r="DK12" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL12" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -5372,6 +5411,9 @@
       <c r="DK13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="DL13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5725,6 +5767,9 @@
       <c r="DK14" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DL14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -6078,6 +6123,9 @@
       <c r="DK15" s="3" t="n">
         <v>21.41</v>
       </c>
+      <c r="DL15" s="3" t="n">
+        <v>21.41</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -6431,6 +6479,9 @@
       <c r="DK16" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DL16" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6784,6 +6835,9 @@
       <c r="DK17" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DL17" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -7137,6 +7191,9 @@
       <c r="DK18" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DL18" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -7490,6 +7547,9 @@
       <c r="DK19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="DL19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -7843,6 +7903,9 @@
       <c r="DK20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DL20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -8196,6 +8259,9 @@
       <c r="DK21" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DL21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -8549,6 +8615,9 @@
       <c r="DK22" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DL22" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -8902,6 +8971,9 @@
       <c r="DK23" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DL23" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -9255,6 +9327,9 @@
       <c r="DK24" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DL24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -9608,6 +9683,9 @@
       <c r="DK25" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DL25" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -9961,6 +10039,9 @@
       <c r="DK26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DL26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -10314,6 +10395,9 @@
       <c r="DK27" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DL27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -10667,6 +10751,9 @@
       <c r="DK28" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DL28" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -11020,6 +11107,9 @@
       <c r="DK29" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DL29" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -11373,6 +11463,9 @@
       <c r="DK30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -11726,6 +11819,9 @@
       <c r="DK31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DL31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -12079,6 +12175,9 @@
       <c r="DK32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DL32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -12432,6 +12531,9 @@
       <c r="DK33" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -12785,6 +12887,9 @@
       <c r="DK34" s="3" t="n">
         <v>21.77</v>
       </c>
+      <c r="DL34" s="3" t="n">
+        <v>21.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -13138,6 +13243,9 @@
       <c r="DK35" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DL35" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -13491,6 +13599,9 @@
       <c r="DK36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DL36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -13844,6 +13955,9 @@
       <c r="DK37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DL37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -14197,6 +14311,9 @@
       <c r="DK38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DL38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -14550,6 +14667,9 @@
       <c r="DK39" s="3" t="n">
         <v>21.98</v>
       </c>
+      <c r="DL39" s="3" t="n">
+        <v>21.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -14903,6 +15023,9 @@
       <c r="DK40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -15256,6 +15379,9 @@
       <c r="DK41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DL41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -15609,6 +15735,9 @@
       <c r="DK42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DL42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -15962,6 +16091,9 @@
       <c r="DK43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DL43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -16315,6 +16447,9 @@
       <c r="DK44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -16668,6 +16803,9 @@
       <c r="DK45" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DL45" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -17021,6 +17159,9 @@
       <c r="DK46" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="DL46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -17374,6 +17515,9 @@
       <c r="DK47" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DL47" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -17727,6 +17871,9 @@
       <c r="DK48" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DL48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -18080,6 +18227,9 @@
       <c r="DK49" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DL49" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -18433,6 +18583,9 @@
       <c r="DK50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="DL50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -18786,6 +18939,9 @@
       <c r="DK51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DL51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -19139,6 +19295,9 @@
       <c r="DK52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DL52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -19492,6 +19651,9 @@
       <c r="DK53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="DL53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -19845,6 +20007,9 @@
       <c r="DK54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -20198,6 +20363,9 @@
       <c r="DK55" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DL55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -20551,6 +20719,9 @@
       <c r="DK56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -20904,6 +21075,9 @@
       <c r="DK57" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DL57" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -21257,6 +21431,9 @@
       <c r="DK58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="DL58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -21610,6 +21787,9 @@
       <c r="DK59" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DL59" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -21963,6 +22143,9 @@
       <c r="DK60" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DL60" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -22316,6 +22499,9 @@
       <c r="DK61" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DL61" s="3" t="n">
+        <v>21.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -22669,6 +22855,9 @@
       <c r="DK62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DL62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -23022,6 +23211,9 @@
       <c r="DK63" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DL63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -23375,6 +23567,9 @@
       <c r="DK64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DL64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -23728,6 +23923,9 @@
       <c r="DK65" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL65" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -24081,6 +24279,9 @@
       <c r="DK66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -24434,6 +24635,9 @@
       <c r="DK67" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL67" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -24787,6 +24991,9 @@
       <c r="DK68" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DL68" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -25140,6 +25347,9 @@
       <c r="DK69" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL69" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -25493,6 +25703,9 @@
       <c r="DK70" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL70" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -25846,6 +26059,9 @@
       <c r="DK71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -26199,6 +26415,9 @@
       <c r="DK72" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DL72" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -26552,6 +26771,9 @@
       <c r="DK73" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL73" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -26905,6 +27127,9 @@
       <c r="DK74" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL74" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -27258,6 +27483,9 @@
       <c r="DK75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -27611,6 +27839,9 @@
       <c r="DK76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -27964,6 +28195,9 @@
       <c r="DK77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="DL77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -28317,6 +28551,9 @@
       <c r="DK78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DL78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -28670,6 +28907,9 @@
       <c r="DK79" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL79" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -29023,6 +29263,9 @@
       <c r="DK80" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL80" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -29376,6 +29619,9 @@
       <c r="DK81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -29729,6 +29975,9 @@
       <c r="DK82" s="3" t="n">
         <v>21.29</v>
       </c>
+      <c r="DL82" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -30082,6 +30331,9 @@
       <c r="DK83" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL83" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -30435,6 +30687,9 @@
       <c r="DK84" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DL84" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -30788,6 +31043,9 @@
       <c r="DK85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="DL85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -31141,6 +31399,9 @@
       <c r="DK86" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL86" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -31494,6 +31755,9 @@
       <c r="DK87" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL87" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -31847,6 +32111,9 @@
       <c r="DK88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -32200,6 +32467,9 @@
       <c r="DK89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DL89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -32553,6 +32823,9 @@
       <c r="DK90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -32906,6 +33179,9 @@
       <c r="DK91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -33259,6 +33535,9 @@
       <c r="DK92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -33612,6 +33891,9 @@
       <c r="DK93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DL93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -33965,6 +34247,9 @@
       <c r="DK94" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DL94" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -34318,6 +34603,9 @@
       <c r="DK95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DL95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -34671,6 +34959,9 @@
       <c r="DK96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="DL96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -35024,6 +35315,9 @@
       <c r="DK97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DL97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -35377,6 +35671,9 @@
       <c r="DK98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DL98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -35730,6 +36027,9 @@
       <c r="DK99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DL99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -36083,6 +36383,9 @@
       <c r="DK100" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DL100" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -36436,6 +36739,9 @@
       <c r="DK101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -36789,6 +37095,9 @@
       <c r="DK102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="DL102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -37142,6 +37451,9 @@
       <c r="DK103" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL103" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -37495,6 +37807,9 @@
       <c r="DK104" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -37848,6 +38163,9 @@
       <c r="DK105" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL105" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -38201,6 +38519,9 @@
       <c r="DK106" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL106" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -38554,6 +38875,9 @@
       <c r="DK107" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DL107" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -38907,6 +39231,9 @@
       <c r="DK108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DL108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -39260,6 +39587,9 @@
       <c r="DK109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -39613,6 +39943,9 @@
       <c r="DK110" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DL110" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -39966,6 +40299,9 @@
       <c r="DK111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DL111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -40319,6 +40655,9 @@
       <c r="DK112" s="3" t="n">
         <v>23.8</v>
       </c>
+      <c r="DL112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -40672,6 +41011,9 @@
       <c r="DK113" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DL113" s="3" t="n">
+        <v>22.55</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -41025,6 +41367,9 @@
       <c r="DK114" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL114" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -41378,6 +41723,9 @@
       <c r="DK115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DL115" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -41731,6 +42079,9 @@
       <c r="DK116" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DL116" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -42084,6 +42435,9 @@
       <c r="DK117" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL117" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -42437,6 +42791,9 @@
       <c r="DK118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DL118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -42790,6 +43147,9 @@
       <c r="DK119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="DL119" s="3" t="n">
+        <v>21.35</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -43143,6 +43503,9 @@
       <c r="DK120" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL120" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -43496,6 +43859,9 @@
       <c r="DK121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DL121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -43849,6 +44215,9 @@
       <c r="DK122" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL122" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -44202,6 +44571,9 @@
       <c r="DK123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DL123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -44555,6 +44927,9 @@
       <c r="DK124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="DL124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -44908,6 +45283,9 @@
       <c r="DK125" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DL125" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -45261,6 +45639,9 @@
       <c r="DK126" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DL126" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -45614,6 +45995,9 @@
       <c r="DK127" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DL127" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -45967,6 +46351,9 @@
       <c r="DK128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="DL128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -46320,6 +46707,9 @@
       <c r="DK129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DL129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -46673,6 +47063,9 @@
       <c r="DK130" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DL130" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -47026,6 +47419,9 @@
       <c r="DK131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="DL131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -47379,6 +47775,9 @@
       <c r="DK132" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DL132" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -47732,6 +48131,9 @@
       <c r="DK133" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DL133" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -48085,6 +48487,9 @@
       <c r="DK134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="DL134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -48438,6 +48843,9 @@
       <c r="DK135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DL135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -48791,6 +49199,9 @@
       <c r="DK136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DL136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -49144,6 +49555,9 @@
       <c r="DK137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DL137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -49497,6 +49911,9 @@
       <c r="DK138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DL138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -49850,6 +50267,9 @@
       <c r="DK139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DL139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -50203,6 +50623,9 @@
       <c r="DK140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DL140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -50556,6 +50979,9 @@
       <c r="DK141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DL141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -50909,6 +51335,9 @@
       <c r="DK142" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DL142" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -51262,6 +51691,9 @@
       <c r="DK143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DL143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -51615,6 +52047,9 @@
       <c r="DK144" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DL144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -51968,6 +52403,9 @@
       <c r="DK145" s="3" t="n">
         <v>23.19</v>
       </c>
+      <c r="DL145" s="3" t="n">
+        <v>23.19</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -52321,6 +52759,9 @@
       <c r="DK146" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DL146" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -52674,6 +53115,9 @@
       <c r="DK147" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DL147" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -53027,6 +53471,9 @@
       <c r="DK148" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DL148" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -53380,6 +53827,9 @@
       <c r="DK149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DL149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -53733,6 +54183,9 @@
       <c r="DK150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DL150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -54086,6 +54539,9 @@
       <c r="DK151" s="3" t="n">
         <v>23.39</v>
       </c>
+      <c r="DL151" s="3" t="n">
+        <v>23.39</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -54439,6 +54895,9 @@
       <c r="DK152" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DL152" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -54792,6 +55251,9 @@
       <c r="DK153" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DL153" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -55145,6 +55607,9 @@
       <c r="DK154" s="3" t="n">
         <v>23.7</v>
       </c>
+      <c r="DL154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -55498,6 +55963,9 @@
       <c r="DK155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DL155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -55851,6 +56319,9 @@
       <c r="DK156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DL156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -56204,6 +56675,9 @@
       <c r="DK157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DL157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -56557,6 +57031,9 @@
       <c r="DK158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DL158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -56910,6 +57387,9 @@
       <c r="DK159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DL159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -57263,6 +57743,9 @@
       <c r="DK160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DL160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -57616,6 +58099,9 @@
       <c r="DK161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DL161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -57969,6 +58455,9 @@
       <c r="DK162" s="3" t="n">
         <v>24.49</v>
       </c>
+      <c r="DL162" s="3" t="n">
+        <v>24.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -58322,6 +58811,9 @@
       <c r="DK163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DL163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -58675,6 +59167,9 @@
       <c r="DK164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="DL164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -58929,9 +59424,12 @@
       <c r="DK165" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DL165" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:DK165"/>
+  <autoFilter ref="A1:DL165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-19 00:12 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DL$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DM$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DL165"/>
+  <dimension ref="A1:DM165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -559,6 +559,7 @@
     <col width="16" customWidth="1" min="114" max="114"/>
     <col width="16" customWidth="1" min="115" max="115"/>
     <col width="16" customWidth="1" min="116" max="116"/>
+    <col width="16" customWidth="1" min="117" max="117"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1142,6 +1143,11 @@
           <t>2026-09-18 16:08</t>
         </is>
       </c>
+      <c r="DM1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-18 19:12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1498,6 +1504,9 @@
       <c r="DL2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="DM2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1854,6 +1863,9 @@
       <c r="DL3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="DM3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2210,6 +2222,9 @@
       <c r="DL4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="DM4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2566,6 +2581,9 @@
       <c r="DL5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DM5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2922,6 +2940,9 @@
       <c r="DL6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DM6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3278,6 +3299,9 @@
       <c r="DL7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="DM7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3634,6 +3658,9 @@
       <c r="DL8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DM8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3990,6 +4017,9 @@
       <c r="DL9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="DM9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4346,6 +4376,9 @@
       <c r="DL10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DM10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4702,6 +4735,9 @@
       <c r="DL11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DM11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -5058,6 +5094,9 @@
       <c r="DL12" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM12" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -5414,6 +5453,9 @@
       <c r="DL13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="DM13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5770,6 +5812,9 @@
       <c r="DL14" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DM14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -6126,6 +6171,9 @@
       <c r="DL15" s="3" t="n">
         <v>21.41</v>
       </c>
+      <c r="DM15" s="3" t="n">
+        <v>21.41</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -6482,6 +6530,9 @@
       <c r="DL16" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DM16" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6838,6 +6889,9 @@
       <c r="DL17" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DM17" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -7194,6 +7248,9 @@
       <c r="DL18" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DM18" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -7550,6 +7607,9 @@
       <c r="DL19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="DM19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -7906,6 +7966,9 @@
       <c r="DL20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DM20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -8262,6 +8325,9 @@
       <c r="DL21" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DM21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -8618,6 +8684,9 @@
       <c r="DL22" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DM22" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -8974,6 +9043,9 @@
       <c r="DL23" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DM23" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -9330,6 +9402,9 @@
       <c r="DL24" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DM24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -9686,6 +9761,9 @@
       <c r="DL25" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DM25" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -10042,6 +10120,9 @@
       <c r="DL26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DM26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -10398,6 +10479,9 @@
       <c r="DL27" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DM27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -10754,6 +10838,9 @@
       <c r="DL28" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DM28" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -11110,6 +11197,9 @@
       <c r="DL29" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DM29" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -11466,6 +11556,9 @@
       <c r="DL30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -11822,6 +11915,9 @@
       <c r="DL31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DM31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -12178,6 +12274,9 @@
       <c r="DL32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DM32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -12534,6 +12633,9 @@
       <c r="DL33" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -12890,6 +12992,9 @@
       <c r="DL34" s="3" t="n">
         <v>21.77</v>
       </c>
+      <c r="DM34" s="3" t="n">
+        <v>21.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -13246,6 +13351,9 @@
       <c r="DL35" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DM35" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -13602,6 +13710,9 @@
       <c r="DL36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DM36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -13958,6 +14069,9 @@
       <c r="DL37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DM37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -14314,6 +14428,9 @@
       <c r="DL38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DM38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -14670,6 +14787,9 @@
       <c r="DL39" s="3" t="n">
         <v>21.98</v>
       </c>
+      <c r="DM39" s="3" t="n">
+        <v>21.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -15026,6 +15146,9 @@
       <c r="DL40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -15382,6 +15505,9 @@
       <c r="DL41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DM41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -15738,6 +15864,9 @@
       <c r="DL42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DM42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -16094,6 +16223,9 @@
       <c r="DL43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DM43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -16450,6 +16582,9 @@
       <c r="DL44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -16806,6 +16941,9 @@
       <c r="DL45" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DM45" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -17162,6 +17300,9 @@
       <c r="DL46" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="DM46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -17518,6 +17659,9 @@
       <c r="DL47" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DM47" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -17874,6 +18018,9 @@
       <c r="DL48" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DM48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -18230,6 +18377,9 @@
       <c r="DL49" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DM49" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -18586,6 +18736,9 @@
       <c r="DL50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="DM50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -18942,6 +19095,9 @@
       <c r="DL51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DM51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -19298,6 +19454,9 @@
       <c r="DL52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DM52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -19654,6 +19813,9 @@
       <c r="DL53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="DM53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -20010,6 +20172,9 @@
       <c r="DL54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -20366,6 +20531,9 @@
       <c r="DL55" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DM55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -20722,6 +20890,9 @@
       <c r="DL56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -21078,6 +21249,9 @@
       <c r="DL57" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DM57" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -21434,6 +21608,9 @@
       <c r="DL58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="DM58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -21790,6 +21967,9 @@
       <c r="DL59" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DM59" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -22146,6 +22326,9 @@
       <c r="DL60" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DM60" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -22502,6 +22685,9 @@
       <c r="DL61" s="3" t="n">
         <v>21.95</v>
       </c>
+      <c r="DM61" s="3" t="n">
+        <v>21.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -22858,6 +23044,9 @@
       <c r="DL62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DM62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -23214,6 +23403,9 @@
       <c r="DL63" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DM63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -23570,6 +23762,9 @@
       <c r="DL64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DM64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -23926,6 +24121,9 @@
       <c r="DL65" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM65" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -24282,6 +24480,9 @@
       <c r="DL66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -24638,6 +24839,9 @@
       <c r="DL67" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM67" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -24994,6 +25198,9 @@
       <c r="DL68" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DM68" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -25350,6 +25557,9 @@
       <c r="DL69" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM69" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -25706,6 +25916,9 @@
       <c r="DL70" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM70" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -26062,6 +26275,9 @@
       <c r="DL71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -26418,6 +26634,9 @@
       <c r="DL72" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DM72" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -26774,6 +26993,9 @@
       <c r="DL73" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM73" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -27130,6 +27352,9 @@
       <c r="DL74" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM74" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -27486,6 +27711,9 @@
       <c r="DL75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -27842,6 +28070,9 @@
       <c r="DL76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -28198,6 +28429,9 @@
       <c r="DL77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="DM77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -28554,6 +28788,9 @@
       <c r="DL78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DM78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -28910,6 +29147,9 @@
       <c r="DL79" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM79" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -29266,6 +29506,9 @@
       <c r="DL80" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM80" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -29622,6 +29865,9 @@
       <c r="DL81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -29978,6 +30224,9 @@
       <c r="DL82" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DM82" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -30334,6 +30583,9 @@
       <c r="DL83" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM83" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -30690,6 +30942,9 @@
       <c r="DL84" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DM84" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -31046,6 +31301,9 @@
       <c r="DL85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="DM85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -31402,6 +31660,9 @@
       <c r="DL86" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM86" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -31758,6 +32019,9 @@
       <c r="DL87" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM87" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -32114,6 +32378,9 @@
       <c r="DL88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -32470,6 +32737,9 @@
       <c r="DL89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DM89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -32826,6 +33096,9 @@
       <c r="DL90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -33182,6 +33455,9 @@
       <c r="DL91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -33538,6 +33814,9 @@
       <c r="DL92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -33894,6 +34173,9 @@
       <c r="DL93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DM93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -34250,6 +34532,9 @@
       <c r="DL94" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DM94" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -34606,6 +34891,9 @@
       <c r="DL95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DM95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -34962,6 +35250,9 @@
       <c r="DL96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="DM96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -35318,6 +35609,9 @@
       <c r="DL97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DM97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -35674,6 +35968,9 @@
       <c r="DL98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DM98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -36030,6 +36327,9 @@
       <c r="DL99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DM99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -36386,6 +36686,9 @@
       <c r="DL100" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DM100" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -36742,6 +37045,9 @@
       <c r="DL101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -37098,6 +37404,9 @@
       <c r="DL102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="DM102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -37454,6 +37763,9 @@
       <c r="DL103" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM103" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -37810,6 +38122,9 @@
       <c r="DL104" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -38166,6 +38481,9 @@
       <c r="DL105" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM105" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -38522,6 +38840,9 @@
       <c r="DL106" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM106" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -38878,6 +39199,9 @@
       <c r="DL107" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DM107" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -39234,6 +39558,9 @@
       <c r="DL108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DM108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -39590,6 +39917,9 @@
       <c r="DL109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -39946,6 +40276,9 @@
       <c r="DL110" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DM110" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -40302,6 +40635,9 @@
       <c r="DL111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DM111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -40658,6 +40994,9 @@
       <c r="DL112" s="3" t="n">
         <v>23.8</v>
       </c>
+      <c r="DM112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -41014,6 +41353,9 @@
       <c r="DL113" s="3" t="n">
         <v>22.55</v>
       </c>
+      <c r="DM113" s="3" t="n">
+        <v>22.55</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -41370,6 +41712,9 @@
       <c r="DL114" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM114" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -41726,6 +42071,9 @@
       <c r="DL115" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DM115" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -42082,6 +42430,9 @@
       <c r="DL116" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DM116" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -42438,6 +42789,9 @@
       <c r="DL117" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM117" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -42794,6 +43148,9 @@
       <c r="DL118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DM118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -43150,6 +43507,9 @@
       <c r="DL119" s="3" t="n">
         <v>21.35</v>
       </c>
+      <c r="DM119" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -43506,6 +43866,9 @@
       <c r="DL120" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM120" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -43862,6 +44225,9 @@
       <c r="DL121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DM121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -44218,6 +44584,9 @@
       <c r="DL122" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DM122" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -44574,6 +44943,9 @@
       <c r="DL123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DM123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -44930,6 +45302,9 @@
       <c r="DL124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="DM124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -45286,6 +45661,9 @@
       <c r="DL125" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DM125" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -45642,6 +46020,9 @@
       <c r="DL126" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DM126" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -45998,6 +46379,9 @@
       <c r="DL127" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DM127" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -46354,6 +46738,9 @@
       <c r="DL128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="DM128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -46710,6 +47097,9 @@
       <c r="DL129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DM129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -47066,6 +47456,9 @@
       <c r="DL130" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DM130" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -47422,6 +47815,9 @@
       <c r="DL131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="DM131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -47778,6 +48174,9 @@
       <c r="DL132" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DM132" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -48134,6 +48533,9 @@
       <c r="DL133" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DM133" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -48490,6 +48892,9 @@
       <c r="DL134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="DM134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -48846,6 +49251,9 @@
       <c r="DL135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DM135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -49202,6 +49610,9 @@
       <c r="DL136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DM136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -49558,6 +49969,9 @@
       <c r="DL137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DM137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -49914,6 +50328,9 @@
       <c r="DL138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DM138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -50270,6 +50687,9 @@
       <c r="DL139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DM139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -50626,6 +51046,9 @@
       <c r="DL140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DM140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -50982,6 +51405,9 @@
       <c r="DL141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DM141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -51338,6 +51764,9 @@
       <c r="DL142" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DM142" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -51694,6 +52123,9 @@
       <c r="DL143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DM143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -52050,6 +52482,9 @@
       <c r="DL144" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DM144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -52406,6 +52841,9 @@
       <c r="DL145" s="3" t="n">
         <v>23.19</v>
       </c>
+      <c r="DM145" s="3" t="n">
+        <v>23.19</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -52762,6 +53200,9 @@
       <c r="DL146" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DM146" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -53118,6 +53559,9 @@
       <c r="DL147" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DM147" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -53474,6 +53918,9 @@
       <c r="DL148" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DM148" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -53830,6 +54277,9 @@
       <c r="DL149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DM149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -54186,6 +54636,9 @@
       <c r="DL150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DM150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -54542,6 +54995,9 @@
       <c r="DL151" s="3" t="n">
         <v>23.39</v>
       </c>
+      <c r="DM151" s="3" t="n">
+        <v>23.39</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -54898,6 +55354,9 @@
       <c r="DL152" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DM152" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -55254,6 +55713,9 @@
       <c r="DL153" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DM153" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -55610,6 +56072,9 @@
       <c r="DL154" s="3" t="n">
         <v>23.7</v>
       </c>
+      <c r="DM154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -55966,6 +56431,9 @@
       <c r="DL155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DM155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -56322,6 +56790,9 @@
       <c r="DL156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DM156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -56678,6 +57149,9 @@
       <c r="DL157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DM157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -57034,6 +57508,9 @@
       <c r="DL158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DM158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -57390,6 +57867,9 @@
       <c r="DL159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DM159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -57746,6 +58226,9 @@
       <c r="DL160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DM160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -58102,6 +58585,9 @@
       <c r="DL161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DM161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -58458,6 +58944,9 @@
       <c r="DL162" s="3" t="n">
         <v>24.49</v>
       </c>
+      <c r="DM162" s="3" t="n">
+        <v>24.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -58814,6 +59303,9 @@
       <c r="DL163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DM163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -59170,6 +59662,9 @@
       <c r="DL164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="DM164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -59427,9 +59922,12 @@
       <c r="DL165" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DM165" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:DL165"/>
+  <autoFilter ref="A1:DM165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-19 03:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DM$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DN$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DM165"/>
+  <dimension ref="A1:DN165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -560,6 +560,7 @@
     <col width="16" customWidth="1" min="115" max="115"/>
     <col width="16" customWidth="1" min="116" max="116"/>
     <col width="16" customWidth="1" min="117" max="117"/>
+    <col width="16" customWidth="1" min="118" max="118"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1148,6 +1149,11 @@
           <t>2026-09-18 19:12</t>
         </is>
       </c>
+      <c r="DN1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-18 22:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1507,6 +1513,9 @@
       <c r="DM2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="DN2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1866,6 +1875,9 @@
       <c r="DM3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="DN3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2225,6 +2237,9 @@
       <c r="DM4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="DN4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2584,6 +2599,9 @@
       <c r="DM5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DN5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2943,6 +2961,9 @@
       <c r="DM6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DN6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3302,6 +3323,9 @@
       <c r="DM7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="DN7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3661,6 +3685,9 @@
       <c r="DM8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DN8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -4020,6 +4047,9 @@
       <c r="DM9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="DN9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4379,6 +4409,9 @@
       <c r="DM10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DN10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4738,6 +4771,9 @@
       <c r="DM11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DN11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -5097,6 +5133,9 @@
       <c r="DM12" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN12" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -5456,6 +5495,9 @@
       <c r="DM13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="DN13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5815,6 +5857,9 @@
       <c r="DM14" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DN14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -6174,6 +6219,9 @@
       <c r="DM15" s="3" t="n">
         <v>21.41</v>
       </c>
+      <c r="DN15" s="3" t="n">
+        <v>21.41</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -6533,6 +6581,9 @@
       <c r="DM16" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DN16" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6892,6 +6943,9 @@
       <c r="DM17" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DN17" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -7251,6 +7305,9 @@
       <c r="DM18" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DN18" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -7610,6 +7667,9 @@
       <c r="DM19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="DN19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -7969,6 +8029,9 @@
       <c r="DM20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DN20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -8328,6 +8391,9 @@
       <c r="DM21" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DN21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -8687,6 +8753,9 @@
       <c r="DM22" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DN22" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -9046,6 +9115,9 @@
       <c r="DM23" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DN23" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -9405,6 +9477,9 @@
       <c r="DM24" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DN24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -9764,6 +9839,9 @@
       <c r="DM25" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DN25" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -10123,6 +10201,9 @@
       <c r="DM26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DN26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -10482,6 +10563,9 @@
       <c r="DM27" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DN27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -10841,6 +10925,9 @@
       <c r="DM28" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DN28" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -11200,6 +11287,9 @@
       <c r="DM29" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DN29" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -11559,6 +11649,9 @@
       <c r="DM30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -11918,6 +12011,9 @@
       <c r="DM31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DN31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -12277,6 +12373,9 @@
       <c r="DM32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DN32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -12636,6 +12735,9 @@
       <c r="DM33" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -12995,6 +13097,9 @@
       <c r="DM34" s="3" t="n">
         <v>21.77</v>
       </c>
+      <c r="DN34" s="3" t="n">
+        <v>21.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -13354,6 +13459,9 @@
       <c r="DM35" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DN35" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -13713,6 +13821,9 @@
       <c r="DM36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DN36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -14072,6 +14183,9 @@
       <c r="DM37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DN37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -14431,6 +14545,9 @@
       <c r="DM38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DN38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -14790,6 +14907,9 @@
       <c r="DM39" s="3" t="n">
         <v>21.98</v>
       </c>
+      <c r="DN39" s="3" t="n">
+        <v>21.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -15149,6 +15269,9 @@
       <c r="DM40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -15508,6 +15631,9 @@
       <c r="DM41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DN41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -15867,6 +15993,9 @@
       <c r="DM42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DN42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -16226,6 +16355,9 @@
       <c r="DM43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DN43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -16585,6 +16717,9 @@
       <c r="DM44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -16944,6 +17079,9 @@
       <c r="DM45" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DN45" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -17303,6 +17441,9 @@
       <c r="DM46" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="DN46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -17662,6 +17803,9 @@
       <c r="DM47" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DN47" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -18021,6 +18165,9 @@
       <c r="DM48" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DN48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -18380,6 +18527,9 @@
       <c r="DM49" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DN49" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -18739,6 +18889,9 @@
       <c r="DM50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="DN50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -19098,6 +19251,9 @@
       <c r="DM51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DN51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -19457,6 +19613,9 @@
       <c r="DM52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DN52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -19816,6 +19975,9 @@
       <c r="DM53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="DN53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -20175,6 +20337,9 @@
       <c r="DM54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -20534,6 +20699,9 @@
       <c r="DM55" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DN55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -20893,6 +21061,9 @@
       <c r="DM56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -21252,6 +21423,9 @@
       <c r="DM57" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DN57" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -21611,6 +21785,9 @@
       <c r="DM58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="DN58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -21970,6 +22147,9 @@
       <c r="DM59" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DN59" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -22329,6 +22509,9 @@
       <c r="DM60" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DN60" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -22688,6 +22871,9 @@
       <c r="DM61" s="3" t="n">
         <v>21.95</v>
       </c>
+      <c r="DN61" s="3" t="n">
+        <v>21.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -23047,6 +23233,9 @@
       <c r="DM62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DN62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -23406,6 +23595,9 @@
       <c r="DM63" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DN63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -23765,6 +23957,9 @@
       <c r="DM64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DN64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -24124,6 +24319,9 @@
       <c r="DM65" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN65" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -24483,6 +24681,9 @@
       <c r="DM66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -24842,6 +25043,9 @@
       <c r="DM67" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN67" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -25201,6 +25405,9 @@
       <c r="DM68" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DN68" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -25560,6 +25767,9 @@
       <c r="DM69" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN69" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -25919,6 +26129,9 @@
       <c r="DM70" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN70" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -26278,6 +26491,9 @@
       <c r="DM71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -26637,6 +26853,9 @@
       <c r="DM72" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DN72" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -26996,6 +27215,9 @@
       <c r="DM73" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN73" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -27355,6 +27577,9 @@
       <c r="DM74" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN74" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -27714,6 +27939,9 @@
       <c r="DM75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -28073,6 +28301,9 @@
       <c r="DM76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -28432,6 +28663,9 @@
       <c r="DM77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="DN77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -28791,6 +29025,9 @@
       <c r="DM78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DN78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -29150,6 +29387,9 @@
       <c r="DM79" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN79" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -29509,6 +29749,9 @@
       <c r="DM80" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN80" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -29868,6 +30111,9 @@
       <c r="DM81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -30227,6 +30473,9 @@
       <c r="DM82" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DN82" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -30586,6 +30835,9 @@
       <c r="DM83" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN83" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -30945,6 +31197,9 @@
       <c r="DM84" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DN84" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -31304,6 +31559,9 @@
       <c r="DM85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="DN85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -31663,6 +31921,9 @@
       <c r="DM86" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN86" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -32022,6 +32283,9 @@
       <c r="DM87" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DN87" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -32381,6 +32645,9 @@
       <c r="DM88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -32740,6 +33007,9 @@
       <c r="DM89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DN89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -33099,6 +33369,9 @@
       <c r="DM90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -33458,6 +33731,9 @@
       <c r="DM91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -33817,6 +34093,9 @@
       <c r="DM92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -34176,6 +34455,9 @@
       <c r="DM93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DN93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -34535,6 +34817,9 @@
       <c r="DM94" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DN94" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -34894,6 +35179,9 @@
       <c r="DM95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DN95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -35253,6 +35541,9 @@
       <c r="DM96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="DN96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -35612,6 +35903,9 @@
       <c r="DM97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DN97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -35971,6 +36265,9 @@
       <c r="DM98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DN98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -36330,6 +36627,9 @@
       <c r="DM99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DN99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -36689,6 +36989,9 @@
       <c r="DM100" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DN100" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -37048,6 +37351,9 @@
       <c r="DM101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -37407,6 +37713,9 @@
       <c r="DM102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="DN102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -37766,6 +38075,9 @@
       <c r="DM103" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN103" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -38125,6 +38437,9 @@
       <c r="DM104" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -38484,6 +38799,9 @@
       <c r="DM105" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN105" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -38843,6 +39161,9 @@
       <c r="DM106" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN106" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -39202,6 +39523,9 @@
       <c r="DM107" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DN107" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -39561,6 +39885,9 @@
       <c r="DM108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DN108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -39920,6 +40247,9 @@
       <c r="DM109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -40279,6 +40609,9 @@
       <c r="DM110" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DN110" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -40638,6 +40971,9 @@
       <c r="DM111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DN111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -40997,6 +41333,9 @@
       <c r="DM112" s="3" t="n">
         <v>23.8</v>
       </c>
+      <c r="DN112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -41356,6 +41695,9 @@
       <c r="DM113" s="3" t="n">
         <v>22.55</v>
       </c>
+      <c r="DN113" s="3" t="n">
+        <v>22.55</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -41715,6 +42057,9 @@
       <c r="DM114" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN114" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -42074,6 +42419,9 @@
       <c r="DM115" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN115" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -42433,6 +42781,9 @@
       <c r="DM116" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DN116" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -42792,6 +43143,9 @@
       <c r="DM117" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN117" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -43151,6 +43505,9 @@
       <c r="DM118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DN118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -43510,6 +43867,9 @@
       <c r="DM119" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN119" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -43869,6 +44229,9 @@
       <c r="DM120" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN120" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -44228,6 +44591,9 @@
       <c r="DM121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DN121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -44587,6 +44953,9 @@
       <c r="DM122" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DN122" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -44946,6 +45315,9 @@
       <c r="DM123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DN123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -45305,6 +45677,9 @@
       <c r="DM124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="DN124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -45664,6 +46039,9 @@
       <c r="DM125" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DN125" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -46023,6 +46401,9 @@
       <c r="DM126" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DN126" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -46382,6 +46763,9 @@
       <c r="DM127" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DN127" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -46741,6 +47125,9 @@
       <c r="DM128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="DN128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -47100,6 +47487,9 @@
       <c r="DM129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DN129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -47459,6 +47849,9 @@
       <c r="DM130" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DN130" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -47818,6 +48211,9 @@
       <c r="DM131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="DN131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -48177,6 +48573,9 @@
       <c r="DM132" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DN132" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -48536,6 +48935,9 @@
       <c r="DM133" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DN133" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -48895,6 +49297,9 @@
       <c r="DM134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="DN134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -49254,6 +49659,9 @@
       <c r="DM135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DN135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -49613,6 +50021,9 @@
       <c r="DM136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DN136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -49972,6 +50383,9 @@
       <c r="DM137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DN137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -50331,6 +50745,9 @@
       <c r="DM138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DN138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -50690,6 +51107,9 @@
       <c r="DM139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DN139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -51049,6 +51469,9 @@
       <c r="DM140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DN140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -51408,6 +51831,9 @@
       <c r="DM141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DN141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -51767,6 +52193,9 @@
       <c r="DM142" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DN142" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -52126,6 +52555,9 @@
       <c r="DM143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DN143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -52485,6 +52917,9 @@
       <c r="DM144" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DN144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -52844,6 +53279,9 @@
       <c r="DM145" s="3" t="n">
         <v>23.19</v>
       </c>
+      <c r="DN145" s="3" t="n">
+        <v>23.19</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -53203,6 +53641,9 @@
       <c r="DM146" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DN146" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -53562,6 +54003,9 @@
       <c r="DM147" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DN147" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -53921,6 +54365,9 @@
       <c r="DM148" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DN148" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -54280,6 +54727,9 @@
       <c r="DM149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DN149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -54639,6 +55089,9 @@
       <c r="DM150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DN150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -54998,6 +55451,9 @@
       <c r="DM151" s="3" t="n">
         <v>23.39</v>
       </c>
+      <c r="DN151" s="3" t="n">
+        <v>23.39</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -55357,6 +55813,9 @@
       <c r="DM152" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DN152" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -55716,6 +56175,9 @@
       <c r="DM153" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DN153" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -56075,6 +56537,9 @@
       <c r="DM154" s="3" t="n">
         <v>23.7</v>
       </c>
+      <c r="DN154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -56434,6 +56899,9 @@
       <c r="DM155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DN155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -56793,6 +57261,9 @@
       <c r="DM156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DN156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -57152,6 +57623,9 @@
       <c r="DM157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DN157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -57511,6 +57985,9 @@
       <c r="DM158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DN158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -57870,6 +58347,9 @@
       <c r="DM159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DN159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -58229,6 +58709,9 @@
       <c r="DM160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DN160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -58588,6 +59071,9 @@
       <c r="DM161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DN161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -58947,6 +59433,9 @@
       <c r="DM162" s="3" t="n">
         <v>24.49</v>
       </c>
+      <c r="DN162" s="3" t="n">
+        <v>24.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -59306,6 +59795,9 @@
       <c r="DM163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DN163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -59665,6 +60157,9 @@
       <c r="DM164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="DN164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -59925,9 +60420,12 @@
       <c r="DM165" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DN165" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:DM165"/>
+  <autoFilter ref="A1:DN165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-19 06:11 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DN$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DO$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DN165"/>
+  <dimension ref="A1:DO165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -561,6 +561,7 @@
     <col width="16" customWidth="1" min="116" max="116"/>
     <col width="16" customWidth="1" min="117" max="117"/>
     <col width="16" customWidth="1" min="118" max="118"/>
+    <col width="16" customWidth="1" min="119" max="119"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1154,6 +1155,11 @@
           <t>2026-09-18 22:09</t>
         </is>
       </c>
+      <c r="DO1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-19 01:11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1516,6 +1522,9 @@
       <c r="DN2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="DO2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1878,6 +1887,9 @@
       <c r="DN3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="DO3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2240,6 +2252,9 @@
       <c r="DN4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="DO4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2602,6 +2617,9 @@
       <c r="DN5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DO5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2964,6 +2982,9 @@
       <c r="DN6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DO6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3326,6 +3347,9 @@
       <c r="DN7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="DO7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3688,6 +3712,9 @@
       <c r="DN8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DO8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -4050,6 +4077,9 @@
       <c r="DN9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="DO9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4412,6 +4442,9 @@
       <c r="DN10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DO10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4774,6 +4807,9 @@
       <c r="DN11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DO11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -5136,6 +5172,9 @@
       <c r="DN12" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO12" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -5498,6 +5537,9 @@
       <c r="DN13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="DO13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5860,6 +5902,9 @@
       <c r="DN14" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DO14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -6222,6 +6267,9 @@
       <c r="DN15" s="3" t="n">
         <v>21.41</v>
       </c>
+      <c r="DO15" s="3" t="n">
+        <v>21.41</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -6584,6 +6632,9 @@
       <c r="DN16" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DO16" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6946,6 +6997,9 @@
       <c r="DN17" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DO17" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -7308,6 +7362,9 @@
       <c r="DN18" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DO18" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -7670,6 +7727,9 @@
       <c r="DN19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="DO19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -8032,6 +8092,9 @@
       <c r="DN20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DO20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -8394,6 +8457,9 @@
       <c r="DN21" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DO21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -8756,6 +8822,9 @@
       <c r="DN22" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DO22" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -9118,6 +9187,9 @@
       <c r="DN23" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DO23" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -9480,6 +9552,9 @@
       <c r="DN24" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DO24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -9842,6 +9917,9 @@
       <c r="DN25" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DO25" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -10204,6 +10282,9 @@
       <c r="DN26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DO26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -10566,6 +10647,9 @@
       <c r="DN27" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DO27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -10928,6 +11012,9 @@
       <c r="DN28" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DO28" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -11290,6 +11377,9 @@
       <c r="DN29" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DO29" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -11652,6 +11742,9 @@
       <c r="DN30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -12014,6 +12107,9 @@
       <c r="DN31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DO31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -12376,6 +12472,9 @@
       <c r="DN32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DO32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -12738,6 +12837,9 @@
       <c r="DN33" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -13100,6 +13202,9 @@
       <c r="DN34" s="3" t="n">
         <v>21.77</v>
       </c>
+      <c r="DO34" s="3" t="n">
+        <v>21.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -13462,6 +13567,9 @@
       <c r="DN35" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DO35" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -13824,6 +13932,9 @@
       <c r="DN36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DO36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -14186,6 +14297,9 @@
       <c r="DN37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DO37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -14548,6 +14662,9 @@
       <c r="DN38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DO38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -14910,6 +15027,9 @@
       <c r="DN39" s="3" t="n">
         <v>21.98</v>
       </c>
+      <c r="DO39" s="3" t="n">
+        <v>21.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -15272,6 +15392,9 @@
       <c r="DN40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -15634,6 +15757,9 @@
       <c r="DN41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DO41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -15996,6 +16122,9 @@
       <c r="DN42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DO42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -16358,6 +16487,9 @@
       <c r="DN43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DO43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -16720,6 +16852,9 @@
       <c r="DN44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -17082,6 +17217,9 @@
       <c r="DN45" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DO45" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -17444,6 +17582,9 @@
       <c r="DN46" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="DO46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -17806,6 +17947,9 @@
       <c r="DN47" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DO47" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -18168,6 +18312,9 @@
       <c r="DN48" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DO48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -18530,6 +18677,9 @@
       <c r="DN49" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DO49" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -18892,6 +19042,9 @@
       <c r="DN50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="DO50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -19254,6 +19407,9 @@
       <c r="DN51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DO51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -19616,6 +19772,9 @@
       <c r="DN52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DO52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -19978,6 +20137,9 @@
       <c r="DN53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="DO53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -20340,6 +20502,9 @@
       <c r="DN54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -20702,6 +20867,9 @@
       <c r="DN55" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DO55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -21064,6 +21232,9 @@
       <c r="DN56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -21426,6 +21597,9 @@
       <c r="DN57" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DO57" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -21788,6 +21962,9 @@
       <c r="DN58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="DO58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -22150,6 +22327,9 @@
       <c r="DN59" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DO59" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -22512,6 +22692,9 @@
       <c r="DN60" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DO60" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -22874,6 +23057,9 @@
       <c r="DN61" s="3" t="n">
         <v>21.95</v>
       </c>
+      <c r="DO61" s="3" t="n">
+        <v>21.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -23236,6 +23422,9 @@
       <c r="DN62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DO62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -23598,6 +23787,9 @@
       <c r="DN63" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DO63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -23960,6 +24152,9 @@
       <c r="DN64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DO64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -24322,6 +24517,9 @@
       <c r="DN65" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO65" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -24684,6 +24882,9 @@
       <c r="DN66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -25046,6 +25247,9 @@
       <c r="DN67" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO67" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -25408,6 +25612,9 @@
       <c r="DN68" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DO68" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -25770,6 +25977,9 @@
       <c r="DN69" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO69" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -26132,6 +26342,9 @@
       <c r="DN70" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO70" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -26494,6 +26707,9 @@
       <c r="DN71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -26856,6 +27072,9 @@
       <c r="DN72" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DO72" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -27218,6 +27437,9 @@
       <c r="DN73" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO73" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -27580,6 +27802,9 @@
       <c r="DN74" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO74" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -27942,6 +28167,9 @@
       <c r="DN75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -28304,6 +28532,9 @@
       <c r="DN76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -28666,6 +28897,9 @@
       <c r="DN77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="DO77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -29028,6 +29262,9 @@
       <c r="DN78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DO78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -29390,6 +29627,9 @@
       <c r="DN79" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO79" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -29752,6 +29992,9 @@
       <c r="DN80" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO80" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -30114,6 +30357,9 @@
       <c r="DN81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -30476,6 +30722,9 @@
       <c r="DN82" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DO82" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -30838,6 +31087,9 @@
       <c r="DN83" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO83" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -31200,6 +31452,9 @@
       <c r="DN84" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO84" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -31562,6 +31817,9 @@
       <c r="DN85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="DO85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -31924,6 +32182,9 @@
       <c r="DN86" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO86" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -32286,6 +32547,9 @@
       <c r="DN87" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DO87" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -32648,6 +32912,9 @@
       <c r="DN88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -33010,6 +33277,9 @@
       <c r="DN89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DO89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -33372,6 +33642,9 @@
       <c r="DN90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -33734,6 +34007,9 @@
       <c r="DN91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -34096,6 +34372,9 @@
       <c r="DN92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -34458,6 +34737,9 @@
       <c r="DN93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DO93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -34820,6 +35102,9 @@
       <c r="DN94" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DO94" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -35182,6 +35467,9 @@
       <c r="DN95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DO95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -35544,6 +35832,9 @@
       <c r="DN96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="DO96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -35906,6 +36197,9 @@
       <c r="DN97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DO97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -36268,6 +36562,9 @@
       <c r="DN98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DO98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -36630,6 +36927,9 @@
       <c r="DN99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DO99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -36992,6 +37292,9 @@
       <c r="DN100" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DO100" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -37354,6 +37657,9 @@
       <c r="DN101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -37716,6 +38022,9 @@
       <c r="DN102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="DO102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -38078,6 +38387,9 @@
       <c r="DN103" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO103" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -38440,6 +38752,9 @@
       <c r="DN104" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -38802,6 +39117,9 @@
       <c r="DN105" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO105" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -39164,6 +39482,9 @@
       <c r="DN106" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO106" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -39526,6 +39847,9 @@
       <c r="DN107" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DO107" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -39888,6 +40212,9 @@
       <c r="DN108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DO108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -40250,6 +40577,9 @@
       <c r="DN109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -40612,6 +40942,9 @@
       <c r="DN110" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DO110" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -40974,6 +41307,9 @@
       <c r="DN111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DO111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -41336,6 +41672,9 @@
       <c r="DN112" s="3" t="n">
         <v>23.8</v>
       </c>
+      <c r="DO112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -41698,6 +42037,9 @@
       <c r="DN113" s="3" t="n">
         <v>22.55</v>
       </c>
+      <c r="DO113" s="3" t="n">
+        <v>22.55</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -42060,6 +42402,9 @@
       <c r="DN114" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO114" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -42422,6 +42767,9 @@
       <c r="DN115" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO115" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -42784,6 +43132,9 @@
       <c r="DN116" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DO116" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -43146,6 +43497,9 @@
       <c r="DN117" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO117" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -43508,6 +43862,9 @@
       <c r="DN118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DO118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -43870,6 +44227,9 @@
       <c r="DN119" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO119" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -44232,6 +44592,9 @@
       <c r="DN120" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO120" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -44594,6 +44957,9 @@
       <c r="DN121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DO121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -44956,6 +45322,9 @@
       <c r="DN122" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DO122" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -45318,6 +45687,9 @@
       <c r="DN123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DO123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -45680,6 +46052,9 @@
       <c r="DN124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="DO124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -46042,6 +46417,9 @@
       <c r="DN125" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DO125" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -46404,6 +46782,9 @@
       <c r="DN126" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DO126" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -46766,6 +47147,9 @@
       <c r="DN127" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DO127" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -47128,6 +47512,9 @@
       <c r="DN128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="DO128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -47490,6 +47877,9 @@
       <c r="DN129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DO129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -47852,6 +48242,9 @@
       <c r="DN130" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DO130" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -48214,6 +48607,9 @@
       <c r="DN131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="DO131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -48576,6 +48972,9 @@
       <c r="DN132" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DO132" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -48938,6 +49337,9 @@
       <c r="DN133" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DO133" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -49300,6 +49702,9 @@
       <c r="DN134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="DO134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -49662,6 +50067,9 @@
       <c r="DN135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DO135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -50024,6 +50432,9 @@
       <c r="DN136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DO136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -50386,6 +50797,9 @@
       <c r="DN137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DO137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -50748,6 +51162,9 @@
       <c r="DN138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DO138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -51110,6 +51527,9 @@
       <c r="DN139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DO139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -51472,6 +51892,9 @@
       <c r="DN140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DO140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -51834,6 +52257,9 @@
       <c r="DN141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DO141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -52196,6 +52622,9 @@
       <c r="DN142" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DO142" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -52558,6 +52987,9 @@
       <c r="DN143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DO143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -52920,6 +53352,9 @@
       <c r="DN144" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DO144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -53282,6 +53717,9 @@
       <c r="DN145" s="3" t="n">
         <v>23.19</v>
       </c>
+      <c r="DO145" s="3" t="n">
+        <v>23.19</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -53644,6 +54082,9 @@
       <c r="DN146" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DO146" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -54006,6 +54447,9 @@
       <c r="DN147" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DO147" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -54368,6 +54812,9 @@
       <c r="DN148" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="DO148" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -54730,6 +55177,9 @@
       <c r="DN149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DO149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -55092,6 +55542,9 @@
       <c r="DN150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DO150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -55454,6 +55907,9 @@
       <c r="DN151" s="3" t="n">
         <v>23.39</v>
       </c>
+      <c r="DO151" s="3" t="n">
+        <v>23.39</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -55816,6 +56272,9 @@
       <c r="DN152" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DO152" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -56178,6 +56637,9 @@
       <c r="DN153" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DO153" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -56540,6 +57002,9 @@
       <c r="DN154" s="3" t="n">
         <v>23.7</v>
       </c>
+      <c r="DO154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -56902,6 +57367,9 @@
       <c r="DN155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DO155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -57264,6 +57732,9 @@
       <c r="DN156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DO156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -57626,6 +58097,9 @@
       <c r="DN157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DO157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -57988,6 +58462,9 @@
       <c r="DN158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DO158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -58350,6 +58827,9 @@
       <c r="DN159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DO159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -58712,6 +59192,9 @@
       <c r="DN160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DO160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -59074,6 +59557,9 @@
       <c r="DN161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DO161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -59436,6 +59922,9 @@
       <c r="DN162" s="3" t="n">
         <v>24.49</v>
       </c>
+      <c r="DO162" s="3" t="n">
+        <v>24.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -59798,6 +60287,9 @@
       <c r="DN163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DO163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -60160,6 +60652,9 @@
       <c r="DN164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="DO164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -60423,9 +60918,12 @@
       <c r="DN165" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DO165" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:DN165"/>
+  <autoFilter ref="A1:DO165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-19 09:09 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DO$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DP$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DO165"/>
+  <dimension ref="A1:DP165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -562,6 +562,7 @@
     <col width="16" customWidth="1" min="117" max="117"/>
     <col width="16" customWidth="1" min="118" max="118"/>
     <col width="16" customWidth="1" min="119" max="119"/>
+    <col width="16" customWidth="1" min="120" max="120"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1160,6 +1161,11 @@
           <t>2026-09-19 01:11</t>
         </is>
       </c>
+      <c r="DP1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-19 04:09</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1525,6 +1531,9 @@
       <c r="DO2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="DP2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1890,6 +1899,9 @@
       <c r="DO3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="DP3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2255,6 +2267,9 @@
       <c r="DO4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="DP4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2620,6 +2635,9 @@
       <c r="DO5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DP5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2985,6 +3003,9 @@
       <c r="DO6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DP6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3350,6 +3371,9 @@
       <c r="DO7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="DP7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3715,6 +3739,9 @@
       <c r="DO8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DP8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -4080,6 +4107,9 @@
       <c r="DO9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="DP9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4445,6 +4475,9 @@
       <c r="DO10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DP10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4810,6 +4843,9 @@
       <c r="DO11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DP11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -5175,6 +5211,9 @@
       <c r="DO12" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP12" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -5540,6 +5579,9 @@
       <c r="DO13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="DP13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5905,6 +5947,9 @@
       <c r="DO14" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DP14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -6270,6 +6315,9 @@
       <c r="DO15" s="3" t="n">
         <v>21.41</v>
       </c>
+      <c r="DP15" s="3" t="n">
+        <v>21.41</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -6635,6 +6683,9 @@
       <c r="DO16" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DP16" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -7000,6 +7051,9 @@
       <c r="DO17" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DP17" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -7365,6 +7419,9 @@
       <c r="DO18" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DP18" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -7730,6 +7787,9 @@
       <c r="DO19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="DP19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -8095,6 +8155,9 @@
       <c r="DO20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DP20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -8460,6 +8523,9 @@
       <c r="DO21" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DP21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -8825,6 +8891,9 @@
       <c r="DO22" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DP22" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -9190,6 +9259,9 @@
       <c r="DO23" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DP23" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -9555,6 +9627,9 @@
       <c r="DO24" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DP24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -9920,6 +9995,9 @@
       <c r="DO25" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DP25" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -10285,6 +10363,9 @@
       <c r="DO26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DP26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -10650,6 +10731,9 @@
       <c r="DO27" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DP27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -11015,6 +11099,9 @@
       <c r="DO28" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DP28" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -11380,6 +11467,9 @@
       <c r="DO29" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DP29" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -11745,6 +11835,9 @@
       <c r="DO30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -12110,6 +12203,9 @@
       <c r="DO31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DP31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -12475,6 +12571,9 @@
       <c r="DO32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DP32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -12840,6 +12939,9 @@
       <c r="DO33" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -13205,6 +13307,9 @@
       <c r="DO34" s="3" t="n">
         <v>21.77</v>
       </c>
+      <c r="DP34" s="3" t="n">
+        <v>21.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -13570,6 +13675,9 @@
       <c r="DO35" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DP35" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -13935,6 +14043,9 @@
       <c r="DO36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DP36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -14300,6 +14411,9 @@
       <c r="DO37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DP37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -14665,6 +14779,9 @@
       <c r="DO38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DP38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -15030,6 +15147,9 @@
       <c r="DO39" s="3" t="n">
         <v>21.98</v>
       </c>
+      <c r="DP39" s="3" t="n">
+        <v>21.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -15395,6 +15515,9 @@
       <c r="DO40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -15760,6 +15883,9 @@
       <c r="DO41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DP41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -16125,6 +16251,9 @@
       <c r="DO42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DP42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -16490,6 +16619,9 @@
       <c r="DO43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DP43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -16855,6 +16987,9 @@
       <c r="DO44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -17220,6 +17355,9 @@
       <c r="DO45" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DP45" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -17585,6 +17723,9 @@
       <c r="DO46" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="DP46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -17950,6 +18091,9 @@
       <c r="DO47" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DP47" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -18315,6 +18459,9 @@
       <c r="DO48" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DP48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -18680,6 +18827,9 @@
       <c r="DO49" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DP49" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -19045,6 +19195,9 @@
       <c r="DO50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="DP50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -19410,6 +19563,9 @@
       <c r="DO51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DP51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -19775,6 +19931,9 @@
       <c r="DO52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DP52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -20140,6 +20299,9 @@
       <c r="DO53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="DP53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -20505,6 +20667,9 @@
       <c r="DO54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -20870,6 +21035,9 @@
       <c r="DO55" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DP55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -21235,6 +21403,9 @@
       <c r="DO56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -21600,6 +21771,9 @@
       <c r="DO57" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DP57" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -21965,6 +22139,9 @@
       <c r="DO58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="DP58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -22330,6 +22507,9 @@
       <c r="DO59" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DP59" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -22695,6 +22875,9 @@
       <c r="DO60" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DP60" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -23060,6 +23243,9 @@
       <c r="DO61" s="3" t="n">
         <v>21.95</v>
       </c>
+      <c r="DP61" s="3" t="n">
+        <v>21.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -23425,6 +23611,9 @@
       <c r="DO62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DP62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -23790,6 +23979,9 @@
       <c r="DO63" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DP63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -24155,6 +24347,9 @@
       <c r="DO64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DP64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -24520,6 +24715,9 @@
       <c r="DO65" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP65" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -24885,6 +25083,9 @@
       <c r="DO66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -25250,6 +25451,9 @@
       <c r="DO67" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP67" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -25615,6 +25819,9 @@
       <c r="DO68" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DP68" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -25980,6 +26187,9 @@
       <c r="DO69" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP69" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -26345,6 +26555,9 @@
       <c r="DO70" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP70" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -26710,6 +26923,9 @@
       <c r="DO71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -27075,6 +27291,9 @@
       <c r="DO72" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DP72" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -27440,6 +27659,9 @@
       <c r="DO73" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP73" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -27805,6 +28027,9 @@
       <c r="DO74" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP74" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -28170,6 +28395,9 @@
       <c r="DO75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -28535,6 +28763,9 @@
       <c r="DO76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -28900,6 +29131,9 @@
       <c r="DO77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="DP77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -29265,6 +29499,9 @@
       <c r="DO78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DP78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -29630,6 +29867,9 @@
       <c r="DO79" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP79" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -29995,6 +30235,9 @@
       <c r="DO80" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP80" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -30360,6 +30603,9 @@
       <c r="DO81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -30725,6 +30971,9 @@
       <c r="DO82" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DP82" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -31090,6 +31339,9 @@
       <c r="DO83" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP83" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -31455,6 +31707,9 @@
       <c r="DO84" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP84" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -31820,6 +32075,9 @@
       <c r="DO85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="DP85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -32185,6 +32443,9 @@
       <c r="DO86" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP86" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -32550,6 +32811,9 @@
       <c r="DO87" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DP87" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -32915,6 +33179,9 @@
       <c r="DO88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -33280,6 +33547,9 @@
       <c r="DO89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DP89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -33645,6 +33915,9 @@
       <c r="DO90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -34010,6 +34283,9 @@
       <c r="DO91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -34375,6 +34651,9 @@
       <c r="DO92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -34740,6 +35019,9 @@
       <c r="DO93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DP93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -35105,6 +35387,9 @@
       <c r="DO94" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DP94" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -35470,6 +35755,9 @@
       <c r="DO95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DP95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -35835,6 +36123,9 @@
       <c r="DO96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="DP96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -36200,6 +36491,9 @@
       <c r="DO97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DP97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -36565,6 +36859,9 @@
       <c r="DO98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DP98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -36930,6 +37227,9 @@
       <c r="DO99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DP99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -37295,6 +37595,9 @@
       <c r="DO100" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DP100" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -37660,6 +37963,9 @@
       <c r="DO101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -38025,6 +38331,9 @@
       <c r="DO102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="DP102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -38390,6 +38699,9 @@
       <c r="DO103" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP103" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -38755,6 +39067,9 @@
       <c r="DO104" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -39120,6 +39435,9 @@
       <c r="DO105" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP105" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -39485,6 +39803,9 @@
       <c r="DO106" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP106" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -39850,6 +40171,9 @@
       <c r="DO107" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DP107" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -40215,6 +40539,9 @@
       <c r="DO108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DP108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -40580,6 +40907,9 @@
       <c r="DO109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -40945,6 +41275,9 @@
       <c r="DO110" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DP110" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -41310,6 +41643,9 @@
       <c r="DO111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DP111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -41675,6 +42011,9 @@
       <c r="DO112" s="3" t="n">
         <v>23.8</v>
       </c>
+      <c r="DP112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -42040,6 +42379,9 @@
       <c r="DO113" s="3" t="n">
         <v>22.55</v>
       </c>
+      <c r="DP113" s="3" t="n">
+        <v>22.55</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -42405,6 +42747,9 @@
       <c r="DO114" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP114" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -42770,6 +43115,9 @@
       <c r="DO115" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP115" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -43135,6 +43483,9 @@
       <c r="DO116" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DP116" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -43500,6 +43851,9 @@
       <c r="DO117" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP117" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -43865,6 +44219,9 @@
       <c r="DO118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DP118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -44230,6 +44587,9 @@
       <c r="DO119" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP119" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -44595,6 +44955,9 @@
       <c r="DO120" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP120" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -44960,6 +45323,9 @@
       <c r="DO121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DP121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -45325,6 +45691,9 @@
       <c r="DO122" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DP122" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -45690,6 +46059,9 @@
       <c r="DO123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DP123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -46055,6 +46427,9 @@
       <c r="DO124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="DP124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -46420,6 +46795,9 @@
       <c r="DO125" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DP125" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -46785,6 +47163,9 @@
       <c r="DO126" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DP126" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -47150,6 +47531,9 @@
       <c r="DO127" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DP127" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -47515,6 +47899,9 @@
       <c r="DO128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="DP128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -47880,6 +48267,9 @@
       <c r="DO129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DP129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -48245,6 +48635,9 @@
       <c r="DO130" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DP130" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -48610,6 +49003,9 @@
       <c r="DO131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="DP131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -48975,6 +49371,9 @@
       <c r="DO132" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DP132" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -49340,6 +49739,9 @@
       <c r="DO133" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DP133" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -49705,6 +50107,9 @@
       <c r="DO134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="DP134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -50070,6 +50475,9 @@
       <c r="DO135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DP135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -50435,6 +50843,9 @@
       <c r="DO136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DP136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -50800,6 +51211,9 @@
       <c r="DO137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DP137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -51165,6 +51579,9 @@
       <c r="DO138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DP138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -51530,6 +51947,9 @@
       <c r="DO139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DP139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -51895,6 +52315,9 @@
       <c r="DO140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DP140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -52260,6 +52683,9 @@
       <c r="DO141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DP141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -52625,6 +53051,9 @@
       <c r="DO142" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DP142" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -52990,6 +53419,9 @@
       <c r="DO143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DP143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -53355,6 +53787,9 @@
       <c r="DO144" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DP144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -53720,6 +54155,9 @@
       <c r="DO145" s="3" t="n">
         <v>23.19</v>
       </c>
+      <c r="DP145" s="3" t="n">
+        <v>23.19</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -54085,6 +54523,9 @@
       <c r="DO146" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DP146" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -54450,6 +54891,9 @@
       <c r="DO147" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DP147" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -54815,6 +55259,9 @@
       <c r="DO148" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="DP148" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -55180,6 +55627,9 @@
       <c r="DO149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DP149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -55545,6 +55995,9 @@
       <c r="DO150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DP150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -55910,6 +56363,9 @@
       <c r="DO151" s="3" t="n">
         <v>23.39</v>
       </c>
+      <c r="DP151" s="3" t="n">
+        <v>23.39</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -56275,6 +56731,9 @@
       <c r="DO152" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DP152" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -56640,6 +57099,9 @@
       <c r="DO153" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DP153" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -57005,6 +57467,9 @@
       <c r="DO154" s="3" t="n">
         <v>23.7</v>
       </c>
+      <c r="DP154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -57370,6 +57835,9 @@
       <c r="DO155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DP155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -57735,6 +58203,9 @@
       <c r="DO156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DP156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -58100,6 +58571,9 @@
       <c r="DO157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DP157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -58465,6 +58939,9 @@
       <c r="DO158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DP158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -58830,6 +59307,9 @@
       <c r="DO159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DP159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -59195,6 +59675,9 @@
       <c r="DO160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DP160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -59560,6 +60043,9 @@
       <c r="DO161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DP161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -59925,6 +60411,9 @@
       <c r="DO162" s="3" t="n">
         <v>24.49</v>
       </c>
+      <c r="DP162" s="3" t="n">
+        <v>24.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -60290,6 +60779,9 @@
       <c r="DO163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DP163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -60655,6 +61147,9 @@
       <c r="DO164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="DP164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -60921,9 +61416,12 @@
       <c r="DO165" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DP165" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:DO165"/>
+  <autoFilter ref="A1:DP165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-19 12:11 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DP$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DQ$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DP165"/>
+  <dimension ref="A1:DQ165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,7 @@
     <col width="16" customWidth="1" min="118" max="118"/>
     <col width="16" customWidth="1" min="119" max="119"/>
     <col width="16" customWidth="1" min="120" max="120"/>
+    <col width="16" customWidth="1" min="121" max="121"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1166,6 +1167,11 @@
           <t>2026-09-19 04:09</t>
         </is>
       </c>
+      <c r="DQ1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-19 07:11</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1534,6 +1540,9 @@
       <c r="DP2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="DQ2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1902,6 +1911,9 @@
       <c r="DP3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="DQ3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2270,6 +2282,9 @@
       <c r="DP4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="DQ4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2638,6 +2653,9 @@
       <c r="DP5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DQ5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -3006,6 +3024,9 @@
       <c r="DP6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DQ6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3374,6 +3395,9 @@
       <c r="DP7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="DQ7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3742,6 +3766,9 @@
       <c r="DP8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DQ8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -4110,6 +4137,9 @@
       <c r="DP9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="DQ9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4478,6 +4508,9 @@
       <c r="DP10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DQ10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4846,6 +4879,9 @@
       <c r="DP11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DQ11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -5214,6 +5250,9 @@
       <c r="DP12" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ12" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -5582,6 +5621,9 @@
       <c r="DP13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="DQ13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5950,6 +5992,9 @@
       <c r="DP14" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DQ14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -6318,6 +6363,9 @@
       <c r="DP15" s="3" t="n">
         <v>21.41</v>
       </c>
+      <c r="DQ15" s="3" t="n">
+        <v>21.41</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -6686,6 +6734,9 @@
       <c r="DP16" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DQ16" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -7054,6 +7105,9 @@
       <c r="DP17" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DQ17" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -7422,6 +7476,9 @@
       <c r="DP18" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DQ18" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -7790,6 +7847,9 @@
       <c r="DP19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="DQ19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -8158,6 +8218,9 @@
       <c r="DP20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DQ20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -8526,6 +8589,9 @@
       <c r="DP21" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DQ21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -8894,6 +8960,9 @@
       <c r="DP22" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DQ22" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -9262,6 +9331,9 @@
       <c r="DP23" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DQ23" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -9630,6 +9702,9 @@
       <c r="DP24" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DQ24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -9998,6 +10073,9 @@
       <c r="DP25" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DQ25" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -10366,6 +10444,9 @@
       <c r="DP26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DQ26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -10734,6 +10815,9 @@
       <c r="DP27" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DQ27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -11102,6 +11186,9 @@
       <c r="DP28" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DQ28" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -11470,6 +11557,9 @@
       <c r="DP29" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DQ29" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -11838,6 +11928,9 @@
       <c r="DP30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -12206,6 +12299,9 @@
       <c r="DP31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DQ31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -12574,6 +12670,9 @@
       <c r="DP32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DQ32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -12942,6 +13041,9 @@
       <c r="DP33" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -13310,6 +13412,9 @@
       <c r="DP34" s="3" t="n">
         <v>21.77</v>
       </c>
+      <c r="DQ34" s="3" t="n">
+        <v>21.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -13678,6 +13783,9 @@
       <c r="DP35" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DQ35" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -14046,6 +14154,9 @@
       <c r="DP36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DQ36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -14414,6 +14525,9 @@
       <c r="DP37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DQ37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -14782,6 +14896,9 @@
       <c r="DP38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DQ38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -15150,6 +15267,9 @@
       <c r="DP39" s="3" t="n">
         <v>21.98</v>
       </c>
+      <c r="DQ39" s="3" t="n">
+        <v>21.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -15518,6 +15638,9 @@
       <c r="DP40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -15886,6 +16009,9 @@
       <c r="DP41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DQ41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -16254,6 +16380,9 @@
       <c r="DP42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DQ42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -16622,6 +16751,9 @@
       <c r="DP43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DQ43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -16990,6 +17122,9 @@
       <c r="DP44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -17358,6 +17493,9 @@
       <c r="DP45" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DQ45" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -17726,6 +17864,9 @@
       <c r="DP46" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="DQ46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -18094,6 +18235,9 @@
       <c r="DP47" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DQ47" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -18462,6 +18606,9 @@
       <c r="DP48" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DQ48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -18830,6 +18977,9 @@
       <c r="DP49" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DQ49" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -19198,6 +19348,9 @@
       <c r="DP50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="DQ50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -19566,6 +19719,9 @@
       <c r="DP51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DQ51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -19934,6 +20090,9 @@
       <c r="DP52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DQ52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -20302,6 +20461,9 @@
       <c r="DP53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="DQ53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -20670,6 +20832,9 @@
       <c r="DP54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -21038,6 +21203,9 @@
       <c r="DP55" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DQ55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -21406,6 +21574,9 @@
       <c r="DP56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -21774,6 +21945,9 @@
       <c r="DP57" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DQ57" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -22142,6 +22316,9 @@
       <c r="DP58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="DQ58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -22510,6 +22687,9 @@
       <c r="DP59" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DQ59" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -22878,6 +23058,9 @@
       <c r="DP60" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DQ60" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -23246,6 +23429,9 @@
       <c r="DP61" s="3" t="n">
         <v>21.95</v>
       </c>
+      <c r="DQ61" s="3" t="n">
+        <v>21.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -23614,6 +23800,9 @@
       <c r="DP62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DQ62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -23982,6 +24171,9 @@
       <c r="DP63" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DQ63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -24350,6 +24542,9 @@
       <c r="DP64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DQ64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -24718,6 +24913,9 @@
       <c r="DP65" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ65" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -25086,6 +25284,9 @@
       <c r="DP66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -25454,6 +25655,9 @@
       <c r="DP67" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ67" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -25822,6 +26026,9 @@
       <c r="DP68" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DQ68" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -26190,6 +26397,9 @@
       <c r="DP69" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ69" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -26558,6 +26768,9 @@
       <c r="DP70" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ70" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -26926,6 +27139,9 @@
       <c r="DP71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -27294,6 +27510,9 @@
       <c r="DP72" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DQ72" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -27662,6 +27881,9 @@
       <c r="DP73" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ73" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -28030,6 +28252,9 @@
       <c r="DP74" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ74" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -28398,6 +28623,9 @@
       <c r="DP75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -28766,6 +28994,9 @@
       <c r="DP76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -29134,6 +29365,9 @@
       <c r="DP77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="DQ77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -29502,6 +29736,9 @@
       <c r="DP78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DQ78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -29870,6 +30107,9 @@
       <c r="DP79" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ79" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -30238,6 +30478,9 @@
       <c r="DP80" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ80" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -30606,6 +30849,9 @@
       <c r="DP81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -30974,6 +31220,9 @@
       <c r="DP82" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DQ82" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -31342,6 +31591,9 @@
       <c r="DP83" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ83" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -31710,6 +31962,9 @@
       <c r="DP84" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ84" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -32078,6 +32333,9 @@
       <c r="DP85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="DQ85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -32446,6 +32704,9 @@
       <c r="DP86" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ86" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -32814,6 +33075,9 @@
       <c r="DP87" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DQ87" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -33182,6 +33446,9 @@
       <c r="DP88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -33550,6 +33817,9 @@
       <c r="DP89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DQ89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -33918,6 +34188,9 @@
       <c r="DP90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -34286,6 +34559,9 @@
       <c r="DP91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -34654,6 +34930,9 @@
       <c r="DP92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -35022,6 +35301,9 @@
       <c r="DP93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DQ93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -35390,6 +35672,9 @@
       <c r="DP94" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DQ94" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -35758,6 +36043,9 @@
       <c r="DP95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DQ95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -36126,6 +36414,9 @@
       <c r="DP96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="DQ96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -36494,6 +36785,9 @@
       <c r="DP97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DQ97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -36862,6 +37156,9 @@
       <c r="DP98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DQ98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -37230,6 +37527,9 @@
       <c r="DP99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DQ99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -37598,6 +37898,9 @@
       <c r="DP100" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DQ100" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -37966,6 +38269,9 @@
       <c r="DP101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -38334,6 +38640,9 @@
       <c r="DP102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="DQ102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -38702,6 +39011,9 @@
       <c r="DP103" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ103" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -39070,6 +39382,9 @@
       <c r="DP104" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -39438,6 +39753,9 @@
       <c r="DP105" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ105" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -39806,6 +40124,9 @@
       <c r="DP106" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ106" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -40174,6 +40495,9 @@
       <c r="DP107" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DQ107" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -40542,6 +40866,9 @@
       <c r="DP108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DQ108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -40910,6 +41237,9 @@
       <c r="DP109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -41278,6 +41608,9 @@
       <c r="DP110" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DQ110" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -41646,6 +41979,9 @@
       <c r="DP111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DQ111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -42014,6 +42350,9 @@
       <c r="DP112" s="3" t="n">
         <v>23.8</v>
       </c>
+      <c r="DQ112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -42382,6 +42721,9 @@
       <c r="DP113" s="3" t="n">
         <v>22.55</v>
       </c>
+      <c r="DQ113" s="3" t="n">
+        <v>22.55</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -42750,6 +43092,9 @@
       <c r="DP114" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ114" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -43118,6 +43463,9 @@
       <c r="DP115" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ115" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -43486,6 +43834,9 @@
       <c r="DP116" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DQ116" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -43854,6 +44205,9 @@
       <c r="DP117" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ117" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -44222,6 +44576,9 @@
       <c r="DP118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DQ118" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -44590,6 +44947,9 @@
       <c r="DP119" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ119" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -44958,6 +45318,9 @@
       <c r="DP120" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ120" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -45326,6 +45689,9 @@
       <c r="DP121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DQ121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -45694,6 +46060,9 @@
       <c r="DP122" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DQ122" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -46062,6 +46431,9 @@
       <c r="DP123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DQ123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -46430,6 +46802,9 @@
       <c r="DP124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="DQ124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -46798,6 +47173,9 @@
       <c r="DP125" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DQ125" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -47166,6 +47544,9 @@
       <c r="DP126" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DQ126" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -47534,6 +47915,9 @@
       <c r="DP127" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DQ127" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -47902,6 +48286,9 @@
       <c r="DP128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="DQ128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -48270,6 +48657,9 @@
       <c r="DP129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DQ129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -48638,6 +49028,9 @@
       <c r="DP130" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DQ130" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -49006,6 +49399,9 @@
       <c r="DP131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="DQ131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -49374,6 +49770,9 @@
       <c r="DP132" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DQ132" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -49742,6 +50141,9 @@
       <c r="DP133" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DQ133" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -50110,6 +50512,9 @@
       <c r="DP134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="DQ134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -50478,6 +50883,9 @@
       <c r="DP135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DQ135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -50846,6 +51254,9 @@
       <c r="DP136" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DQ136" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -51214,6 +51625,9 @@
       <c r="DP137" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DQ137" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -51582,6 +51996,9 @@
       <c r="DP138" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DQ138" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -51950,6 +52367,9 @@
       <c r="DP139" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DQ139" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -52318,6 +52738,9 @@
       <c r="DP140" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DQ140" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -52686,6 +53109,9 @@
       <c r="DP141" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DQ141" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -53054,6 +53480,9 @@
       <c r="DP142" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DQ142" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -53422,6 +53851,9 @@
       <c r="DP143" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DQ143" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -53790,6 +54222,9 @@
       <c r="DP144" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DQ144" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -54158,6 +54593,9 @@
       <c r="DP145" s="3" t="n">
         <v>23.19</v>
       </c>
+      <c r="DQ145" s="3" t="n">
+        <v>23.19</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -54526,6 +54964,9 @@
       <c r="DP146" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DQ146" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -54894,6 +55335,9 @@
       <c r="DP147" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DQ147" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -55262,6 +55706,9 @@
       <c r="DP148" s="3" t="n">
         <v>23.49</v>
       </c>
+      <c r="DQ148" s="3" t="n">
+        <v>23.49</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -55630,6 +56077,9 @@
       <c r="DP149" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DQ149" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -55998,6 +56448,9 @@
       <c r="DP150" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DQ150" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -56366,6 +56819,9 @@
       <c r="DP151" s="3" t="n">
         <v>23.39</v>
       </c>
+      <c r="DQ151" s="3" t="n">
+        <v>23.39</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -56734,6 +57190,9 @@
       <c r="DP152" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DQ152" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -57102,6 +57561,9 @@
       <c r="DP153" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DQ153" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -57470,6 +57932,9 @@
       <c r="DP154" s="3" t="n">
         <v>23.7</v>
       </c>
+      <c r="DQ154" s="3" t="n">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -57838,6 +58303,9 @@
       <c r="DP155" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DQ155" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -58206,6 +58674,9 @@
       <c r="DP156" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DQ156" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -58574,6 +59045,9 @@
       <c r="DP157" s="3" t="n">
         <v>23.6</v>
       </c>
+      <c r="DQ157" s="3" t="n">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -58942,6 +59416,9 @@
       <c r="DP158" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DQ158" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -59310,6 +59787,9 @@
       <c r="DP159" s="3" t="n">
         <v>23.99</v>
       </c>
+      <c r="DQ159" s="3" t="n">
+        <v>23.99</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -59678,6 +60158,9 @@
       <c r="DP160" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DQ160" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -60046,6 +60529,9 @@
       <c r="DP161" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DQ161" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -60414,6 +60900,9 @@
       <c r="DP162" s="3" t="n">
         <v>24.49</v>
       </c>
+      <c r="DQ162" s="3" t="n">
+        <v>24.49</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -60782,6 +61271,9 @@
       <c r="DP163" s="3" t="n">
         <v>23</v>
       </c>
+      <c r="DQ163" s="3" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -61150,6 +61642,9 @@
       <c r="DP164" s="3" t="n">
         <v>24.25</v>
       </c>
+      <c r="DQ164" s="3" t="n">
+        <v>24.25</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -61419,9 +61914,12 @@
       <c r="DP165" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DQ165" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:DP165"/>
+  <autoFilter ref="A1:DQ165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualiza precios Facilito 2026-09-19 15:08 UTC
</commit_message>
<xml_diff>
--- a/historial/Chiclayo_GasoholRegular_historial.xlsx
+++ b/historial/Chiclayo_GasoholRegular_historial.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DQ$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2026-09'!$A$1:$DR$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DQ165"/>
+  <dimension ref="A1:DR165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -564,6 +564,7 @@
     <col width="16" customWidth="1" min="119" max="119"/>
     <col width="16" customWidth="1" min="120" max="120"/>
     <col width="16" customWidth="1" min="121" max="121"/>
+    <col width="16" customWidth="1" min="122" max="122"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1172,6 +1173,11 @@
           <t>2026-09-19 07:11</t>
         </is>
       </c>
+      <c r="DR1" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-19 10:08</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1543,6 +1549,9 @@
       <c r="DQ2" s="3" t="n">
         <v>13.45</v>
       </c>
+      <c r="DR2" s="3" t="n">
+        <v>13.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1914,6 +1923,9 @@
       <c r="DQ3" s="3" t="n">
         <v>16</v>
       </c>
+      <c r="DR3" s="3" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2285,6 +2297,9 @@
       <c r="DQ4" s="3" t="n">
         <v>17.95</v>
       </c>
+      <c r="DR4" s="3" t="n">
+        <v>17.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2656,6 +2671,9 @@
       <c r="DQ5" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DR5" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -3027,6 +3045,9 @@
       <c r="DQ6" s="3" t="n">
         <v>18</v>
       </c>
+      <c r="DR6" s="3" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3398,6 +3419,9 @@
       <c r="DQ7" s="3" t="n">
         <v>19.49</v>
       </c>
+      <c r="DR7" s="3" t="n">
+        <v>19.49</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3769,6 +3793,9 @@
       <c r="DQ8" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DR8" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -4140,6 +4167,9 @@
       <c r="DQ9" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="DR9" s="3" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -4511,6 +4541,9 @@
       <c r="DQ10" s="3" t="n">
         <v>21.5</v>
       </c>
+      <c r="DR10" s="3" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -4882,6 +4915,9 @@
       <c r="DQ11" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DR11" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -5253,6 +5289,9 @@
       <c r="DQ12" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR12" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -5624,6 +5663,9 @@
       <c r="DQ13" s="3" t="n">
         <v>20.2</v>
       </c>
+      <c r="DR13" s="3" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5995,6 +6037,9 @@
       <c r="DQ14" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DR14" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -6366,6 +6411,9 @@
       <c r="DQ15" s="3" t="n">
         <v>21.41</v>
       </c>
+      <c r="DR15" s="3" t="n">
+        <v>21.41</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -6737,6 +6785,9 @@
       <c r="DQ16" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DR16" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -7108,6 +7159,9 @@
       <c r="DQ17" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DR17" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -7479,6 +7533,9 @@
       <c r="DQ18" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DR18" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -7850,6 +7907,9 @@
       <c r="DQ19" s="3" t="n">
         <v>21.52</v>
       </c>
+      <c r="DR19" s="3" t="n">
+        <v>21.52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -8221,6 +8281,9 @@
       <c r="DQ20" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DR20" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -8592,6 +8655,9 @@
       <c r="DQ21" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DR21" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -8963,6 +9029,9 @@
       <c r="DQ22" s="3" t="n">
         <v>22.49</v>
       </c>
+      <c r="DR22" s="3" t="n">
+        <v>22.49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -9334,6 +9403,9 @@
       <c r="DQ23" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DR23" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -9705,6 +9777,9 @@
       <c r="DQ24" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DR24" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -10076,6 +10151,9 @@
       <c r="DQ25" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DR25" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -10447,6 +10525,9 @@
       <c r="DQ26" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DR26" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -10818,6 +10899,9 @@
       <c r="DQ27" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DR27" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -11189,6 +11273,9 @@
       <c r="DQ28" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DR28" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -11560,6 +11647,9 @@
       <c r="DQ29" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DR29" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -11931,6 +12021,9 @@
       <c r="DQ30" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR30" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -12302,6 +12395,9 @@
       <c r="DQ31" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DR31" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -12673,6 +12769,9 @@
       <c r="DQ32" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DR32" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -13044,6 +13143,9 @@
       <c r="DQ33" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR33" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -13415,6 +13517,9 @@
       <c r="DQ34" s="3" t="n">
         <v>21.77</v>
       </c>
+      <c r="DR34" s="3" t="n">
+        <v>21.77</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -13786,6 +13891,9 @@
       <c r="DQ35" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DR35" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -14157,6 +14265,9 @@
       <c r="DQ36" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DR36" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -14528,6 +14639,9 @@
       <c r="DQ37" s="3" t="n">
         <v>20.99</v>
       </c>
+      <c r="DR37" s="3" t="n">
+        <v>20.99</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -14899,6 +15013,9 @@
       <c r="DQ38" s="3" t="n">
         <v>21.65</v>
       </c>
+      <c r="DR38" s="3" t="n">
+        <v>21.65</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -15270,6 +15387,9 @@
       <c r="DQ39" s="3" t="n">
         <v>21.98</v>
       </c>
+      <c r="DR39" s="3" t="n">
+        <v>21.98</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -15641,6 +15761,9 @@
       <c r="DQ40" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR40" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -16012,6 +16135,9 @@
       <c r="DQ41" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DR41" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -16383,6 +16509,9 @@
       <c r="DQ42" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DR42" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -16754,6 +16883,9 @@
       <c r="DQ43" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DR43" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -17125,6 +17257,9 @@
       <c r="DQ44" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR44" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -17496,6 +17631,9 @@
       <c r="DQ45" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DR45" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -17867,6 +18005,9 @@
       <c r="DQ46" s="3" t="n">
         <v>21.85</v>
       </c>
+      <c r="DR46" s="3" t="n">
+        <v>21.85</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -18238,6 +18379,9 @@
       <c r="DQ47" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DR47" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -18609,6 +18753,9 @@
       <c r="DQ48" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DR48" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -18980,6 +19127,9 @@
       <c r="DQ49" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DR49" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -19351,6 +19501,9 @@
       <c r="DQ50" s="3" t="n">
         <v>22.7</v>
       </c>
+      <c r="DR50" s="3" t="n">
+        <v>22.7</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -19722,6 +19875,9 @@
       <c r="DQ51" s="3" t="n">
         <v>21.79</v>
       </c>
+      <c r="DR51" s="3" t="n">
+        <v>21.79</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -20093,6 +20249,9 @@
       <c r="DQ52" s="3" t="n">
         <v>22.35</v>
       </c>
+      <c r="DR52" s="3" t="n">
+        <v>22.35</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -20464,6 +20623,9 @@
       <c r="DQ53" s="3" t="n">
         <v>22.39</v>
       </c>
+      <c r="DR53" s="3" t="n">
+        <v>22.39</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -20835,6 +20997,9 @@
       <c r="DQ54" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR54" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -21206,6 +21371,9 @@
       <c r="DQ55" s="3" t="n">
         <v>22.3</v>
       </c>
+      <c r="DR55" s="3" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -21577,6 +21745,9 @@
       <c r="DQ56" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR56" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -21948,6 +22119,9 @@
       <c r="DQ57" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DR57" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -22319,6 +22493,9 @@
       <c r="DQ58" s="3" t="n">
         <v>22.75</v>
       </c>
+      <c r="DR58" s="3" t="n">
+        <v>22.75</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -22690,6 +22867,9 @@
       <c r="DQ59" s="3" t="n">
         <v>22.99</v>
       </c>
+      <c r="DR59" s="3" t="n">
+        <v>22.99</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -23061,6 +23241,9 @@
       <c r="DQ60" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DR60" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -23432,6 +23615,9 @@
       <c r="DQ61" s="3" t="n">
         <v>21.95</v>
       </c>
+      <c r="DR61" s="3" t="n">
+        <v>21.95</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -23803,6 +23989,9 @@
       <c r="DQ62" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DR62" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -24174,6 +24363,9 @@
       <c r="DQ63" s="3" t="n">
         <v>22.95</v>
       </c>
+      <c r="DR63" s="3" t="n">
+        <v>22.95</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -24545,6 +24737,9 @@
       <c r="DQ64" s="3" t="n">
         <v>22.79</v>
       </c>
+      <c r="DR64" s="3" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -24916,6 +25111,9 @@
       <c r="DQ65" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR65" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -25287,6 +25485,9 @@
       <c r="DQ66" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR66" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -25658,6 +25859,9 @@
       <c r="DQ67" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR67" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -26029,6 +26233,9 @@
       <c r="DQ68" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DR68" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -26400,6 +26607,9 @@
       <c r="DQ69" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR69" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -26771,6 +26981,9 @@
       <c r="DQ70" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR70" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -27142,6 +27355,9 @@
       <c r="DQ71" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR71" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -27513,6 +27729,9 @@
       <c r="DQ72" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DR72" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -27884,6 +28103,9 @@
       <c r="DQ73" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR73" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -28255,6 +28477,9 @@
       <c r="DQ74" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR74" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -28626,6 +28851,9 @@
       <c r="DQ75" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR75" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -28997,6 +29225,9 @@
       <c r="DQ76" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR76" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -29368,6 +29599,9 @@
       <c r="DQ77" s="3" t="n">
         <v>21.94</v>
       </c>
+      <c r="DR77" s="3" t="n">
+        <v>21.94</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -29739,6 +29973,9 @@
       <c r="DQ78" s="3" t="n">
         <v>22.59</v>
       </c>
+      <c r="DR78" s="3" t="n">
+        <v>22.59</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -30110,6 +30347,9 @@
       <c r="DQ79" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR79" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -30481,6 +30721,9 @@
       <c r="DQ80" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR80" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -30852,6 +31095,9 @@
       <c r="DQ81" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR81" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -31223,6 +31469,9 @@
       <c r="DQ82" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DR82" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -31594,6 +31843,9 @@
       <c r="DQ83" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR83" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -31965,6 +32217,9 @@
       <c r="DQ84" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR84" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -32336,6 +32591,9 @@
       <c r="DQ85" s="3" t="n">
         <v>22.69</v>
       </c>
+      <c r="DR85" s="3" t="n">
+        <v>22.69</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -32707,6 +32965,9 @@
       <c r="DQ86" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR86" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -33078,6 +33339,9 @@
       <c r="DQ87" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DR87" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -33449,6 +33713,9 @@
       <c r="DQ88" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR88" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -33820,6 +34087,9 @@
       <c r="DQ89" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DR89" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -34191,6 +34461,9 @@
       <c r="DQ90" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR90" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -34562,6 +34835,9 @@
       <c r="DQ91" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR91" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -34933,6 +35209,9 @@
       <c r="DQ92" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR92" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -35304,6 +35583,9 @@
       <c r="DQ93" s="3" t="n">
         <v>21.89</v>
       </c>
+      <c r="DR93" s="3" t="n">
+        <v>21.89</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -35675,6 +35957,9 @@
       <c r="DQ94" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DR94" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -36046,6 +36331,9 @@
       <c r="DQ95" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DR95" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -36417,6 +36705,9 @@
       <c r="DQ96" s="3" t="n">
         <v>21.4</v>
       </c>
+      <c r="DR96" s="3" t="n">
+        <v>21.4</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -36788,6 +37079,9 @@
       <c r="DQ97" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DR97" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -37159,6 +37453,9 @@
       <c r="DQ98" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DR98" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -37530,6 +37827,9 @@
       <c r="DQ99" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DR99" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -37901,6 +38201,9 @@
       <c r="DQ100" s="3" t="n">
         <v>21.49</v>
       </c>
+      <c r="DR100" s="3" t="n">
+        <v>21.49</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -38272,6 +38575,9 @@
       <c r="DQ101" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR101" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -38643,6 +38949,9 @@
       <c r="DQ102" s="3" t="n">
         <v>23.79</v>
       </c>
+      <c r="DR102" s="3" t="n">
+        <v>23.79</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -39014,6 +39323,9 @@
       <c r="DQ103" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR103" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -39385,6 +39697,9 @@
       <c r="DQ104" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR104" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -39756,6 +40071,9 @@
       <c r="DQ105" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR105" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -40127,6 +40445,9 @@
       <c r="DQ106" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR106" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -40498,6 +40819,9 @@
       <c r="DQ107" s="3" t="n">
         <v>21.59</v>
       </c>
+      <c r="DR107" s="3" t="n">
+        <v>21.59</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -40869,6 +41193,9 @@
       <c r="DQ108" s="3" t="n">
         <v>21.66</v>
       </c>
+      <c r="DR108" s="3" t="n">
+        <v>21.66</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -41240,6 +41567,9 @@
       <c r="DQ109" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR109" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -41611,6 +41941,9 @@
       <c r="DQ110" s="3" t="n">
         <v>21.39</v>
       </c>
+      <c r="DR110" s="3" t="n">
+        <v>21.39</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -41982,6 +42315,9 @@
       <c r="DQ111" s="3" t="n">
         <v>21.9</v>
       </c>
+      <c r="DR111" s="3" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -42353,6 +42689,9 @@
       <c r="DQ112" s="3" t="n">
         <v>23.8</v>
       </c>
+      <c r="DR112" s="3" t="n">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -42724,6 +43063,9 @@
       <c r="DQ113" s="3" t="n">
         <v>22.55</v>
       </c>
+      <c r="DR113" s="3" t="n">
+        <v>22.55</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -43095,6 +43437,9 @@
       <c r="DQ114" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR114" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -43466,6 +43811,9 @@
       <c r="DQ115" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR115" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -43837,6 +44185,9 @@
       <c r="DQ116" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DR116" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -44208,6 +44559,9 @@
       <c r="DQ117" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR117" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -44579,6 +44933,9 @@
       <c r="DQ118" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DR118" s="3" t="n">
+        <v>21.8</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -44950,6 +45307,9 @@
       <c r="DQ119" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR119" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -45321,6 +45681,9 @@
       <c r="DQ120" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR120" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -45692,6 +46055,9 @@
       <c r="DQ121" s="3" t="n">
         <v>21.55</v>
       </c>
+      <c r="DR121" s="3" t="n">
+        <v>21.55</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -46063,6 +46429,9 @@
       <c r="DQ122" s="3" t="n">
         <v>21.99</v>
       </c>
+      <c r="DR122" s="3" t="n">
+        <v>21.99</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -46434,6 +46803,9 @@
       <c r="DQ123" s="3" t="n">
         <v>21.69</v>
       </c>
+      <c r="DR123" s="3" t="n">
+        <v>21.69</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -46805,6 +47177,9 @@
       <c r="DQ124" s="3" t="n">
         <v>22.4</v>
       </c>
+      <c r="DR124" s="3" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -47176,6 +47551,9 @@
       <c r="DQ125" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DR125" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -47547,6 +47925,9 @@
       <c r="DQ126" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DR126" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -47918,6 +48299,9 @@
       <c r="DQ127" s="3" t="n">
         <v>22.09</v>
       </c>
+      <c r="DR127" s="3" t="n">
+        <v>22.09</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -48289,6 +48673,9 @@
       <c r="DQ128" s="3" t="n">
         <v>22.2</v>
       </c>
+      <c r="DR128" s="3" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -48660,6 +49047,9 @@
       <c r="DQ129" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DR129" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -49031,6 +49421,9 @@
       <c r="DQ130" s="3" t="n">
         <v>23.5</v>
       </c>
+      <c r="DR130" s="3" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -49402,6 +49795,9 @@
       <c r="DQ131" s="3" t="n">
         <v>22</v>
       </c>
+      <c r="DR131" s="3" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -49773,6 +50169,9 @@
       <c r="DQ132" s="3" t="n">
         <v>22.19</v>
       </c>
+      <c r="DR132" s="3" t="n">
+        <v>22.19</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -50144,6 +50543,9 @@
       <c r="DQ133" s="3" t="n">
         <v>22.6</v>
       </c>
+      <c r="DR133" s="3" t="n">
+        <v>22.6</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -50515,6 +50917,9 @@
       <c r="DQ134" s="3" t="n">
         <v>23.4</v>
       </c>
+      <c r="DR134" s="3" t="n">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -50886,6 +51291,9 @@
       <c r="DQ135" s="3" t="n">
         <v>22.5</v>
       </c>
+      <c r="DR135" s="3" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="i